<commit_message>
feat(studio): seating room, simpler 2D plan and size list
The living area becomes a seating room: the sofa, a table in front of
it and two flat-pack chairs facing it from the glass. The chairs stand
where the bed drawer pulled out, so the bed now stores under its
lift-up deck. The 2D section is titled 2D only; its plan is redrawn as
plain outlines (one shape per piece, no carcass detail or zone
dimensions) and the checks table gives way to six sizes from
render/plan.json and one line saying every layout check passes.

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01KRyNxX68L5feJKbJnBKRyV
</commit_message>
<xml_diff>
--- a/public/designs/studio/data/bom.xlsx
+++ b/public/designs/studio/data/bom.xlsx
@@ -491,10 +491,10 @@
         </is>
       </c>
       <c r="B7" t="n">
-        <v>1175440</v>
+        <v>1175980</v>
       </c>
       <c r="C7" t="n">
-        <v>3526320</v>
+        <v>3527940</v>
       </c>
     </row>
     <row r="8">
@@ -634,10 +634,10 @@
         </is>
       </c>
       <c r="B18" t="n">
-        <v>202751</v>
+        <v>196751</v>
       </c>
       <c r="C18" t="n">
-        <v>608253</v>
+        <v>590253</v>
       </c>
     </row>
     <row r="19">
@@ -736,10 +736,10 @@
         </is>
       </c>
       <c r="B26" t="n">
-        <v>2003820</v>
+        <v>2003001</v>
       </c>
       <c r="C26" t="n">
-        <v>6739859</v>
+        <v>6737402</v>
       </c>
     </row>
     <row r="27">
@@ -749,10 +749,10 @@
         </is>
       </c>
       <c r="B27" t="n">
-        <v>15362617</v>
+        <v>15356338</v>
       </c>
       <c r="C27" t="n">
-        <v>51672250</v>
+        <v>51653413</v>
       </c>
     </row>
     <row r="29">
@@ -763,7 +763,7 @@
       </c>
       <c r="B29" t="inlineStr"/>
       <c r="C29" t="n">
-        <v>35010</v>
+        <v>34998</v>
       </c>
     </row>
   </sheetData>
@@ -777,7 +777,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:K138"/>
+  <dimension ref="A1:K137"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -1063,7 +1063,7 @@
         </is>
       </c>
       <c r="E6" t="n">
-        <v>92.40000000000001</v>
+        <v>93.3</v>
       </c>
       <c r="F6" t="inlineStr">
         <is>
@@ -1084,7 +1084,7 @@
         </is>
       </c>
       <c r="J6" t="n">
-        <v>55440</v>
+        <v>55980</v>
       </c>
       <c r="K6" t="inlineStr">
         <is>
@@ -3517,19 +3517,19 @@
       </c>
       <c r="D56" t="inlineStr">
         <is>
-          <t>Castors 50 mm for the drawer</t>
+          <t>Gas struts + lift-up hinges for the deck panels</t>
         </is>
       </c>
       <c r="E56" t="n">
-        <v>4</v>
+        <v>2</v>
       </c>
       <c r="F56" t="inlineStr">
         <is>
-          <t>each</t>
+          <t>set</t>
         </is>
       </c>
       <c r="G56" t="n">
-        <v>1500</v>
+        <v>12000</v>
       </c>
       <c r="H56" t="inlineStr">
         <is>
@@ -3542,14 +3542,14 @@
         </is>
       </c>
       <c r="J56" t="n">
-        <v>6000</v>
+        <v>24000</v>
       </c>
       <c r="K56" t="inlineStr"/>
     </row>
     <row r="57">
       <c r="A57" t="inlineStr">
         <is>
-          <t>K4</t>
+          <t>K5</t>
         </is>
       </c>
       <c r="B57" t="inlineStr">
@@ -3564,11 +3564,11 @@
       </c>
       <c r="D57" t="inlineStr">
         <is>
-          <t>Gas struts + lift-up hinges for the deck panels</t>
+          <t>Coat hooks, hanging rail by the door and a folding luggage rack</t>
         </is>
       </c>
       <c r="E57" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="F57" t="inlineStr">
         <is>
@@ -3576,7 +3576,7 @@
         </is>
       </c>
       <c r="G57" t="n">
-        <v>12000</v>
+        <v>8000</v>
       </c>
       <c r="H57" t="inlineStr">
         <is>
@@ -3589,29 +3589,29 @@
         </is>
       </c>
       <c r="J57" t="n">
-        <v>24000</v>
+        <v>8000</v>
       </c>
       <c r="K57" t="inlineStr"/>
     </row>
     <row r="58">
       <c r="A58" t="inlineStr">
         <is>
-          <t>K5</t>
+          <t>K6</t>
         </is>
       </c>
       <c r="B58" t="inlineStr">
         <is>
-          <t>hardware</t>
+          <t>furnishing</t>
         </is>
       </c>
       <c r="C58" t="inlineStr">
         <is>
-          <t>carpentry</t>
+          <t>furnishing</t>
         </is>
       </c>
       <c r="D58" t="inlineStr">
         <is>
-          <t>Coat hooks, hanging rail by the door and a folding luggage rack</t>
+          <t>Compact two-seat sofa about 1150 x 850, washable covers</t>
         </is>
       </c>
       <c r="E58" t="n">
@@ -3619,11 +3619,11 @@
       </c>
       <c r="F58" t="inlineStr">
         <is>
-          <t>set</t>
+          <t>each</t>
         </is>
       </c>
       <c r="G58" t="n">
-        <v>8000</v>
+        <v>450000</v>
       </c>
       <c r="H58" t="inlineStr">
         <is>
@@ -3636,9 +3636,13 @@
         </is>
       </c>
       <c r="J58" t="n">
-        <v>8000</v>
-      </c>
-      <c r="K58" t="inlineStr"/>
+        <v>450000</v>
+      </c>
+      <c r="K58" t="inlineStr">
+        <is>
+          <t>compact two-seat sofa, washable covers</t>
+        </is>
+      </c>
     </row>
     <row r="59">
       <c r="A59" t="inlineStr">
@@ -3658,7 +3662,7 @@
       </c>
       <c r="D59" t="inlineStr">
         <is>
-          <t>Compact two-seat sofa about 1150 x 850, washable covers</t>
+          <t>Blackout curtain + track for the 3 m slider</t>
         </is>
       </c>
       <c r="E59" t="n">
@@ -3666,11 +3670,11 @@
       </c>
       <c r="F59" t="inlineStr">
         <is>
-          <t>each</t>
+          <t>set</t>
         </is>
       </c>
       <c r="G59" t="n">
-        <v>450000</v>
+        <v>60000</v>
       </c>
       <c r="H59" t="inlineStr">
         <is>
@@ -3683,13 +3687,9 @@
         </is>
       </c>
       <c r="J59" t="n">
-        <v>450000</v>
-      </c>
-      <c r="K59" t="inlineStr">
-        <is>
-          <t>compact two-seat sofa, washable covers</t>
-        </is>
-      </c>
+        <v>60000</v>
+      </c>
+      <c r="K59" t="inlineStr"/>
     </row>
     <row r="60">
       <c r="A60" t="inlineStr">
@@ -3699,17 +3699,17 @@
       </c>
       <c r="B60" t="inlineStr">
         <is>
-          <t>furnishing</t>
+          <t>glazing</t>
         </is>
       </c>
       <c r="C60" t="inlineStr">
         <is>
-          <t>furnishing</t>
+          <t>glazier</t>
         </is>
       </c>
       <c r="D60" t="inlineStr">
         <is>
-          <t>Blackout curtain + track for the 3 m slider</t>
+          <t>Insect screens: slider (sliding), W1, vents</t>
         </is>
       </c>
       <c r="E60" t="n">
@@ -3721,7 +3721,7 @@
         </is>
       </c>
       <c r="G60" t="n">
-        <v>60000</v>
+        <v>90000</v>
       </c>
       <c r="H60" t="inlineStr">
         <is>
@@ -3734,29 +3734,29 @@
         </is>
       </c>
       <c r="J60" t="n">
-        <v>60000</v>
+        <v>90000</v>
       </c>
       <c r="K60" t="inlineStr"/>
     </row>
     <row r="61">
       <c r="A61" t="inlineStr">
         <is>
-          <t>K6</t>
+          <t>K8</t>
         </is>
       </c>
       <c r="B61" t="inlineStr">
         <is>
-          <t>glazing</t>
+          <t>electrical</t>
         </is>
       </c>
       <c r="C61" t="inlineStr">
         <is>
-          <t>glazier</t>
+          <t>electrical</t>
         </is>
       </c>
       <c r="D61" t="inlineStr">
         <is>
-          <t>Insect screens: slider (sliding), W1, vents</t>
+          <t>Unit board on the back wall by the galley</t>
         </is>
       </c>
       <c r="E61" t="n">
@@ -3764,11 +3764,11 @@
       </c>
       <c r="F61" t="inlineStr">
         <is>
-          <t>set</t>
+          <t>each</t>
         </is>
       </c>
       <c r="G61" t="n">
-        <v>90000</v>
+        <v>45000</v>
       </c>
       <c r="H61" t="inlineStr">
         <is>
@@ -3781,9 +3781,13 @@
         </is>
       </c>
       <c r="J61" t="n">
-        <v>90000</v>
-      </c>
-      <c r="K61" t="inlineStr"/>
+        <v>45000</v>
+      </c>
+      <c r="K61" t="inlineStr">
+        <is>
+          <t>enclosure, 12 ways</t>
+        </is>
+      </c>
     </row>
     <row r="62">
       <c r="A62" t="inlineStr">
@@ -3803,7 +3807,7 @@
       </c>
       <c r="D62" t="inlineStr">
         <is>
-          <t>Unit board on the back wall by the galley</t>
+          <t>Ceiling light, bed</t>
         </is>
       </c>
       <c r="E62" t="n">
@@ -3815,7 +3819,7 @@
         </is>
       </c>
       <c r="G62" t="n">
-        <v>45000</v>
+        <v>15000</v>
       </c>
       <c r="H62" t="inlineStr">
         <is>
@@ -3828,13 +3832,9 @@
         </is>
       </c>
       <c r="J62" t="n">
-        <v>45000</v>
-      </c>
-      <c r="K62" t="inlineStr">
-        <is>
-          <t>enclosure, 12 ways</t>
-        </is>
-      </c>
+        <v>15000</v>
+      </c>
+      <c r="K62" t="inlineStr"/>
     </row>
     <row r="63">
       <c r="A63" t="inlineStr">
@@ -3854,7 +3854,7 @@
       </c>
       <c r="D63" t="inlineStr">
         <is>
-          <t>Ceiling light, bed</t>
+          <t>Ceiling light, living</t>
         </is>
       </c>
       <c r="E63" t="n">
@@ -3901,7 +3901,7 @@
       </c>
       <c r="D64" t="inlineStr">
         <is>
-          <t>Ceiling light, living</t>
+          <t>Ceiling light, galley</t>
         </is>
       </c>
       <c r="E64" t="n">
@@ -3948,7 +3948,7 @@
       </c>
       <c r="D65" t="inlineStr">
         <is>
-          <t>Ceiling light, galley</t>
+          <t>Bathroom light IP65</t>
         </is>
       </c>
       <c r="E65" t="n">
@@ -3995,7 +3995,7 @@
       </c>
       <c r="D66" t="inlineStr">
         <is>
-          <t>Bathroom light IP65</t>
+          <t>Reading light 1</t>
         </is>
       </c>
       <c r="E66" t="n">
@@ -4042,7 +4042,7 @@
       </c>
       <c r="D67" t="inlineStr">
         <is>
-          <t>Reading light 1</t>
+          <t>Reading light 2</t>
         </is>
       </c>
       <c r="E67" t="n">
@@ -4089,7 +4089,7 @@
       </c>
       <c r="D68" t="inlineStr">
         <is>
-          <t>Reading light 2</t>
+          <t>Under-cabinet LED strip</t>
         </is>
       </c>
       <c r="E68" t="n">
@@ -4136,7 +4136,7 @@
       </c>
       <c r="D69" t="inlineStr">
         <is>
-          <t>Under-cabinet LED strip</t>
+          <t>Deck light IP65</t>
         </is>
       </c>
       <c r="E69" t="n">
@@ -4183,7 +4183,7 @@
       </c>
       <c r="D70" t="inlineStr">
         <is>
-          <t>Deck light IP65</t>
+          <t>Roof terrace lights IP65 (x2)</t>
         </is>
       </c>
       <c r="E70" t="n">
@@ -4230,7 +4230,7 @@
       </c>
       <c r="D71" t="inlineStr">
         <is>
-          <t>Roof terrace lights IP65 (x2)</t>
+          <t>Stair light IP65</t>
         </is>
       </c>
       <c r="E71" t="n">
@@ -4277,7 +4277,7 @@
       </c>
       <c r="D72" t="inlineStr">
         <is>
-          <t>Stair light IP65</t>
+          <t>Entry: living + kitchen + deck</t>
         </is>
       </c>
       <c r="E72" t="n">
@@ -4289,7 +4289,7 @@
         </is>
       </c>
       <c r="G72" t="n">
-        <v>15000</v>
+        <v>3500</v>
       </c>
       <c r="H72" t="inlineStr">
         <is>
@@ -4302,7 +4302,7 @@
         </is>
       </c>
       <c r="J72" t="n">
-        <v>15000</v>
+        <v>3500</v>
       </c>
       <c r="K72" t="inlineStr"/>
     </row>
@@ -4324,7 +4324,7 @@
       </c>
       <c r="D73" t="inlineStr">
         <is>
-          <t>Entry: living + kitchen + deck</t>
+          <t>Bed: ceiling light (2-way)</t>
         </is>
       </c>
       <c r="E73" t="n">
@@ -4371,7 +4371,7 @@
       </c>
       <c r="D74" t="inlineStr">
         <is>
-          <t>Bed: ceiling light (2-way)</t>
+          <t>Bathroom light + fan (outside)</t>
         </is>
       </c>
       <c r="E74" t="n">
@@ -4418,7 +4418,7 @@
       </c>
       <c r="D75" t="inlineStr">
         <is>
-          <t>Bathroom light + fan (outside)</t>
+          <t>Roof and stair lights (IP65, stair foot)</t>
         </is>
       </c>
       <c r="E75" t="n">
@@ -4465,7 +4465,7 @@
       </c>
       <c r="D76" t="inlineStr">
         <is>
-          <t>Roof and stair lights (IP65, stair foot)</t>
+          <t>Bedside socket + USB-C 1</t>
         </is>
       </c>
       <c r="E76" t="n">
@@ -4477,7 +4477,7 @@
         </is>
       </c>
       <c r="G76" t="n">
-        <v>3500</v>
+        <v>15000</v>
       </c>
       <c r="H76" t="inlineStr">
         <is>
@@ -4490,7 +4490,7 @@
         </is>
       </c>
       <c r="J76" t="n">
-        <v>3500</v>
+        <v>15000</v>
       </c>
       <c r="K76" t="inlineStr"/>
     </row>
@@ -4512,7 +4512,7 @@
       </c>
       <c r="D77" t="inlineStr">
         <is>
-          <t>Bedside socket + USB-C 1</t>
+          <t>Bedside socket + USB-C 2</t>
         </is>
       </c>
       <c r="E77" t="n">
@@ -4559,7 +4559,7 @@
       </c>
       <c r="D78" t="inlineStr">
         <is>
-          <t>Bedside socket + USB-C 2</t>
+          <t>Socket by the sofa</t>
         </is>
       </c>
       <c r="E78" t="n">
@@ -4571,7 +4571,7 @@
         </is>
       </c>
       <c r="G78" t="n">
-        <v>15000</v>
+        <v>5000</v>
       </c>
       <c r="H78" t="inlineStr">
         <is>
@@ -4584,7 +4584,7 @@
         </is>
       </c>
       <c r="J78" t="n">
-        <v>15000</v>
+        <v>5000</v>
       </c>
       <c r="K78" t="inlineStr"/>
     </row>
@@ -4606,7 +4606,7 @@
       </c>
       <c r="D79" t="inlineStr">
         <is>
-          <t>Socket by the sofa</t>
+          <t>Socket, living (front strip)</t>
         </is>
       </c>
       <c r="E79" t="n">
@@ -4653,7 +4653,7 @@
       </c>
       <c r="D80" t="inlineStr">
         <is>
-          <t>Socket, living (front strip)</t>
+          <t>Deck socket IP66</t>
         </is>
       </c>
       <c r="E80" t="n">
@@ -4700,7 +4700,7 @@
       </c>
       <c r="D81" t="inlineStr">
         <is>
-          <t>Deck socket IP66</t>
+          <t>Worktop socket 1 (double)</t>
         </is>
       </c>
       <c r="E81" t="n">
@@ -4747,7 +4747,7 @@
       </c>
       <c r="D82" t="inlineStr">
         <is>
-          <t>Worktop socket 1 (double)</t>
+          <t>Worktop socket 2 (double, back wall)</t>
         </is>
       </c>
       <c r="E82" t="n">
@@ -4794,7 +4794,7 @@
       </c>
       <c r="D83" t="inlineStr">
         <is>
-          <t>Worktop socket 2 (double, back wall)</t>
+          <t>Fridge socket</t>
         </is>
       </c>
       <c r="E83" t="n">
@@ -4841,7 +4841,7 @@
       </c>
       <c r="D84" t="inlineStr">
         <is>
-          <t>Fridge socket</t>
+          <t>Hob connection unit</t>
         </is>
       </c>
       <c r="E84" t="n">
@@ -4853,7 +4853,7 @@
         </is>
       </c>
       <c r="G84" t="n">
-        <v>5000</v>
+        <v>9000</v>
       </c>
       <c r="H84" t="inlineStr">
         <is>
@@ -4866,7 +4866,7 @@
         </is>
       </c>
       <c r="J84" t="n">
-        <v>5000</v>
+        <v>9000</v>
       </c>
       <c r="K84" t="inlineStr"/>
     </row>
@@ -4888,7 +4888,7 @@
       </c>
       <c r="D85" t="inlineStr">
         <is>
-          <t>Hob connection unit</t>
+          <t>Heater DP switch + timer</t>
         </is>
       </c>
       <c r="E85" t="n">
@@ -4935,7 +4935,7 @@
       </c>
       <c r="D86" t="inlineStr">
         <is>
-          <t>Heater DP switch + timer</t>
+          <t>Bathroom extract 100 mm (in W1 panel)</t>
         </is>
       </c>
       <c r="E86" t="n">
@@ -4947,7 +4947,7 @@
         </is>
       </c>
       <c r="G86" t="n">
-        <v>9000</v>
+        <v>35000</v>
       </c>
       <c r="H86" t="inlineStr">
         <is>
@@ -4960,7 +4960,7 @@
         </is>
       </c>
       <c r="J86" t="n">
-        <v>9000</v>
+        <v>35000</v>
       </c>
       <c r="K86" t="inlineStr"/>
     </row>
@@ -4982,7 +4982,7 @@
       </c>
       <c r="D87" t="inlineStr">
         <is>
-          <t>Bathroom extract 100 mm (in W1 panel)</t>
+          <t>Wall fan</t>
         </is>
       </c>
       <c r="E87" t="n">
@@ -5029,7 +5029,7 @@
       </c>
       <c r="D88" t="inlineStr">
         <is>
-          <t>Wall fan</t>
+          <t>AC provision: isolator</t>
         </is>
       </c>
       <c r="E88" t="n">
@@ -5041,7 +5041,7 @@
         </is>
       </c>
       <c r="G88" t="n">
-        <v>35000</v>
+        <v>9000</v>
       </c>
       <c r="H88" t="inlineStr">
         <is>
@@ -5054,7 +5054,7 @@
         </is>
       </c>
       <c r="J88" t="n">
-        <v>35000</v>
+        <v>9000</v>
       </c>
       <c r="K88" t="inlineStr"/>
     </row>
@@ -5076,19 +5076,19 @@
       </c>
       <c r="D89" t="inlineStr">
         <is>
-          <t>AC provision: isolator</t>
+          <t>Cable 1.5 mm2 T+E/singles in conduit, Lighting (incl. bathroom IP65, deck, roof, stair)</t>
         </is>
       </c>
       <c r="E89" t="n">
-        <v>1</v>
+        <v>89</v>
       </c>
       <c r="F89" t="inlineStr">
         <is>
-          <t>each</t>
+          <t>m</t>
         </is>
       </c>
       <c r="G89" t="n">
-        <v>9000</v>
+        <v>500</v>
       </c>
       <c r="H89" t="inlineStr">
         <is>
@@ -5101,9 +5101,13 @@
         </is>
       </c>
       <c r="J89" t="n">
-        <v>9000</v>
-      </c>
-      <c r="K89" t="inlineStr"/>
+        <v>44500</v>
+      </c>
+      <c r="K89" t="inlineStr">
+        <is>
+          <t>per m</t>
+        </is>
+      </c>
     </row>
     <row r="90">
       <c r="A90" t="inlineStr">
@@ -5123,11 +5127,11 @@
       </c>
       <c r="D90" t="inlineStr">
         <is>
-          <t>Cable 1.5 mm2 T+E/singles in conduit, Lighting (incl. bathroom IP65, deck, roof, stair)</t>
+          <t>Cable 2.5 mm2 T+E/singles in conduit, Sockets: bedside USB, living, deck</t>
         </is>
       </c>
       <c r="E90" t="n">
-        <v>89</v>
+        <v>29</v>
       </c>
       <c r="F90" t="inlineStr">
         <is>
@@ -5135,7 +5139,7 @@
         </is>
       </c>
       <c r="G90" t="n">
-        <v>500</v>
+        <v>750</v>
       </c>
       <c r="H90" t="inlineStr">
         <is>
@@ -5148,7 +5152,7 @@
         </is>
       </c>
       <c r="J90" t="n">
-        <v>44500</v>
+        <v>21750</v>
       </c>
       <c r="K90" t="inlineStr">
         <is>
@@ -5174,11 +5178,11 @@
       </c>
       <c r="D91" t="inlineStr">
         <is>
-          <t>Cable 2.5 mm2 T+E/singles in conduit, Sockets: bedside USB, living, deck</t>
+          <t>Cable 2.5 mm2 T+E/singles in conduit, Kitchen sockets and fridge</t>
         </is>
       </c>
       <c r="E91" t="n">
-        <v>29</v>
+        <v>13</v>
       </c>
       <c r="F91" t="inlineStr">
         <is>
@@ -5199,7 +5203,7 @@
         </is>
       </c>
       <c r="J91" t="n">
-        <v>21750</v>
+        <v>9750</v>
       </c>
       <c r="K91" t="inlineStr">
         <is>
@@ -5225,11 +5229,11 @@
       </c>
       <c r="D92" t="inlineStr">
         <is>
-          <t>Cable 2.5 mm2 T+E/singles in conduit, Kitchen sockets and fridge</t>
+          <t>Cable 4.0 mm2 T+E/singles in conduit, Induction hob</t>
         </is>
       </c>
       <c r="E92" t="n">
-        <v>13</v>
+        <v>8</v>
       </c>
       <c r="F92" t="inlineStr">
         <is>
@@ -5237,7 +5241,7 @@
         </is>
       </c>
       <c r="G92" t="n">
-        <v>750</v>
+        <v>1200</v>
       </c>
       <c r="H92" t="inlineStr">
         <is>
@@ -5250,7 +5254,7 @@
         </is>
       </c>
       <c r="J92" t="n">
-        <v>9750</v>
+        <v>9600</v>
       </c>
       <c r="K92" t="inlineStr">
         <is>
@@ -5276,11 +5280,11 @@
       </c>
       <c r="D93" t="inlineStr">
         <is>
-          <t>Cable 4.0 mm2 T+E/singles in conduit, Induction hob</t>
+          <t>Cable 2.5 mm2 T+E/singles in conduit, 80 L water heater</t>
         </is>
       </c>
       <c r="E93" t="n">
-        <v>8</v>
+        <v>7</v>
       </c>
       <c r="F93" t="inlineStr">
         <is>
@@ -5288,7 +5292,7 @@
         </is>
       </c>
       <c r="G93" t="n">
-        <v>1200</v>
+        <v>750</v>
       </c>
       <c r="H93" t="inlineStr">
         <is>
@@ -5301,7 +5305,7 @@
         </is>
       </c>
       <c r="J93" t="n">
-        <v>9600</v>
+        <v>5250</v>
       </c>
       <c r="K93" t="inlineStr">
         <is>
@@ -5327,11 +5331,11 @@
       </c>
       <c r="D94" t="inlineStr">
         <is>
-          <t>Cable 2.5 mm2 T+E/singles in conduit, 80 L water heater</t>
+          <t>Cable 1.5 mm2 T+E/singles in conduit, Extract fan and wall fan</t>
         </is>
       </c>
       <c r="E94" t="n">
-        <v>7</v>
+        <v>12</v>
       </c>
       <c r="F94" t="inlineStr">
         <is>
@@ -5339,7 +5343,7 @@
         </is>
       </c>
       <c r="G94" t="n">
-        <v>750</v>
+        <v>500</v>
       </c>
       <c r="H94" t="inlineStr">
         <is>
@@ -5352,7 +5356,7 @@
         </is>
       </c>
       <c r="J94" t="n">
-        <v>5250</v>
+        <v>6000</v>
       </c>
       <c r="K94" t="inlineStr">
         <is>
@@ -5378,11 +5382,11 @@
       </c>
       <c r="D95" t="inlineStr">
         <is>
-          <t>Cable 1.5 mm2 T+E/singles in conduit, Extract fan and wall fan</t>
+          <t>Cable 2.5 mm2 T+E/singles in conduit, AC provision</t>
         </is>
       </c>
       <c r="E95" t="n">
-        <v>12</v>
+        <v>7</v>
       </c>
       <c r="F95" t="inlineStr">
         <is>
@@ -5390,7 +5394,7 @@
         </is>
       </c>
       <c r="G95" t="n">
-        <v>500</v>
+        <v>750</v>
       </c>
       <c r="H95" t="inlineStr">
         <is>
@@ -5403,7 +5407,7 @@
         </is>
       </c>
       <c r="J95" t="n">
-        <v>6000</v>
+        <v>5250</v>
       </c>
       <c r="K95" t="inlineStr">
         <is>
@@ -5429,11 +5433,11 @@
       </c>
       <c r="D96" t="inlineStr">
         <is>
-          <t>Cable 2.5 mm2 T+E/singles in conduit, AC provision</t>
+          <t>PVC conduit 20 mm + boxes</t>
         </is>
       </c>
       <c r="E96" t="n">
-        <v>7</v>
+        <v>60</v>
       </c>
       <c r="F96" t="inlineStr">
         <is>
@@ -5441,7 +5445,7 @@
         </is>
       </c>
       <c r="G96" t="n">
-        <v>750</v>
+        <v>600</v>
       </c>
       <c r="H96" t="inlineStr">
         <is>
@@ -5454,7 +5458,7 @@
         </is>
       </c>
       <c r="J96" t="n">
-        <v>5250</v>
+        <v>36000</v>
       </c>
       <c r="K96" t="inlineStr">
         <is>
@@ -5480,19 +5484,19 @@
       </c>
       <c r="D97" t="inlineStr">
         <is>
-          <t>PVC conduit 20 mm + boxes</t>
+          <t>Surge protection device type 2</t>
         </is>
       </c>
       <c r="E97" t="n">
-        <v>60</v>
+        <v>1</v>
       </c>
       <c r="F97" t="inlineStr">
         <is>
-          <t>m</t>
+          <t>each</t>
         </is>
       </c>
       <c r="G97" t="n">
-        <v>600</v>
+        <v>60000</v>
       </c>
       <c r="H97" t="inlineStr">
         <is>
@@ -5505,13 +5509,9 @@
         </is>
       </c>
       <c r="J97" t="n">
-        <v>36000</v>
-      </c>
-      <c r="K97" t="inlineStr">
-        <is>
-          <t>per m</t>
-        </is>
-      </c>
+        <v>60000</v>
+      </c>
+      <c r="K97" t="inlineStr"/>
     </row>
     <row r="98">
       <c r="A98" t="inlineStr">
@@ -5531,7 +5531,7 @@
       </c>
       <c r="D98" t="inlineStr">
         <is>
-          <t>Surge protection device type 2</t>
+          <t>RCD 40 A 30 mA type A (or RCBOs)</t>
         </is>
       </c>
       <c r="E98" t="n">
@@ -5543,7 +5543,7 @@
         </is>
       </c>
       <c r="G98" t="n">
-        <v>60000</v>
+        <v>45000</v>
       </c>
       <c r="H98" t="inlineStr">
         <is>
@@ -5556,7 +5556,7 @@
         </is>
       </c>
       <c r="J98" t="n">
-        <v>60000</v>
+        <v>45000</v>
       </c>
       <c r="K98" t="inlineStr"/>
     </row>
@@ -5578,11 +5578,11 @@
       </c>
       <c r="D99" t="inlineStr">
         <is>
-          <t>RCD 40 A 30 mA type A (or RCBOs)</t>
+          <t>MCBs (B6 x2, B16 x5, B20 x1)</t>
         </is>
       </c>
       <c r="E99" t="n">
-        <v>1</v>
+        <v>8</v>
       </c>
       <c r="F99" t="inlineStr">
         <is>
@@ -5590,7 +5590,7 @@
         </is>
       </c>
       <c r="G99" t="n">
-        <v>45000</v>
+        <v>6000</v>
       </c>
       <c r="H99" t="inlineStr">
         <is>
@@ -5603,7 +5603,7 @@
         </is>
       </c>
       <c r="J99" t="n">
-        <v>45000</v>
+        <v>48000</v>
       </c>
       <c r="K99" t="inlineStr"/>
     </row>
@@ -5625,19 +5625,19 @@
       </c>
       <c r="D100" t="inlineStr">
         <is>
-          <t>MCBs (B6 x2, B16 x5, B20 x1)</t>
+          <t>Main switch 40 A DP + check meter (DIN kWh)</t>
         </is>
       </c>
       <c r="E100" t="n">
-        <v>8</v>
+        <v>1</v>
       </c>
       <c r="F100" t="inlineStr">
         <is>
-          <t>each</t>
+          <t>set</t>
         </is>
       </c>
       <c r="G100" t="n">
-        <v>6000</v>
+        <v>40000</v>
       </c>
       <c r="H100" t="inlineStr">
         <is>
@@ -5650,7 +5650,7 @@
         </is>
       </c>
       <c r="J100" t="n">
-        <v>48000</v>
+        <v>40000</v>
       </c>
       <c r="K100" t="inlineStr"/>
     </row>
@@ -5672,7 +5672,7 @@
       </c>
       <c r="D101" t="inlineStr">
         <is>
-          <t>Main switch 40 A DP + check meter (DIN kWh)</t>
+          <t>Earth rod 1.5 m copper-bonded + clamp + inspection pit</t>
         </is>
       </c>
       <c r="E101" t="n">
@@ -5680,11 +5680,11 @@
       </c>
       <c r="F101" t="inlineStr">
         <is>
-          <t>set</t>
+          <t>each</t>
         </is>
       </c>
       <c r="G101" t="n">
-        <v>40000</v>
+        <v>35000</v>
       </c>
       <c r="H101" t="inlineStr">
         <is>
@@ -5697,7 +5697,7 @@
         </is>
       </c>
       <c r="J101" t="n">
-        <v>40000</v>
+        <v>35000</v>
       </c>
       <c r="K101" t="inlineStr"/>
     </row>
@@ -5709,7 +5709,7 @@
       </c>
       <c r="B102" t="inlineStr">
         <is>
-          <t>electrical</t>
+          <t>safety</t>
         </is>
       </c>
       <c r="C102" t="inlineStr">
@@ -5719,11 +5719,11 @@
       </c>
       <c r="D102" t="inlineStr">
         <is>
-          <t>Earth rod 1.5 m copper-bonded + clamp + inspection pit</t>
+          <t>Smoke alarm (10-year) + heat alarm (kitchen)</t>
         </is>
       </c>
       <c r="E102" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="F102" t="inlineStr">
         <is>
@@ -5731,7 +5731,7 @@
         </is>
       </c>
       <c r="G102" t="n">
-        <v>35000</v>
+        <v>20000</v>
       </c>
       <c r="H102" t="inlineStr">
         <is>
@@ -5744,7 +5744,7 @@
         </is>
       </c>
       <c r="J102" t="n">
-        <v>35000</v>
+        <v>40000</v>
       </c>
       <c r="K102" t="inlineStr"/>
     </row>
@@ -5761,24 +5761,24 @@
       </c>
       <c r="C103" t="inlineStr">
         <is>
-          <t>electrical</t>
+          <t>furnishing</t>
         </is>
       </c>
       <c r="D103" t="inlineStr">
         <is>
-          <t>Smoke alarm (10-year) + heat alarm (kitchen)</t>
+          <t>Fire extinguisher 2 kg ABC + fire blanket</t>
         </is>
       </c>
       <c r="E103" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="F103" t="inlineStr">
         <is>
-          <t>each</t>
+          <t>set</t>
         </is>
       </c>
       <c r="G103" t="n">
-        <v>20000</v>
+        <v>55000</v>
       </c>
       <c r="H103" t="inlineStr">
         <is>
@@ -5791,41 +5791,41 @@
         </is>
       </c>
       <c r="J103" t="n">
-        <v>40000</v>
+        <v>55000</v>
       </c>
       <c r="K103" t="inlineStr"/>
     </row>
     <row r="104">
       <c r="A104" t="inlineStr">
         <is>
-          <t>K8</t>
+          <t>K9</t>
         </is>
       </c>
       <c r="B104" t="inlineStr">
         <is>
-          <t>safety</t>
+          <t>plumbing</t>
         </is>
       </c>
       <c r="C104" t="inlineStr">
         <is>
-          <t>furnishing</t>
+          <t>plumbing</t>
         </is>
       </c>
       <c r="D104" t="inlineStr">
         <is>
-          <t>Fire extinguisher 2 kg ABC + fire blanket</t>
+          <t>PPR PN20 pipe DN20</t>
         </is>
       </c>
       <c r="E104" t="n">
-        <v>1</v>
+        <v>8.800000000000001</v>
       </c>
       <c r="F104" t="inlineStr">
         <is>
-          <t>set</t>
+          <t>m</t>
         </is>
       </c>
       <c r="G104" t="n">
-        <v>55000</v>
+        <v>2000</v>
       </c>
       <c r="H104" t="inlineStr">
         <is>
@@ -5838,9 +5838,13 @@
         </is>
       </c>
       <c r="J104" t="n">
-        <v>55000</v>
-      </c>
-      <c r="K104" t="inlineStr"/>
+        <v>17600</v>
+      </c>
+      <c r="K104" t="inlineStr">
+        <is>
+          <t>per m</t>
+        </is>
+      </c>
     </row>
     <row r="105">
       <c r="A105" t="inlineStr">
@@ -5860,11 +5864,11 @@
       </c>
       <c r="D105" t="inlineStr">
         <is>
-          <t>PPR PN20 pipe DN20</t>
+          <t>PPR PN20 pipe DN25</t>
         </is>
       </c>
       <c r="E105" t="n">
-        <v>8.800000000000001</v>
+        <v>4.6</v>
       </c>
       <c r="F105" t="inlineStr">
         <is>
@@ -5872,7 +5876,7 @@
         </is>
       </c>
       <c r="G105" t="n">
-        <v>2000</v>
+        <v>2800</v>
       </c>
       <c r="H105" t="inlineStr">
         <is>
@@ -5885,7 +5889,7 @@
         </is>
       </c>
       <c r="J105" t="n">
-        <v>17600</v>
+        <v>12880</v>
       </c>
       <c r="K105" t="inlineStr">
         <is>
@@ -5911,11 +5915,11 @@
       </c>
       <c r="D106" t="inlineStr">
         <is>
-          <t>PPR PN20 pipe DN25</t>
+          <t>PPR PN20 pipe (hot) DN20</t>
         </is>
       </c>
       <c r="E106" t="n">
-        <v>4.6</v>
+        <v>4.5</v>
       </c>
       <c r="F106" t="inlineStr">
         <is>
@@ -5923,7 +5927,7 @@
         </is>
       </c>
       <c r="G106" t="n">
-        <v>2800</v>
+        <v>2000</v>
       </c>
       <c r="H106" t="inlineStr">
         <is>
@@ -5936,7 +5940,7 @@
         </is>
       </c>
       <c r="J106" t="n">
-        <v>12880</v>
+        <v>9000</v>
       </c>
       <c r="K106" t="inlineStr">
         <is>
@@ -5962,11 +5966,11 @@
       </c>
       <c r="D107" t="inlineStr">
         <is>
-          <t>PPR PN20 pipe (hot) DN20</t>
+          <t>uPVC soil pipe DN110</t>
         </is>
       </c>
       <c r="E107" t="n">
-        <v>4.5</v>
+        <v>4.2</v>
       </c>
       <c r="F107" t="inlineStr">
         <is>
@@ -5974,7 +5978,7 @@
         </is>
       </c>
       <c r="G107" t="n">
-        <v>2000</v>
+        <v>7000</v>
       </c>
       <c r="H107" t="inlineStr">
         <is>
@@ -5987,7 +5991,7 @@
         </is>
       </c>
       <c r="J107" t="n">
-        <v>9000</v>
+        <v>29400</v>
       </c>
       <c r="K107" t="inlineStr">
         <is>
@@ -6013,11 +6017,11 @@
       </c>
       <c r="D108" t="inlineStr">
         <is>
-          <t>uPVC soil pipe DN110</t>
+          <t>PPR PN20 pipe (tempered) DN20</t>
         </is>
       </c>
       <c r="E108" t="n">
-        <v>4.2</v>
+        <v>5.5</v>
       </c>
       <c r="F108" t="inlineStr">
         <is>
@@ -6025,7 +6029,7 @@
         </is>
       </c>
       <c r="G108" t="n">
-        <v>7000</v>
+        <v>2000</v>
       </c>
       <c r="H108" t="inlineStr">
         <is>
@@ -6038,7 +6042,7 @@
         </is>
       </c>
       <c r="J108" t="n">
-        <v>29400</v>
+        <v>11000</v>
       </c>
       <c r="K108" t="inlineStr">
         <is>
@@ -6064,11 +6068,11 @@
       </c>
       <c r="D109" t="inlineStr">
         <is>
-          <t>PPR PN20 pipe (tempered) DN20</t>
+          <t>uPVC vent pipe DN75</t>
         </is>
       </c>
       <c r="E109" t="n">
-        <v>5.5</v>
+        <v>7.9</v>
       </c>
       <c r="F109" t="inlineStr">
         <is>
@@ -6076,7 +6080,7 @@
         </is>
       </c>
       <c r="G109" t="n">
-        <v>2000</v>
+        <v>4500</v>
       </c>
       <c r="H109" t="inlineStr">
         <is>
@@ -6089,7 +6093,7 @@
         </is>
       </c>
       <c r="J109" t="n">
-        <v>11000</v>
+        <v>35550</v>
       </c>
       <c r="K109" t="inlineStr">
         <is>
@@ -6115,11 +6119,11 @@
       </c>
       <c r="D110" t="inlineStr">
         <is>
-          <t>uPVC vent pipe DN75</t>
+          <t>uPVC waste pipe DN40</t>
         </is>
       </c>
       <c r="E110" t="n">
-        <v>7.9</v>
+        <v>1.5</v>
       </c>
       <c r="F110" t="inlineStr">
         <is>
@@ -6127,7 +6131,7 @@
         </is>
       </c>
       <c r="G110" t="n">
-        <v>4500</v>
+        <v>2500</v>
       </c>
       <c r="H110" t="inlineStr">
         <is>
@@ -6140,7 +6144,7 @@
         </is>
       </c>
       <c r="J110" t="n">
-        <v>35550</v>
+        <v>3750</v>
       </c>
       <c r="K110" t="inlineStr">
         <is>
@@ -6166,11 +6170,11 @@
       </c>
       <c r="D111" t="inlineStr">
         <is>
-          <t>uPVC waste pipe DN40</t>
+          <t>uPVC waste pipe DN50</t>
         </is>
       </c>
       <c r="E111" t="n">
-        <v>1.5</v>
+        <v>5.7</v>
       </c>
       <c r="F111" t="inlineStr">
         <is>
@@ -6178,7 +6182,7 @@
         </is>
       </c>
       <c r="G111" t="n">
-        <v>2500</v>
+        <v>3000</v>
       </c>
       <c r="H111" t="inlineStr">
         <is>
@@ -6191,7 +6195,7 @@
         </is>
       </c>
       <c r="J111" t="n">
-        <v>3750</v>
+        <v>17100</v>
       </c>
       <c r="K111" t="inlineStr">
         <is>
@@ -6217,19 +6221,19 @@
       </c>
       <c r="D112" t="inlineStr">
         <is>
-          <t>uPVC waste pipe DN50</t>
+          <t>Pipe fittings and clips (allowance)</t>
         </is>
       </c>
       <c r="E112" t="n">
-        <v>5.7</v>
+        <v>1</v>
       </c>
       <c r="F112" t="inlineStr">
         <is>
-          <t>m</t>
+          <t>set</t>
         </is>
       </c>
       <c r="G112" t="n">
-        <v>3000</v>
+        <v>120000</v>
       </c>
       <c r="H112" t="inlineStr">
         <is>
@@ -6242,13 +6246,9 @@
         </is>
       </c>
       <c r="J112" t="n">
-        <v>17100</v>
-      </c>
-      <c r="K112" t="inlineStr">
-        <is>
-          <t>per m</t>
-        </is>
-      </c>
+        <v>120000</v>
+      </c>
+      <c r="K112" t="inlineStr"/>
     </row>
     <row r="113">
       <c r="A113" t="inlineStr">
@@ -6268,7 +6268,7 @@
       </c>
       <c r="D113" t="inlineStr">
         <is>
-          <t>Pipe fittings and clips (allowance)</t>
+          <t>Thermostatic mixing valve (TMV) 41-44 C</t>
         </is>
       </c>
       <c r="E113" t="n">
@@ -6276,11 +6276,11 @@
       </c>
       <c r="F113" t="inlineStr">
         <is>
-          <t>set</t>
+          <t>each</t>
         </is>
       </c>
       <c r="G113" t="n">
-        <v>120000</v>
+        <v>60000</v>
       </c>
       <c r="H113" t="inlineStr">
         <is>
@@ -6293,7 +6293,7 @@
         </is>
       </c>
       <c r="J113" t="n">
-        <v>120000</v>
+        <v>60000</v>
       </c>
       <c r="K113" t="inlineStr"/>
     </row>
@@ -6315,7 +6315,7 @@
       </c>
       <c r="D114" t="inlineStr">
         <is>
-          <t>Thermostatic mixing valve (TMV) 41-44 C</t>
+          <t>Thermostatic shower valve + 6-7 L/min head + rail</t>
         </is>
       </c>
       <c r="E114" t="n">
@@ -6323,11 +6323,11 @@
       </c>
       <c r="F114" t="inlineStr">
         <is>
-          <t>each</t>
+          <t>set</t>
         </is>
       </c>
       <c r="G114" t="n">
-        <v>60000</v>
+        <v>90000</v>
       </c>
       <c r="H114" t="inlineStr">
         <is>
@@ -6340,7 +6340,7 @@
         </is>
       </c>
       <c r="J114" t="n">
-        <v>60000</v>
+        <v>90000</v>
       </c>
       <c r="K114" t="inlineStr"/>
     </row>
@@ -6362,7 +6362,7 @@
       </c>
       <c r="D115" t="inlineStr">
         <is>
-          <t>Thermostatic shower valve + 6-7 L/min head + rail</t>
+          <t>Electric storage water heater 80 L, 2 kW, with T&amp;P valve</t>
         </is>
       </c>
       <c r="E115" t="n">
@@ -6370,11 +6370,11 @@
       </c>
       <c r="F115" t="inlineStr">
         <is>
-          <t>set</t>
+          <t>each</t>
         </is>
       </c>
       <c r="G115" t="n">
-        <v>90000</v>
+        <v>300000</v>
       </c>
       <c r="H115" t="inlineStr">
         <is>
@@ -6387,9 +6387,13 @@
         </is>
       </c>
       <c r="J115" t="n">
-        <v>90000</v>
-      </c>
-      <c r="K115" t="inlineStr"/>
+        <v>300000</v>
+      </c>
+      <c r="K115" t="inlineStr">
+        <is>
+          <t>80 L not found; 50 L listed at RWF 144,000-252,000 (STU-P01, STU-P02)</t>
+        </is>
+      </c>
     </row>
     <row r="116">
       <c r="A116" t="inlineStr">
@@ -6409,11 +6413,11 @@
       </c>
       <c r="D116" t="inlineStr">
         <is>
-          <t>Electric storage water heater 80 L, 2 kW, with T&amp;P valve</t>
+          <t>Angle valves with filters</t>
         </is>
       </c>
       <c r="E116" t="n">
-        <v>1</v>
+        <v>5</v>
       </c>
       <c r="F116" t="inlineStr">
         <is>
@@ -6421,7 +6425,7 @@
         </is>
       </c>
       <c r="G116" t="n">
-        <v>300000</v>
+        <v>6000</v>
       </c>
       <c r="H116" t="inlineStr">
         <is>
@@ -6434,13 +6438,9 @@
         </is>
       </c>
       <c r="J116" t="n">
-        <v>300000</v>
-      </c>
-      <c r="K116" t="inlineStr">
-        <is>
-          <t>80 L not found; 50 L listed at RWF 144,000-252,000 (STU-P01, STU-P02)</t>
-        </is>
-      </c>
+        <v>30000</v>
+      </c>
+      <c r="K116" t="inlineStr"/>
     </row>
     <row r="117">
       <c r="A117" t="inlineStr">
@@ -6460,19 +6460,19 @@
       </c>
       <c r="D117" t="inlineStr">
         <is>
-          <t>Angle valves with filters</t>
+          <t>Air admittance valve 110 mm (spare) + rodding eyes</t>
         </is>
       </c>
       <c r="E117" t="n">
-        <v>5</v>
+        <v>1</v>
       </c>
       <c r="F117" t="inlineStr">
         <is>
-          <t>each</t>
+          <t>set</t>
         </is>
       </c>
       <c r="G117" t="n">
-        <v>6000</v>
+        <v>30000</v>
       </c>
       <c r="H117" t="inlineStr">
         <is>
@@ -6507,7 +6507,7 @@
       </c>
       <c r="D118" t="inlineStr">
         <is>
-          <t>Air admittance valve 110 mm (spare) + rodding eyes</t>
+          <t>Stop valve + Y-filter + check water meter</t>
         </is>
       </c>
       <c r="E118" t="n">
@@ -6519,7 +6519,7 @@
         </is>
       </c>
       <c r="G118" t="n">
-        <v>30000</v>
+        <v>45000</v>
       </c>
       <c r="H118" t="inlineStr">
         <is>
@@ -6532,29 +6532,29 @@
         </is>
       </c>
       <c r="J118" t="n">
-        <v>30000</v>
+        <v>45000</v>
       </c>
       <c r="K118" t="inlineStr"/>
     </row>
     <row r="119">
       <c r="A119" t="inlineStr">
         <is>
-          <t>K9</t>
+          <t>K10</t>
         </is>
       </c>
       <c r="B119" t="inlineStr">
         <is>
-          <t>plumbing</t>
+          <t>steel</t>
         </is>
       </c>
       <c r="C119" t="inlineStr">
         <is>
-          <t>plumbing</t>
+          <t>welding</t>
         </is>
       </c>
       <c r="D119" t="inlineStr">
         <is>
-          <t>Stop valve + Y-filter + check water meter</t>
+          <t>W1 infill: 2 mm steel + 40 mm EPS, welded into the old door frame (0-1,150)</t>
         </is>
       </c>
       <c r="E119" t="n">
@@ -6562,11 +6562,11 @@
       </c>
       <c r="F119" t="inlineStr">
         <is>
-          <t>set</t>
+          <t>each</t>
         </is>
       </c>
       <c r="G119" t="n">
-        <v>45000</v>
+        <v>180000</v>
       </c>
       <c r="H119" t="inlineStr">
         <is>
@@ -6579,9 +6579,13 @@
         </is>
       </c>
       <c r="J119" t="n">
-        <v>45000</v>
-      </c>
-      <c r="K119" t="inlineStr"/>
+        <v>180000</v>
+      </c>
+      <c r="K119" t="inlineStr">
+        <is>
+          <t>incl. welding</t>
+        </is>
+      </c>
     </row>
     <row r="120">
       <c r="A120" t="inlineStr">
@@ -6591,17 +6595,17 @@
       </c>
       <c r="B120" t="inlineStr">
         <is>
-          <t>steel</t>
+          <t>glazing</t>
         </is>
       </c>
       <c r="C120" t="inlineStr">
         <is>
-          <t>welding</t>
+          <t>glazier</t>
         </is>
       </c>
       <c r="D120" t="inlineStr">
         <is>
-          <t>W1 infill: 2 mm steel + 40 mm EPS, welded into the old door frame (0-1,150)</t>
+          <t>W1 obscure louvre window 520 x 890 + insect mesh + fan panel</t>
         </is>
       </c>
       <c r="E120" t="n">
@@ -6613,7 +6617,7 @@
         </is>
       </c>
       <c r="G120" t="n">
-        <v>180000</v>
+        <v>120000</v>
       </c>
       <c r="H120" t="inlineStr">
         <is>
@@ -6626,13 +6630,9 @@
         </is>
       </c>
       <c r="J120" t="n">
-        <v>180000</v>
-      </c>
-      <c r="K120" t="inlineStr">
-        <is>
-          <t>incl. welding</t>
-        </is>
-      </c>
+        <v>120000</v>
+      </c>
+      <c r="K120" t="inlineStr"/>
     </row>
     <row r="121">
       <c r="A121" t="inlineStr">
@@ -6642,17 +6642,17 @@
       </c>
       <c r="B121" t="inlineStr">
         <is>
-          <t>glazing</t>
+          <t>steel</t>
         </is>
       </c>
       <c r="C121" t="inlineStr">
         <is>
-          <t>glazier</t>
+          <t>welding</t>
         </is>
       </c>
       <c r="D121" t="inlineStr">
         <is>
-          <t>W1 obscure louvre window 520 x 890 + insect mesh + fan panel</t>
+          <t>Seal and lock the end-B cargo doors (weld tabs, sealant)</t>
         </is>
       </c>
       <c r="E121" t="n">
@@ -6664,7 +6664,7 @@
         </is>
       </c>
       <c r="G121" t="n">
-        <v>120000</v>
+        <v>60000</v>
       </c>
       <c r="H121" t="inlineStr">
         <is>
@@ -6677,7 +6677,7 @@
         </is>
       </c>
       <c r="J121" t="n">
-        <v>120000</v>
+        <v>60000</v>
       </c>
       <c r="K121" t="inlineStr"/>
     </row>
@@ -6694,16 +6694,16 @@
       </c>
       <c r="C122" t="inlineStr">
         <is>
-          <t>welding</t>
+          <t>masonry</t>
         </is>
       </c>
       <c r="D122" t="inlineStr">
         <is>
-          <t>Seal and lock the end-B cargo doors (weld tabs, sealant)</t>
+          <t>Level the corner castings: concrete pads or steel shims (rock corner)</t>
         </is>
       </c>
       <c r="E122" t="n">
-        <v>1</v>
+        <v>4</v>
       </c>
       <c r="F122" t="inlineStr">
         <is>
@@ -6711,7 +6711,7 @@
         </is>
       </c>
       <c r="G122" t="n">
-        <v>60000</v>
+        <v>25000</v>
       </c>
       <c r="H122" t="inlineStr">
         <is>
@@ -6724,7 +6724,7 @@
         </is>
       </c>
       <c r="J122" t="n">
-        <v>60000</v>
+        <v>100000</v>
       </c>
       <c r="K122" t="inlineStr"/>
     </row>
@@ -6741,24 +6741,24 @@
       </c>
       <c r="C123" t="inlineStr">
         <is>
-          <t>masonry</t>
+          <t>welding</t>
         </is>
       </c>
       <c r="D123" t="inlineStr">
         <is>
-          <t>Level the corner castings: concrete pads or steel shims (rock corner)</t>
+          <t>Steel hanging rail for wall units + heater bracket</t>
         </is>
       </c>
       <c r="E123" t="n">
-        <v>4</v>
+        <v>1</v>
       </c>
       <c r="F123" t="inlineStr">
         <is>
-          <t>each</t>
+          <t>set</t>
         </is>
       </c>
       <c r="G123" t="n">
-        <v>25000</v>
+        <v>40000</v>
       </c>
       <c r="H123" t="inlineStr">
         <is>
@@ -6771,7 +6771,7 @@
         </is>
       </c>
       <c r="J123" t="n">
-        <v>100000</v>
+        <v>40000</v>
       </c>
       <c r="K123" t="inlineStr"/>
     </row>
@@ -6783,17 +6783,17 @@
       </c>
       <c r="B124" t="inlineStr">
         <is>
-          <t>steel</t>
+          <t>hardware</t>
         </is>
       </c>
       <c r="C124" t="inlineStr">
         <is>
-          <t>welding</t>
+          <t>glazier</t>
         </is>
       </c>
       <c r="D124" t="inlineStr">
         <is>
-          <t>Steel hanging rail for wall units + heater bracket</t>
+          <t>Keyed lock + secondary bolt for the slider</t>
         </is>
       </c>
       <c r="E124" t="n">
@@ -6805,7 +6805,7 @@
         </is>
       </c>
       <c r="G124" t="n">
-        <v>40000</v>
+        <v>45000</v>
       </c>
       <c r="H124" t="inlineStr">
         <is>
@@ -6818,7 +6818,7 @@
         </is>
       </c>
       <c r="J124" t="n">
-        <v>40000</v>
+        <v>45000</v>
       </c>
       <c r="K124" t="inlineStr"/>
     </row>
@@ -6830,7 +6830,7 @@
       </c>
       <c r="B125" t="inlineStr">
         <is>
-          <t>hardware</t>
+          <t>glazing</t>
         </is>
       </c>
       <c r="C125" t="inlineStr">
@@ -6840,7 +6840,7 @@
       </c>
       <c r="D125" t="inlineStr">
         <is>
-          <t>Keyed lock + secondary bolt for the slider</t>
+          <t>Louvred trickle-vent strip with mesh (10,000 mm2)</t>
         </is>
       </c>
       <c r="E125" t="n">
@@ -6848,11 +6848,11 @@
       </c>
       <c r="F125" t="inlineStr">
         <is>
-          <t>set</t>
+          <t>each</t>
         </is>
       </c>
       <c r="G125" t="n">
-        <v>45000</v>
+        <v>30000</v>
       </c>
       <c r="H125" t="inlineStr">
         <is>
@@ -6865,7 +6865,7 @@
         </is>
       </c>
       <c r="J125" t="n">
-        <v>45000</v>
+        <v>30000</v>
       </c>
       <c r="K125" t="inlineStr"/>
     </row>
@@ -6877,17 +6877,17 @@
       </c>
       <c r="B126" t="inlineStr">
         <is>
-          <t>glazing</t>
+          <t>steel</t>
         </is>
       </c>
       <c r="C126" t="inlineStr">
         <is>
-          <t>glazier</t>
+          <t>welding</t>
         </is>
       </c>
       <c r="D126" t="inlineStr">
         <is>
-          <t>Louvred trickle-vent strip with mesh (10,000 mm2)</t>
+          <t>AC wall sleeve 75 mm (provision, back wall, one hole)</t>
         </is>
       </c>
       <c r="E126" t="n">
@@ -6899,7 +6899,7 @@
         </is>
       </c>
       <c r="G126" t="n">
-        <v>30000</v>
+        <v>15000</v>
       </c>
       <c r="H126" t="inlineStr">
         <is>
@@ -6912,19 +6912,19 @@
         </is>
       </c>
       <c r="J126" t="n">
-        <v>30000</v>
+        <v>15000</v>
       </c>
       <c r="K126" t="inlineStr"/>
     </row>
     <row r="127">
       <c r="A127" t="inlineStr">
         <is>
-          <t>K10</t>
+          <t>K11</t>
         </is>
       </c>
       <c r="B127" t="inlineStr">
         <is>
-          <t>steel</t>
+          <t>roofing</t>
         </is>
       </c>
       <c r="C127" t="inlineStr">
@@ -6934,7 +6934,7 @@
       </c>
       <c r="D127" t="inlineStr">
         <is>
-          <t>AC wall sleeve 75 mm (provision, back wall, one hole)</t>
+          <t>Gutter + downpipe to the rainwater tank (deck canopy)</t>
         </is>
       </c>
       <c r="E127" t="n">
@@ -6942,11 +6942,11 @@
       </c>
       <c r="F127" t="inlineStr">
         <is>
-          <t>each</t>
+          <t>set</t>
         </is>
       </c>
       <c r="G127" t="n">
-        <v>15000</v>
+        <v>90000</v>
       </c>
       <c r="H127" t="inlineStr">
         <is>
@@ -6959,7 +6959,7 @@
         </is>
       </c>
       <c r="J127" t="n">
-        <v>15000</v>
+        <v>90000</v>
       </c>
       <c r="K127" t="inlineStr"/>
     </row>
@@ -6971,17 +6971,17 @@
       </c>
       <c r="B128" t="inlineStr">
         <is>
-          <t>roofing</t>
+          <t>electrical</t>
         </is>
       </c>
       <c r="C128" t="inlineStr">
         <is>
-          <t>welding</t>
+          <t>electrical</t>
         </is>
       </c>
       <c r="D128" t="inlineStr">
         <is>
-          <t>Gutter + downpipe to the rainwater tank (deck canopy)</t>
+          <t>Bonding: 16 mm2 green-yellow from the frame to the earth bar</t>
         </is>
       </c>
       <c r="E128" t="n">
@@ -6993,7 +6993,7 @@
         </is>
       </c>
       <c r="G128" t="n">
-        <v>90000</v>
+        <v>25000</v>
       </c>
       <c r="H128" t="inlineStr">
         <is>
@@ -7006,41 +7006,41 @@
         </is>
       </c>
       <c r="J128" t="n">
-        <v>90000</v>
+        <v>25000</v>
       </c>
       <c r="K128" t="inlineStr"/>
     </row>
     <row r="129">
       <c r="A129" t="inlineStr">
         <is>
-          <t>K11</t>
+          <t>K1</t>
         </is>
       </c>
       <c r="B129" t="inlineStr">
         <is>
-          <t>electrical</t>
+          <t>timber</t>
         </is>
       </c>
       <c r="C129" t="inlineStr">
         <is>
-          <t>electrical</t>
+          <t>carpentry</t>
         </is>
       </c>
       <c r="D129" t="inlineStr">
         <is>
-          <t>Bonding: 16 mm2 green-yellow from the frame to the earth bar</t>
+          <t>Battens 38 x 50 treated, 2.4 m</t>
         </is>
       </c>
       <c r="E129" t="n">
-        <v>1</v>
+        <v>19.8</v>
       </c>
       <c r="F129" t="inlineStr">
         <is>
-          <t>set</t>
+          <t>each</t>
         </is>
       </c>
       <c r="G129" t="n">
-        <v>25000</v>
+        <v>2500</v>
       </c>
       <c r="H129" t="inlineStr">
         <is>
@@ -7053,14 +7053,18 @@
         </is>
       </c>
       <c r="J129" t="n">
-        <v>25000</v>
-      </c>
-      <c r="K129" t="inlineStr"/>
+        <v>49500</v>
+      </c>
+      <c r="K129" t="inlineStr">
+        <is>
+          <t>38 x 50 treated, 2.4 m</t>
+        </is>
+      </c>
     </row>
     <row r="130">
       <c r="A130" t="inlineStr">
         <is>
-          <t>K1</t>
+          <t>K2</t>
         </is>
       </c>
       <c r="B130" t="inlineStr">
@@ -7075,11 +7079,11 @@
       </c>
       <c r="D130" t="inlineStr">
         <is>
-          <t>Battens 38 x 50 treated, 2.4 m</t>
+          <t>Studs 40 x 40 treated, 2.4 m</t>
         </is>
       </c>
       <c r="E130" t="n">
-        <v>19.8</v>
+        <v>5.5</v>
       </c>
       <c r="F130" t="inlineStr">
         <is>
@@ -7087,7 +7091,7 @@
         </is>
       </c>
       <c r="G130" t="n">
-        <v>2500</v>
+        <v>3000</v>
       </c>
       <c r="H130" t="inlineStr">
         <is>
@@ -7100,45 +7104,41 @@
         </is>
       </c>
       <c r="J130" t="n">
-        <v>49500</v>
+        <v>16500</v>
       </c>
       <c r="K130" t="inlineStr">
         <is>
-          <t>38 x 50 treated, 2.4 m</t>
+          <t>40 x 40, 2.4 m</t>
         </is>
       </c>
     </row>
     <row r="131">
       <c r="A131" t="inlineStr">
         <is>
-          <t>K2</t>
+          <t>labour</t>
         </is>
       </c>
       <c r="B131" t="inlineStr">
         <is>
-          <t>timber</t>
-        </is>
-      </c>
-      <c r="C131" t="inlineStr">
-        <is>
-          <t>carpentry</t>
-        </is>
-      </c>
+          <t>labour</t>
+        </is>
+      </c>
+      <c r="C131" t="inlineStr"/>
       <c r="D131" t="inlineStr">
         <is>
-          <t>Studs 40 x 40 treated, 2.4 m</t>
+          <t>Carpentry workshop: cutting, edging, drilling, labelling (per unit kit)</t>
         </is>
       </c>
       <c r="E131" t="n">
-        <v>5.5</v>
+        <v>1</v>
       </c>
       <c r="F131" t="inlineStr">
         <is>
-          <t>each</t>
+          <t>lot</t>
         </is>
       </c>
       <c r="G131" t="n">
-        <v>3000</v>
+        <v>450000</v>
       </c>
       <c r="H131" t="inlineStr">
         <is>
@@ -7151,13 +7151,9 @@
         </is>
       </c>
       <c r="J131" t="n">
-        <v>16500</v>
-      </c>
-      <c r="K131" t="inlineStr">
-        <is>
-          <t>40 x 40, 2.4 m</t>
-        </is>
-      </c>
+        <v>450000</v>
+      </c>
+      <c r="K131" t="inlineStr"/>
     </row>
     <row r="132">
       <c r="A132" t="inlineStr">
@@ -7173,7 +7169,7 @@
       <c r="C132" t="inlineStr"/>
       <c r="D132" t="inlineStr">
         <is>
-          <t>Carpentry workshop: cutting, edging, drilling, labelling (per unit kit)</t>
+          <t>Site carpentry and assembly: 2 people x 8 days</t>
         </is>
       </c>
       <c r="E132" t="n">
@@ -7185,7 +7181,7 @@
         </is>
       </c>
       <c r="G132" t="n">
-        <v>450000</v>
+        <v>320000</v>
       </c>
       <c r="H132" t="inlineStr">
         <is>
@@ -7198,7 +7194,7 @@
         </is>
       </c>
       <c r="J132" t="n">
-        <v>450000</v>
+        <v>320000</v>
       </c>
       <c r="K132" t="inlineStr"/>
     </row>
@@ -7216,7 +7212,7 @@
       <c r="C133" t="inlineStr"/>
       <c r="D133" t="inlineStr">
         <is>
-          <t>Site carpentry and assembly: 2 people x 8 days</t>
+          <t>Electrician (RURA class A), install + certificate</t>
         </is>
       </c>
       <c r="E133" t="n">
@@ -7228,7 +7224,7 @@
         </is>
       </c>
       <c r="G133" t="n">
-        <v>320000</v>
+        <v>250000</v>
       </c>
       <c r="H133" t="inlineStr">
         <is>
@@ -7241,7 +7237,7 @@
         </is>
       </c>
       <c r="J133" t="n">
-        <v>320000</v>
+        <v>250000</v>
       </c>
       <c r="K133" t="inlineStr"/>
     </row>
@@ -7259,7 +7255,7 @@
       <c r="C134" t="inlineStr"/>
       <c r="D134" t="inlineStr">
         <is>
-          <t>Electrician (RURA class A), install + certificate</t>
+          <t>Plumber, install + tests</t>
         </is>
       </c>
       <c r="E134" t="n">
@@ -7271,7 +7267,7 @@
         </is>
       </c>
       <c r="G134" t="n">
-        <v>250000</v>
+        <v>200000</v>
       </c>
       <c r="H134" t="inlineStr">
         <is>
@@ -7284,7 +7280,7 @@
         </is>
       </c>
       <c r="J134" t="n">
-        <v>250000</v>
+        <v>200000</v>
       </c>
       <c r="K134" t="inlineStr"/>
     </row>
@@ -7302,7 +7298,7 @@
       <c r="C135" t="inlineStr"/>
       <c r="D135" t="inlineStr">
         <is>
-          <t>Plumber, install + tests</t>
+          <t>Tiler: wet walls and floor</t>
         </is>
       </c>
       <c r="E135" t="n">
@@ -7314,7 +7310,7 @@
         </is>
       </c>
       <c r="G135" t="n">
-        <v>200000</v>
+        <v>150000</v>
       </c>
       <c r="H135" t="inlineStr">
         <is>
@@ -7327,7 +7323,7 @@
         </is>
       </c>
       <c r="J135" t="n">
-        <v>200000</v>
+        <v>150000</v>
       </c>
       <c r="K135" t="inlineStr"/>
     </row>
@@ -7345,7 +7341,7 @@
       <c r="C136" t="inlineStr"/>
       <c r="D136" t="inlineStr">
         <is>
-          <t>Tiler: wet walls and floor</t>
+          <t>Welder: W1, roof frame, deck canopy, stair (per unit)</t>
         </is>
       </c>
       <c r="E136" t="n">
@@ -7357,7 +7353,7 @@
         </is>
       </c>
       <c r="G136" t="n">
-        <v>150000</v>
+        <v>600000</v>
       </c>
       <c r="H136" t="inlineStr">
         <is>
@@ -7370,7 +7366,7 @@
         </is>
       </c>
       <c r="J136" t="n">
-        <v>150000</v>
+        <v>600000</v>
       </c>
       <c r="K136" t="inlineStr"/>
     </row>
@@ -7388,7 +7384,7 @@
       <c r="C137" t="inlineStr"/>
       <c r="D137" t="inlineStr">
         <is>
-          <t>Welder: W1, roof frame, deck canopy, stair (per unit)</t>
+          <t>Transport Kigali to site (share of 2 truck trips)</t>
         </is>
       </c>
       <c r="E137" t="n">
@@ -7400,7 +7396,7 @@
         </is>
       </c>
       <c r="G137" t="n">
-        <v>600000</v>
+        <v>120000</v>
       </c>
       <c r="H137" t="inlineStr">
         <is>
@@ -7413,52 +7409,9 @@
         </is>
       </c>
       <c r="J137" t="n">
-        <v>600000</v>
+        <v>120000</v>
       </c>
       <c r="K137" t="inlineStr"/>
-    </row>
-    <row r="138">
-      <c r="A138" t="inlineStr">
-        <is>
-          <t>labour</t>
-        </is>
-      </c>
-      <c r="B138" t="inlineStr">
-        <is>
-          <t>labour</t>
-        </is>
-      </c>
-      <c r="C138" t="inlineStr"/>
-      <c r="D138" t="inlineStr">
-        <is>
-          <t>Transport Kigali to site (share of 2 truck trips)</t>
-        </is>
-      </c>
-      <c r="E138" t="n">
-        <v>1</v>
-      </c>
-      <c r="F138" t="inlineStr">
-        <is>
-          <t>lot</t>
-        </is>
-      </c>
-      <c r="G138" t="n">
-        <v>120000</v>
-      </c>
-      <c r="H138" t="inlineStr">
-        <is>
-          <t>A</t>
-        </is>
-      </c>
-      <c r="I138" t="inlineStr">
-        <is>
-          <t>AS-21</t>
-        </is>
-      </c>
-      <c r="J138" t="n">
-        <v>120000</v>
-      </c>
-      <c r="K138" t="inlineStr"/>
     </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>

</xml_diff>

<commit_message>
feat(studio): centre the seating group, clear of the bed and the entrance
The sofa, table and chairs now sit centred between the bed and the
galley aisle (about 100 mm from the bed, a 900 mm aisle), and the
table and chairs move back from the sliding glass so the entrance
stays clear. The layout re-centres the group if the survey moves the
partition.

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01KRyNxX68L5feJKbJnBKRyV
</commit_message>
<xml_diff>
--- a/public/designs/studio/data/bom.xlsx
+++ b/public/designs/studio/data/bom.xlsx
@@ -491,10 +491,10 @@
         </is>
       </c>
       <c r="B7" t="n">
-        <v>1175980</v>
+        <v>1175440</v>
       </c>
       <c r="C7" t="n">
-        <v>3527940</v>
+        <v>3526320</v>
       </c>
     </row>
     <row r="8">
@@ -736,10 +736,10 @@
         </is>
       </c>
       <c r="B26" t="n">
-        <v>2003001</v>
+        <v>2002920</v>
       </c>
       <c r="C26" t="n">
-        <v>6737402</v>
+        <v>6737159</v>
       </c>
     </row>
     <row r="27">
@@ -749,10 +749,10 @@
         </is>
       </c>
       <c r="B27" t="n">
-        <v>15356338</v>
+        <v>15355717</v>
       </c>
       <c r="C27" t="n">
-        <v>51653413</v>
+        <v>51651550</v>
       </c>
     </row>
     <row r="29">
@@ -763,7 +763,7 @@
       </c>
       <c r="B29" t="inlineStr"/>
       <c r="C29" t="n">
-        <v>34998</v>
+        <v>34996</v>
       </c>
     </row>
   </sheetData>
@@ -1063,7 +1063,7 @@
         </is>
       </c>
       <c r="E6" t="n">
-        <v>93.3</v>
+        <v>92.40000000000001</v>
       </c>
       <c r="F6" t="inlineStr">
         <is>
@@ -1084,7 +1084,7 @@
         </is>
       </c>
       <c r="J6" t="n">
-        <v>55980</v>
+        <v>55440</v>
       </c>
       <c r="K6" t="inlineStr">
         <is>

</xml_diff>

<commit_message>
feat(studio): shower, WC and basin in one row, basin outside the door
The bathroom fixtures now stand in one row against end wall B: the
shower, then the WC, then the basin. A short cross wall with a 600 mm
sliding door closes the shower and WC; the basin and mirror cabinet
sit outside it in a wash lobby under the W1 window, open to the galley.
The WC is a short-projection model so 600 mm stays clear in front of
it even if the survey moves the partition 150 mm. The extract fan
moves to one 110 mm hole in the back wall. All checks pass at
-150/0/+150 mm.

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01KRyNxX68L5feJKbJnBKRyV
</commit_message>
<xml_diff>
--- a/public/designs/studio/data/bom.xlsx
+++ b/public/designs/studio/data/bom.xlsx
@@ -491,10 +491,10 @@
         </is>
       </c>
       <c r="B7" t="n">
-        <v>1175440</v>
+        <v>1175200</v>
       </c>
       <c r="C7" t="n">
-        <v>3526320</v>
+        <v>3525600</v>
       </c>
     </row>
     <row r="8">
@@ -504,10 +504,10 @@
         </is>
       </c>
       <c r="B8" t="n">
-        <v>891280</v>
+        <v>884280</v>
       </c>
       <c r="C8" t="n">
-        <v>2673840</v>
+        <v>2652840</v>
       </c>
     </row>
     <row r="9">
@@ -517,10 +517,10 @@
         </is>
       </c>
       <c r="B9" t="n">
-        <v>757100</v>
+        <v>755100</v>
       </c>
       <c r="C9" t="n">
-        <v>2271300</v>
+        <v>2265300</v>
       </c>
     </row>
     <row r="10">
@@ -565,27 +565,27 @@
     <row r="13">
       <c r="A13" t="inlineStr">
         <is>
-          <t>wet walls</t>
+          <t>furnishing</t>
         </is>
       </c>
       <c r="B13" t="n">
-        <v>523960</v>
+        <v>510000</v>
       </c>
       <c r="C13" t="n">
-        <v>1571880</v>
+        <v>1530000</v>
       </c>
     </row>
     <row r="14">
       <c r="A14" t="inlineStr">
         <is>
-          <t>furnishing</t>
+          <t>wet walls</t>
         </is>
       </c>
       <c r="B14" t="n">
-        <v>510000</v>
+        <v>478680</v>
       </c>
       <c r="C14" t="n">
-        <v>1530000</v>
+        <v>1436040</v>
       </c>
     </row>
     <row r="15">
@@ -699,10 +699,10 @@
         </is>
       </c>
       <c r="B23" t="n">
-        <v>66000</v>
+        <v>69300</v>
       </c>
       <c r="C23" t="n">
-        <v>198000</v>
+        <v>207900</v>
       </c>
     </row>
     <row r="24">
@@ -736,10 +736,10 @@
         </is>
       </c>
       <c r="B26" t="n">
-        <v>2002920</v>
+        <v>1995237</v>
       </c>
       <c r="C26" t="n">
-        <v>6737159</v>
+        <v>6714110</v>
       </c>
     </row>
     <row r="27">
@@ -749,10 +749,10 @@
         </is>
       </c>
       <c r="B27" t="n">
-        <v>15355717</v>
+        <v>15296814</v>
       </c>
       <c r="C27" t="n">
-        <v>51651550</v>
+        <v>51474841</v>
       </c>
     </row>
     <row r="29">
@@ -763,7 +763,7 @@
       </c>
       <c r="B29" t="inlineStr"/>
       <c r="C29" t="n">
-        <v>34996</v>
+        <v>34877</v>
       </c>
     </row>
   </sheetData>
@@ -777,7 +777,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:K137"/>
+  <dimension ref="A1:K139"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -1063,7 +1063,7 @@
         </is>
       </c>
       <c r="E6" t="n">
-        <v>92.40000000000001</v>
+        <v>92</v>
       </c>
       <c r="F6" t="inlineStr">
         <is>
@@ -1084,7 +1084,7 @@
         </is>
       </c>
       <c r="J6" t="n">
-        <v>55440</v>
+        <v>55200</v>
       </c>
       <c r="K6" t="inlineStr">
         <is>
@@ -2294,7 +2294,7 @@
       </c>
       <c r="D31" t="inlineStr">
         <is>
-          <t>Door leaf 700 x 2,000, moisture-resistant, lever + privacy lock</t>
+          <t>Sliding door leaf 640 x 2,050 on a top track, moisture-resistant, privacy latch</t>
         </is>
       </c>
       <c r="E31" t="n">
@@ -2447,7 +2447,7 @@
         </is>
       </c>
       <c r="E34" t="n">
-        <v>5.23</v>
+        <v>3.95</v>
       </c>
       <c r="F34" t="inlineStr">
         <is>
@@ -2468,7 +2468,7 @@
         </is>
       </c>
       <c r="J34" t="n">
-        <v>73220</v>
+        <v>55300</v>
       </c>
       <c r="K34" t="inlineStr">
         <is>
@@ -2498,7 +2498,7 @@
         </is>
       </c>
       <c r="E35" t="n">
-        <v>5.75</v>
+        <v>4.35</v>
       </c>
       <c r="F35" t="inlineStr">
         <is>
@@ -2519,7 +2519,7 @@
         </is>
       </c>
       <c r="J35" t="n">
-        <v>92000</v>
+        <v>69600</v>
       </c>
       <c r="K35" t="inlineStr">
         <is>
@@ -2545,11 +2545,11 @@
       </c>
       <c r="D36" t="inlineStr">
         <is>
-          <t>Cement board 12 mm + liquid membrane, front wall (around W1)</t>
+          <t>Cement board 12 mm + liquid membrane, partition, bath face</t>
         </is>
       </c>
       <c r="E36" t="n">
-        <v>3.06</v>
+        <v>3.95</v>
       </c>
       <c r="F36" t="inlineStr">
         <is>
@@ -2570,7 +2570,7 @@
         </is>
       </c>
       <c r="J36" t="n">
-        <v>42840</v>
+        <v>55300</v>
       </c>
       <c r="K36" t="inlineStr">
         <is>
@@ -2596,11 +2596,11 @@
       </c>
       <c r="D37" t="inlineStr">
         <is>
-          <t>Wall tiles + adhesive + grout, front wall (around W1)</t>
+          <t>Wall tiles + adhesive + grout, partition, bath face</t>
         </is>
       </c>
       <c r="E37" t="n">
-        <v>3.37</v>
+        <v>4.35</v>
       </c>
       <c r="F37" t="inlineStr">
         <is>
@@ -2621,7 +2621,7 @@
         </is>
       </c>
       <c r="J37" t="n">
-        <v>53920</v>
+        <v>69600</v>
       </c>
       <c r="K37" t="inlineStr">
         <is>
@@ -2647,11 +2647,11 @@
       </c>
       <c r="D38" t="inlineStr">
         <is>
-          <t>Cement board 12 mm + liquid membrane, partition, bath face</t>
+          <t>Cement board 12 mm + liquid membrane, cross wall, bath face</t>
         </is>
       </c>
       <c r="E38" t="n">
-        <v>5.23</v>
+        <v>3.06</v>
       </c>
       <c r="F38" t="inlineStr">
         <is>
@@ -2672,7 +2672,7 @@
         </is>
       </c>
       <c r="J38" t="n">
-        <v>73220</v>
+        <v>42840</v>
       </c>
       <c r="K38" t="inlineStr">
         <is>
@@ -2698,11 +2698,11 @@
       </c>
       <c r="D39" t="inlineStr">
         <is>
-          <t>Wall tiles + adhesive + grout, partition, bath face</t>
+          <t>Wall tiles + adhesive + grout, cross wall, bath face</t>
         </is>
       </c>
       <c r="E39" t="n">
-        <v>5.75</v>
+        <v>3.37</v>
       </c>
       <c r="F39" t="inlineStr">
         <is>
@@ -2723,7 +2723,7 @@
         </is>
       </c>
       <c r="J39" t="n">
-        <v>92000</v>
+        <v>53920</v>
       </c>
       <c r="K39" t="inlineStr">
         <is>
@@ -2739,7 +2739,7 @@
       </c>
       <c r="B40" t="inlineStr">
         <is>
-          <t>finishes</t>
+          <t>wet walls</t>
         </is>
       </c>
       <c r="C40" t="inlineStr">
@@ -2749,11 +2749,11 @@
       </c>
       <c r="D40" t="inlineStr">
         <is>
-          <t>Safety vinyl sheet, coved 100 mm up the walls</t>
+          <t>Cement board 12 mm + liquid membrane, splashback behind the basin (end wall B, wash lobby)</t>
         </is>
       </c>
       <c r="E40" t="n">
-        <v>3.7</v>
+        <v>1.12</v>
       </c>
       <c r="F40" t="inlineStr">
         <is>
@@ -2761,7 +2761,7 @@
         </is>
       </c>
       <c r="G40" t="n">
-        <v>15000</v>
+        <v>14000</v>
       </c>
       <c r="H40" t="inlineStr">
         <is>
@@ -2774,11 +2774,11 @@
         </is>
       </c>
       <c r="J40" t="n">
-        <v>55500</v>
+        <v>15680</v>
       </c>
       <c r="K40" t="inlineStr">
         <is>
-          <t>per m2</t>
+          <t>per m2 incl. membrane</t>
         </is>
       </c>
     </row>
@@ -2790,29 +2790,29 @@
       </c>
       <c r="B41" t="inlineStr">
         <is>
-          <t>sanitaryware</t>
+          <t>wet walls</t>
         </is>
       </c>
       <c r="C41" t="inlineStr">
         <is>
-          <t>plumbing</t>
+          <t>tiling</t>
         </is>
       </c>
       <c r="D41" t="inlineStr">
         <is>
-          <t>Shower tray 1200 x 900, low profile, 90 mm waste</t>
+          <t>Wall tiles + adhesive + grout, splashback behind the basin (end wall B, wash lobby)</t>
         </is>
       </c>
       <c r="E41" t="n">
-        <v>1</v>
+        <v>1.23</v>
       </c>
       <c r="F41" t="inlineStr">
         <is>
-          <t>each</t>
+          <t>m2</t>
         </is>
       </c>
       <c r="G41" t="n">
-        <v>120000</v>
+        <v>16000</v>
       </c>
       <c r="H41" t="inlineStr">
         <is>
@@ -2825,9 +2825,13 @@
         </is>
       </c>
       <c r="J41" t="n">
-        <v>120000</v>
-      </c>
-      <c r="K41" t="inlineStr"/>
+        <v>19680</v>
+      </c>
+      <c r="K41" t="inlineStr">
+        <is>
+          <t>per m2 incl. adhesive and grout</t>
+        </is>
+      </c>
     </row>
     <row r="42">
       <c r="A42" t="inlineStr">
@@ -2837,29 +2841,29 @@
       </c>
       <c r="B42" t="inlineStr">
         <is>
-          <t>sanitaryware</t>
+          <t>finishes</t>
         </is>
       </c>
       <c r="C42" t="inlineStr">
         <is>
-          <t>plumbing</t>
+          <t>tiling</t>
         </is>
       </c>
       <c r="D42" t="inlineStr">
         <is>
-          <t>Fixed glass shower screen 700 x 2,000, 8 mm toughened</t>
+          <t>Safety vinyl sheet, coved 100 mm up the walls (bathroom and wash lobby)</t>
         </is>
       </c>
       <c r="E42" t="n">
-        <v>1</v>
+        <v>3.7</v>
       </c>
       <c r="F42" t="inlineStr">
         <is>
-          <t>each</t>
+          <t>m2</t>
         </is>
       </c>
       <c r="G42" t="n">
-        <v>180000</v>
+        <v>15000</v>
       </c>
       <c r="H42" t="inlineStr">
         <is>
@@ -2872,9 +2876,13 @@
         </is>
       </c>
       <c r="J42" t="n">
-        <v>180000</v>
-      </c>
-      <c r="K42" t="inlineStr"/>
+        <v>55500</v>
+      </c>
+      <c r="K42" t="inlineStr">
+        <is>
+          <t>per m2</t>
+        </is>
+      </c>
     </row>
     <row r="43">
       <c r="A43" t="inlineStr">
@@ -2894,7 +2902,7 @@
       </c>
       <c r="D43" t="inlineStr">
         <is>
-          <t>Close-coupled WC, floor outlet, dual flush</t>
+          <t>Shower tray 1200 x 900, low profile, 90 mm waste</t>
         </is>
       </c>
       <c r="E43" t="n">
@@ -2906,7 +2914,7 @@
         </is>
       </c>
       <c r="G43" t="n">
-        <v>150000</v>
+        <v>120000</v>
       </c>
       <c r="H43" t="inlineStr">
         <is>
@@ -2919,7 +2927,7 @@
         </is>
       </c>
       <c r="J43" t="n">
-        <v>150000</v>
+        <v>120000</v>
       </c>
       <c r="K43" t="inlineStr"/>
     </row>
@@ -2941,7 +2949,7 @@
       </c>
       <c r="D44" t="inlineStr">
         <is>
-          <t>Wall basin 400 x 300 + mixer + bottle trap</t>
+          <t>Fixed glass shower screen 700 x 2,000, 8 mm toughened</t>
         </is>
       </c>
       <c r="E44" t="n">
@@ -2953,7 +2961,7 @@
         </is>
       </c>
       <c r="G44" t="n">
-        <v>90000</v>
+        <v>180000</v>
       </c>
       <c r="H44" t="inlineStr">
         <is>
@@ -2966,7 +2974,7 @@
         </is>
       </c>
       <c r="J44" t="n">
-        <v>90000</v>
+        <v>180000</v>
       </c>
       <c r="K44" t="inlineStr"/>
     </row>
@@ -2978,17 +2986,17 @@
       </c>
       <c r="B45" t="inlineStr">
         <is>
-          <t>glazing</t>
+          <t>sanitaryware</t>
         </is>
       </c>
       <c r="C45" t="inlineStr">
         <is>
-          <t>carpentry</t>
+          <t>plumbing</t>
         </is>
       </c>
       <c r="D45" t="inlineStr">
         <is>
-          <t>Mirror 4 mm bonded to the cabinet door</t>
+          <t>Short-projection close-coupled WC (550 deep), floor outlet, dual flush, back to end wall B</t>
         </is>
       </c>
       <c r="E45" t="n">
@@ -3000,7 +3008,7 @@
         </is>
       </c>
       <c r="G45" t="n">
-        <v>25000</v>
+        <v>150000</v>
       </c>
       <c r="H45" t="inlineStr">
         <is>
@@ -3013,7 +3021,7 @@
         </is>
       </c>
       <c r="J45" t="n">
-        <v>25000</v>
+        <v>150000</v>
       </c>
       <c r="K45" t="inlineStr"/>
     </row>
@@ -3025,17 +3033,17 @@
       </c>
       <c r="B46" t="inlineStr">
         <is>
-          <t>accessories</t>
+          <t>sanitaryware</t>
         </is>
       </c>
       <c r="C46" t="inlineStr">
         <is>
-          <t>carpentry</t>
+          <t>plumbing</t>
         </is>
       </c>
       <c r="D46" t="inlineStr">
         <is>
-          <t>Towel rail, robe hook, toilet-roll holder, shower shelf</t>
+          <t>Wall basin 400 x 300 + mixer + bottle trap (wash lobby)</t>
         </is>
       </c>
       <c r="E46" t="n">
@@ -3043,11 +3051,11 @@
       </c>
       <c r="F46" t="inlineStr">
         <is>
-          <t>set</t>
+          <t>each</t>
         </is>
       </c>
       <c r="G46" t="n">
-        <v>40000</v>
+        <v>90000</v>
       </c>
       <c r="H46" t="inlineStr">
         <is>
@@ -3060,19 +3068,19 @@
         </is>
       </c>
       <c r="J46" t="n">
-        <v>40000</v>
+        <v>90000</v>
       </c>
       <c r="K46" t="inlineStr"/>
     </row>
     <row r="47">
       <c r="A47" t="inlineStr">
         <is>
-          <t>K3</t>
+          <t>K2</t>
         </is>
       </c>
       <c r="B47" t="inlineStr">
         <is>
-          <t>hardware</t>
+          <t>glazing</t>
         </is>
       </c>
       <c r="C47" t="inlineStr">
@@ -3082,11 +3090,11 @@
       </c>
       <c r="D47" t="inlineStr">
         <is>
-          <t>Hob base adjustable legs</t>
+          <t>Mirror 4 mm bonded to the cabinet door</t>
         </is>
       </c>
       <c r="E47" t="n">
-        <v>4</v>
+        <v>1</v>
       </c>
       <c r="F47" t="inlineStr">
         <is>
@@ -3094,7 +3102,7 @@
         </is>
       </c>
       <c r="G47" t="n">
-        <v>1500</v>
+        <v>25000</v>
       </c>
       <c r="H47" t="inlineStr">
         <is>
@@ -3107,19 +3115,19 @@
         </is>
       </c>
       <c r="J47" t="n">
-        <v>6000</v>
+        <v>25000</v>
       </c>
       <c r="K47" t="inlineStr"/>
     </row>
     <row r="48">
       <c r="A48" t="inlineStr">
         <is>
-          <t>K3</t>
+          <t>K2</t>
         </is>
       </c>
       <c r="B48" t="inlineStr">
         <is>
-          <t>hardware</t>
+          <t>accessories</t>
         </is>
       </c>
       <c r="C48" t="inlineStr">
@@ -3129,19 +3137,19 @@
       </c>
       <c r="D48" t="inlineStr">
         <is>
-          <t>Sink base adjustable legs</t>
+          <t>Towel rail, robe hook, toilet-roll holder, shower shelf</t>
         </is>
       </c>
       <c r="E48" t="n">
-        <v>4</v>
+        <v>1</v>
       </c>
       <c r="F48" t="inlineStr">
         <is>
-          <t>each</t>
+          <t>set</t>
         </is>
       </c>
       <c r="G48" t="n">
-        <v>1500</v>
+        <v>40000</v>
       </c>
       <c r="H48" t="inlineStr">
         <is>
@@ -3154,7 +3162,7 @@
         </is>
       </c>
       <c r="J48" t="n">
-        <v>6000</v>
+        <v>40000</v>
       </c>
       <c r="K48" t="inlineStr"/>
     </row>
@@ -3166,21 +3174,21 @@
       </c>
       <c r="B49" t="inlineStr">
         <is>
-          <t>appliances</t>
+          <t>hardware</t>
         </is>
       </c>
       <c r="C49" t="inlineStr">
         <is>
-          <t>electrical</t>
+          <t>carpentry</t>
         </is>
       </c>
       <c r="D49" t="inlineStr">
         <is>
-          <t>Two-zone induction hob, 300 mm domino, about 3.5 kW</t>
+          <t>Hob base adjustable legs</t>
         </is>
       </c>
       <c r="E49" t="n">
-        <v>1</v>
+        <v>4</v>
       </c>
       <c r="F49" t="inlineStr">
         <is>
@@ -3188,7 +3196,7 @@
         </is>
       </c>
       <c r="G49" t="n">
-        <v>250000</v>
+        <v>1500</v>
       </c>
       <c r="H49" t="inlineStr">
         <is>
@@ -3201,13 +3209,9 @@
         </is>
       </c>
       <c r="J49" t="n">
-        <v>250000</v>
-      </c>
-      <c r="K49" t="inlineStr">
-        <is>
-          <t>2-zone induction domino</t>
-        </is>
-      </c>
+        <v>6000</v>
+      </c>
+      <c r="K49" t="inlineStr"/>
     </row>
     <row r="50">
       <c r="A50" t="inlineStr">
@@ -3217,21 +3221,21 @@
       </c>
       <c r="B50" t="inlineStr">
         <is>
-          <t>sanitaryware</t>
+          <t>hardware</t>
         </is>
       </c>
       <c r="C50" t="inlineStr">
         <is>
-          <t>plumbing</t>
+          <t>carpentry</t>
         </is>
       </c>
       <c r="D50" t="inlineStr">
         <is>
-          <t>Inset stainless sink 430 x 400, single bowl</t>
+          <t>Sink base adjustable legs</t>
         </is>
       </c>
       <c r="E50" t="n">
-        <v>1</v>
+        <v>4</v>
       </c>
       <c r="F50" t="inlineStr">
         <is>
@@ -3239,7 +3243,7 @@
         </is>
       </c>
       <c r="G50" t="n">
-        <v>70000</v>
+        <v>1500</v>
       </c>
       <c r="H50" t="inlineStr">
         <is>
@@ -3252,7 +3256,7 @@
         </is>
       </c>
       <c r="J50" t="n">
-        <v>70000</v>
+        <v>6000</v>
       </c>
       <c r="K50" t="inlineStr"/>
     </row>
@@ -3264,17 +3268,17 @@
       </c>
       <c r="B51" t="inlineStr">
         <is>
-          <t>sanitaryware</t>
+          <t>appliances</t>
         </is>
       </c>
       <c r="C51" t="inlineStr">
         <is>
-          <t>plumbing</t>
+          <t>electrical</t>
         </is>
       </c>
       <c r="D51" t="inlineStr">
         <is>
-          <t>Kitchen mixer tap</t>
+          <t>Two-zone induction hob, 300 mm domino, about 3.5 kW</t>
         </is>
       </c>
       <c r="E51" t="n">
@@ -3286,7 +3290,7 @@
         </is>
       </c>
       <c r="G51" t="n">
-        <v>45000</v>
+        <v>250000</v>
       </c>
       <c r="H51" t="inlineStr">
         <is>
@@ -3299,9 +3303,13 @@
         </is>
       </c>
       <c r="J51" t="n">
-        <v>45000</v>
-      </c>
-      <c r="K51" t="inlineStr"/>
+        <v>250000</v>
+      </c>
+      <c r="K51" t="inlineStr">
+        <is>
+          <t>2-zone induction domino</t>
+        </is>
+      </c>
     </row>
     <row r="52">
       <c r="A52" t="inlineStr">
@@ -3311,17 +3319,17 @@
       </c>
       <c r="B52" t="inlineStr">
         <is>
-          <t>appliances</t>
+          <t>sanitaryware</t>
         </is>
       </c>
       <c r="C52" t="inlineStr">
         <is>
-          <t>electrical</t>
+          <t>plumbing</t>
         </is>
       </c>
       <c r="D52" t="inlineStr">
         <is>
-          <t>Under-counter fridge about 90 L (A-class)</t>
+          <t>Inset stainless sink 430 x 400, single bowl</t>
         </is>
       </c>
       <c r="E52" t="n">
@@ -3333,26 +3341,22 @@
         </is>
       </c>
       <c r="G52" t="n">
-        <v>265000</v>
+        <v>70000</v>
       </c>
       <c r="H52" t="inlineStr">
         <is>
-          <t>V</t>
+          <t>A</t>
         </is>
       </c>
       <c r="I52" t="inlineStr">
         <is>
-          <t>STU-P03</t>
+          <t>AS-21</t>
         </is>
       </c>
       <c r="J52" t="n">
-        <v>265000</v>
-      </c>
-      <c r="K52" t="inlineStr">
-        <is>
-          <t>90 L mini fridge, Kanis 2026-10-26</t>
-        </is>
-      </c>
+        <v>70000</v>
+      </c>
+      <c r="K52" t="inlineStr"/>
     </row>
     <row r="53">
       <c r="A53" t="inlineStr">
@@ -3362,17 +3366,17 @@
       </c>
       <c r="B53" t="inlineStr">
         <is>
-          <t>appliances</t>
+          <t>sanitaryware</t>
         </is>
       </c>
       <c r="C53" t="inlineStr">
         <is>
-          <t>electrical</t>
+          <t>plumbing</t>
         </is>
       </c>
       <c r="D53" t="inlineStr">
         <is>
-          <t>Recirculating hood 300-450 mm, charcoal filter</t>
+          <t>Kitchen mixer tap</t>
         </is>
       </c>
       <c r="E53" t="n">
@@ -3384,7 +3388,7 @@
         </is>
       </c>
       <c r="G53" t="n">
-        <v>90000</v>
+        <v>45000</v>
       </c>
       <c r="H53" t="inlineStr">
         <is>
@@ -3397,7 +3401,7 @@
         </is>
       </c>
       <c r="J53" t="n">
-        <v>90000</v>
+        <v>45000</v>
       </c>
       <c r="K53" t="inlineStr"/>
     </row>
@@ -3409,17 +3413,17 @@
       </c>
       <c r="B54" t="inlineStr">
         <is>
-          <t>plumbing</t>
+          <t>appliances</t>
         </is>
       </c>
       <c r="C54" t="inlineStr">
         <is>
-          <t>plumbing</t>
+          <t>electrical</t>
         </is>
       </c>
       <c r="D54" t="inlineStr">
         <is>
-          <t>Under-sink drinking-water filter + faucet</t>
+          <t>Under-counter fridge about 90 L (A-class)</t>
         </is>
       </c>
       <c r="E54" t="n">
@@ -3431,42 +3435,46 @@
         </is>
       </c>
       <c r="G54" t="n">
-        <v>80000</v>
+        <v>265000</v>
       </c>
       <c r="H54" t="inlineStr">
         <is>
-          <t>A</t>
+          <t>V</t>
         </is>
       </c>
       <c r="I54" t="inlineStr">
         <is>
-          <t>AS-21</t>
+          <t>STU-P03</t>
         </is>
       </c>
       <c r="J54" t="n">
-        <v>80000</v>
-      </c>
-      <c r="K54" t="inlineStr"/>
+        <v>265000</v>
+      </c>
+      <c r="K54" t="inlineStr">
+        <is>
+          <t>90 L mini fridge, Kanis 2026-10-26</t>
+        </is>
+      </c>
     </row>
     <row r="55">
       <c r="A55" t="inlineStr">
         <is>
-          <t>K4</t>
+          <t>K3</t>
         </is>
       </c>
       <c r="B55" t="inlineStr">
         <is>
-          <t>bedding</t>
+          <t>appliances</t>
         </is>
       </c>
       <c r="C55" t="inlineStr">
         <is>
-          <t>furnishing</t>
+          <t>electrical</t>
         </is>
       </c>
       <c r="D55" t="inlineStr">
         <is>
-          <t>Mattress up to 1,600 x 2,000 (local size, e.g. 5 x 6 ft), 200 mm</t>
+          <t>Recirculating hood 300-450 mm, charcoal filter</t>
         </is>
       </c>
       <c r="E55" t="n">
@@ -3478,7 +3486,7 @@
         </is>
       </c>
       <c r="G55" t="n">
-        <v>180000</v>
+        <v>90000</v>
       </c>
       <c r="H55" t="inlineStr">
         <is>
@@ -3491,45 +3499,41 @@
         </is>
       </c>
       <c r="J55" t="n">
-        <v>180000</v>
-      </c>
-      <c r="K55" t="inlineStr">
-        <is>
-          <t>local foam, size to field-check (STU-51)</t>
-        </is>
-      </c>
+        <v>90000</v>
+      </c>
+      <c r="K55" t="inlineStr"/>
     </row>
     <row r="56">
       <c r="A56" t="inlineStr">
         <is>
-          <t>K4</t>
+          <t>K3</t>
         </is>
       </c>
       <c r="B56" t="inlineStr">
         <is>
-          <t>hardware</t>
+          <t>plumbing</t>
         </is>
       </c>
       <c r="C56" t="inlineStr">
         <is>
-          <t>carpentry</t>
+          <t>plumbing</t>
         </is>
       </c>
       <c r="D56" t="inlineStr">
         <is>
-          <t>Gas struts + lift-up hinges for the deck panels</t>
+          <t>Under-sink drinking-water filter + faucet</t>
         </is>
       </c>
       <c r="E56" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="F56" t="inlineStr">
         <is>
-          <t>set</t>
+          <t>each</t>
         </is>
       </c>
       <c r="G56" t="n">
-        <v>12000</v>
+        <v>80000</v>
       </c>
       <c r="H56" t="inlineStr">
         <is>
@@ -3542,29 +3546,29 @@
         </is>
       </c>
       <c r="J56" t="n">
-        <v>24000</v>
+        <v>80000</v>
       </c>
       <c r="K56" t="inlineStr"/>
     </row>
     <row r="57">
       <c r="A57" t="inlineStr">
         <is>
-          <t>K5</t>
+          <t>K4</t>
         </is>
       </c>
       <c r="B57" t="inlineStr">
         <is>
-          <t>hardware</t>
+          <t>bedding</t>
         </is>
       </c>
       <c r="C57" t="inlineStr">
         <is>
-          <t>carpentry</t>
+          <t>furnishing</t>
         </is>
       </c>
       <c r="D57" t="inlineStr">
         <is>
-          <t>Coat hooks, hanging rail by the door and a folding luggage rack</t>
+          <t>Mattress up to 1,600 x 2,000 (local size, e.g. 5 x 6 ft), 200 mm</t>
         </is>
       </c>
       <c r="E57" t="n">
@@ -3572,11 +3576,11 @@
       </c>
       <c r="F57" t="inlineStr">
         <is>
-          <t>set</t>
+          <t>each</t>
         </is>
       </c>
       <c r="G57" t="n">
-        <v>8000</v>
+        <v>180000</v>
       </c>
       <c r="H57" t="inlineStr">
         <is>
@@ -3589,41 +3593,45 @@
         </is>
       </c>
       <c r="J57" t="n">
-        <v>8000</v>
-      </c>
-      <c r="K57" t="inlineStr"/>
+        <v>180000</v>
+      </c>
+      <c r="K57" t="inlineStr">
+        <is>
+          <t>local foam, size to field-check (STU-51)</t>
+        </is>
+      </c>
     </row>
     <row r="58">
       <c r="A58" t="inlineStr">
         <is>
-          <t>K6</t>
+          <t>K4</t>
         </is>
       </c>
       <c r="B58" t="inlineStr">
         <is>
-          <t>furnishing</t>
+          <t>hardware</t>
         </is>
       </c>
       <c r="C58" t="inlineStr">
         <is>
-          <t>furnishing</t>
+          <t>carpentry</t>
         </is>
       </c>
       <c r="D58" t="inlineStr">
         <is>
-          <t>Compact two-seat sofa about 1150 x 850, washable covers</t>
+          <t>Gas struts + lift-up hinges for the deck panels</t>
         </is>
       </c>
       <c r="E58" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="F58" t="inlineStr">
         <is>
-          <t>each</t>
+          <t>set</t>
         </is>
       </c>
       <c r="G58" t="n">
-        <v>450000</v>
+        <v>12000</v>
       </c>
       <c r="H58" t="inlineStr">
         <is>
@@ -3636,33 +3644,29 @@
         </is>
       </c>
       <c r="J58" t="n">
-        <v>450000</v>
-      </c>
-      <c r="K58" t="inlineStr">
-        <is>
-          <t>compact two-seat sofa, washable covers</t>
-        </is>
-      </c>
+        <v>24000</v>
+      </c>
+      <c r="K58" t="inlineStr"/>
     </row>
     <row r="59">
       <c r="A59" t="inlineStr">
         <is>
-          <t>K6</t>
+          <t>K5</t>
         </is>
       </c>
       <c r="B59" t="inlineStr">
         <is>
-          <t>furnishing</t>
+          <t>hardware</t>
         </is>
       </c>
       <c r="C59" t="inlineStr">
         <is>
-          <t>furnishing</t>
+          <t>carpentry</t>
         </is>
       </c>
       <c r="D59" t="inlineStr">
         <is>
-          <t>Blackout curtain + track for the 3 m slider</t>
+          <t>Coat hooks, hanging rail by the door and a folding luggage rack</t>
         </is>
       </c>
       <c r="E59" t="n">
@@ -3674,7 +3678,7 @@
         </is>
       </c>
       <c r="G59" t="n">
-        <v>60000</v>
+        <v>8000</v>
       </c>
       <c r="H59" t="inlineStr">
         <is>
@@ -3687,7 +3691,7 @@
         </is>
       </c>
       <c r="J59" t="n">
-        <v>60000</v>
+        <v>8000</v>
       </c>
       <c r="K59" t="inlineStr"/>
     </row>
@@ -3699,17 +3703,17 @@
       </c>
       <c r="B60" t="inlineStr">
         <is>
-          <t>glazing</t>
+          <t>furnishing</t>
         </is>
       </c>
       <c r="C60" t="inlineStr">
         <is>
-          <t>glazier</t>
+          <t>furnishing</t>
         </is>
       </c>
       <c r="D60" t="inlineStr">
         <is>
-          <t>Insect screens: slider (sliding), W1, vents</t>
+          <t>Compact two-seat sofa about 1150 x 850, washable covers</t>
         </is>
       </c>
       <c r="E60" t="n">
@@ -3717,11 +3721,11 @@
       </c>
       <c r="F60" t="inlineStr">
         <is>
-          <t>set</t>
+          <t>each</t>
         </is>
       </c>
       <c r="G60" t="n">
-        <v>90000</v>
+        <v>450000</v>
       </c>
       <c r="H60" t="inlineStr">
         <is>
@@ -3734,29 +3738,33 @@
         </is>
       </c>
       <c r="J60" t="n">
-        <v>90000</v>
-      </c>
-      <c r="K60" t="inlineStr"/>
+        <v>450000</v>
+      </c>
+      <c r="K60" t="inlineStr">
+        <is>
+          <t>compact two-seat sofa, washable covers</t>
+        </is>
+      </c>
     </row>
     <row r="61">
       <c r="A61" t="inlineStr">
         <is>
-          <t>K8</t>
+          <t>K6</t>
         </is>
       </c>
       <c r="B61" t="inlineStr">
         <is>
-          <t>electrical</t>
+          <t>furnishing</t>
         </is>
       </c>
       <c r="C61" t="inlineStr">
         <is>
-          <t>electrical</t>
+          <t>furnishing</t>
         </is>
       </c>
       <c r="D61" t="inlineStr">
         <is>
-          <t>Unit board on the back wall by the galley</t>
+          <t>Blackout curtain + track for the 3 m slider</t>
         </is>
       </c>
       <c r="E61" t="n">
@@ -3764,11 +3772,11 @@
       </c>
       <c r="F61" t="inlineStr">
         <is>
-          <t>each</t>
+          <t>set</t>
         </is>
       </c>
       <c r="G61" t="n">
-        <v>45000</v>
+        <v>60000</v>
       </c>
       <c r="H61" t="inlineStr">
         <is>
@@ -3781,33 +3789,29 @@
         </is>
       </c>
       <c r="J61" t="n">
-        <v>45000</v>
-      </c>
-      <c r="K61" t="inlineStr">
-        <is>
-          <t>enclosure, 12 ways</t>
-        </is>
-      </c>
+        <v>60000</v>
+      </c>
+      <c r="K61" t="inlineStr"/>
     </row>
     <row r="62">
       <c r="A62" t="inlineStr">
         <is>
-          <t>K8</t>
+          <t>K6</t>
         </is>
       </c>
       <c r="B62" t="inlineStr">
         <is>
-          <t>electrical</t>
+          <t>glazing</t>
         </is>
       </c>
       <c r="C62" t="inlineStr">
         <is>
-          <t>electrical</t>
+          <t>glazier</t>
         </is>
       </c>
       <c r="D62" t="inlineStr">
         <is>
-          <t>Ceiling light, bed</t>
+          <t>Insect screens: slider (sliding), W1, vents</t>
         </is>
       </c>
       <c r="E62" t="n">
@@ -3815,11 +3819,11 @@
       </c>
       <c r="F62" t="inlineStr">
         <is>
-          <t>each</t>
+          <t>set</t>
         </is>
       </c>
       <c r="G62" t="n">
-        <v>15000</v>
+        <v>90000</v>
       </c>
       <c r="H62" t="inlineStr">
         <is>
@@ -3832,7 +3836,7 @@
         </is>
       </c>
       <c r="J62" t="n">
-        <v>15000</v>
+        <v>90000</v>
       </c>
       <c r="K62" t="inlineStr"/>
     </row>
@@ -3854,7 +3858,7 @@
       </c>
       <c r="D63" t="inlineStr">
         <is>
-          <t>Ceiling light, living</t>
+          <t>Unit board on the back wall by the galley</t>
         </is>
       </c>
       <c r="E63" t="n">
@@ -3866,7 +3870,7 @@
         </is>
       </c>
       <c r="G63" t="n">
-        <v>15000</v>
+        <v>45000</v>
       </c>
       <c r="H63" t="inlineStr">
         <is>
@@ -3879,9 +3883,13 @@
         </is>
       </c>
       <c r="J63" t="n">
-        <v>15000</v>
-      </c>
-      <c r="K63" t="inlineStr"/>
+        <v>45000</v>
+      </c>
+      <c r="K63" t="inlineStr">
+        <is>
+          <t>enclosure, 12 ways</t>
+        </is>
+      </c>
     </row>
     <row r="64">
       <c r="A64" t="inlineStr">
@@ -3901,7 +3909,7 @@
       </c>
       <c r="D64" t="inlineStr">
         <is>
-          <t>Ceiling light, galley</t>
+          <t>Ceiling light, bed</t>
         </is>
       </c>
       <c r="E64" t="n">
@@ -3948,7 +3956,7 @@
       </c>
       <c r="D65" t="inlineStr">
         <is>
-          <t>Bathroom light IP65</t>
+          <t>Ceiling light, living</t>
         </is>
       </c>
       <c r="E65" t="n">
@@ -3995,7 +4003,7 @@
       </c>
       <c r="D66" t="inlineStr">
         <is>
-          <t>Reading light 1</t>
+          <t>Ceiling light, galley</t>
         </is>
       </c>
       <c r="E66" t="n">
@@ -4042,7 +4050,7 @@
       </c>
       <c r="D67" t="inlineStr">
         <is>
-          <t>Reading light 2</t>
+          <t>Bathroom light IP65</t>
         </is>
       </c>
       <c r="E67" t="n">
@@ -4089,7 +4097,7 @@
       </c>
       <c r="D68" t="inlineStr">
         <is>
-          <t>Under-cabinet LED strip</t>
+          <t>Reading light 1</t>
         </is>
       </c>
       <c r="E68" t="n">
@@ -4136,7 +4144,7 @@
       </c>
       <c r="D69" t="inlineStr">
         <is>
-          <t>Deck light IP65</t>
+          <t>Reading light 2</t>
         </is>
       </c>
       <c r="E69" t="n">
@@ -4183,7 +4191,7 @@
       </c>
       <c r="D70" t="inlineStr">
         <is>
-          <t>Roof terrace lights IP65 (x2)</t>
+          <t>Under-cabinet LED strip</t>
         </is>
       </c>
       <c r="E70" t="n">
@@ -4230,7 +4238,7 @@
       </c>
       <c r="D71" t="inlineStr">
         <is>
-          <t>Stair light IP65</t>
+          <t>Deck light IP65</t>
         </is>
       </c>
       <c r="E71" t="n">
@@ -4277,7 +4285,7 @@
       </c>
       <c r="D72" t="inlineStr">
         <is>
-          <t>Entry: living + kitchen + deck</t>
+          <t>Roof terrace lights IP65 (x2)</t>
         </is>
       </c>
       <c r="E72" t="n">
@@ -4289,7 +4297,7 @@
         </is>
       </c>
       <c r="G72" t="n">
-        <v>3500</v>
+        <v>15000</v>
       </c>
       <c r="H72" t="inlineStr">
         <is>
@@ -4302,7 +4310,7 @@
         </is>
       </c>
       <c r="J72" t="n">
-        <v>3500</v>
+        <v>15000</v>
       </c>
       <c r="K72" t="inlineStr"/>
     </row>
@@ -4324,7 +4332,7 @@
       </c>
       <c r="D73" t="inlineStr">
         <is>
-          <t>Bed: ceiling light (2-way)</t>
+          <t>Stair light IP65</t>
         </is>
       </c>
       <c r="E73" t="n">
@@ -4336,7 +4344,7 @@
         </is>
       </c>
       <c r="G73" t="n">
-        <v>3500</v>
+        <v>15000</v>
       </c>
       <c r="H73" t="inlineStr">
         <is>
@@ -4349,7 +4357,7 @@
         </is>
       </c>
       <c r="J73" t="n">
-        <v>3500</v>
+        <v>15000</v>
       </c>
       <c r="K73" t="inlineStr"/>
     </row>
@@ -4371,7 +4379,7 @@
       </c>
       <c r="D74" t="inlineStr">
         <is>
-          <t>Bathroom light + fan (outside)</t>
+          <t>Entry: living + kitchen + deck</t>
         </is>
       </c>
       <c r="E74" t="n">
@@ -4418,7 +4426,7 @@
       </c>
       <c r="D75" t="inlineStr">
         <is>
-          <t>Roof and stair lights (IP65, stair foot)</t>
+          <t>Bed: ceiling light (2-way)</t>
         </is>
       </c>
       <c r="E75" t="n">
@@ -4465,7 +4473,7 @@
       </c>
       <c r="D76" t="inlineStr">
         <is>
-          <t>Bedside socket + USB-C 1</t>
+          <t>Bathroom light + fan (outside)</t>
         </is>
       </c>
       <c r="E76" t="n">
@@ -4477,7 +4485,7 @@
         </is>
       </c>
       <c r="G76" t="n">
-        <v>15000</v>
+        <v>3500</v>
       </c>
       <c r="H76" t="inlineStr">
         <is>
@@ -4490,7 +4498,7 @@
         </is>
       </c>
       <c r="J76" t="n">
-        <v>15000</v>
+        <v>3500</v>
       </c>
       <c r="K76" t="inlineStr"/>
     </row>
@@ -4512,7 +4520,7 @@
       </c>
       <c r="D77" t="inlineStr">
         <is>
-          <t>Bedside socket + USB-C 2</t>
+          <t>Roof and stair lights (IP65, stair foot)</t>
         </is>
       </c>
       <c r="E77" t="n">
@@ -4524,7 +4532,7 @@
         </is>
       </c>
       <c r="G77" t="n">
-        <v>15000</v>
+        <v>3500</v>
       </c>
       <c r="H77" t="inlineStr">
         <is>
@@ -4537,7 +4545,7 @@
         </is>
       </c>
       <c r="J77" t="n">
-        <v>15000</v>
+        <v>3500</v>
       </c>
       <c r="K77" t="inlineStr"/>
     </row>
@@ -4559,7 +4567,7 @@
       </c>
       <c r="D78" t="inlineStr">
         <is>
-          <t>Socket by the sofa</t>
+          <t>Bedside socket + USB-C 1</t>
         </is>
       </c>
       <c r="E78" t="n">
@@ -4571,7 +4579,7 @@
         </is>
       </c>
       <c r="G78" t="n">
-        <v>5000</v>
+        <v>15000</v>
       </c>
       <c r="H78" t="inlineStr">
         <is>
@@ -4584,7 +4592,7 @@
         </is>
       </c>
       <c r="J78" t="n">
-        <v>5000</v>
+        <v>15000</v>
       </c>
       <c r="K78" t="inlineStr"/>
     </row>
@@ -4606,7 +4614,7 @@
       </c>
       <c r="D79" t="inlineStr">
         <is>
-          <t>Socket, living (front strip)</t>
+          <t>Bedside socket + USB-C 2</t>
         </is>
       </c>
       <c r="E79" t="n">
@@ -4618,7 +4626,7 @@
         </is>
       </c>
       <c r="G79" t="n">
-        <v>5000</v>
+        <v>15000</v>
       </c>
       <c r="H79" t="inlineStr">
         <is>
@@ -4631,7 +4639,7 @@
         </is>
       </c>
       <c r="J79" t="n">
-        <v>5000</v>
+        <v>15000</v>
       </c>
       <c r="K79" t="inlineStr"/>
     </row>
@@ -4653,7 +4661,7 @@
       </c>
       <c r="D80" t="inlineStr">
         <is>
-          <t>Deck socket IP66</t>
+          <t>Socket by the sofa</t>
         </is>
       </c>
       <c r="E80" t="n">
@@ -4700,7 +4708,7 @@
       </c>
       <c r="D81" t="inlineStr">
         <is>
-          <t>Worktop socket 1 (double)</t>
+          <t>Socket, living (front strip)</t>
         </is>
       </c>
       <c r="E81" t="n">
@@ -4747,7 +4755,7 @@
       </c>
       <c r="D82" t="inlineStr">
         <is>
-          <t>Worktop socket 2 (double, back wall)</t>
+          <t>Deck socket IP66</t>
         </is>
       </c>
       <c r="E82" t="n">
@@ -4794,7 +4802,7 @@
       </c>
       <c r="D83" t="inlineStr">
         <is>
-          <t>Fridge socket</t>
+          <t>Worktop socket 1 (double)</t>
         </is>
       </c>
       <c r="E83" t="n">
@@ -4841,7 +4849,7 @@
       </c>
       <c r="D84" t="inlineStr">
         <is>
-          <t>Hob connection unit</t>
+          <t>Worktop socket 2 (double, back wall)</t>
         </is>
       </c>
       <c r="E84" t="n">
@@ -4853,7 +4861,7 @@
         </is>
       </c>
       <c r="G84" t="n">
-        <v>9000</v>
+        <v>5000</v>
       </c>
       <c r="H84" t="inlineStr">
         <is>
@@ -4866,7 +4874,7 @@
         </is>
       </c>
       <c r="J84" t="n">
-        <v>9000</v>
+        <v>5000</v>
       </c>
       <c r="K84" t="inlineStr"/>
     </row>
@@ -4888,7 +4896,7 @@
       </c>
       <c r="D85" t="inlineStr">
         <is>
-          <t>Heater DP switch + timer</t>
+          <t>Fridge socket</t>
         </is>
       </c>
       <c r="E85" t="n">
@@ -4900,7 +4908,7 @@
         </is>
       </c>
       <c r="G85" t="n">
-        <v>9000</v>
+        <v>5000</v>
       </c>
       <c r="H85" t="inlineStr">
         <is>
@@ -4913,7 +4921,7 @@
         </is>
       </c>
       <c r="J85" t="n">
-        <v>9000</v>
+        <v>5000</v>
       </c>
       <c r="K85" t="inlineStr"/>
     </row>
@@ -4935,7 +4943,7 @@
       </c>
       <c r="D86" t="inlineStr">
         <is>
-          <t>Bathroom extract 100 mm (in W1 panel)</t>
+          <t>Hob connection unit</t>
         </is>
       </c>
       <c r="E86" t="n">
@@ -4947,7 +4955,7 @@
         </is>
       </c>
       <c r="G86" t="n">
-        <v>35000</v>
+        <v>9000</v>
       </c>
       <c r="H86" t="inlineStr">
         <is>
@@ -4960,7 +4968,7 @@
         </is>
       </c>
       <c r="J86" t="n">
-        <v>35000</v>
+        <v>9000</v>
       </c>
       <c r="K86" t="inlineStr"/>
     </row>
@@ -4982,7 +4990,7 @@
       </c>
       <c r="D87" t="inlineStr">
         <is>
-          <t>Wall fan</t>
+          <t>Heater DP switch + timer</t>
         </is>
       </c>
       <c r="E87" t="n">
@@ -4994,7 +5002,7 @@
         </is>
       </c>
       <c r="G87" t="n">
-        <v>35000</v>
+        <v>9000</v>
       </c>
       <c r="H87" t="inlineStr">
         <is>
@@ -5007,7 +5015,7 @@
         </is>
       </c>
       <c r="J87" t="n">
-        <v>35000</v>
+        <v>9000</v>
       </c>
       <c r="K87" t="inlineStr"/>
     </row>
@@ -5029,7 +5037,7 @@
       </c>
       <c r="D88" t="inlineStr">
         <is>
-          <t>AC provision: isolator</t>
+          <t>Bathroom extract 100 mm (one 110 mm hole in the back wall)</t>
         </is>
       </c>
       <c r="E88" t="n">
@@ -5041,7 +5049,7 @@
         </is>
       </c>
       <c r="G88" t="n">
-        <v>9000</v>
+        <v>35000</v>
       </c>
       <c r="H88" t="inlineStr">
         <is>
@@ -5054,7 +5062,7 @@
         </is>
       </c>
       <c r="J88" t="n">
-        <v>9000</v>
+        <v>35000</v>
       </c>
       <c r="K88" t="inlineStr"/>
     </row>
@@ -5076,19 +5084,19 @@
       </c>
       <c r="D89" t="inlineStr">
         <is>
-          <t>Cable 1.5 mm2 T+E/singles in conduit, Lighting (incl. bathroom IP65, deck, roof, stair)</t>
+          <t>Wall fan</t>
         </is>
       </c>
       <c r="E89" t="n">
-        <v>89</v>
+        <v>1</v>
       </c>
       <c r="F89" t="inlineStr">
         <is>
-          <t>m</t>
+          <t>each</t>
         </is>
       </c>
       <c r="G89" t="n">
-        <v>500</v>
+        <v>35000</v>
       </c>
       <c r="H89" t="inlineStr">
         <is>
@@ -5101,13 +5109,9 @@
         </is>
       </c>
       <c r="J89" t="n">
-        <v>44500</v>
-      </c>
-      <c r="K89" t="inlineStr">
-        <is>
-          <t>per m</t>
-        </is>
-      </c>
+        <v>35000</v>
+      </c>
+      <c r="K89" t="inlineStr"/>
     </row>
     <row r="90">
       <c r="A90" t="inlineStr">
@@ -5127,19 +5131,19 @@
       </c>
       <c r="D90" t="inlineStr">
         <is>
-          <t>Cable 2.5 mm2 T+E/singles in conduit, Sockets: bedside USB, living, deck</t>
+          <t>AC provision: isolator</t>
         </is>
       </c>
       <c r="E90" t="n">
-        <v>29</v>
+        <v>1</v>
       </c>
       <c r="F90" t="inlineStr">
         <is>
-          <t>m</t>
+          <t>each</t>
         </is>
       </c>
       <c r="G90" t="n">
-        <v>750</v>
+        <v>9000</v>
       </c>
       <c r="H90" t="inlineStr">
         <is>
@@ -5152,13 +5156,9 @@
         </is>
       </c>
       <c r="J90" t="n">
-        <v>21750</v>
-      </c>
-      <c r="K90" t="inlineStr">
-        <is>
-          <t>per m</t>
-        </is>
-      </c>
+        <v>9000</v>
+      </c>
+      <c r="K90" t="inlineStr"/>
     </row>
     <row r="91">
       <c r="A91" t="inlineStr">
@@ -5178,11 +5178,11 @@
       </c>
       <c r="D91" t="inlineStr">
         <is>
-          <t>Cable 2.5 mm2 T+E/singles in conduit, Kitchen sockets and fridge</t>
+          <t>Cable 1.5 mm2 T+E/singles in conduit, Lighting (incl. bathroom IP65, deck, roof, stair)</t>
         </is>
       </c>
       <c r="E91" t="n">
-        <v>13</v>
+        <v>89</v>
       </c>
       <c r="F91" t="inlineStr">
         <is>
@@ -5190,7 +5190,7 @@
         </is>
       </c>
       <c r="G91" t="n">
-        <v>750</v>
+        <v>500</v>
       </c>
       <c r="H91" t="inlineStr">
         <is>
@@ -5203,7 +5203,7 @@
         </is>
       </c>
       <c r="J91" t="n">
-        <v>9750</v>
+        <v>44500</v>
       </c>
       <c r="K91" t="inlineStr">
         <is>
@@ -5229,11 +5229,11 @@
       </c>
       <c r="D92" t="inlineStr">
         <is>
-          <t>Cable 4.0 mm2 T+E/singles in conduit, Induction hob</t>
+          <t>Cable 2.5 mm2 T+E/singles in conduit, Sockets: bedside USB, living, deck</t>
         </is>
       </c>
       <c r="E92" t="n">
-        <v>8</v>
+        <v>29</v>
       </c>
       <c r="F92" t="inlineStr">
         <is>
@@ -5241,7 +5241,7 @@
         </is>
       </c>
       <c r="G92" t="n">
-        <v>1200</v>
+        <v>750</v>
       </c>
       <c r="H92" t="inlineStr">
         <is>
@@ -5254,7 +5254,7 @@
         </is>
       </c>
       <c r="J92" t="n">
-        <v>9600</v>
+        <v>21750</v>
       </c>
       <c r="K92" t="inlineStr">
         <is>
@@ -5280,11 +5280,11 @@
       </c>
       <c r="D93" t="inlineStr">
         <is>
-          <t>Cable 2.5 mm2 T+E/singles in conduit, 80 L water heater</t>
+          <t>Cable 2.5 mm2 T+E/singles in conduit, Kitchen sockets and fridge</t>
         </is>
       </c>
       <c r="E93" t="n">
-        <v>7</v>
+        <v>13</v>
       </c>
       <c r="F93" t="inlineStr">
         <is>
@@ -5305,7 +5305,7 @@
         </is>
       </c>
       <c r="J93" t="n">
-        <v>5250</v>
+        <v>9750</v>
       </c>
       <c r="K93" t="inlineStr">
         <is>
@@ -5331,11 +5331,11 @@
       </c>
       <c r="D94" t="inlineStr">
         <is>
-          <t>Cable 1.5 mm2 T+E/singles in conduit, Extract fan and wall fan</t>
+          <t>Cable 4.0 mm2 T+E/singles in conduit, Induction hob</t>
         </is>
       </c>
       <c r="E94" t="n">
-        <v>12</v>
+        <v>8</v>
       </c>
       <c r="F94" t="inlineStr">
         <is>
@@ -5343,7 +5343,7 @@
         </is>
       </c>
       <c r="G94" t="n">
-        <v>500</v>
+        <v>1200</v>
       </c>
       <c r="H94" t="inlineStr">
         <is>
@@ -5356,7 +5356,7 @@
         </is>
       </c>
       <c r="J94" t="n">
-        <v>6000</v>
+        <v>9600</v>
       </c>
       <c r="K94" t="inlineStr">
         <is>
@@ -5382,7 +5382,7 @@
       </c>
       <c r="D95" t="inlineStr">
         <is>
-          <t>Cable 2.5 mm2 T+E/singles in conduit, AC provision</t>
+          <t>Cable 2.5 mm2 T+E/singles in conduit, 80 L water heater</t>
         </is>
       </c>
       <c r="E95" t="n">
@@ -5433,11 +5433,11 @@
       </c>
       <c r="D96" t="inlineStr">
         <is>
-          <t>PVC conduit 20 mm + boxes</t>
+          <t>Cable 1.5 mm2 T+E/singles in conduit, Extract fan and wall fan</t>
         </is>
       </c>
       <c r="E96" t="n">
-        <v>60</v>
+        <v>8</v>
       </c>
       <c r="F96" t="inlineStr">
         <is>
@@ -5445,7 +5445,7 @@
         </is>
       </c>
       <c r="G96" t="n">
-        <v>600</v>
+        <v>500</v>
       </c>
       <c r="H96" t="inlineStr">
         <is>
@@ -5458,7 +5458,7 @@
         </is>
       </c>
       <c r="J96" t="n">
-        <v>36000</v>
+        <v>4000</v>
       </c>
       <c r="K96" t="inlineStr">
         <is>
@@ -5484,19 +5484,19 @@
       </c>
       <c r="D97" t="inlineStr">
         <is>
-          <t>Surge protection device type 2</t>
+          <t>Cable 2.5 mm2 T+E/singles in conduit, AC provision</t>
         </is>
       </c>
       <c r="E97" t="n">
-        <v>1</v>
+        <v>7</v>
       </c>
       <c r="F97" t="inlineStr">
         <is>
-          <t>each</t>
+          <t>m</t>
         </is>
       </c>
       <c r="G97" t="n">
-        <v>60000</v>
+        <v>750</v>
       </c>
       <c r="H97" t="inlineStr">
         <is>
@@ -5509,9 +5509,13 @@
         </is>
       </c>
       <c r="J97" t="n">
-        <v>60000</v>
-      </c>
-      <c r="K97" t="inlineStr"/>
+        <v>5250</v>
+      </c>
+      <c r="K97" t="inlineStr">
+        <is>
+          <t>per m</t>
+        </is>
+      </c>
     </row>
     <row r="98">
       <c r="A98" t="inlineStr">
@@ -5531,19 +5535,19 @@
       </c>
       <c r="D98" t="inlineStr">
         <is>
-          <t>RCD 40 A 30 mA type A (or RCBOs)</t>
+          <t>PVC conduit 20 mm + boxes</t>
         </is>
       </c>
       <c r="E98" t="n">
-        <v>1</v>
+        <v>60</v>
       </c>
       <c r="F98" t="inlineStr">
         <is>
-          <t>each</t>
+          <t>m</t>
         </is>
       </c>
       <c r="G98" t="n">
-        <v>45000</v>
+        <v>600</v>
       </c>
       <c r="H98" t="inlineStr">
         <is>
@@ -5556,9 +5560,13 @@
         </is>
       </c>
       <c r="J98" t="n">
-        <v>45000</v>
-      </c>
-      <c r="K98" t="inlineStr"/>
+        <v>36000</v>
+      </c>
+      <c r="K98" t="inlineStr">
+        <is>
+          <t>per m</t>
+        </is>
+      </c>
     </row>
     <row r="99">
       <c r="A99" t="inlineStr">
@@ -5578,11 +5586,11 @@
       </c>
       <c r="D99" t="inlineStr">
         <is>
-          <t>MCBs (B6 x2, B16 x5, B20 x1)</t>
+          <t>Surge protection device type 2</t>
         </is>
       </c>
       <c r="E99" t="n">
-        <v>8</v>
+        <v>1</v>
       </c>
       <c r="F99" t="inlineStr">
         <is>
@@ -5590,7 +5598,7 @@
         </is>
       </c>
       <c r="G99" t="n">
-        <v>6000</v>
+        <v>60000</v>
       </c>
       <c r="H99" t="inlineStr">
         <is>
@@ -5603,7 +5611,7 @@
         </is>
       </c>
       <c r="J99" t="n">
-        <v>48000</v>
+        <v>60000</v>
       </c>
       <c r="K99" t="inlineStr"/>
     </row>
@@ -5625,7 +5633,7 @@
       </c>
       <c r="D100" t="inlineStr">
         <is>
-          <t>Main switch 40 A DP + check meter (DIN kWh)</t>
+          <t>RCD 40 A 30 mA type A (or RCBOs)</t>
         </is>
       </c>
       <c r="E100" t="n">
@@ -5633,11 +5641,11 @@
       </c>
       <c r="F100" t="inlineStr">
         <is>
-          <t>set</t>
+          <t>each</t>
         </is>
       </c>
       <c r="G100" t="n">
-        <v>40000</v>
+        <v>45000</v>
       </c>
       <c r="H100" t="inlineStr">
         <is>
@@ -5650,7 +5658,7 @@
         </is>
       </c>
       <c r="J100" t="n">
-        <v>40000</v>
+        <v>45000</v>
       </c>
       <c r="K100" t="inlineStr"/>
     </row>
@@ -5672,11 +5680,11 @@
       </c>
       <c r="D101" t="inlineStr">
         <is>
-          <t>Earth rod 1.5 m copper-bonded + clamp + inspection pit</t>
+          <t>MCBs (B6 x2, B16 x5, B20 x1)</t>
         </is>
       </c>
       <c r="E101" t="n">
-        <v>1</v>
+        <v>8</v>
       </c>
       <c r="F101" t="inlineStr">
         <is>
@@ -5684,7 +5692,7 @@
         </is>
       </c>
       <c r="G101" t="n">
-        <v>35000</v>
+        <v>6000</v>
       </c>
       <c r="H101" t="inlineStr">
         <is>
@@ -5697,7 +5705,7 @@
         </is>
       </c>
       <c r="J101" t="n">
-        <v>35000</v>
+        <v>48000</v>
       </c>
       <c r="K101" t="inlineStr"/>
     </row>
@@ -5709,7 +5717,7 @@
       </c>
       <c r="B102" t="inlineStr">
         <is>
-          <t>safety</t>
+          <t>electrical</t>
         </is>
       </c>
       <c r="C102" t="inlineStr">
@@ -5719,19 +5727,19 @@
       </c>
       <c r="D102" t="inlineStr">
         <is>
-          <t>Smoke alarm (10-year) + heat alarm (kitchen)</t>
+          <t>Main switch 40 A DP + check meter (DIN kWh)</t>
         </is>
       </c>
       <c r="E102" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="F102" t="inlineStr">
         <is>
-          <t>each</t>
+          <t>set</t>
         </is>
       </c>
       <c r="G102" t="n">
-        <v>20000</v>
+        <v>40000</v>
       </c>
       <c r="H102" t="inlineStr">
         <is>
@@ -5756,17 +5764,17 @@
       </c>
       <c r="B103" t="inlineStr">
         <is>
-          <t>safety</t>
+          <t>electrical</t>
         </is>
       </c>
       <c r="C103" t="inlineStr">
         <is>
-          <t>furnishing</t>
+          <t>electrical</t>
         </is>
       </c>
       <c r="D103" t="inlineStr">
         <is>
-          <t>Fire extinguisher 2 kg ABC + fire blanket</t>
+          <t>Earth rod 1.5 m copper-bonded + clamp + inspection pit</t>
         </is>
       </c>
       <c r="E103" t="n">
@@ -5774,11 +5782,11 @@
       </c>
       <c r="F103" t="inlineStr">
         <is>
-          <t>set</t>
+          <t>each</t>
         </is>
       </c>
       <c r="G103" t="n">
-        <v>55000</v>
+        <v>35000</v>
       </c>
       <c r="H103" t="inlineStr">
         <is>
@@ -5791,41 +5799,41 @@
         </is>
       </c>
       <c r="J103" t="n">
-        <v>55000</v>
+        <v>35000</v>
       </c>
       <c r="K103" t="inlineStr"/>
     </row>
     <row r="104">
       <c r="A104" t="inlineStr">
         <is>
-          <t>K9</t>
+          <t>K8</t>
         </is>
       </c>
       <c r="B104" t="inlineStr">
         <is>
-          <t>plumbing</t>
+          <t>safety</t>
         </is>
       </c>
       <c r="C104" t="inlineStr">
         <is>
-          <t>plumbing</t>
+          <t>electrical</t>
         </is>
       </c>
       <c r="D104" t="inlineStr">
         <is>
-          <t>PPR PN20 pipe DN20</t>
+          <t>Smoke alarm (10-year) + heat alarm (kitchen)</t>
         </is>
       </c>
       <c r="E104" t="n">
-        <v>8.800000000000001</v>
+        <v>2</v>
       </c>
       <c r="F104" t="inlineStr">
         <is>
-          <t>m</t>
+          <t>each</t>
         </is>
       </c>
       <c r="G104" t="n">
-        <v>2000</v>
+        <v>20000</v>
       </c>
       <c r="H104" t="inlineStr">
         <is>
@@ -5838,45 +5846,41 @@
         </is>
       </c>
       <c r="J104" t="n">
-        <v>17600</v>
-      </c>
-      <c r="K104" t="inlineStr">
-        <is>
-          <t>per m</t>
-        </is>
-      </c>
+        <v>40000</v>
+      </c>
+      <c r="K104" t="inlineStr"/>
     </row>
     <row r="105">
       <c r="A105" t="inlineStr">
         <is>
-          <t>K9</t>
+          <t>K8</t>
         </is>
       </c>
       <c r="B105" t="inlineStr">
         <is>
-          <t>plumbing</t>
+          <t>safety</t>
         </is>
       </c>
       <c r="C105" t="inlineStr">
         <is>
-          <t>plumbing</t>
+          <t>furnishing</t>
         </is>
       </c>
       <c r="D105" t="inlineStr">
         <is>
-          <t>PPR PN20 pipe DN25</t>
+          <t>Fire extinguisher 2 kg ABC + fire blanket</t>
         </is>
       </c>
       <c r="E105" t="n">
-        <v>4.6</v>
+        <v>1</v>
       </c>
       <c r="F105" t="inlineStr">
         <is>
-          <t>m</t>
+          <t>set</t>
         </is>
       </c>
       <c r="G105" t="n">
-        <v>2800</v>
+        <v>55000</v>
       </c>
       <c r="H105" t="inlineStr">
         <is>
@@ -5889,13 +5893,9 @@
         </is>
       </c>
       <c r="J105" t="n">
-        <v>12880</v>
-      </c>
-      <c r="K105" t="inlineStr">
-        <is>
-          <t>per m</t>
-        </is>
-      </c>
+        <v>55000</v>
+      </c>
+      <c r="K105" t="inlineStr"/>
     </row>
     <row r="106">
       <c r="A106" t="inlineStr">
@@ -5915,11 +5915,11 @@
       </c>
       <c r="D106" t="inlineStr">
         <is>
-          <t>PPR PN20 pipe (hot) DN20</t>
+          <t>PPR PN20 pipe DN20</t>
         </is>
       </c>
       <c r="E106" t="n">
-        <v>4.5</v>
+        <v>8.4</v>
       </c>
       <c r="F106" t="inlineStr">
         <is>
@@ -5940,7 +5940,7 @@
         </is>
       </c>
       <c r="J106" t="n">
-        <v>9000</v>
+        <v>16800</v>
       </c>
       <c r="K106" t="inlineStr">
         <is>
@@ -5966,11 +5966,11 @@
       </c>
       <c r="D107" t="inlineStr">
         <is>
-          <t>uPVC soil pipe DN110</t>
+          <t>PPR PN20 pipe DN25</t>
         </is>
       </c>
       <c r="E107" t="n">
-        <v>4.2</v>
+        <v>4.6</v>
       </c>
       <c r="F107" t="inlineStr">
         <is>
@@ -5978,7 +5978,7 @@
         </is>
       </c>
       <c r="G107" t="n">
-        <v>7000</v>
+        <v>2800</v>
       </c>
       <c r="H107" t="inlineStr">
         <is>
@@ -5991,7 +5991,7 @@
         </is>
       </c>
       <c r="J107" t="n">
-        <v>29400</v>
+        <v>12880</v>
       </c>
       <c r="K107" t="inlineStr">
         <is>
@@ -6017,11 +6017,11 @@
       </c>
       <c r="D108" t="inlineStr">
         <is>
-          <t>PPR PN20 pipe (tempered) DN20</t>
+          <t>PPR PN20 pipe (hot) DN20</t>
         </is>
       </c>
       <c r="E108" t="n">
-        <v>5.5</v>
+        <v>4.5</v>
       </c>
       <c r="F108" t="inlineStr">
         <is>
@@ -6042,7 +6042,7 @@
         </is>
       </c>
       <c r="J108" t="n">
-        <v>11000</v>
+        <v>9000</v>
       </c>
       <c r="K108" t="inlineStr">
         <is>
@@ -6068,11 +6068,11 @@
       </c>
       <c r="D109" t="inlineStr">
         <is>
-          <t>uPVC vent pipe DN75</t>
+          <t>uPVC soil pipe DN110</t>
         </is>
       </c>
       <c r="E109" t="n">
-        <v>7.9</v>
+        <v>2.7</v>
       </c>
       <c r="F109" t="inlineStr">
         <is>
@@ -6080,7 +6080,7 @@
         </is>
       </c>
       <c r="G109" t="n">
-        <v>4500</v>
+        <v>7000</v>
       </c>
       <c r="H109" t="inlineStr">
         <is>
@@ -6093,7 +6093,7 @@
         </is>
       </c>
       <c r="J109" t="n">
-        <v>35550</v>
+        <v>18900</v>
       </c>
       <c r="K109" t="inlineStr">
         <is>
@@ -6119,11 +6119,11 @@
       </c>
       <c r="D110" t="inlineStr">
         <is>
-          <t>uPVC waste pipe DN40</t>
+          <t>PPR PN20 pipe (tempered) DN20</t>
         </is>
       </c>
       <c r="E110" t="n">
-        <v>1.5</v>
+        <v>6.4</v>
       </c>
       <c r="F110" t="inlineStr">
         <is>
@@ -6131,7 +6131,7 @@
         </is>
       </c>
       <c r="G110" t="n">
-        <v>2500</v>
+        <v>2000</v>
       </c>
       <c r="H110" t="inlineStr">
         <is>
@@ -6144,7 +6144,7 @@
         </is>
       </c>
       <c r="J110" t="n">
-        <v>3750</v>
+        <v>12800</v>
       </c>
       <c r="K110" t="inlineStr">
         <is>
@@ -6170,11 +6170,11 @@
       </c>
       <c r="D111" t="inlineStr">
         <is>
-          <t>uPVC waste pipe DN50</t>
+          <t>uPVC vent pipe DN75</t>
         </is>
       </c>
       <c r="E111" t="n">
-        <v>5.7</v>
+        <v>7.9</v>
       </c>
       <c r="F111" t="inlineStr">
         <is>
@@ -6182,7 +6182,7 @@
         </is>
       </c>
       <c r="G111" t="n">
-        <v>3000</v>
+        <v>4500</v>
       </c>
       <c r="H111" t="inlineStr">
         <is>
@@ -6195,7 +6195,7 @@
         </is>
       </c>
       <c r="J111" t="n">
-        <v>17100</v>
+        <v>35550</v>
       </c>
       <c r="K111" t="inlineStr">
         <is>
@@ -6221,19 +6221,19 @@
       </c>
       <c r="D112" t="inlineStr">
         <is>
-          <t>Pipe fittings and clips (allowance)</t>
+          <t>uPVC waste pipe DN40</t>
         </is>
       </c>
       <c r="E112" t="n">
-        <v>1</v>
+        <v>2.5</v>
       </c>
       <c r="F112" t="inlineStr">
         <is>
-          <t>set</t>
+          <t>m</t>
         </is>
       </c>
       <c r="G112" t="n">
-        <v>120000</v>
+        <v>2500</v>
       </c>
       <c r="H112" t="inlineStr">
         <is>
@@ -6246,9 +6246,13 @@
         </is>
       </c>
       <c r="J112" t="n">
-        <v>120000</v>
-      </c>
-      <c r="K112" t="inlineStr"/>
+        <v>6250</v>
+      </c>
+      <c r="K112" t="inlineStr">
+        <is>
+          <t>per m</t>
+        </is>
+      </c>
     </row>
     <row r="113">
       <c r="A113" t="inlineStr">
@@ -6268,19 +6272,19 @@
       </c>
       <c r="D113" t="inlineStr">
         <is>
-          <t>Thermostatic mixing valve (TMV) 41-44 C</t>
+          <t>uPVC waste pipe DN50</t>
         </is>
       </c>
       <c r="E113" t="n">
-        <v>1</v>
+        <v>5.7</v>
       </c>
       <c r="F113" t="inlineStr">
         <is>
-          <t>each</t>
+          <t>m</t>
         </is>
       </c>
       <c r="G113" t="n">
-        <v>60000</v>
+        <v>3000</v>
       </c>
       <c r="H113" t="inlineStr">
         <is>
@@ -6293,9 +6297,13 @@
         </is>
       </c>
       <c r="J113" t="n">
-        <v>60000</v>
-      </c>
-      <c r="K113" t="inlineStr"/>
+        <v>17100</v>
+      </c>
+      <c r="K113" t="inlineStr">
+        <is>
+          <t>per m</t>
+        </is>
+      </c>
     </row>
     <row r="114">
       <c r="A114" t="inlineStr">
@@ -6315,7 +6323,7 @@
       </c>
       <c r="D114" t="inlineStr">
         <is>
-          <t>Thermostatic shower valve + 6-7 L/min head + rail</t>
+          <t>Pipe fittings and clips (allowance)</t>
         </is>
       </c>
       <c r="E114" t="n">
@@ -6327,7 +6335,7 @@
         </is>
       </c>
       <c r="G114" t="n">
-        <v>90000</v>
+        <v>120000</v>
       </c>
       <c r="H114" t="inlineStr">
         <is>
@@ -6340,7 +6348,7 @@
         </is>
       </c>
       <c r="J114" t="n">
-        <v>90000</v>
+        <v>120000</v>
       </c>
       <c r="K114" t="inlineStr"/>
     </row>
@@ -6362,7 +6370,7 @@
       </c>
       <c r="D115" t="inlineStr">
         <is>
-          <t>Electric storage water heater 80 L, 2 kW, with T&amp;P valve</t>
+          <t>Thermostatic mixing valve (TMV) 41-44 C</t>
         </is>
       </c>
       <c r="E115" t="n">
@@ -6374,7 +6382,7 @@
         </is>
       </c>
       <c r="G115" t="n">
-        <v>300000</v>
+        <v>60000</v>
       </c>
       <c r="H115" t="inlineStr">
         <is>
@@ -6387,13 +6395,9 @@
         </is>
       </c>
       <c r="J115" t="n">
-        <v>300000</v>
-      </c>
-      <c r="K115" t="inlineStr">
-        <is>
-          <t>80 L not found; 50 L listed at RWF 144,000-252,000 (STU-P01, STU-P02)</t>
-        </is>
-      </c>
+        <v>60000</v>
+      </c>
+      <c r="K115" t="inlineStr"/>
     </row>
     <row r="116">
       <c r="A116" t="inlineStr">
@@ -6413,19 +6417,19 @@
       </c>
       <c r="D116" t="inlineStr">
         <is>
-          <t>Angle valves with filters</t>
+          <t>Thermostatic shower valve + 6-7 L/min head + rail</t>
         </is>
       </c>
       <c r="E116" t="n">
-        <v>5</v>
+        <v>1</v>
       </c>
       <c r="F116" t="inlineStr">
         <is>
-          <t>each</t>
+          <t>set</t>
         </is>
       </c>
       <c r="G116" t="n">
-        <v>6000</v>
+        <v>90000</v>
       </c>
       <c r="H116" t="inlineStr">
         <is>
@@ -6438,7 +6442,7 @@
         </is>
       </c>
       <c r="J116" t="n">
-        <v>30000</v>
+        <v>90000</v>
       </c>
       <c r="K116" t="inlineStr"/>
     </row>
@@ -6460,7 +6464,7 @@
       </c>
       <c r="D117" t="inlineStr">
         <is>
-          <t>Air admittance valve 110 mm (spare) + rodding eyes</t>
+          <t>Electric storage water heater 80 L, 2 kW, with T&amp;P valve</t>
         </is>
       </c>
       <c r="E117" t="n">
@@ -6468,11 +6472,11 @@
       </c>
       <c r="F117" t="inlineStr">
         <is>
-          <t>set</t>
+          <t>each</t>
         </is>
       </c>
       <c r="G117" t="n">
-        <v>30000</v>
+        <v>300000</v>
       </c>
       <c r="H117" t="inlineStr">
         <is>
@@ -6485,9 +6489,13 @@
         </is>
       </c>
       <c r="J117" t="n">
-        <v>30000</v>
-      </c>
-      <c r="K117" t="inlineStr"/>
+        <v>300000</v>
+      </c>
+      <c r="K117" t="inlineStr">
+        <is>
+          <t>80 L not found; 50 L listed at RWF 144,000-252,000 (STU-P01, STU-P02)</t>
+        </is>
+      </c>
     </row>
     <row r="118">
       <c r="A118" t="inlineStr">
@@ -6507,19 +6515,19 @@
       </c>
       <c r="D118" t="inlineStr">
         <is>
-          <t>Stop valve + Y-filter + check water meter</t>
+          <t>Angle valves with filters</t>
         </is>
       </c>
       <c r="E118" t="n">
-        <v>1</v>
+        <v>5</v>
       </c>
       <c r="F118" t="inlineStr">
         <is>
-          <t>set</t>
+          <t>each</t>
         </is>
       </c>
       <c r="G118" t="n">
-        <v>45000</v>
+        <v>6000</v>
       </c>
       <c r="H118" t="inlineStr">
         <is>
@@ -6532,29 +6540,29 @@
         </is>
       </c>
       <c r="J118" t="n">
-        <v>45000</v>
+        <v>30000</v>
       </c>
       <c r="K118" t="inlineStr"/>
     </row>
     <row r="119">
       <c r="A119" t="inlineStr">
         <is>
-          <t>K10</t>
+          <t>K9</t>
         </is>
       </c>
       <c r="B119" t="inlineStr">
         <is>
-          <t>steel</t>
+          <t>plumbing</t>
         </is>
       </c>
       <c r="C119" t="inlineStr">
         <is>
-          <t>welding</t>
+          <t>plumbing</t>
         </is>
       </c>
       <c r="D119" t="inlineStr">
         <is>
-          <t>W1 infill: 2 mm steel + 40 mm EPS, welded into the old door frame (0-1,150)</t>
+          <t>Air admittance valve 110 mm (spare) + rodding eyes</t>
         </is>
       </c>
       <c r="E119" t="n">
@@ -6562,11 +6570,11 @@
       </c>
       <c r="F119" t="inlineStr">
         <is>
-          <t>each</t>
+          <t>set</t>
         </is>
       </c>
       <c r="G119" t="n">
-        <v>180000</v>
+        <v>30000</v>
       </c>
       <c r="H119" t="inlineStr">
         <is>
@@ -6579,33 +6587,29 @@
         </is>
       </c>
       <c r="J119" t="n">
-        <v>180000</v>
-      </c>
-      <c r="K119" t="inlineStr">
-        <is>
-          <t>incl. welding</t>
-        </is>
-      </c>
+        <v>30000</v>
+      </c>
+      <c r="K119" t="inlineStr"/>
     </row>
     <row r="120">
       <c r="A120" t="inlineStr">
         <is>
-          <t>K10</t>
+          <t>K9</t>
         </is>
       </c>
       <c r="B120" t="inlineStr">
         <is>
-          <t>glazing</t>
+          <t>plumbing</t>
         </is>
       </c>
       <c r="C120" t="inlineStr">
         <is>
-          <t>glazier</t>
+          <t>plumbing</t>
         </is>
       </c>
       <c r="D120" t="inlineStr">
         <is>
-          <t>W1 obscure louvre window 520 x 890 + insect mesh + fan panel</t>
+          <t>Stop valve + Y-filter + check water meter</t>
         </is>
       </c>
       <c r="E120" t="n">
@@ -6613,11 +6617,11 @@
       </c>
       <c r="F120" t="inlineStr">
         <is>
-          <t>each</t>
+          <t>set</t>
         </is>
       </c>
       <c r="G120" t="n">
-        <v>120000</v>
+        <v>45000</v>
       </c>
       <c r="H120" t="inlineStr">
         <is>
@@ -6630,7 +6634,7 @@
         </is>
       </c>
       <c r="J120" t="n">
-        <v>120000</v>
+        <v>45000</v>
       </c>
       <c r="K120" t="inlineStr"/>
     </row>
@@ -6652,7 +6656,7 @@
       </c>
       <c r="D121" t="inlineStr">
         <is>
-          <t>Seal and lock the end-B cargo doors (weld tabs, sealant)</t>
+          <t>W1 infill: 2 mm steel + 40 mm EPS, welded into the old door frame (0-1,150)</t>
         </is>
       </c>
       <c r="E121" t="n">
@@ -6664,7 +6668,7 @@
         </is>
       </c>
       <c r="G121" t="n">
-        <v>60000</v>
+        <v>180000</v>
       </c>
       <c r="H121" t="inlineStr">
         <is>
@@ -6677,9 +6681,13 @@
         </is>
       </c>
       <c r="J121" t="n">
-        <v>60000</v>
-      </c>
-      <c r="K121" t="inlineStr"/>
+        <v>180000</v>
+      </c>
+      <c r="K121" t="inlineStr">
+        <is>
+          <t>incl. welding</t>
+        </is>
+      </c>
     </row>
     <row r="122">
       <c r="A122" t="inlineStr">
@@ -6689,21 +6697,21 @@
       </c>
       <c r="B122" t="inlineStr">
         <is>
-          <t>steel</t>
+          <t>glazing</t>
         </is>
       </c>
       <c r="C122" t="inlineStr">
         <is>
-          <t>masonry</t>
+          <t>glazier</t>
         </is>
       </c>
       <c r="D122" t="inlineStr">
         <is>
-          <t>Level the corner castings: concrete pads or steel shims (rock corner)</t>
+          <t>W1 obscure louvre window 520 x 890 + insect mesh (wash lobby)</t>
         </is>
       </c>
       <c r="E122" t="n">
-        <v>4</v>
+        <v>1</v>
       </c>
       <c r="F122" t="inlineStr">
         <is>
@@ -6711,7 +6719,7 @@
         </is>
       </c>
       <c r="G122" t="n">
-        <v>25000</v>
+        <v>120000</v>
       </c>
       <c r="H122" t="inlineStr">
         <is>
@@ -6724,7 +6732,7 @@
         </is>
       </c>
       <c r="J122" t="n">
-        <v>100000</v>
+        <v>120000</v>
       </c>
       <c r="K122" t="inlineStr"/>
     </row>
@@ -6746,7 +6754,7 @@
       </c>
       <c r="D123" t="inlineStr">
         <is>
-          <t>Steel hanging rail for wall units + heater bracket</t>
+          <t>Seal and lock the end-B cargo doors (weld tabs, sealant)</t>
         </is>
       </c>
       <c r="E123" t="n">
@@ -6754,11 +6762,11 @@
       </c>
       <c r="F123" t="inlineStr">
         <is>
-          <t>set</t>
+          <t>each</t>
         </is>
       </c>
       <c r="G123" t="n">
-        <v>40000</v>
+        <v>60000</v>
       </c>
       <c r="H123" t="inlineStr">
         <is>
@@ -6771,7 +6779,7 @@
         </is>
       </c>
       <c r="J123" t="n">
-        <v>40000</v>
+        <v>60000</v>
       </c>
       <c r="K123" t="inlineStr"/>
     </row>
@@ -6783,29 +6791,29 @@
       </c>
       <c r="B124" t="inlineStr">
         <is>
-          <t>hardware</t>
+          <t>steel</t>
         </is>
       </c>
       <c r="C124" t="inlineStr">
         <is>
-          <t>glazier</t>
+          <t>masonry</t>
         </is>
       </c>
       <c r="D124" t="inlineStr">
         <is>
-          <t>Keyed lock + secondary bolt for the slider</t>
+          <t>Level the corner castings: concrete pads or steel shims (rock corner)</t>
         </is>
       </c>
       <c r="E124" t="n">
-        <v>1</v>
+        <v>4</v>
       </c>
       <c r="F124" t="inlineStr">
         <is>
-          <t>set</t>
+          <t>each</t>
         </is>
       </c>
       <c r="G124" t="n">
-        <v>45000</v>
+        <v>25000</v>
       </c>
       <c r="H124" t="inlineStr">
         <is>
@@ -6818,7 +6826,7 @@
         </is>
       </c>
       <c r="J124" t="n">
-        <v>45000</v>
+        <v>100000</v>
       </c>
       <c r="K124" t="inlineStr"/>
     </row>
@@ -6830,17 +6838,17 @@
       </c>
       <c r="B125" t="inlineStr">
         <is>
-          <t>glazing</t>
+          <t>steel</t>
         </is>
       </c>
       <c r="C125" t="inlineStr">
         <is>
-          <t>glazier</t>
+          <t>welding</t>
         </is>
       </c>
       <c r="D125" t="inlineStr">
         <is>
-          <t>Louvred trickle-vent strip with mesh (10,000 mm2)</t>
+          <t>Steel hanging rail for wall units + heater bracket</t>
         </is>
       </c>
       <c r="E125" t="n">
@@ -6848,11 +6856,11 @@
       </c>
       <c r="F125" t="inlineStr">
         <is>
-          <t>each</t>
+          <t>set</t>
         </is>
       </c>
       <c r="G125" t="n">
-        <v>30000</v>
+        <v>40000</v>
       </c>
       <c r="H125" t="inlineStr">
         <is>
@@ -6865,7 +6873,7 @@
         </is>
       </c>
       <c r="J125" t="n">
-        <v>30000</v>
+        <v>40000</v>
       </c>
       <c r="K125" t="inlineStr"/>
     </row>
@@ -6877,17 +6885,17 @@
       </c>
       <c r="B126" t="inlineStr">
         <is>
-          <t>steel</t>
+          <t>hardware</t>
         </is>
       </c>
       <c r="C126" t="inlineStr">
         <is>
-          <t>welding</t>
+          <t>glazier</t>
         </is>
       </c>
       <c r="D126" t="inlineStr">
         <is>
-          <t>AC wall sleeve 75 mm (provision, back wall, one hole)</t>
+          <t>Keyed lock + secondary bolt for the slider</t>
         </is>
       </c>
       <c r="E126" t="n">
@@ -6895,11 +6903,11 @@
       </c>
       <c r="F126" t="inlineStr">
         <is>
-          <t>each</t>
+          <t>set</t>
         </is>
       </c>
       <c r="G126" t="n">
-        <v>15000</v>
+        <v>45000</v>
       </c>
       <c r="H126" t="inlineStr">
         <is>
@@ -6912,29 +6920,29 @@
         </is>
       </c>
       <c r="J126" t="n">
-        <v>15000</v>
+        <v>45000</v>
       </c>
       <c r="K126" t="inlineStr"/>
     </row>
     <row r="127">
       <c r="A127" t="inlineStr">
         <is>
-          <t>K11</t>
+          <t>K10</t>
         </is>
       </c>
       <c r="B127" t="inlineStr">
         <is>
-          <t>roofing</t>
+          <t>glazing</t>
         </is>
       </c>
       <c r="C127" t="inlineStr">
         <is>
-          <t>welding</t>
+          <t>glazier</t>
         </is>
       </c>
       <c r="D127" t="inlineStr">
         <is>
-          <t>Gutter + downpipe to the rainwater tank (deck canopy)</t>
+          <t>Louvred trickle-vent strip with mesh (10,000 mm2)</t>
         </is>
       </c>
       <c r="E127" t="n">
@@ -6942,11 +6950,11 @@
       </c>
       <c r="F127" t="inlineStr">
         <is>
-          <t>set</t>
+          <t>each</t>
         </is>
       </c>
       <c r="G127" t="n">
-        <v>90000</v>
+        <v>30000</v>
       </c>
       <c r="H127" t="inlineStr">
         <is>
@@ -6959,29 +6967,29 @@
         </is>
       </c>
       <c r="J127" t="n">
-        <v>90000</v>
+        <v>30000</v>
       </c>
       <c r="K127" t="inlineStr"/>
     </row>
     <row r="128">
       <c r="A128" t="inlineStr">
         <is>
-          <t>K11</t>
+          <t>K10</t>
         </is>
       </c>
       <c r="B128" t="inlineStr">
         <is>
-          <t>electrical</t>
+          <t>steel</t>
         </is>
       </c>
       <c r="C128" t="inlineStr">
         <is>
-          <t>electrical</t>
+          <t>welding</t>
         </is>
       </c>
       <c r="D128" t="inlineStr">
         <is>
-          <t>Bonding: 16 mm2 green-yellow from the frame to the earth bar</t>
+          <t>AC wall sleeve 75 mm (provision, back wall, one hole)</t>
         </is>
       </c>
       <c r="E128" t="n">
@@ -6989,11 +6997,11 @@
       </c>
       <c r="F128" t="inlineStr">
         <is>
-          <t>set</t>
+          <t>each</t>
         </is>
       </c>
       <c r="G128" t="n">
-        <v>25000</v>
+        <v>15000</v>
       </c>
       <c r="H128" t="inlineStr">
         <is>
@@ -7006,41 +7014,41 @@
         </is>
       </c>
       <c r="J128" t="n">
-        <v>25000</v>
+        <v>15000</v>
       </c>
       <c r="K128" t="inlineStr"/>
     </row>
     <row r="129">
       <c r="A129" t="inlineStr">
         <is>
-          <t>K1</t>
+          <t>K11</t>
         </is>
       </c>
       <c r="B129" t="inlineStr">
         <is>
-          <t>timber</t>
+          <t>roofing</t>
         </is>
       </c>
       <c r="C129" t="inlineStr">
         <is>
-          <t>carpentry</t>
+          <t>welding</t>
         </is>
       </c>
       <c r="D129" t="inlineStr">
         <is>
-          <t>Battens 38 x 50 treated, 2.4 m</t>
+          <t>Gutter + downpipe to the rainwater tank (deck canopy)</t>
         </is>
       </c>
       <c r="E129" t="n">
-        <v>19.8</v>
+        <v>1</v>
       </c>
       <c r="F129" t="inlineStr">
         <is>
-          <t>each</t>
+          <t>set</t>
         </is>
       </c>
       <c r="G129" t="n">
-        <v>2500</v>
+        <v>90000</v>
       </c>
       <c r="H129" t="inlineStr">
         <is>
@@ -7053,45 +7061,41 @@
         </is>
       </c>
       <c r="J129" t="n">
-        <v>49500</v>
-      </c>
-      <c r="K129" t="inlineStr">
-        <is>
-          <t>38 x 50 treated, 2.4 m</t>
-        </is>
-      </c>
+        <v>90000</v>
+      </c>
+      <c r="K129" t="inlineStr"/>
     </row>
     <row r="130">
       <c r="A130" t="inlineStr">
         <is>
-          <t>K2</t>
+          <t>K11</t>
         </is>
       </c>
       <c r="B130" t="inlineStr">
         <is>
-          <t>timber</t>
+          <t>electrical</t>
         </is>
       </c>
       <c r="C130" t="inlineStr">
         <is>
-          <t>carpentry</t>
+          <t>electrical</t>
         </is>
       </c>
       <c r="D130" t="inlineStr">
         <is>
-          <t>Studs 40 x 40 treated, 2.4 m</t>
+          <t>Bonding: 16 mm2 green-yellow from the frame to the earth bar</t>
         </is>
       </c>
       <c r="E130" t="n">
-        <v>5.5</v>
+        <v>1</v>
       </c>
       <c r="F130" t="inlineStr">
         <is>
-          <t>each</t>
+          <t>set</t>
         </is>
       </c>
       <c r="G130" t="n">
-        <v>3000</v>
+        <v>25000</v>
       </c>
       <c r="H130" t="inlineStr">
         <is>
@@ -7104,41 +7108,41 @@
         </is>
       </c>
       <c r="J130" t="n">
-        <v>16500</v>
-      </c>
-      <c r="K130" t="inlineStr">
-        <is>
-          <t>40 x 40, 2.4 m</t>
-        </is>
-      </c>
+        <v>25000</v>
+      </c>
+      <c r="K130" t="inlineStr"/>
     </row>
     <row r="131">
       <c r="A131" t="inlineStr">
         <is>
-          <t>labour</t>
+          <t>K1</t>
         </is>
       </c>
       <c r="B131" t="inlineStr">
         <is>
-          <t>labour</t>
-        </is>
-      </c>
-      <c r="C131" t="inlineStr"/>
+          <t>timber</t>
+        </is>
+      </c>
+      <c r="C131" t="inlineStr">
+        <is>
+          <t>carpentry</t>
+        </is>
+      </c>
       <c r="D131" t="inlineStr">
         <is>
-          <t>Carpentry workshop: cutting, edging, drilling, labelling (per unit kit)</t>
+          <t>Battens 38 x 50 treated, 2.4 m</t>
         </is>
       </c>
       <c r="E131" t="n">
-        <v>1</v>
+        <v>19.8</v>
       </c>
       <c r="F131" t="inlineStr">
         <is>
-          <t>lot</t>
+          <t>each</t>
         </is>
       </c>
       <c r="G131" t="n">
-        <v>450000</v>
+        <v>2500</v>
       </c>
       <c r="H131" t="inlineStr">
         <is>
@@ -7151,37 +7155,45 @@
         </is>
       </c>
       <c r="J131" t="n">
-        <v>450000</v>
-      </c>
-      <c r="K131" t="inlineStr"/>
+        <v>49500</v>
+      </c>
+      <c r="K131" t="inlineStr">
+        <is>
+          <t>38 x 50 treated, 2.4 m</t>
+        </is>
+      </c>
     </row>
     <row r="132">
       <c r="A132" t="inlineStr">
         <is>
-          <t>labour</t>
+          <t>K2</t>
         </is>
       </c>
       <c r="B132" t="inlineStr">
         <is>
-          <t>labour</t>
-        </is>
-      </c>
-      <c r="C132" t="inlineStr"/>
+          <t>timber</t>
+        </is>
+      </c>
+      <c r="C132" t="inlineStr">
+        <is>
+          <t>carpentry</t>
+        </is>
+      </c>
       <c r="D132" t="inlineStr">
         <is>
-          <t>Site carpentry and assembly: 2 people x 8 days</t>
+          <t>Studs 40 x 40 treated, 2.4 m</t>
         </is>
       </c>
       <c r="E132" t="n">
-        <v>1</v>
+        <v>6.6</v>
       </c>
       <c r="F132" t="inlineStr">
         <is>
-          <t>lot</t>
+          <t>each</t>
         </is>
       </c>
       <c r="G132" t="n">
-        <v>320000</v>
+        <v>3000</v>
       </c>
       <c r="H132" t="inlineStr">
         <is>
@@ -7194,9 +7206,13 @@
         </is>
       </c>
       <c r="J132" t="n">
-        <v>320000</v>
-      </c>
-      <c r="K132" t="inlineStr"/>
+        <v>19800</v>
+      </c>
+      <c r="K132" t="inlineStr">
+        <is>
+          <t>40 x 40, 2.4 m</t>
+        </is>
+      </c>
     </row>
     <row r="133">
       <c r="A133" t="inlineStr">
@@ -7212,7 +7228,7 @@
       <c r="C133" t="inlineStr"/>
       <c r="D133" t="inlineStr">
         <is>
-          <t>Electrician (RURA class A), install + certificate</t>
+          <t>Carpentry workshop: cutting, edging, drilling, labelling (per unit kit)</t>
         </is>
       </c>
       <c r="E133" t="n">
@@ -7224,7 +7240,7 @@
         </is>
       </c>
       <c r="G133" t="n">
-        <v>250000</v>
+        <v>450000</v>
       </c>
       <c r="H133" t="inlineStr">
         <is>
@@ -7237,7 +7253,7 @@
         </is>
       </c>
       <c r="J133" t="n">
-        <v>250000</v>
+        <v>450000</v>
       </c>
       <c r="K133" t="inlineStr"/>
     </row>
@@ -7255,7 +7271,7 @@
       <c r="C134" t="inlineStr"/>
       <c r="D134" t="inlineStr">
         <is>
-          <t>Plumber, install + tests</t>
+          <t>Site carpentry and assembly: 2 people x 8 days</t>
         </is>
       </c>
       <c r="E134" t="n">
@@ -7267,7 +7283,7 @@
         </is>
       </c>
       <c r="G134" t="n">
-        <v>200000</v>
+        <v>320000</v>
       </c>
       <c r="H134" t="inlineStr">
         <is>
@@ -7280,7 +7296,7 @@
         </is>
       </c>
       <c r="J134" t="n">
-        <v>200000</v>
+        <v>320000</v>
       </c>
       <c r="K134" t="inlineStr"/>
     </row>
@@ -7298,7 +7314,7 @@
       <c r="C135" t="inlineStr"/>
       <c r="D135" t="inlineStr">
         <is>
-          <t>Tiler: wet walls and floor</t>
+          <t>Electrician (RURA class A), install + certificate</t>
         </is>
       </c>
       <c r="E135" t="n">
@@ -7310,7 +7326,7 @@
         </is>
       </c>
       <c r="G135" t="n">
-        <v>150000</v>
+        <v>250000</v>
       </c>
       <c r="H135" t="inlineStr">
         <is>
@@ -7323,7 +7339,7 @@
         </is>
       </c>
       <c r="J135" t="n">
-        <v>150000</v>
+        <v>250000</v>
       </c>
       <c r="K135" t="inlineStr"/>
     </row>
@@ -7341,7 +7357,7 @@
       <c r="C136" t="inlineStr"/>
       <c r="D136" t="inlineStr">
         <is>
-          <t>Welder: W1, roof frame, deck canopy, stair (per unit)</t>
+          <t>Plumber, install + tests</t>
         </is>
       </c>
       <c r="E136" t="n">
@@ -7353,7 +7369,7 @@
         </is>
       </c>
       <c r="G136" t="n">
-        <v>600000</v>
+        <v>200000</v>
       </c>
       <c r="H136" t="inlineStr">
         <is>
@@ -7366,7 +7382,7 @@
         </is>
       </c>
       <c r="J136" t="n">
-        <v>600000</v>
+        <v>200000</v>
       </c>
       <c r="K136" t="inlineStr"/>
     </row>
@@ -7384,7 +7400,7 @@
       <c r="C137" t="inlineStr"/>
       <c r="D137" t="inlineStr">
         <is>
-          <t>Transport Kigali to site (share of 2 truck trips)</t>
+          <t>Tiler: wet walls and floor</t>
         </is>
       </c>
       <c r="E137" t="n">
@@ -7396,22 +7412,108 @@
         </is>
       </c>
       <c r="G137" t="n">
+        <v>150000</v>
+      </c>
+      <c r="H137" t="inlineStr">
+        <is>
+          <t>A</t>
+        </is>
+      </c>
+      <c r="I137" t="inlineStr">
+        <is>
+          <t>AS-21</t>
+        </is>
+      </c>
+      <c r="J137" t="n">
+        <v>150000</v>
+      </c>
+      <c r="K137" t="inlineStr"/>
+    </row>
+    <row r="138">
+      <c r="A138" t="inlineStr">
+        <is>
+          <t>labour</t>
+        </is>
+      </c>
+      <c r="B138" t="inlineStr">
+        <is>
+          <t>labour</t>
+        </is>
+      </c>
+      <c r="C138" t="inlineStr"/>
+      <c r="D138" t="inlineStr">
+        <is>
+          <t>Welder: W1, roof frame, deck canopy, stair (per unit)</t>
+        </is>
+      </c>
+      <c r="E138" t="n">
+        <v>1</v>
+      </c>
+      <c r="F138" t="inlineStr">
+        <is>
+          <t>lot</t>
+        </is>
+      </c>
+      <c r="G138" t="n">
+        <v>600000</v>
+      </c>
+      <c r="H138" t="inlineStr">
+        <is>
+          <t>A</t>
+        </is>
+      </c>
+      <c r="I138" t="inlineStr">
+        <is>
+          <t>AS-21</t>
+        </is>
+      </c>
+      <c r="J138" t="n">
+        <v>600000</v>
+      </c>
+      <c r="K138" t="inlineStr"/>
+    </row>
+    <row r="139">
+      <c r="A139" t="inlineStr">
+        <is>
+          <t>labour</t>
+        </is>
+      </c>
+      <c r="B139" t="inlineStr">
+        <is>
+          <t>labour</t>
+        </is>
+      </c>
+      <c r="C139" t="inlineStr"/>
+      <c r="D139" t="inlineStr">
+        <is>
+          <t>Transport Kigali to site (share of 2 truck trips)</t>
+        </is>
+      </c>
+      <c r="E139" t="n">
+        <v>1</v>
+      </c>
+      <c r="F139" t="inlineStr">
+        <is>
+          <t>lot</t>
+        </is>
+      </c>
+      <c r="G139" t="n">
         <v>120000</v>
       </c>
-      <c r="H137" t="inlineStr">
-        <is>
-          <t>A</t>
-        </is>
-      </c>
-      <c r="I137" t="inlineStr">
-        <is>
-          <t>AS-21</t>
-        </is>
-      </c>
-      <c r="J137" t="n">
+      <c r="H139" t="inlineStr">
+        <is>
+          <t>A</t>
+        </is>
+      </c>
+      <c r="I139" t="inlineStr">
+        <is>
+          <t>AS-21</t>
+        </is>
+      </c>
+      <c r="J139" t="n">
         <v>120000</v>
       </c>
-      <c r="K137" t="inlineStr"/>
+      <c r="K139" t="inlineStr"/>
     </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>

</xml_diff>

<commit_message>
feat(studio): narrower bathroom, low wide sofa, full-width 2D plan
The bathroom is now only as long as a short-projection WC and its
600 mm front zone need (1,150 mm), with a 1,000 x 900 shower and a
600 mm door opening into the bathroom; the partition and galley move
about 170 mm toward end B. Because the bathroom, not the glazing, now
places the partition, the survey band no longer moves the layout.
The sofa is lower and wider (1,300 x 750, 700 high) and the seating
group sits centred with about 110 mm to the bed and a 909 mm aisle,
the chairs well back from the glass. The 2D section drops the size
list and shows the plan across the full width.

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01KRyNxX68L5feJKbJnBKRyV
</commit_message>
<xml_diff>
--- a/public/designs/studio/data/bom.xlsx
+++ b/public/designs/studio/data/bom.xlsx
@@ -504,10 +504,10 @@
         </is>
       </c>
       <c r="B8" t="n">
-        <v>884280</v>
+        <v>882020</v>
       </c>
       <c r="C8" t="n">
-        <v>2652840</v>
+        <v>2646060</v>
       </c>
     </row>
     <row r="9">
@@ -517,10 +517,10 @@
         </is>
       </c>
       <c r="B9" t="n">
-        <v>755100</v>
+        <v>757350</v>
       </c>
       <c r="C9" t="n">
-        <v>2265300</v>
+        <v>2272050</v>
       </c>
     </row>
     <row r="10">
@@ -556,10 +556,10 @@
         </is>
       </c>
       <c r="B12" t="n">
-        <v>538100</v>
+        <v>537800</v>
       </c>
       <c r="C12" t="n">
-        <v>1614300</v>
+        <v>1613400</v>
       </c>
     </row>
     <row r="13">
@@ -582,10 +582,10 @@
         </is>
       </c>
       <c r="B14" t="n">
-        <v>478680</v>
+        <v>454000</v>
       </c>
       <c r="C14" t="n">
-        <v>1436040</v>
+        <v>1362000</v>
       </c>
     </row>
     <row r="15">
@@ -699,10 +699,10 @@
         </is>
       </c>
       <c r="B23" t="n">
-        <v>69300</v>
+        <v>66000</v>
       </c>
       <c r="C23" t="n">
-        <v>207900</v>
+        <v>198000</v>
       </c>
     </row>
     <row r="24">
@@ -736,10 +736,10 @@
         </is>
       </c>
       <c r="B26" t="n">
-        <v>1995237</v>
+        <v>1990993</v>
       </c>
       <c r="C26" t="n">
-        <v>6714110</v>
+        <v>6701379</v>
       </c>
     </row>
     <row r="27">
@@ -749,10 +749,10 @@
         </is>
       </c>
       <c r="B27" t="n">
-        <v>15296814</v>
+        <v>15264280</v>
       </c>
       <c r="C27" t="n">
-        <v>51474841</v>
+        <v>51377240</v>
       </c>
     </row>
     <row r="29">
@@ -763,7 +763,7 @@
       </c>
       <c r="B29" t="inlineStr"/>
       <c r="C29" t="n">
-        <v>34877</v>
+        <v>34811</v>
       </c>
     </row>
   </sheetData>
@@ -2145,7 +2145,7 @@
         </is>
       </c>
       <c r="E28" t="n">
-        <v>10.7</v>
+        <v>11.1</v>
       </c>
       <c r="F28" t="inlineStr">
         <is>
@@ -2166,7 +2166,7 @@
         </is>
       </c>
       <c r="J28" t="n">
-        <v>192600</v>
+        <v>199800</v>
       </c>
       <c r="K28" t="inlineStr">
         <is>
@@ -2294,7 +2294,7 @@
       </c>
       <c r="D31" t="inlineStr">
         <is>
-          <t>Sliding door leaf 640 x 2,050 on a top track, moisture-resistant, privacy latch</t>
+          <t>Door leaf 564 x 2,030, moisture-resistant, opens into the bathroom, privacy lock</t>
         </is>
       </c>
       <c r="E31" t="n">
@@ -2345,7 +2345,7 @@
         </is>
       </c>
       <c r="E32" t="n">
-        <v>3.06</v>
+        <v>2.67</v>
       </c>
       <c r="F32" t="inlineStr">
         <is>
@@ -2366,7 +2366,7 @@
         </is>
       </c>
       <c r="J32" t="n">
-        <v>42840</v>
+        <v>37380</v>
       </c>
       <c r="K32" t="inlineStr">
         <is>
@@ -2396,7 +2396,7 @@
         </is>
       </c>
       <c r="E33" t="n">
-        <v>3.37</v>
+        <v>2.94</v>
       </c>
       <c r="F33" t="inlineStr">
         <is>
@@ -2417,7 +2417,7 @@
         </is>
       </c>
       <c r="J33" t="n">
-        <v>53920</v>
+        <v>47040</v>
       </c>
       <c r="K33" t="inlineStr">
         <is>
@@ -2651,7 +2651,7 @@
         </is>
       </c>
       <c r="E38" t="n">
-        <v>3.06</v>
+        <v>2.67</v>
       </c>
       <c r="F38" t="inlineStr">
         <is>
@@ -2672,7 +2672,7 @@
         </is>
       </c>
       <c r="J38" t="n">
-        <v>42840</v>
+        <v>37380</v>
       </c>
       <c r="K38" t="inlineStr">
         <is>
@@ -2702,7 +2702,7 @@
         </is>
       </c>
       <c r="E39" t="n">
-        <v>3.37</v>
+        <v>2.94</v>
       </c>
       <c r="F39" t="inlineStr">
         <is>
@@ -2723,7 +2723,7 @@
         </is>
       </c>
       <c r="J39" t="n">
-        <v>53920</v>
+        <v>47040</v>
       </c>
       <c r="K39" t="inlineStr">
         <is>
@@ -2855,7 +2855,7 @@
         </is>
       </c>
       <c r="E42" t="n">
-        <v>3.7</v>
+        <v>3.2</v>
       </c>
       <c r="F42" t="inlineStr">
         <is>
@@ -2876,7 +2876,7 @@
         </is>
       </c>
       <c r="J42" t="n">
-        <v>55500</v>
+        <v>48000</v>
       </c>
       <c r="K42" t="inlineStr">
         <is>
@@ -2902,7 +2902,7 @@
       </c>
       <c r="D43" t="inlineStr">
         <is>
-          <t>Shower tray 1200 x 900, low profile, 90 mm waste</t>
+          <t>Shower tray 1000 x 900, low profile, 90 mm waste</t>
         </is>
       </c>
       <c r="E43" t="n">
@@ -3713,7 +3713,7 @@
       </c>
       <c r="D60" t="inlineStr">
         <is>
-          <t>Compact two-seat sofa about 1150 x 850, washable covers</t>
+          <t>Low two-seat sofa about 1300 x 750, 700 high, washable covers</t>
         </is>
       </c>
       <c r="E60" t="n">
@@ -5182,7 +5182,7 @@
         </is>
       </c>
       <c r="E91" t="n">
-        <v>89</v>
+        <v>91</v>
       </c>
       <c r="F91" t="inlineStr">
         <is>
@@ -5203,7 +5203,7 @@
         </is>
       </c>
       <c r="J91" t="n">
-        <v>44500</v>
+        <v>45500</v>
       </c>
       <c r="K91" t="inlineStr">
         <is>
@@ -5233,7 +5233,7 @@
         </is>
       </c>
       <c r="E92" t="n">
-        <v>29</v>
+        <v>30</v>
       </c>
       <c r="F92" t="inlineStr">
         <is>
@@ -5254,7 +5254,7 @@
         </is>
       </c>
       <c r="J92" t="n">
-        <v>21750</v>
+        <v>22500</v>
       </c>
       <c r="K92" t="inlineStr">
         <is>
@@ -5437,7 +5437,7 @@
         </is>
       </c>
       <c r="E96" t="n">
-        <v>8</v>
+        <v>9</v>
       </c>
       <c r="F96" t="inlineStr">
         <is>
@@ -5458,7 +5458,7 @@
         </is>
       </c>
       <c r="J96" t="n">
-        <v>4000</v>
+        <v>4500</v>
       </c>
       <c r="K96" t="inlineStr">
         <is>
@@ -5970,7 +5970,7 @@
         </is>
       </c>
       <c r="E107" t="n">
-        <v>4.6</v>
+        <v>4.4</v>
       </c>
       <c r="F107" t="inlineStr">
         <is>
@@ -5991,7 +5991,7 @@
         </is>
       </c>
       <c r="J107" t="n">
-        <v>12880</v>
+        <v>12320</v>
       </c>
       <c r="K107" t="inlineStr">
         <is>
@@ -6123,7 +6123,7 @@
         </is>
       </c>
       <c r="E110" t="n">
-        <v>6.4</v>
+        <v>6</v>
       </c>
       <c r="F110" t="inlineStr">
         <is>
@@ -6144,7 +6144,7 @@
         </is>
       </c>
       <c r="J110" t="n">
-        <v>12800</v>
+        <v>12000</v>
       </c>
       <c r="K110" t="inlineStr">
         <is>
@@ -6276,7 +6276,7 @@
         </is>
       </c>
       <c r="E113" t="n">
-        <v>5.7</v>
+        <v>5.4</v>
       </c>
       <c r="F113" t="inlineStr">
         <is>
@@ -6297,7 +6297,7 @@
         </is>
       </c>
       <c r="J113" t="n">
-        <v>17100</v>
+        <v>16200</v>
       </c>
       <c r="K113" t="inlineStr">
         <is>
@@ -7185,7 +7185,7 @@
         </is>
       </c>
       <c r="E132" t="n">
-        <v>6.6</v>
+        <v>5.5</v>
       </c>
       <c r="F132" t="inlineStr">
         <is>
@@ -7206,7 +7206,7 @@
         </is>
       </c>
       <c r="J132" t="n">
-        <v>19800</v>
+        <v>16500</v>
       </c>
       <c r="K132" t="inlineStr">
         <is>

</xml_diff>

<commit_message>
feat(studio): mahogany furniture, off-white walls, slimmer table legs
The joinery (bed, bedside table, table, chairs, galley and overhead
cabinet, sofa legs) takes a natural mahogany-tone stain under satin PU,
and the living linings are painted off-white over a vapour-retarding
primer; the finishes table and the bill of materials say so (a K7
stain line, the K1 paint line). The render shows both, and the seating
table stands on slimmer legs in the drawing and the render.

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01KRyNxX68L5feJKbJnBKRyV
</commit_message>
<xml_diff>
--- a/public/designs/studio/data/bom.xlsx
+++ b/public/designs/studio/data/bom.xlsx
@@ -539,40 +539,40 @@
     <row r="11">
       <c r="A11" t="inlineStr">
         <is>
-          <t>appliances</t>
+          <t>finishes</t>
         </is>
       </c>
       <c r="B11" t="n">
-        <v>605000</v>
+        <v>621800</v>
       </c>
       <c r="C11" t="n">
-        <v>1815000</v>
+        <v>1865400</v>
       </c>
     </row>
     <row r="12">
       <c r="A12" t="inlineStr">
         <is>
-          <t>furnishing</t>
+          <t>appliances</t>
         </is>
       </c>
       <c r="B12" t="n">
-        <v>545000</v>
+        <v>605000</v>
       </c>
       <c r="C12" t="n">
-        <v>1635000</v>
+        <v>1815000</v>
       </c>
     </row>
     <row r="13">
       <c r="A13" t="inlineStr">
         <is>
-          <t>finishes</t>
+          <t>furnishing</t>
         </is>
       </c>
       <c r="B13" t="n">
-        <v>537800</v>
+        <v>545000</v>
       </c>
       <c r="C13" t="n">
-        <v>1613400</v>
+        <v>1635000</v>
       </c>
     </row>
     <row r="14">
@@ -736,10 +736,10 @@
         </is>
       </c>
       <c r="B26" t="n">
-        <v>2027770</v>
+        <v>2040370</v>
       </c>
       <c r="C26" t="n">
-        <v>6811711</v>
+        <v>6849511</v>
       </c>
     </row>
     <row r="27">
@@ -749,10 +749,10 @@
         </is>
       </c>
       <c r="B27" t="n">
-        <v>15546239</v>
+        <v>15642839</v>
       </c>
       <c r="C27" t="n">
-        <v>52223118</v>
+        <v>52512918</v>
       </c>
     </row>
     <row r="29">
@@ -763,7 +763,7 @@
       </c>
       <c r="B29" t="inlineStr"/>
       <c r="C29" t="n">
-        <v>35384</v>
+        <v>35580</v>
       </c>
     </row>
   </sheetData>
@@ -777,7 +777,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:K139"/>
+  <dimension ref="A1:K140"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -2243,7 +2243,7 @@
       </c>
       <c r="D30" t="inlineStr">
         <is>
-          <t>Vapour-retarding PU varnish for linings</t>
+          <t>Vapour-retarding primer + off-white paint for the linings</t>
         </is>
       </c>
       <c r="E30" t="n">
@@ -3898,34 +3898,34 @@
     <row r="64">
       <c r="A64" t="inlineStr">
         <is>
-          <t>K8</t>
+          <t>K7</t>
         </is>
       </c>
       <c r="B64" t="inlineStr">
         <is>
-          <t>electrical</t>
+          <t>finishes</t>
         </is>
       </c>
       <c r="C64" t="inlineStr">
         <is>
-          <t>electrical</t>
+          <t>painting</t>
         </is>
       </c>
       <c r="D64" t="inlineStr">
         <is>
-          <t>Unit board on the back wall by the galley</t>
+          <t>Joinery finish: natural mahogany-tone stain + satin PU varnish (all furniture)</t>
         </is>
       </c>
       <c r="E64" t="n">
-        <v>1</v>
+        <v>6</v>
       </c>
       <c r="F64" t="inlineStr">
         <is>
-          <t>each</t>
+          <t>L</t>
         </is>
       </c>
       <c r="G64" t="n">
-        <v>45000</v>
+        <v>14000</v>
       </c>
       <c r="H64" t="inlineStr">
         <is>
@@ -3938,11 +3938,11 @@
         </is>
       </c>
       <c r="J64" t="n">
-        <v>45000</v>
+        <v>84000</v>
       </c>
       <c r="K64" t="inlineStr">
         <is>
-          <t>enclosure, 12 ways</t>
+          <t>mahogany-tone wood stain + satin PU varnish, per L</t>
         </is>
       </c>
     </row>
@@ -3964,7 +3964,7 @@
       </c>
       <c r="D65" t="inlineStr">
         <is>
-          <t>Ceiling light, bed</t>
+          <t>Unit board on the back wall by the galley</t>
         </is>
       </c>
       <c r="E65" t="n">
@@ -3976,7 +3976,7 @@
         </is>
       </c>
       <c r="G65" t="n">
-        <v>15000</v>
+        <v>45000</v>
       </c>
       <c r="H65" t="inlineStr">
         <is>
@@ -3989,9 +3989,13 @@
         </is>
       </c>
       <c r="J65" t="n">
-        <v>15000</v>
-      </c>
-      <c r="K65" t="inlineStr"/>
+        <v>45000</v>
+      </c>
+      <c r="K65" t="inlineStr">
+        <is>
+          <t>enclosure, 12 ways</t>
+        </is>
+      </c>
     </row>
     <row r="66">
       <c r="A66" t="inlineStr">
@@ -4011,7 +4015,7 @@
       </c>
       <c r="D66" t="inlineStr">
         <is>
-          <t>Ceiling light, living</t>
+          <t>Ceiling light, bed</t>
         </is>
       </c>
       <c r="E66" t="n">
@@ -4058,7 +4062,7 @@
       </c>
       <c r="D67" t="inlineStr">
         <is>
-          <t>Ceiling light, galley</t>
+          <t>Ceiling light, living</t>
         </is>
       </c>
       <c r="E67" t="n">
@@ -4105,7 +4109,7 @@
       </c>
       <c r="D68" t="inlineStr">
         <is>
-          <t>Bathroom light IP65</t>
+          <t>Ceiling light, galley</t>
         </is>
       </c>
       <c r="E68" t="n">
@@ -4152,7 +4156,7 @@
       </c>
       <c r="D69" t="inlineStr">
         <is>
-          <t>Wall reading light over the bed (wall side)</t>
+          <t>Bathroom light IP65</t>
         </is>
       </c>
       <c r="E69" t="n">
@@ -4199,7 +4203,7 @@
       </c>
       <c r="D70" t="inlineStr">
         <is>
-          <t>Under-cabinet LED strip</t>
+          <t>Wall reading light over the bed (wall side)</t>
         </is>
       </c>
       <c r="E70" t="n">
@@ -4246,7 +4250,7 @@
       </c>
       <c r="D71" t="inlineStr">
         <is>
-          <t>Deck light IP65</t>
+          <t>Under-cabinet LED strip</t>
         </is>
       </c>
       <c r="E71" t="n">
@@ -4293,7 +4297,7 @@
       </c>
       <c r="D72" t="inlineStr">
         <is>
-          <t>Roof terrace lights IP65 (x2)</t>
+          <t>Deck light IP65</t>
         </is>
       </c>
       <c r="E72" t="n">
@@ -4340,7 +4344,7 @@
       </c>
       <c r="D73" t="inlineStr">
         <is>
-          <t>Stair light IP65</t>
+          <t>Roof terrace lights IP65 (x2)</t>
         </is>
       </c>
       <c r="E73" t="n">
@@ -4387,7 +4391,7 @@
       </c>
       <c r="D74" t="inlineStr">
         <is>
-          <t>Entry: living + kitchen + deck</t>
+          <t>Stair light IP65</t>
         </is>
       </c>
       <c r="E74" t="n">
@@ -4399,7 +4403,7 @@
         </is>
       </c>
       <c r="G74" t="n">
-        <v>3500</v>
+        <v>15000</v>
       </c>
       <c r="H74" t="inlineStr">
         <is>
@@ -4412,7 +4416,7 @@
         </is>
       </c>
       <c r="J74" t="n">
-        <v>3500</v>
+        <v>15000</v>
       </c>
       <c r="K74" t="inlineStr"/>
     </row>
@@ -4434,7 +4438,7 @@
       </c>
       <c r="D75" t="inlineStr">
         <is>
-          <t>Bed: ceiling light (2-way), over the bedside table</t>
+          <t>Entry: living + kitchen + deck</t>
         </is>
       </c>
       <c r="E75" t="n">
@@ -4481,7 +4485,7 @@
       </c>
       <c r="D76" t="inlineStr">
         <is>
-          <t>Bathroom light + fan (outside)</t>
+          <t>Bed: ceiling light (2-way), over the bedside table</t>
         </is>
       </c>
       <c r="E76" t="n">
@@ -4528,7 +4532,7 @@
       </c>
       <c r="D77" t="inlineStr">
         <is>
-          <t>Roof and stair lights (IP65, stair foot)</t>
+          <t>Bathroom light + fan (outside)</t>
         </is>
       </c>
       <c r="E77" t="n">
@@ -4575,7 +4579,7 @@
       </c>
       <c r="D78" t="inlineStr">
         <is>
-          <t>Socket + USB-C in the headboard (wall side)</t>
+          <t>Roof and stair lights (IP65, stair foot)</t>
         </is>
       </c>
       <c r="E78" t="n">
@@ -4587,7 +4591,7 @@
         </is>
       </c>
       <c r="G78" t="n">
-        <v>15000</v>
+        <v>3500</v>
       </c>
       <c r="H78" t="inlineStr">
         <is>
@@ -4600,7 +4604,7 @@
         </is>
       </c>
       <c r="J78" t="n">
-        <v>15000</v>
+        <v>3500</v>
       </c>
       <c r="K78" t="inlineStr"/>
     </row>
@@ -4622,7 +4626,7 @@
       </c>
       <c r="D79" t="inlineStr">
         <is>
-          <t>Bedside socket + USB-C (reading lamp)</t>
+          <t>Socket + USB-C in the headboard (wall side)</t>
         </is>
       </c>
       <c r="E79" t="n">
@@ -4669,7 +4673,7 @@
       </c>
       <c r="D80" t="inlineStr">
         <is>
-          <t>Socket by the sofa</t>
+          <t>Bedside socket + USB-C (reading lamp)</t>
         </is>
       </c>
       <c r="E80" t="n">
@@ -4681,7 +4685,7 @@
         </is>
       </c>
       <c r="G80" t="n">
-        <v>5000</v>
+        <v>15000</v>
       </c>
       <c r="H80" t="inlineStr">
         <is>
@@ -4694,7 +4698,7 @@
         </is>
       </c>
       <c r="J80" t="n">
-        <v>5000</v>
+        <v>15000</v>
       </c>
       <c r="K80" t="inlineStr"/>
     </row>
@@ -4716,7 +4720,7 @@
       </c>
       <c r="D81" t="inlineStr">
         <is>
-          <t>Socket, living (front strip)</t>
+          <t>Socket by the sofa</t>
         </is>
       </c>
       <c r="E81" t="n">
@@ -4763,7 +4767,7 @@
       </c>
       <c r="D82" t="inlineStr">
         <is>
-          <t>Deck socket IP66</t>
+          <t>Socket, living (front strip)</t>
         </is>
       </c>
       <c r="E82" t="n">
@@ -4810,7 +4814,7 @@
       </c>
       <c r="D83" t="inlineStr">
         <is>
-          <t>Worktop socket 1 (double)</t>
+          <t>Deck socket IP66</t>
         </is>
       </c>
       <c r="E83" t="n">
@@ -4857,7 +4861,7 @@
       </c>
       <c r="D84" t="inlineStr">
         <is>
-          <t>Worktop socket 2 (double, back wall)</t>
+          <t>Worktop socket 1 (double)</t>
         </is>
       </c>
       <c r="E84" t="n">
@@ -4904,7 +4908,7 @@
       </c>
       <c r="D85" t="inlineStr">
         <is>
-          <t>Fridge socket</t>
+          <t>Worktop socket 2 (double, back wall)</t>
         </is>
       </c>
       <c r="E85" t="n">
@@ -4951,7 +4955,7 @@
       </c>
       <c r="D86" t="inlineStr">
         <is>
-          <t>Hob connection unit</t>
+          <t>Fridge socket</t>
         </is>
       </c>
       <c r="E86" t="n">
@@ -4963,7 +4967,7 @@
         </is>
       </c>
       <c r="G86" t="n">
-        <v>9000</v>
+        <v>5000</v>
       </c>
       <c r="H86" t="inlineStr">
         <is>
@@ -4976,7 +4980,7 @@
         </is>
       </c>
       <c r="J86" t="n">
-        <v>9000</v>
+        <v>5000</v>
       </c>
       <c r="K86" t="inlineStr"/>
     </row>
@@ -4998,7 +5002,7 @@
       </c>
       <c r="D87" t="inlineStr">
         <is>
-          <t>Heater DP switch + timer</t>
+          <t>Hob connection unit</t>
         </is>
       </c>
       <c r="E87" t="n">
@@ -5045,7 +5049,7 @@
       </c>
       <c r="D88" t="inlineStr">
         <is>
-          <t>Bathroom extract 100 mm (one 110 mm hole in the back wall)</t>
+          <t>Heater DP switch + timer</t>
         </is>
       </c>
       <c r="E88" t="n">
@@ -5057,7 +5061,7 @@
         </is>
       </c>
       <c r="G88" t="n">
-        <v>35000</v>
+        <v>9000</v>
       </c>
       <c r="H88" t="inlineStr">
         <is>
@@ -5070,7 +5074,7 @@
         </is>
       </c>
       <c r="J88" t="n">
-        <v>35000</v>
+        <v>9000</v>
       </c>
       <c r="K88" t="inlineStr"/>
     </row>
@@ -5092,7 +5096,7 @@
       </c>
       <c r="D89" t="inlineStr">
         <is>
-          <t>Wall fan</t>
+          <t>Bathroom extract 100 mm (one 110 mm hole in the back wall)</t>
         </is>
       </c>
       <c r="E89" t="n">
@@ -5139,7 +5143,7 @@
       </c>
       <c r="D90" t="inlineStr">
         <is>
-          <t>AC provision: isolator</t>
+          <t>Wall fan</t>
         </is>
       </c>
       <c r="E90" t="n">
@@ -5151,7 +5155,7 @@
         </is>
       </c>
       <c r="G90" t="n">
-        <v>9000</v>
+        <v>35000</v>
       </c>
       <c r="H90" t="inlineStr">
         <is>
@@ -5164,7 +5168,7 @@
         </is>
       </c>
       <c r="J90" t="n">
-        <v>9000</v>
+        <v>35000</v>
       </c>
       <c r="K90" t="inlineStr"/>
     </row>
@@ -5186,19 +5190,19 @@
       </c>
       <c r="D91" t="inlineStr">
         <is>
-          <t>Cable 1.5 mm2 T+E/singles in conduit, Lighting (incl. bathroom IP65, deck, roof, stair)</t>
+          <t>AC provision: isolator</t>
         </is>
       </c>
       <c r="E91" t="n">
-        <v>85</v>
+        <v>1</v>
       </c>
       <c r="F91" t="inlineStr">
         <is>
-          <t>m</t>
+          <t>each</t>
         </is>
       </c>
       <c r="G91" t="n">
-        <v>500</v>
+        <v>9000</v>
       </c>
       <c r="H91" t="inlineStr">
         <is>
@@ -5211,13 +5215,9 @@
         </is>
       </c>
       <c r="J91" t="n">
-        <v>42500</v>
-      </c>
-      <c r="K91" t="inlineStr">
-        <is>
-          <t>per m</t>
-        </is>
-      </c>
+        <v>9000</v>
+      </c>
+      <c r="K91" t="inlineStr"/>
     </row>
     <row r="92">
       <c r="A92" t="inlineStr">
@@ -5237,11 +5237,11 @@
       </c>
       <c r="D92" t="inlineStr">
         <is>
-          <t>Cable 2.5 mm2 T+E/singles in conduit, Sockets: bedside USB, living, deck</t>
+          <t>Cable 1.5 mm2 T+E/singles in conduit, Lighting (incl. bathroom IP65, deck, roof, stair)</t>
         </is>
       </c>
       <c r="E92" t="n">
-        <v>30</v>
+        <v>85</v>
       </c>
       <c r="F92" t="inlineStr">
         <is>
@@ -5249,7 +5249,7 @@
         </is>
       </c>
       <c r="G92" t="n">
-        <v>750</v>
+        <v>500</v>
       </c>
       <c r="H92" t="inlineStr">
         <is>
@@ -5262,7 +5262,7 @@
         </is>
       </c>
       <c r="J92" t="n">
-        <v>22500</v>
+        <v>42500</v>
       </c>
       <c r="K92" t="inlineStr">
         <is>
@@ -5288,11 +5288,11 @@
       </c>
       <c r="D93" t="inlineStr">
         <is>
-          <t>Cable 2.5 mm2 T+E/singles in conduit, Kitchen sockets and fridge</t>
+          <t>Cable 2.5 mm2 T+E/singles in conduit, Sockets: bedside USB, living, deck</t>
         </is>
       </c>
       <c r="E93" t="n">
-        <v>13</v>
+        <v>30</v>
       </c>
       <c r="F93" t="inlineStr">
         <is>
@@ -5313,7 +5313,7 @@
         </is>
       </c>
       <c r="J93" t="n">
-        <v>9750</v>
+        <v>22500</v>
       </c>
       <c r="K93" t="inlineStr">
         <is>
@@ -5339,11 +5339,11 @@
       </c>
       <c r="D94" t="inlineStr">
         <is>
-          <t>Cable 4.0 mm2 T+E/singles in conduit, Induction hob</t>
+          <t>Cable 2.5 mm2 T+E/singles in conduit, Kitchen sockets and fridge</t>
         </is>
       </c>
       <c r="E94" t="n">
-        <v>8</v>
+        <v>13</v>
       </c>
       <c r="F94" t="inlineStr">
         <is>
@@ -5351,7 +5351,7 @@
         </is>
       </c>
       <c r="G94" t="n">
-        <v>1200</v>
+        <v>750</v>
       </c>
       <c r="H94" t="inlineStr">
         <is>
@@ -5364,7 +5364,7 @@
         </is>
       </c>
       <c r="J94" t="n">
-        <v>9600</v>
+        <v>9750</v>
       </c>
       <c r="K94" t="inlineStr">
         <is>
@@ -5390,11 +5390,11 @@
       </c>
       <c r="D95" t="inlineStr">
         <is>
-          <t>Cable 2.5 mm2 T+E/singles in conduit, 80 L water heater</t>
+          <t>Cable 4.0 mm2 T+E/singles in conduit, Induction hob</t>
         </is>
       </c>
       <c r="E95" t="n">
-        <v>7</v>
+        <v>8</v>
       </c>
       <c r="F95" t="inlineStr">
         <is>
@@ -5402,7 +5402,7 @@
         </is>
       </c>
       <c r="G95" t="n">
-        <v>750</v>
+        <v>1200</v>
       </c>
       <c r="H95" t="inlineStr">
         <is>
@@ -5415,7 +5415,7 @@
         </is>
       </c>
       <c r="J95" t="n">
-        <v>5250</v>
+        <v>9600</v>
       </c>
       <c r="K95" t="inlineStr">
         <is>
@@ -5441,11 +5441,11 @@
       </c>
       <c r="D96" t="inlineStr">
         <is>
-          <t>Cable 1.5 mm2 T+E/singles in conduit, Extract fan and wall fan</t>
+          <t>Cable 2.5 mm2 T+E/singles in conduit, 80 L water heater</t>
         </is>
       </c>
       <c r="E96" t="n">
-        <v>9</v>
+        <v>7</v>
       </c>
       <c r="F96" t="inlineStr">
         <is>
@@ -5453,7 +5453,7 @@
         </is>
       </c>
       <c r="G96" t="n">
-        <v>500</v>
+        <v>750</v>
       </c>
       <c r="H96" t="inlineStr">
         <is>
@@ -5466,7 +5466,7 @@
         </is>
       </c>
       <c r="J96" t="n">
-        <v>4500</v>
+        <v>5250</v>
       </c>
       <c r="K96" t="inlineStr">
         <is>
@@ -5492,11 +5492,11 @@
       </c>
       <c r="D97" t="inlineStr">
         <is>
-          <t>Cable 2.5 mm2 T+E/singles in conduit, AC provision</t>
+          <t>Cable 1.5 mm2 T+E/singles in conduit, Extract fan and wall fan</t>
         </is>
       </c>
       <c r="E97" t="n">
-        <v>7</v>
+        <v>9</v>
       </c>
       <c r="F97" t="inlineStr">
         <is>
@@ -5504,7 +5504,7 @@
         </is>
       </c>
       <c r="G97" t="n">
-        <v>750</v>
+        <v>500</v>
       </c>
       <c r="H97" t="inlineStr">
         <is>
@@ -5517,7 +5517,7 @@
         </is>
       </c>
       <c r="J97" t="n">
-        <v>5250</v>
+        <v>4500</v>
       </c>
       <c r="K97" t="inlineStr">
         <is>
@@ -5543,11 +5543,11 @@
       </c>
       <c r="D98" t="inlineStr">
         <is>
-          <t>PVC conduit 20 mm + boxes</t>
+          <t>Cable 2.5 mm2 T+E/singles in conduit, AC provision</t>
         </is>
       </c>
       <c r="E98" t="n">
-        <v>60</v>
+        <v>7</v>
       </c>
       <c r="F98" t="inlineStr">
         <is>
@@ -5555,7 +5555,7 @@
         </is>
       </c>
       <c r="G98" t="n">
-        <v>600</v>
+        <v>750</v>
       </c>
       <c r="H98" t="inlineStr">
         <is>
@@ -5568,7 +5568,7 @@
         </is>
       </c>
       <c r="J98" t="n">
-        <v>36000</v>
+        <v>5250</v>
       </c>
       <c r="K98" t="inlineStr">
         <is>
@@ -5594,19 +5594,19 @@
       </c>
       <c r="D99" t="inlineStr">
         <is>
-          <t>Surge protection device type 2</t>
+          <t>PVC conduit 20 mm + boxes</t>
         </is>
       </c>
       <c r="E99" t="n">
-        <v>1</v>
+        <v>60</v>
       </c>
       <c r="F99" t="inlineStr">
         <is>
-          <t>each</t>
+          <t>m</t>
         </is>
       </c>
       <c r="G99" t="n">
-        <v>60000</v>
+        <v>600</v>
       </c>
       <c r="H99" t="inlineStr">
         <is>
@@ -5619,9 +5619,13 @@
         </is>
       </c>
       <c r="J99" t="n">
-        <v>60000</v>
-      </c>
-      <c r="K99" t="inlineStr"/>
+        <v>36000</v>
+      </c>
+      <c r="K99" t="inlineStr">
+        <is>
+          <t>per m</t>
+        </is>
+      </c>
     </row>
     <row r="100">
       <c r="A100" t="inlineStr">
@@ -5641,7 +5645,7 @@
       </c>
       <c r="D100" t="inlineStr">
         <is>
-          <t>RCD 40 A 30 mA type A (or RCBOs)</t>
+          <t>Surge protection device type 2</t>
         </is>
       </c>
       <c r="E100" t="n">
@@ -5653,7 +5657,7 @@
         </is>
       </c>
       <c r="G100" t="n">
-        <v>45000</v>
+        <v>60000</v>
       </c>
       <c r="H100" t="inlineStr">
         <is>
@@ -5666,7 +5670,7 @@
         </is>
       </c>
       <c r="J100" t="n">
-        <v>45000</v>
+        <v>60000</v>
       </c>
       <c r="K100" t="inlineStr"/>
     </row>
@@ -5688,11 +5692,11 @@
       </c>
       <c r="D101" t="inlineStr">
         <is>
-          <t>MCBs (B6 x2, B16 x5, B20 x1)</t>
+          <t>RCD 40 A 30 mA type A (or RCBOs)</t>
         </is>
       </c>
       <c r="E101" t="n">
-        <v>8</v>
+        <v>1</v>
       </c>
       <c r="F101" t="inlineStr">
         <is>
@@ -5700,7 +5704,7 @@
         </is>
       </c>
       <c r="G101" t="n">
-        <v>6000</v>
+        <v>45000</v>
       </c>
       <c r="H101" t="inlineStr">
         <is>
@@ -5713,7 +5717,7 @@
         </is>
       </c>
       <c r="J101" t="n">
-        <v>48000</v>
+        <v>45000</v>
       </c>
       <c r="K101" t="inlineStr"/>
     </row>
@@ -5735,19 +5739,19 @@
       </c>
       <c r="D102" t="inlineStr">
         <is>
-          <t>Main switch 40 A DP + check meter (DIN kWh)</t>
+          <t>MCBs (B6 x2, B16 x5, B20 x1)</t>
         </is>
       </c>
       <c r="E102" t="n">
-        <v>1</v>
+        <v>8</v>
       </c>
       <c r="F102" t="inlineStr">
         <is>
-          <t>set</t>
+          <t>each</t>
         </is>
       </c>
       <c r="G102" t="n">
-        <v>40000</v>
+        <v>6000</v>
       </c>
       <c r="H102" t="inlineStr">
         <is>
@@ -5760,7 +5764,7 @@
         </is>
       </c>
       <c r="J102" t="n">
-        <v>40000</v>
+        <v>48000</v>
       </c>
       <c r="K102" t="inlineStr"/>
     </row>
@@ -5782,7 +5786,7 @@
       </c>
       <c r="D103" t="inlineStr">
         <is>
-          <t>Earth rod 1.5 m copper-bonded + clamp + inspection pit</t>
+          <t>Main switch 40 A DP + check meter (DIN kWh)</t>
         </is>
       </c>
       <c r="E103" t="n">
@@ -5790,11 +5794,11 @@
       </c>
       <c r="F103" t="inlineStr">
         <is>
-          <t>each</t>
+          <t>set</t>
         </is>
       </c>
       <c r="G103" t="n">
-        <v>35000</v>
+        <v>40000</v>
       </c>
       <c r="H103" t="inlineStr">
         <is>
@@ -5807,7 +5811,7 @@
         </is>
       </c>
       <c r="J103" t="n">
-        <v>35000</v>
+        <v>40000</v>
       </c>
       <c r="K103" t="inlineStr"/>
     </row>
@@ -5819,7 +5823,7 @@
       </c>
       <c r="B104" t="inlineStr">
         <is>
-          <t>safety</t>
+          <t>electrical</t>
         </is>
       </c>
       <c r="C104" t="inlineStr">
@@ -5829,11 +5833,11 @@
       </c>
       <c r="D104" t="inlineStr">
         <is>
-          <t>Smoke alarm (10-year) + heat alarm (kitchen)</t>
+          <t>Earth rod 1.5 m copper-bonded + clamp + inspection pit</t>
         </is>
       </c>
       <c r="E104" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="F104" t="inlineStr">
         <is>
@@ -5841,7 +5845,7 @@
         </is>
       </c>
       <c r="G104" t="n">
-        <v>20000</v>
+        <v>35000</v>
       </c>
       <c r="H104" t="inlineStr">
         <is>
@@ -5854,7 +5858,7 @@
         </is>
       </c>
       <c r="J104" t="n">
-        <v>40000</v>
+        <v>35000</v>
       </c>
       <c r="K104" t="inlineStr"/>
     </row>
@@ -5871,24 +5875,24 @@
       </c>
       <c r="C105" t="inlineStr">
         <is>
-          <t>furnishing</t>
+          <t>electrical</t>
         </is>
       </c>
       <c r="D105" t="inlineStr">
         <is>
-          <t>Fire extinguisher 2 kg ABC + fire blanket</t>
+          <t>Smoke alarm (10-year) + heat alarm (kitchen)</t>
         </is>
       </c>
       <c r="E105" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="F105" t="inlineStr">
         <is>
-          <t>set</t>
+          <t>each</t>
         </is>
       </c>
       <c r="G105" t="n">
-        <v>55000</v>
+        <v>20000</v>
       </c>
       <c r="H105" t="inlineStr">
         <is>
@@ -5901,41 +5905,41 @@
         </is>
       </c>
       <c r="J105" t="n">
-        <v>55000</v>
+        <v>40000</v>
       </c>
       <c r="K105" t="inlineStr"/>
     </row>
     <row r="106">
       <c r="A106" t="inlineStr">
         <is>
-          <t>K9</t>
+          <t>K8</t>
         </is>
       </c>
       <c r="B106" t="inlineStr">
         <is>
-          <t>plumbing</t>
+          <t>safety</t>
         </is>
       </c>
       <c r="C106" t="inlineStr">
         <is>
-          <t>plumbing</t>
+          <t>furnishing</t>
         </is>
       </c>
       <c r="D106" t="inlineStr">
         <is>
-          <t>PPR PN20 pipe DN20</t>
+          <t>Fire extinguisher 2 kg ABC + fire blanket</t>
         </is>
       </c>
       <c r="E106" t="n">
-        <v>9.1</v>
+        <v>1</v>
       </c>
       <c r="F106" t="inlineStr">
         <is>
-          <t>m</t>
+          <t>set</t>
         </is>
       </c>
       <c r="G106" t="n">
-        <v>2000</v>
+        <v>55000</v>
       </c>
       <c r="H106" t="inlineStr">
         <is>
@@ -5948,13 +5952,9 @@
         </is>
       </c>
       <c r="J106" t="n">
-        <v>18200</v>
-      </c>
-      <c r="K106" t="inlineStr">
-        <is>
-          <t>per m</t>
-        </is>
-      </c>
+        <v>55000</v>
+      </c>
+      <c r="K106" t="inlineStr"/>
     </row>
     <row r="107">
       <c r="A107" t="inlineStr">
@@ -5974,11 +5974,11 @@
       </c>
       <c r="D107" t="inlineStr">
         <is>
-          <t>PPR PN20 pipe DN25</t>
+          <t>PPR PN20 pipe DN20</t>
         </is>
       </c>
       <c r="E107" t="n">
-        <v>4.4</v>
+        <v>9.1</v>
       </c>
       <c r="F107" t="inlineStr">
         <is>
@@ -5986,7 +5986,7 @@
         </is>
       </c>
       <c r="G107" t="n">
-        <v>2800</v>
+        <v>2000</v>
       </c>
       <c r="H107" t="inlineStr">
         <is>
@@ -5999,7 +5999,7 @@
         </is>
       </c>
       <c r="J107" t="n">
-        <v>12320</v>
+        <v>18200</v>
       </c>
       <c r="K107" t="inlineStr">
         <is>
@@ -6025,11 +6025,11 @@
       </c>
       <c r="D108" t="inlineStr">
         <is>
-          <t>PPR PN20 pipe (hot) DN20</t>
+          <t>PPR PN20 pipe DN25</t>
         </is>
       </c>
       <c r="E108" t="n">
-        <v>4.5</v>
+        <v>4.4</v>
       </c>
       <c r="F108" t="inlineStr">
         <is>
@@ -6037,7 +6037,7 @@
         </is>
       </c>
       <c r="G108" t="n">
-        <v>2000</v>
+        <v>2800</v>
       </c>
       <c r="H108" t="inlineStr">
         <is>
@@ -6050,7 +6050,7 @@
         </is>
       </c>
       <c r="J108" t="n">
-        <v>9000</v>
+        <v>12320</v>
       </c>
       <c r="K108" t="inlineStr">
         <is>
@@ -6076,11 +6076,11 @@
       </c>
       <c r="D109" t="inlineStr">
         <is>
-          <t>uPVC soil pipe DN110</t>
+          <t>PPR PN20 pipe (hot) DN20</t>
         </is>
       </c>
       <c r="E109" t="n">
-        <v>2.7</v>
+        <v>4.5</v>
       </c>
       <c r="F109" t="inlineStr">
         <is>
@@ -6088,7 +6088,7 @@
         </is>
       </c>
       <c r="G109" t="n">
-        <v>7000</v>
+        <v>2000</v>
       </c>
       <c r="H109" t="inlineStr">
         <is>
@@ -6101,7 +6101,7 @@
         </is>
       </c>
       <c r="J109" t="n">
-        <v>18900</v>
+        <v>9000</v>
       </c>
       <c r="K109" t="inlineStr">
         <is>
@@ -6127,11 +6127,11 @@
       </c>
       <c r="D110" t="inlineStr">
         <is>
-          <t>PPR PN20 pipe (tempered) DN20</t>
+          <t>uPVC soil pipe DN110</t>
         </is>
       </c>
       <c r="E110" t="n">
-        <v>6</v>
+        <v>2.7</v>
       </c>
       <c r="F110" t="inlineStr">
         <is>
@@ -6139,7 +6139,7 @@
         </is>
       </c>
       <c r="G110" t="n">
-        <v>2000</v>
+        <v>7000</v>
       </c>
       <c r="H110" t="inlineStr">
         <is>
@@ -6152,7 +6152,7 @@
         </is>
       </c>
       <c r="J110" t="n">
-        <v>12000</v>
+        <v>18900</v>
       </c>
       <c r="K110" t="inlineStr">
         <is>
@@ -6178,11 +6178,11 @@
       </c>
       <c r="D111" t="inlineStr">
         <is>
-          <t>uPVC vent pipe DN75</t>
+          <t>PPR PN20 pipe (tempered) DN20</t>
         </is>
       </c>
       <c r="E111" t="n">
-        <v>7.9</v>
+        <v>6</v>
       </c>
       <c r="F111" t="inlineStr">
         <is>
@@ -6190,7 +6190,7 @@
         </is>
       </c>
       <c r="G111" t="n">
-        <v>4500</v>
+        <v>2000</v>
       </c>
       <c r="H111" t="inlineStr">
         <is>
@@ -6203,7 +6203,7 @@
         </is>
       </c>
       <c r="J111" t="n">
-        <v>35550</v>
+        <v>12000</v>
       </c>
       <c r="K111" t="inlineStr">
         <is>
@@ -6229,11 +6229,11 @@
       </c>
       <c r="D112" t="inlineStr">
         <is>
-          <t>uPVC waste pipe DN40</t>
+          <t>uPVC vent pipe DN75</t>
         </is>
       </c>
       <c r="E112" t="n">
-        <v>2.5</v>
+        <v>7.9</v>
       </c>
       <c r="F112" t="inlineStr">
         <is>
@@ -6241,7 +6241,7 @@
         </is>
       </c>
       <c r="G112" t="n">
-        <v>2500</v>
+        <v>4500</v>
       </c>
       <c r="H112" t="inlineStr">
         <is>
@@ -6254,7 +6254,7 @@
         </is>
       </c>
       <c r="J112" t="n">
-        <v>6250</v>
+        <v>35550</v>
       </c>
       <c r="K112" t="inlineStr">
         <is>
@@ -6280,11 +6280,11 @@
       </c>
       <c r="D113" t="inlineStr">
         <is>
-          <t>uPVC waste pipe DN50</t>
+          <t>uPVC waste pipe DN40</t>
         </is>
       </c>
       <c r="E113" t="n">
-        <v>5.5</v>
+        <v>2.5</v>
       </c>
       <c r="F113" t="inlineStr">
         <is>
@@ -6292,7 +6292,7 @@
         </is>
       </c>
       <c r="G113" t="n">
-        <v>3000</v>
+        <v>2500</v>
       </c>
       <c r="H113" t="inlineStr">
         <is>
@@ -6305,7 +6305,7 @@
         </is>
       </c>
       <c r="J113" t="n">
-        <v>16500</v>
+        <v>6250</v>
       </c>
       <c r="K113" t="inlineStr">
         <is>
@@ -6331,19 +6331,19 @@
       </c>
       <c r="D114" t="inlineStr">
         <is>
-          <t>Pipe fittings and clips (allowance)</t>
+          <t>uPVC waste pipe DN50</t>
         </is>
       </c>
       <c r="E114" t="n">
-        <v>1</v>
+        <v>5.5</v>
       </c>
       <c r="F114" t="inlineStr">
         <is>
-          <t>set</t>
+          <t>m</t>
         </is>
       </c>
       <c r="G114" t="n">
-        <v>120000</v>
+        <v>3000</v>
       </c>
       <c r="H114" t="inlineStr">
         <is>
@@ -6356,9 +6356,13 @@
         </is>
       </c>
       <c r="J114" t="n">
-        <v>120000</v>
-      </c>
-      <c r="K114" t="inlineStr"/>
+        <v>16500</v>
+      </c>
+      <c r="K114" t="inlineStr">
+        <is>
+          <t>per m</t>
+        </is>
+      </c>
     </row>
     <row r="115">
       <c r="A115" t="inlineStr">
@@ -6378,7 +6382,7 @@
       </c>
       <c r="D115" t="inlineStr">
         <is>
-          <t>Thermostatic mixing valve (TMV) 41-44 C</t>
+          <t>Pipe fittings and clips (allowance)</t>
         </is>
       </c>
       <c r="E115" t="n">
@@ -6386,11 +6390,11 @@
       </c>
       <c r="F115" t="inlineStr">
         <is>
-          <t>each</t>
+          <t>set</t>
         </is>
       </c>
       <c r="G115" t="n">
-        <v>60000</v>
+        <v>120000</v>
       </c>
       <c r="H115" t="inlineStr">
         <is>
@@ -6403,7 +6407,7 @@
         </is>
       </c>
       <c r="J115" t="n">
-        <v>60000</v>
+        <v>120000</v>
       </c>
       <c r="K115" t="inlineStr"/>
     </row>
@@ -6425,7 +6429,7 @@
       </c>
       <c r="D116" t="inlineStr">
         <is>
-          <t>Thermostatic shower valve + 6-7 L/min head + rail</t>
+          <t>Thermostatic mixing valve (TMV) 41-44 C</t>
         </is>
       </c>
       <c r="E116" t="n">
@@ -6433,11 +6437,11 @@
       </c>
       <c r="F116" t="inlineStr">
         <is>
-          <t>set</t>
+          <t>each</t>
         </is>
       </c>
       <c r="G116" t="n">
-        <v>90000</v>
+        <v>60000</v>
       </c>
       <c r="H116" t="inlineStr">
         <is>
@@ -6450,7 +6454,7 @@
         </is>
       </c>
       <c r="J116" t="n">
-        <v>90000</v>
+        <v>60000</v>
       </c>
       <c r="K116" t="inlineStr"/>
     </row>
@@ -6472,7 +6476,7 @@
       </c>
       <c r="D117" t="inlineStr">
         <is>
-          <t>Electric storage water heater 80 L, 2 kW, with T&amp;P valve</t>
+          <t>Thermostatic shower valve + 6-7 L/min head + rail</t>
         </is>
       </c>
       <c r="E117" t="n">
@@ -6480,11 +6484,11 @@
       </c>
       <c r="F117" t="inlineStr">
         <is>
-          <t>each</t>
+          <t>set</t>
         </is>
       </c>
       <c r="G117" t="n">
-        <v>300000</v>
+        <v>90000</v>
       </c>
       <c r="H117" t="inlineStr">
         <is>
@@ -6497,13 +6501,9 @@
         </is>
       </c>
       <c r="J117" t="n">
-        <v>300000</v>
-      </c>
-      <c r="K117" t="inlineStr">
-        <is>
-          <t>80 L not found; 50 L listed at RWF 144,000-252,000 (STU-P01, STU-P02)</t>
-        </is>
-      </c>
+        <v>90000</v>
+      </c>
+      <c r="K117" t="inlineStr"/>
     </row>
     <row r="118">
       <c r="A118" t="inlineStr">
@@ -6523,11 +6523,11 @@
       </c>
       <c r="D118" t="inlineStr">
         <is>
-          <t>Angle valves with filters</t>
+          <t>Electric storage water heater 80 L, 2 kW, with T&amp;P valve</t>
         </is>
       </c>
       <c r="E118" t="n">
-        <v>5</v>
+        <v>1</v>
       </c>
       <c r="F118" t="inlineStr">
         <is>
@@ -6535,7 +6535,7 @@
         </is>
       </c>
       <c r="G118" t="n">
-        <v>6000</v>
+        <v>300000</v>
       </c>
       <c r="H118" t="inlineStr">
         <is>
@@ -6548,9 +6548,13 @@
         </is>
       </c>
       <c r="J118" t="n">
-        <v>30000</v>
-      </c>
-      <c r="K118" t="inlineStr"/>
+        <v>300000</v>
+      </c>
+      <c r="K118" t="inlineStr">
+        <is>
+          <t>80 L not found; 50 L listed at RWF 144,000-252,000 (STU-P01, STU-P02)</t>
+        </is>
+      </c>
     </row>
     <row r="119">
       <c r="A119" t="inlineStr">
@@ -6570,19 +6574,19 @@
       </c>
       <c r="D119" t="inlineStr">
         <is>
-          <t>Air admittance valve 110 mm (spare) + rodding eyes</t>
+          <t>Angle valves with filters</t>
         </is>
       </c>
       <c r="E119" t="n">
-        <v>1</v>
+        <v>5</v>
       </c>
       <c r="F119" t="inlineStr">
         <is>
-          <t>set</t>
+          <t>each</t>
         </is>
       </c>
       <c r="G119" t="n">
-        <v>30000</v>
+        <v>6000</v>
       </c>
       <c r="H119" t="inlineStr">
         <is>
@@ -6617,7 +6621,7 @@
       </c>
       <c r="D120" t="inlineStr">
         <is>
-          <t>Stop valve + Y-filter + check water meter</t>
+          <t>Air admittance valve 110 mm (spare) + rodding eyes</t>
         </is>
       </c>
       <c r="E120" t="n">
@@ -6629,7 +6633,7 @@
         </is>
       </c>
       <c r="G120" t="n">
-        <v>45000</v>
+        <v>30000</v>
       </c>
       <c r="H120" t="inlineStr">
         <is>
@@ -6642,29 +6646,29 @@
         </is>
       </c>
       <c r="J120" t="n">
-        <v>45000</v>
+        <v>30000</v>
       </c>
       <c r="K120" t="inlineStr"/>
     </row>
     <row r="121">
       <c r="A121" t="inlineStr">
         <is>
-          <t>K10</t>
+          <t>K9</t>
         </is>
       </c>
       <c r="B121" t="inlineStr">
         <is>
-          <t>steel</t>
+          <t>plumbing</t>
         </is>
       </c>
       <c r="C121" t="inlineStr">
         <is>
-          <t>welding</t>
+          <t>plumbing</t>
         </is>
       </c>
       <c r="D121" t="inlineStr">
         <is>
-          <t>W1 infill: 2 mm steel + 40 mm EPS, welded into the old door frame (0-1,150)</t>
+          <t>Stop valve + Y-filter + check water meter</t>
         </is>
       </c>
       <c r="E121" t="n">
@@ -6672,11 +6676,11 @@
       </c>
       <c r="F121" t="inlineStr">
         <is>
-          <t>each</t>
+          <t>set</t>
         </is>
       </c>
       <c r="G121" t="n">
-        <v>180000</v>
+        <v>45000</v>
       </c>
       <c r="H121" t="inlineStr">
         <is>
@@ -6689,13 +6693,9 @@
         </is>
       </c>
       <c r="J121" t="n">
-        <v>180000</v>
-      </c>
-      <c r="K121" t="inlineStr">
-        <is>
-          <t>incl. welding</t>
-        </is>
-      </c>
+        <v>45000</v>
+      </c>
+      <c r="K121" t="inlineStr"/>
     </row>
     <row r="122">
       <c r="A122" t="inlineStr">
@@ -6705,17 +6705,17 @@
       </c>
       <c r="B122" t="inlineStr">
         <is>
-          <t>glazing</t>
+          <t>steel</t>
         </is>
       </c>
       <c r="C122" t="inlineStr">
         <is>
-          <t>glazier</t>
+          <t>welding</t>
         </is>
       </c>
       <c r="D122" t="inlineStr">
         <is>
-          <t>W1 obscure louvre window 520 x 890 + insect mesh (wash lobby)</t>
+          <t>W1 infill: 2 mm steel + 40 mm EPS, welded into the old door frame (0-1,150)</t>
         </is>
       </c>
       <c r="E122" t="n">
@@ -6727,7 +6727,7 @@
         </is>
       </c>
       <c r="G122" t="n">
-        <v>120000</v>
+        <v>180000</v>
       </c>
       <c r="H122" t="inlineStr">
         <is>
@@ -6740,9 +6740,13 @@
         </is>
       </c>
       <c r="J122" t="n">
-        <v>120000</v>
-      </c>
-      <c r="K122" t="inlineStr"/>
+        <v>180000</v>
+      </c>
+      <c r="K122" t="inlineStr">
+        <is>
+          <t>incl. welding</t>
+        </is>
+      </c>
     </row>
     <row r="123">
       <c r="A123" t="inlineStr">
@@ -6752,17 +6756,17 @@
       </c>
       <c r="B123" t="inlineStr">
         <is>
-          <t>steel</t>
+          <t>glazing</t>
         </is>
       </c>
       <c r="C123" t="inlineStr">
         <is>
-          <t>welding</t>
+          <t>glazier</t>
         </is>
       </c>
       <c r="D123" t="inlineStr">
         <is>
-          <t>Seal and lock the end-B cargo doors (weld tabs, sealant)</t>
+          <t>W1 obscure louvre window 520 x 890 + insect mesh (wash lobby)</t>
         </is>
       </c>
       <c r="E123" t="n">
@@ -6774,7 +6778,7 @@
         </is>
       </c>
       <c r="G123" t="n">
-        <v>60000</v>
+        <v>120000</v>
       </c>
       <c r="H123" t="inlineStr">
         <is>
@@ -6787,7 +6791,7 @@
         </is>
       </c>
       <c r="J123" t="n">
-        <v>60000</v>
+        <v>120000</v>
       </c>
       <c r="K123" t="inlineStr"/>
     </row>
@@ -6804,16 +6808,16 @@
       </c>
       <c r="C124" t="inlineStr">
         <is>
-          <t>masonry</t>
+          <t>welding</t>
         </is>
       </c>
       <c r="D124" t="inlineStr">
         <is>
-          <t>Level the corner castings: concrete pads or steel shims (rock corner)</t>
+          <t>Seal and lock the end-B cargo doors (weld tabs, sealant)</t>
         </is>
       </c>
       <c r="E124" t="n">
-        <v>4</v>
+        <v>1</v>
       </c>
       <c r="F124" t="inlineStr">
         <is>
@@ -6821,7 +6825,7 @@
         </is>
       </c>
       <c r="G124" t="n">
-        <v>25000</v>
+        <v>60000</v>
       </c>
       <c r="H124" t="inlineStr">
         <is>
@@ -6834,7 +6838,7 @@
         </is>
       </c>
       <c r="J124" t="n">
-        <v>100000</v>
+        <v>60000</v>
       </c>
       <c r="K124" t="inlineStr"/>
     </row>
@@ -6851,24 +6855,24 @@
       </c>
       <c r="C125" t="inlineStr">
         <is>
-          <t>welding</t>
+          <t>masonry</t>
         </is>
       </c>
       <c r="D125" t="inlineStr">
         <is>
-          <t>Steel hanging rail for wall units + heater bracket</t>
+          <t>Level the corner castings: concrete pads or steel shims (rock corner)</t>
         </is>
       </c>
       <c r="E125" t="n">
-        <v>1</v>
+        <v>4</v>
       </c>
       <c r="F125" t="inlineStr">
         <is>
-          <t>set</t>
+          <t>each</t>
         </is>
       </c>
       <c r="G125" t="n">
-        <v>40000</v>
+        <v>25000</v>
       </c>
       <c r="H125" t="inlineStr">
         <is>
@@ -6881,7 +6885,7 @@
         </is>
       </c>
       <c r="J125" t="n">
-        <v>40000</v>
+        <v>100000</v>
       </c>
       <c r="K125" t="inlineStr"/>
     </row>
@@ -6893,17 +6897,17 @@
       </c>
       <c r="B126" t="inlineStr">
         <is>
-          <t>hardware</t>
+          <t>steel</t>
         </is>
       </c>
       <c r="C126" t="inlineStr">
         <is>
-          <t>glazier</t>
+          <t>welding</t>
         </is>
       </c>
       <c r="D126" t="inlineStr">
         <is>
-          <t>Keyed lock + secondary bolt for the slider</t>
+          <t>Steel hanging rail for wall units + heater bracket</t>
         </is>
       </c>
       <c r="E126" t="n">
@@ -6915,7 +6919,7 @@
         </is>
       </c>
       <c r="G126" t="n">
-        <v>45000</v>
+        <v>40000</v>
       </c>
       <c r="H126" t="inlineStr">
         <is>
@@ -6928,7 +6932,7 @@
         </is>
       </c>
       <c r="J126" t="n">
-        <v>45000</v>
+        <v>40000</v>
       </c>
       <c r="K126" t="inlineStr"/>
     </row>
@@ -6940,7 +6944,7 @@
       </c>
       <c r="B127" t="inlineStr">
         <is>
-          <t>glazing</t>
+          <t>hardware</t>
         </is>
       </c>
       <c r="C127" t="inlineStr">
@@ -6950,7 +6954,7 @@
       </c>
       <c r="D127" t="inlineStr">
         <is>
-          <t>Louvred trickle-vent strip with mesh (10,000 mm2)</t>
+          <t>Keyed lock + secondary bolt for the slider</t>
         </is>
       </c>
       <c r="E127" t="n">
@@ -6958,11 +6962,11 @@
       </c>
       <c r="F127" t="inlineStr">
         <is>
-          <t>each</t>
+          <t>set</t>
         </is>
       </c>
       <c r="G127" t="n">
-        <v>30000</v>
+        <v>45000</v>
       </c>
       <c r="H127" t="inlineStr">
         <is>
@@ -6975,7 +6979,7 @@
         </is>
       </c>
       <c r="J127" t="n">
-        <v>30000</v>
+        <v>45000</v>
       </c>
       <c r="K127" t="inlineStr"/>
     </row>
@@ -6987,17 +6991,17 @@
       </c>
       <c r="B128" t="inlineStr">
         <is>
-          <t>steel</t>
+          <t>glazing</t>
         </is>
       </c>
       <c r="C128" t="inlineStr">
         <is>
-          <t>welding</t>
+          <t>glazier</t>
         </is>
       </c>
       <c r="D128" t="inlineStr">
         <is>
-          <t>AC wall sleeve 75 mm (provision, back wall, one hole)</t>
+          <t>Louvred trickle-vent strip with mesh (10,000 mm2)</t>
         </is>
       </c>
       <c r="E128" t="n">
@@ -7009,7 +7013,7 @@
         </is>
       </c>
       <c r="G128" t="n">
-        <v>15000</v>
+        <v>30000</v>
       </c>
       <c r="H128" t="inlineStr">
         <is>
@@ -7022,19 +7026,19 @@
         </is>
       </c>
       <c r="J128" t="n">
-        <v>15000</v>
+        <v>30000</v>
       </c>
       <c r="K128" t="inlineStr"/>
     </row>
     <row r="129">
       <c r="A129" t="inlineStr">
         <is>
-          <t>K11</t>
+          <t>K10</t>
         </is>
       </c>
       <c r="B129" t="inlineStr">
         <is>
-          <t>roofing</t>
+          <t>steel</t>
         </is>
       </c>
       <c r="C129" t="inlineStr">
@@ -7044,7 +7048,7 @@
       </c>
       <c r="D129" t="inlineStr">
         <is>
-          <t>Gutter + downpipe to the rainwater tank (deck canopy)</t>
+          <t>AC wall sleeve 75 mm (provision, back wall, one hole)</t>
         </is>
       </c>
       <c r="E129" t="n">
@@ -7052,11 +7056,11 @@
       </c>
       <c r="F129" t="inlineStr">
         <is>
-          <t>set</t>
+          <t>each</t>
         </is>
       </c>
       <c r="G129" t="n">
-        <v>90000</v>
+        <v>15000</v>
       </c>
       <c r="H129" t="inlineStr">
         <is>
@@ -7069,7 +7073,7 @@
         </is>
       </c>
       <c r="J129" t="n">
-        <v>90000</v>
+        <v>15000</v>
       </c>
       <c r="K129" t="inlineStr"/>
     </row>
@@ -7081,17 +7085,17 @@
       </c>
       <c r="B130" t="inlineStr">
         <is>
-          <t>electrical</t>
+          <t>roofing</t>
         </is>
       </c>
       <c r="C130" t="inlineStr">
         <is>
-          <t>electrical</t>
+          <t>welding</t>
         </is>
       </c>
       <c r="D130" t="inlineStr">
         <is>
-          <t>Bonding: 16 mm2 green-yellow from the frame to the earth bar</t>
+          <t>Gutter + downpipe to the rainwater tank (deck canopy)</t>
         </is>
       </c>
       <c r="E130" t="n">
@@ -7103,7 +7107,7 @@
         </is>
       </c>
       <c r="G130" t="n">
-        <v>25000</v>
+        <v>90000</v>
       </c>
       <c r="H130" t="inlineStr">
         <is>
@@ -7116,41 +7120,41 @@
         </is>
       </c>
       <c r="J130" t="n">
-        <v>25000</v>
+        <v>90000</v>
       </c>
       <c r="K130" t="inlineStr"/>
     </row>
     <row r="131">
       <c r="A131" t="inlineStr">
         <is>
-          <t>K1</t>
+          <t>K11</t>
         </is>
       </c>
       <c r="B131" t="inlineStr">
         <is>
-          <t>timber</t>
+          <t>electrical</t>
         </is>
       </c>
       <c r="C131" t="inlineStr">
         <is>
-          <t>carpentry</t>
+          <t>electrical</t>
         </is>
       </c>
       <c r="D131" t="inlineStr">
         <is>
-          <t>Battens 38 x 50 treated, 2.4 m</t>
+          <t>Bonding: 16 mm2 green-yellow from the frame to the earth bar</t>
         </is>
       </c>
       <c r="E131" t="n">
-        <v>19.8</v>
+        <v>1</v>
       </c>
       <c r="F131" t="inlineStr">
         <is>
-          <t>each</t>
+          <t>set</t>
         </is>
       </c>
       <c r="G131" t="n">
-        <v>2500</v>
+        <v>25000</v>
       </c>
       <c r="H131" t="inlineStr">
         <is>
@@ -7163,18 +7167,14 @@
         </is>
       </c>
       <c r="J131" t="n">
-        <v>49500</v>
-      </c>
-      <c r="K131" t="inlineStr">
-        <is>
-          <t>38 x 50 treated, 2.4 m</t>
-        </is>
-      </c>
+        <v>25000</v>
+      </c>
+      <c r="K131" t="inlineStr"/>
     </row>
     <row r="132">
       <c r="A132" t="inlineStr">
         <is>
-          <t>K2</t>
+          <t>K1</t>
         </is>
       </c>
       <c r="B132" t="inlineStr">
@@ -7189,11 +7189,11 @@
       </c>
       <c r="D132" t="inlineStr">
         <is>
-          <t>Studs 40 x 40 treated, 2.4 m</t>
+          <t>Battens 38 x 50 treated, 2.4 m</t>
         </is>
       </c>
       <c r="E132" t="n">
-        <v>5.5</v>
+        <v>19.8</v>
       </c>
       <c r="F132" t="inlineStr">
         <is>
@@ -7201,7 +7201,7 @@
         </is>
       </c>
       <c r="G132" t="n">
-        <v>3000</v>
+        <v>2500</v>
       </c>
       <c r="H132" t="inlineStr">
         <is>
@@ -7214,41 +7214,45 @@
         </is>
       </c>
       <c r="J132" t="n">
-        <v>16500</v>
+        <v>49500</v>
       </c>
       <c r="K132" t="inlineStr">
         <is>
-          <t>40 x 40, 2.4 m</t>
+          <t>38 x 50 treated, 2.4 m</t>
         </is>
       </c>
     </row>
     <row r="133">
       <c r="A133" t="inlineStr">
         <is>
-          <t>labour</t>
+          <t>K2</t>
         </is>
       </c>
       <c r="B133" t="inlineStr">
         <is>
-          <t>labour</t>
-        </is>
-      </c>
-      <c r="C133" t="inlineStr"/>
+          <t>timber</t>
+        </is>
+      </c>
+      <c r="C133" t="inlineStr">
+        <is>
+          <t>carpentry</t>
+        </is>
+      </c>
       <c r="D133" t="inlineStr">
         <is>
-          <t>Carpentry workshop: cutting, edging, drilling, labelling (per unit kit)</t>
+          <t>Studs 40 x 40 treated, 2.4 m</t>
         </is>
       </c>
       <c r="E133" t="n">
-        <v>1</v>
+        <v>5.5</v>
       </c>
       <c r="F133" t="inlineStr">
         <is>
-          <t>lot</t>
+          <t>each</t>
         </is>
       </c>
       <c r="G133" t="n">
-        <v>450000</v>
+        <v>3000</v>
       </c>
       <c r="H133" t="inlineStr">
         <is>
@@ -7261,9 +7265,13 @@
         </is>
       </c>
       <c r="J133" t="n">
-        <v>450000</v>
-      </c>
-      <c r="K133" t="inlineStr"/>
+        <v>16500</v>
+      </c>
+      <c r="K133" t="inlineStr">
+        <is>
+          <t>40 x 40, 2.4 m</t>
+        </is>
+      </c>
     </row>
     <row r="134">
       <c r="A134" t="inlineStr">
@@ -7279,7 +7287,7 @@
       <c r="C134" t="inlineStr"/>
       <c r="D134" t="inlineStr">
         <is>
-          <t>Site carpentry and assembly: 2 people x 8 days</t>
+          <t>Carpentry workshop: cutting, edging, drilling, labelling (per unit kit)</t>
         </is>
       </c>
       <c r="E134" t="n">
@@ -7291,7 +7299,7 @@
         </is>
       </c>
       <c r="G134" t="n">
-        <v>320000</v>
+        <v>450000</v>
       </c>
       <c r="H134" t="inlineStr">
         <is>
@@ -7304,7 +7312,7 @@
         </is>
       </c>
       <c r="J134" t="n">
-        <v>320000</v>
+        <v>450000</v>
       </c>
       <c r="K134" t="inlineStr"/>
     </row>
@@ -7322,7 +7330,7 @@
       <c r="C135" t="inlineStr"/>
       <c r="D135" t="inlineStr">
         <is>
-          <t>Electrician (RURA class A), install + certificate</t>
+          <t>Site carpentry and assembly: 2 people x 8 days</t>
         </is>
       </c>
       <c r="E135" t="n">
@@ -7334,7 +7342,7 @@
         </is>
       </c>
       <c r="G135" t="n">
-        <v>250000</v>
+        <v>320000</v>
       </c>
       <c r="H135" t="inlineStr">
         <is>
@@ -7347,7 +7355,7 @@
         </is>
       </c>
       <c r="J135" t="n">
-        <v>250000</v>
+        <v>320000</v>
       </c>
       <c r="K135" t="inlineStr"/>
     </row>
@@ -7365,7 +7373,7 @@
       <c r="C136" t="inlineStr"/>
       <c r="D136" t="inlineStr">
         <is>
-          <t>Plumber, install + tests</t>
+          <t>Electrician (RURA class A), install + certificate</t>
         </is>
       </c>
       <c r="E136" t="n">
@@ -7377,7 +7385,7 @@
         </is>
       </c>
       <c r="G136" t="n">
-        <v>200000</v>
+        <v>250000</v>
       </c>
       <c r="H136" t="inlineStr">
         <is>
@@ -7390,7 +7398,7 @@
         </is>
       </c>
       <c r="J136" t="n">
-        <v>200000</v>
+        <v>250000</v>
       </c>
       <c r="K136" t="inlineStr"/>
     </row>
@@ -7408,7 +7416,7 @@
       <c r="C137" t="inlineStr"/>
       <c r="D137" t="inlineStr">
         <is>
-          <t>Tiler: wet walls and floor</t>
+          <t>Plumber, install + tests</t>
         </is>
       </c>
       <c r="E137" t="n">
@@ -7420,7 +7428,7 @@
         </is>
       </c>
       <c r="G137" t="n">
-        <v>150000</v>
+        <v>200000</v>
       </c>
       <c r="H137" t="inlineStr">
         <is>
@@ -7433,7 +7441,7 @@
         </is>
       </c>
       <c r="J137" t="n">
-        <v>150000</v>
+        <v>200000</v>
       </c>
       <c r="K137" t="inlineStr"/>
     </row>
@@ -7451,7 +7459,7 @@
       <c r="C138" t="inlineStr"/>
       <c r="D138" t="inlineStr">
         <is>
-          <t>Welder: W1, roof frame, deck canopy, stair (per unit)</t>
+          <t>Tiler: wet walls and floor</t>
         </is>
       </c>
       <c r="E138" t="n">
@@ -7463,7 +7471,7 @@
         </is>
       </c>
       <c r="G138" t="n">
-        <v>600000</v>
+        <v>150000</v>
       </c>
       <c r="H138" t="inlineStr">
         <is>
@@ -7476,7 +7484,7 @@
         </is>
       </c>
       <c r="J138" t="n">
-        <v>600000</v>
+        <v>150000</v>
       </c>
       <c r="K138" t="inlineStr"/>
     </row>
@@ -7494,7 +7502,7 @@
       <c r="C139" t="inlineStr"/>
       <c r="D139" t="inlineStr">
         <is>
-          <t>Transport Kigali to site (share of 2 truck trips)</t>
+          <t>Welder: W1, roof frame, deck canopy, stair (per unit)</t>
         </is>
       </c>
       <c r="E139" t="n">
@@ -7506,22 +7514,65 @@
         </is>
       </c>
       <c r="G139" t="n">
+        <v>600000</v>
+      </c>
+      <c r="H139" t="inlineStr">
+        <is>
+          <t>A</t>
+        </is>
+      </c>
+      <c r="I139" t="inlineStr">
+        <is>
+          <t>AS-21</t>
+        </is>
+      </c>
+      <c r="J139" t="n">
+        <v>600000</v>
+      </c>
+      <c r="K139" t="inlineStr"/>
+    </row>
+    <row r="140">
+      <c r="A140" t="inlineStr">
+        <is>
+          <t>labour</t>
+        </is>
+      </c>
+      <c r="B140" t="inlineStr">
+        <is>
+          <t>labour</t>
+        </is>
+      </c>
+      <c r="C140" t="inlineStr"/>
+      <c r="D140" t="inlineStr">
+        <is>
+          <t>Transport Kigali to site (share of 2 truck trips)</t>
+        </is>
+      </c>
+      <c r="E140" t="n">
+        <v>1</v>
+      </c>
+      <c r="F140" t="inlineStr">
+        <is>
+          <t>lot</t>
+        </is>
+      </c>
+      <c r="G140" t="n">
         <v>120000</v>
       </c>
-      <c r="H139" t="inlineStr">
-        <is>
-          <t>A</t>
-        </is>
-      </c>
-      <c r="I139" t="inlineStr">
-        <is>
-          <t>AS-21</t>
-        </is>
-      </c>
-      <c r="J139" t="n">
+      <c r="H140" t="inlineStr">
+        <is>
+          <t>A</t>
+        </is>
+      </c>
+      <c r="I140" t="inlineStr">
+        <is>
+          <t>AS-21</t>
+        </is>
+      </c>
+      <c r="J140" t="n">
         <v>120000</v>
       </c>
-      <c r="K139" t="inlineStr"/>
+      <c r="K140" t="inlineStr"/>
     </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>

</xml_diff>

<commit_message>
feat(studio): natural oak furniture, darker grey sofa, smoked-oak floor
The founder preferred another wood to mahogany: the joinery takes a
natural oak-tone stain, the sofa a soft dark grey cover, and the SPC
floor a darker smoked-oak decor, so the light wood stands out. The
render, the finishes table and the bill of materials follow.

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01KRyNxX68L5feJKbJnBKRyV
</commit_message>
<xml_diff>
--- a/public/designs/studio/data/bom.xlsx
+++ b/public/designs/studio/data/bom.xlsx
@@ -2141,7 +2141,7 @@
       </c>
       <c r="D28" t="inlineStr">
         <is>
-          <t>SPC flooring 5 mm + underlay (living area)</t>
+          <t>SPC flooring 5 mm, smoked-oak decor, + underlay (living area)</t>
         </is>
       </c>
       <c r="E28" t="n">
@@ -3768,7 +3768,7 @@
       </c>
       <c r="D61" t="inlineStr">
         <is>
-          <t>Low two-seat sofa about 1300 x 750, 700 high, washable covers</t>
+          <t>Low two-seat sofa about 1300 x 750, 700 high, soft dark grey washable covers</t>
         </is>
       </c>
       <c r="E61" t="n">
@@ -3913,7 +3913,7 @@
       </c>
       <c r="D64" t="inlineStr">
         <is>
-          <t>Joinery finish: natural mahogany-tone stain + satin PU varnish (all furniture)</t>
+          <t>Joinery finish: natural oak-tone stain + satin PU varnish (all furniture)</t>
         </is>
       </c>
       <c r="E64" t="n">
@@ -3942,7 +3942,7 @@
       </c>
       <c r="K64" t="inlineStr">
         <is>
-          <t>mahogany-tone wood stain + satin PU varnish, per L</t>
+          <t>oak-tone wood stain + satin PU varnish, per L</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
feat(studio): golden knotty pine joinery, lower seating table
The furniture takes the founder's reference wood: golden knotty pine
(pine-faced ply or solid pine, clear matte varnish, knots kept); the
render draws it procedurally after the photo. The seating table drops
to 550 mm with the chair seats at 400; the finishes table, the bill of
materials and the D-020 note follow.

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01KRyNxX68L5feJKbJnBKRyV
</commit_message>
<xml_diff>
--- a/public/designs/studio/data/bom.xlsx
+++ b/public/designs/studio/data/bom.xlsx
@@ -491,10 +491,10 @@
         </is>
       </c>
       <c r="B7" t="n">
-        <v>1208160</v>
+        <v>1207800</v>
       </c>
       <c r="C7" t="n">
-        <v>3624480</v>
+        <v>3623400</v>
       </c>
     </row>
     <row r="8">
@@ -736,10 +736,10 @@
         </is>
       </c>
       <c r="B26" t="n">
-        <v>2040370</v>
+        <v>2040316</v>
       </c>
       <c r="C26" t="n">
-        <v>6849511</v>
+        <v>6849349</v>
       </c>
     </row>
     <row r="27">
@@ -749,10 +749,10 @@
         </is>
       </c>
       <c r="B27" t="n">
-        <v>15642839</v>
+        <v>15642425</v>
       </c>
       <c r="C27" t="n">
-        <v>52512918</v>
+        <v>52511676</v>
       </c>
     </row>
     <row r="29">
@@ -763,7 +763,7 @@
       </c>
       <c r="B29" t="inlineStr"/>
       <c r="C29" t="n">
-        <v>35580</v>
+        <v>35579</v>
       </c>
     </row>
   </sheetData>
@@ -1063,7 +1063,7 @@
         </is>
       </c>
       <c r="E6" t="n">
-        <v>88.59999999999999</v>
+        <v>88</v>
       </c>
       <c r="F6" t="inlineStr">
         <is>
@@ -1084,7 +1084,7 @@
         </is>
       </c>
       <c r="J6" t="n">
-        <v>53160</v>
+        <v>52800</v>
       </c>
       <c r="K6" t="inlineStr">
         <is>
@@ -3913,7 +3913,7 @@
       </c>
       <c r="D64" t="inlineStr">
         <is>
-          <t>Joinery finish: natural oak-tone stain + satin PU varnish (all furniture)</t>
+          <t>Joinery finish: clear matte PU varnish over golden pine, knots kept (all furniture)</t>
         </is>
       </c>
       <c r="E64" t="n">
@@ -3942,7 +3942,7 @@
       </c>
       <c r="K64" t="inlineStr">
         <is>
-          <t>oak-tone wood stain + satin PU varnish, per L</t>
+          <t>clear matte PU varnish for pine joinery, per L</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
feat(studio): calmer, darker honey pine
The founder found the knotty pine too busy: the joinery keeps pine but
takes a darker honey-tone stain under clear matte varnish, with faint
grain and only a few soft knots. Render, finishes table and bill of
materials follow.

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01KRyNxX68L5feJKbJnBKRyV
</commit_message>
<xml_diff>
--- a/public/designs/studio/data/bom.xlsx
+++ b/public/designs/studio/data/bom.xlsx
@@ -3913,7 +3913,7 @@
       </c>
       <c r="D64" t="inlineStr">
         <is>
-          <t>Joinery finish: clear matte PU varnish over golden pine, knots kept (all furniture)</t>
+          <t>Joinery finish: honey-tone stain + clear matte PU varnish over pine (all furniture)</t>
         </is>
       </c>
       <c r="E64" t="n">
@@ -3942,7 +3942,7 @@
       </c>
       <c r="K64" t="inlineStr">
         <is>
-          <t>clear matte PU varnish for pine joinery, per L</t>
+          <t>honey-tone stain + clear matte PU varnish for pine, per L</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
feat(studio): slatted bed, bedroom rail and the bed piece by piece
The bed top is now 20 wooden slats laid across the bed with an 11.6 mm
gap, on two new ledgers and the spine (the founder's call), replacing
two drilled deck panels. Low rails get one bolt on their centreline:
the shared two-bolt pattern put a hole outside the 80 and 60 mm rails.
The studio now needs one fewer 18 mm sheet.

/en/studio: the bedroom pieces become a horizontal rail of product
cards after databayt.org's products rail (native scroll-snap, no
Embla), rendered on a transparent ground. A new Bed section breaks
kit K4 into its 41 pieces: the stock to buy and where, one cutting
diagram per sheet, each piece's size and its cut, edge, drill and
finish steps, then the assembly. bed_parts.py nests the bed alone and
writes the data the section and room.html?bed= read.

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01KUWWUBfSNDQyavvXAD1cc3
</commit_message>
<xml_diff>
--- a/public/designs/studio/data/bom.xlsx
+++ b/public/designs/studio/data/bom.xlsx
@@ -491,10 +491,10 @@
         </is>
       </c>
       <c r="B7" t="n">
-        <v>1254120</v>
+        <v>1251420</v>
       </c>
       <c r="C7" t="n">
-        <v>3762360</v>
+        <v>3754260</v>
       </c>
     </row>
     <row r="8">
@@ -647,10 +647,10 @@
         </is>
       </c>
       <c r="B19" t="n">
-        <v>170273</v>
+        <v>171218</v>
       </c>
       <c r="C19" t="n">
-        <v>510819</v>
+        <v>513654</v>
       </c>
     </row>
     <row r="20">
@@ -736,10 +736,10 @@
         </is>
       </c>
       <c r="B26" t="n">
-        <v>2047384</v>
+        <v>2047121</v>
       </c>
       <c r="C26" t="n">
-        <v>6870553</v>
+        <v>6869763</v>
       </c>
     </row>
     <row r="27">
@@ -749,10 +749,10 @@
         </is>
       </c>
       <c r="B27" t="n">
-        <v>15696613</v>
+        <v>15694595</v>
       </c>
       <c r="C27" t="n">
-        <v>52674240</v>
+        <v>52668185</v>
       </c>
     </row>
     <row r="29">
@@ -763,7 +763,7 @@
       </c>
       <c r="B29" t="inlineStr"/>
       <c r="C29" t="n">
-        <v>35689</v>
+        <v>35685</v>
       </c>
     </row>
   </sheetData>
@@ -961,7 +961,7 @@
         </is>
       </c>
       <c r="E4" t="n">
-        <v>9</v>
+        <v>8</v>
       </c>
       <c r="F4" t="inlineStr">
         <is>
@@ -982,7 +982,7 @@
         </is>
       </c>
       <c r="J4" t="n">
-        <v>405000</v>
+        <v>360000</v>
       </c>
       <c r="K4" t="inlineStr">
         <is>
@@ -1063,7 +1063,7 @@
         </is>
       </c>
       <c r="E6" t="n">
-        <v>90.2</v>
+        <v>160.7</v>
       </c>
       <c r="F6" t="inlineStr">
         <is>
@@ -1084,7 +1084,7 @@
         </is>
       </c>
       <c r="J6" t="n">
-        <v>54120</v>
+        <v>96420</v>
       </c>
       <c r="K6" t="inlineStr">
         <is>
@@ -1208,7 +1208,7 @@
         </is>
       </c>
       <c r="E9" t="n">
-        <v>31.5</v>
+        <v>29.4</v>
       </c>
       <c r="F9" t="inlineStr">
         <is>
@@ -1229,7 +1229,7 @@
         </is>
       </c>
       <c r="J9" t="n">
-        <v>18900</v>
+        <v>17640</v>
       </c>
       <c r="K9" t="inlineStr"/>
     </row>
@@ -1349,7 +1349,7 @@
         </is>
       </c>
       <c r="E12" t="n">
-        <v>298.2</v>
+        <v>445.2</v>
       </c>
       <c r="F12" t="inlineStr">
         <is>
@@ -1370,7 +1370,7 @@
         </is>
       </c>
       <c r="J12" t="n">
-        <v>4473</v>
+        <v>6678</v>
       </c>
       <c r="K12" t="inlineStr"/>
     </row>

</xml_diff>

<commit_message>
feat(studio): electrical plans one studio from its own power inlet
The studio no longer assumes a site board and feeder. It plugs in through
a 63 A IP67 inlet on the back wall, so any 230 V source (grid, site board,
generator, inverter) can feed it; the section now covers the installation
from the inlet to every circuit.

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01MmmvYpwvCkLHKUJEnNsLYF
</commit_message>
<xml_diff>
--- a/public/designs/studio/data/bom.xlsx
+++ b/public/designs/studio/data/bom.xlsx
@@ -530,10 +530,10 @@
         </is>
       </c>
       <c r="B10" t="n">
-        <v>739350</v>
+        <v>814350</v>
       </c>
       <c r="C10" t="n">
-        <v>2218050</v>
+        <v>2443050</v>
       </c>
     </row>
     <row r="11">
@@ -736,10 +736,10 @@
         </is>
       </c>
       <c r="B26" t="n">
-        <v>2047121</v>
+        <v>2058371</v>
       </c>
       <c r="C26" t="n">
-        <v>6869763</v>
+        <v>6903513</v>
       </c>
     </row>
     <row r="27">
@@ -749,10 +749,10 @@
         </is>
       </c>
       <c r="B27" t="n">
-        <v>15694595</v>
+        <v>15780845</v>
       </c>
       <c r="C27" t="n">
-        <v>52668185</v>
+        <v>52926935</v>
       </c>
     </row>
     <row r="29">
@@ -763,7 +763,7 @@
       </c>
       <c r="B29" t="inlineStr"/>
       <c r="C29" t="n">
-        <v>35685</v>
+        <v>35861</v>
       </c>
     </row>
   </sheetData>
@@ -777,7 +777,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:K140"/>
+  <dimension ref="A1:K143"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -4019,7 +4019,7 @@
       </c>
       <c r="D66" t="inlineStr">
         <is>
-          <t>Ceiling light, bed</t>
+          <t>Power inlet 63 A IP67 (IEC 60309 blue, 2P+E), outside behind the board</t>
         </is>
       </c>
       <c r="E66" t="n">
@@ -4031,7 +4031,7 @@
         </is>
       </c>
       <c r="G66" t="n">
-        <v>15000</v>
+        <v>45000</v>
       </c>
       <c r="H66" t="inlineStr">
         <is>
@@ -4044,9 +4044,13 @@
         </is>
       </c>
       <c r="J66" t="n">
-        <v>15000</v>
-      </c>
-      <c r="K66" t="inlineStr"/>
+        <v>45000</v>
+      </c>
+      <c r="K66" t="inlineStr">
+        <is>
+          <t>surface, IP67</t>
+        </is>
+      </c>
     </row>
     <row r="67">
       <c r="A67" t="inlineStr">
@@ -4066,7 +4070,7 @@
       </c>
       <c r="D67" t="inlineStr">
         <is>
-          <t>Ceiling light, living</t>
+          <t>Ceiling light, bed</t>
         </is>
       </c>
       <c r="E67" t="n">
@@ -4113,7 +4117,7 @@
       </c>
       <c r="D68" t="inlineStr">
         <is>
-          <t>Ceiling light, galley</t>
+          <t>Ceiling light, living</t>
         </is>
       </c>
       <c r="E68" t="n">
@@ -4160,7 +4164,7 @@
       </c>
       <c r="D69" t="inlineStr">
         <is>
-          <t>Bathroom light IP65</t>
+          <t>Ceiling light, galley</t>
         </is>
       </c>
       <c r="E69" t="n">
@@ -4207,7 +4211,7 @@
       </c>
       <c r="D70" t="inlineStr">
         <is>
-          <t>Wall reading light over the bed (wall side)</t>
+          <t>Bathroom light IP65</t>
         </is>
       </c>
       <c r="E70" t="n">
@@ -4254,7 +4258,7 @@
       </c>
       <c r="D71" t="inlineStr">
         <is>
-          <t>Under-cabinet LED strip</t>
+          <t>Wall reading light over the bed (wall side)</t>
         </is>
       </c>
       <c r="E71" t="n">
@@ -4301,7 +4305,7 @@
       </c>
       <c r="D72" t="inlineStr">
         <is>
-          <t>Deck light IP65</t>
+          <t>Under-cabinet LED strip</t>
         </is>
       </c>
       <c r="E72" t="n">
@@ -4348,7 +4352,7 @@
       </c>
       <c r="D73" t="inlineStr">
         <is>
-          <t>Roof terrace lights IP65 (x2)</t>
+          <t>Deck light IP65</t>
         </is>
       </c>
       <c r="E73" t="n">
@@ -4395,7 +4399,7 @@
       </c>
       <c r="D74" t="inlineStr">
         <is>
-          <t>Stair light IP65</t>
+          <t>Roof terrace lights IP65 (x2)</t>
         </is>
       </c>
       <c r="E74" t="n">
@@ -4442,7 +4446,7 @@
       </c>
       <c r="D75" t="inlineStr">
         <is>
-          <t>Entry: living + kitchen + deck</t>
+          <t>Stair light IP65</t>
         </is>
       </c>
       <c r="E75" t="n">
@@ -4454,7 +4458,7 @@
         </is>
       </c>
       <c r="G75" t="n">
-        <v>3500</v>
+        <v>15000</v>
       </c>
       <c r="H75" t="inlineStr">
         <is>
@@ -4467,7 +4471,7 @@
         </is>
       </c>
       <c r="J75" t="n">
-        <v>3500</v>
+        <v>15000</v>
       </c>
       <c r="K75" t="inlineStr"/>
     </row>
@@ -4489,7 +4493,7 @@
       </c>
       <c r="D76" t="inlineStr">
         <is>
-          <t>Bed: ceiling light (2-way), over the bedside table</t>
+          <t>Entry: living + kitchen + deck</t>
         </is>
       </c>
       <c r="E76" t="n">
@@ -4536,7 +4540,7 @@
       </c>
       <c r="D77" t="inlineStr">
         <is>
-          <t>Bathroom light + fan (outside)</t>
+          <t>Bed: ceiling light (2-way), over the bedside table</t>
         </is>
       </c>
       <c r="E77" t="n">
@@ -4583,7 +4587,7 @@
       </c>
       <c r="D78" t="inlineStr">
         <is>
-          <t>Roof and stair lights (IP65, stair foot)</t>
+          <t>Bathroom light + fan (outside)</t>
         </is>
       </c>
       <c r="E78" t="n">
@@ -4630,7 +4634,7 @@
       </c>
       <c r="D79" t="inlineStr">
         <is>
-          <t>Socket + USB-C in the headboard (wall side)</t>
+          <t>Roof and stair lights (IP65, stair foot)</t>
         </is>
       </c>
       <c r="E79" t="n">
@@ -4642,7 +4646,7 @@
         </is>
       </c>
       <c r="G79" t="n">
-        <v>15000</v>
+        <v>3500</v>
       </c>
       <c r="H79" t="inlineStr">
         <is>
@@ -4655,7 +4659,7 @@
         </is>
       </c>
       <c r="J79" t="n">
-        <v>15000</v>
+        <v>3500</v>
       </c>
       <c r="K79" t="inlineStr"/>
     </row>
@@ -4677,7 +4681,7 @@
       </c>
       <c r="D80" t="inlineStr">
         <is>
-          <t>Bedside socket + USB-C (reading lamp)</t>
+          <t>Socket + USB-C in the headboard (wall side)</t>
         </is>
       </c>
       <c r="E80" t="n">
@@ -4724,7 +4728,7 @@
       </c>
       <c r="D81" t="inlineStr">
         <is>
-          <t>Socket by the sofa</t>
+          <t>Bedside socket + USB-C (reading lamp)</t>
         </is>
       </c>
       <c r="E81" t="n">
@@ -4736,7 +4740,7 @@
         </is>
       </c>
       <c r="G81" t="n">
-        <v>5000</v>
+        <v>15000</v>
       </c>
       <c r="H81" t="inlineStr">
         <is>
@@ -4749,7 +4753,7 @@
         </is>
       </c>
       <c r="J81" t="n">
-        <v>5000</v>
+        <v>15000</v>
       </c>
       <c r="K81" t="inlineStr"/>
     </row>
@@ -4771,7 +4775,7 @@
       </c>
       <c r="D82" t="inlineStr">
         <is>
-          <t>Socket, living (front strip)</t>
+          <t>Socket by the sofa</t>
         </is>
       </c>
       <c r="E82" t="n">
@@ -4818,7 +4822,7 @@
       </c>
       <c r="D83" t="inlineStr">
         <is>
-          <t>Deck socket IP66</t>
+          <t>Socket, living (front strip)</t>
         </is>
       </c>
       <c r="E83" t="n">
@@ -4865,7 +4869,7 @@
       </c>
       <c r="D84" t="inlineStr">
         <is>
-          <t>Worktop socket 1 (double)</t>
+          <t>Deck socket IP66</t>
         </is>
       </c>
       <c r="E84" t="n">
@@ -4912,7 +4916,7 @@
       </c>
       <c r="D85" t="inlineStr">
         <is>
-          <t>Worktop socket 2 (double, back wall)</t>
+          <t>Worktop socket 1 (double)</t>
         </is>
       </c>
       <c r="E85" t="n">
@@ -4959,7 +4963,7 @@
       </c>
       <c r="D86" t="inlineStr">
         <is>
-          <t>Fridge socket</t>
+          <t>Worktop socket 2 (double, back wall)</t>
         </is>
       </c>
       <c r="E86" t="n">
@@ -5006,7 +5010,7 @@
       </c>
       <c r="D87" t="inlineStr">
         <is>
-          <t>Hob connection unit</t>
+          <t>Fridge socket</t>
         </is>
       </c>
       <c r="E87" t="n">
@@ -5018,7 +5022,7 @@
         </is>
       </c>
       <c r="G87" t="n">
-        <v>9000</v>
+        <v>5000</v>
       </c>
       <c r="H87" t="inlineStr">
         <is>
@@ -5031,7 +5035,7 @@
         </is>
       </c>
       <c r="J87" t="n">
-        <v>9000</v>
+        <v>5000</v>
       </c>
       <c r="K87" t="inlineStr"/>
     </row>
@@ -5053,7 +5057,7 @@
       </c>
       <c r="D88" t="inlineStr">
         <is>
-          <t>Heater DP switch + timer</t>
+          <t>Hob connection unit</t>
         </is>
       </c>
       <c r="E88" t="n">
@@ -5100,7 +5104,7 @@
       </c>
       <c r="D89" t="inlineStr">
         <is>
-          <t>Bathroom extract 100 mm (one 110 mm hole in the back wall)</t>
+          <t>Heater DP switch + timer</t>
         </is>
       </c>
       <c r="E89" t="n">
@@ -5112,7 +5116,7 @@
         </is>
       </c>
       <c r="G89" t="n">
-        <v>35000</v>
+        <v>9000</v>
       </c>
       <c r="H89" t="inlineStr">
         <is>
@@ -5125,7 +5129,7 @@
         </is>
       </c>
       <c r="J89" t="n">
-        <v>35000</v>
+        <v>9000</v>
       </c>
       <c r="K89" t="inlineStr"/>
     </row>
@@ -5147,7 +5151,7 @@
       </c>
       <c r="D90" t="inlineStr">
         <is>
-          <t>Wall fan</t>
+          <t>Bathroom extract 100 mm (one 110 mm hole in the back wall)</t>
         </is>
       </c>
       <c r="E90" t="n">
@@ -5194,7 +5198,7 @@
       </c>
       <c r="D91" t="inlineStr">
         <is>
-          <t>AC provision: isolator</t>
+          <t>Wall fan</t>
         </is>
       </c>
       <c r="E91" t="n">
@@ -5206,7 +5210,7 @@
         </is>
       </c>
       <c r="G91" t="n">
-        <v>9000</v>
+        <v>35000</v>
       </c>
       <c r="H91" t="inlineStr">
         <is>
@@ -5219,7 +5223,7 @@
         </is>
       </c>
       <c r="J91" t="n">
-        <v>9000</v>
+        <v>35000</v>
       </c>
       <c r="K91" t="inlineStr"/>
     </row>
@@ -5241,19 +5245,19 @@
       </c>
       <c r="D92" t="inlineStr">
         <is>
-          <t>Cable 1.5 mm2 T+E/singles in conduit, Lighting (incl. bathroom IP65, deck, roof, stair)</t>
+          <t>AC provision: isolator</t>
         </is>
       </c>
       <c r="E92" t="n">
-        <v>85</v>
+        <v>1</v>
       </c>
       <c r="F92" t="inlineStr">
         <is>
-          <t>m</t>
+          <t>each</t>
         </is>
       </c>
       <c r="G92" t="n">
-        <v>500</v>
+        <v>9000</v>
       </c>
       <c r="H92" t="inlineStr">
         <is>
@@ -5266,13 +5270,9 @@
         </is>
       </c>
       <c r="J92" t="n">
-        <v>42500</v>
-      </c>
-      <c r="K92" t="inlineStr">
-        <is>
-          <t>per m</t>
-        </is>
-      </c>
+        <v>9000</v>
+      </c>
+      <c r="K92" t="inlineStr"/>
     </row>
     <row r="93">
       <c r="A93" t="inlineStr">
@@ -5292,11 +5292,11 @@
       </c>
       <c r="D93" t="inlineStr">
         <is>
-          <t>Cable 2.5 mm2 T+E/singles in conduit, Sockets: bedside USB, living, deck</t>
+          <t>Cable 1.5 mm2 T+E/singles in conduit, Lighting (incl. bathroom IP65, deck, roof, stair)</t>
         </is>
       </c>
       <c r="E93" t="n">
-        <v>30</v>
+        <v>85</v>
       </c>
       <c r="F93" t="inlineStr">
         <is>
@@ -5304,7 +5304,7 @@
         </is>
       </c>
       <c r="G93" t="n">
-        <v>750</v>
+        <v>500</v>
       </c>
       <c r="H93" t="inlineStr">
         <is>
@@ -5317,7 +5317,7 @@
         </is>
       </c>
       <c r="J93" t="n">
-        <v>22500</v>
+        <v>42500</v>
       </c>
       <c r="K93" t="inlineStr">
         <is>
@@ -5343,11 +5343,11 @@
       </c>
       <c r="D94" t="inlineStr">
         <is>
-          <t>Cable 2.5 mm2 T+E/singles in conduit, Kitchen sockets and fridge</t>
+          <t>Cable 2.5 mm2 T+E/singles in conduit, Sockets: bedside USB, living, deck</t>
         </is>
       </c>
       <c r="E94" t="n">
-        <v>13</v>
+        <v>30</v>
       </c>
       <c r="F94" t="inlineStr">
         <is>
@@ -5368,7 +5368,7 @@
         </is>
       </c>
       <c r="J94" t="n">
-        <v>9750</v>
+        <v>22500</v>
       </c>
       <c r="K94" t="inlineStr">
         <is>
@@ -5394,11 +5394,11 @@
       </c>
       <c r="D95" t="inlineStr">
         <is>
-          <t>Cable 4.0 mm2 T+E/singles in conduit, Induction hob</t>
+          <t>Cable 2.5 mm2 T+E/singles in conduit, Kitchen sockets and fridge</t>
         </is>
       </c>
       <c r="E95" t="n">
-        <v>8</v>
+        <v>13</v>
       </c>
       <c r="F95" t="inlineStr">
         <is>
@@ -5406,7 +5406,7 @@
         </is>
       </c>
       <c r="G95" t="n">
-        <v>1200</v>
+        <v>750</v>
       </c>
       <c r="H95" t="inlineStr">
         <is>
@@ -5419,7 +5419,7 @@
         </is>
       </c>
       <c r="J95" t="n">
-        <v>9600</v>
+        <v>9750</v>
       </c>
       <c r="K95" t="inlineStr">
         <is>
@@ -5445,11 +5445,11 @@
       </c>
       <c r="D96" t="inlineStr">
         <is>
-          <t>Cable 2.5 mm2 T+E/singles in conduit, 80 L water heater</t>
+          <t>Cable 4.0 mm2 T+E/singles in conduit, Induction hob</t>
         </is>
       </c>
       <c r="E96" t="n">
-        <v>7</v>
+        <v>8</v>
       </c>
       <c r="F96" t="inlineStr">
         <is>
@@ -5457,7 +5457,7 @@
         </is>
       </c>
       <c r="G96" t="n">
-        <v>750</v>
+        <v>1200</v>
       </c>
       <c r="H96" t="inlineStr">
         <is>
@@ -5470,7 +5470,7 @@
         </is>
       </c>
       <c r="J96" t="n">
-        <v>5250</v>
+        <v>9600</v>
       </c>
       <c r="K96" t="inlineStr">
         <is>
@@ -5496,11 +5496,11 @@
       </c>
       <c r="D97" t="inlineStr">
         <is>
-          <t>Cable 1.5 mm2 T+E/singles in conduit, Extract fan and wall fan</t>
+          <t>Cable 2.5 mm2 T+E/singles in conduit, 80 L water heater</t>
         </is>
       </c>
       <c r="E97" t="n">
-        <v>9</v>
+        <v>7</v>
       </c>
       <c r="F97" t="inlineStr">
         <is>
@@ -5508,7 +5508,7 @@
         </is>
       </c>
       <c r="G97" t="n">
-        <v>500</v>
+        <v>750</v>
       </c>
       <c r="H97" t="inlineStr">
         <is>
@@ -5521,7 +5521,7 @@
         </is>
       </c>
       <c r="J97" t="n">
-        <v>4500</v>
+        <v>5250</v>
       </c>
       <c r="K97" t="inlineStr">
         <is>
@@ -5547,11 +5547,11 @@
       </c>
       <c r="D98" t="inlineStr">
         <is>
-          <t>Cable 2.5 mm2 T+E/singles in conduit, AC provision</t>
+          <t>Cable 1.5 mm2 T+E/singles in conduit, Extract fan and wall fan</t>
         </is>
       </c>
       <c r="E98" t="n">
-        <v>7</v>
+        <v>9</v>
       </c>
       <c r="F98" t="inlineStr">
         <is>
@@ -5559,7 +5559,7 @@
         </is>
       </c>
       <c r="G98" t="n">
-        <v>750</v>
+        <v>500</v>
       </c>
       <c r="H98" t="inlineStr">
         <is>
@@ -5572,7 +5572,7 @@
         </is>
       </c>
       <c r="J98" t="n">
-        <v>5250</v>
+        <v>4500</v>
       </c>
       <c r="K98" t="inlineStr">
         <is>
@@ -5598,11 +5598,11 @@
       </c>
       <c r="D99" t="inlineStr">
         <is>
-          <t>PVC conduit 20 mm + boxes</t>
+          <t>Cable 2.5 mm2 T+E/singles in conduit, AC provision</t>
         </is>
       </c>
       <c r="E99" t="n">
-        <v>60</v>
+        <v>7</v>
       </c>
       <c r="F99" t="inlineStr">
         <is>
@@ -5610,7 +5610,7 @@
         </is>
       </c>
       <c r="G99" t="n">
-        <v>600</v>
+        <v>750</v>
       </c>
       <c r="H99" t="inlineStr">
         <is>
@@ -5623,7 +5623,7 @@
         </is>
       </c>
       <c r="J99" t="n">
-        <v>36000</v>
+        <v>5250</v>
       </c>
       <c r="K99" t="inlineStr">
         <is>
@@ -5649,19 +5649,19 @@
       </c>
       <c r="D100" t="inlineStr">
         <is>
-          <t>Surge protection device type 2</t>
+          <t>Cable 10 mm2 tails, inlet to main switch, through a gland in the back wall</t>
         </is>
       </c>
       <c r="E100" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="F100" t="inlineStr">
         <is>
-          <t>each</t>
+          <t>m</t>
         </is>
       </c>
       <c r="G100" t="n">
-        <v>60000</v>
+        <v>2500</v>
       </c>
       <c r="H100" t="inlineStr">
         <is>
@@ -5674,9 +5674,13 @@
         </is>
       </c>
       <c r="J100" t="n">
-        <v>60000</v>
-      </c>
-      <c r="K100" t="inlineStr"/>
+        <v>5000</v>
+      </c>
+      <c r="K100" t="inlineStr">
+        <is>
+          <t>per m</t>
+        </is>
+      </c>
     </row>
     <row r="101">
       <c r="A101" t="inlineStr">
@@ -5696,7 +5700,7 @@
       </c>
       <c r="D101" t="inlineStr">
         <is>
-          <t>RCD 40 A 30 mA type A (or RCBOs)</t>
+          <t>Matching 63 A plug (IEC 60309 blue), for whatever supply cable</t>
         </is>
       </c>
       <c r="E101" t="n">
@@ -5708,7 +5712,7 @@
         </is>
       </c>
       <c r="G101" t="n">
-        <v>45000</v>
+        <v>25000</v>
       </c>
       <c r="H101" t="inlineStr">
         <is>
@@ -5721,9 +5725,13 @@
         </is>
       </c>
       <c r="J101" t="n">
-        <v>45000</v>
-      </c>
-      <c r="K101" t="inlineStr"/>
+        <v>25000</v>
+      </c>
+      <c r="K101" t="inlineStr">
+        <is>
+          <t>IP67</t>
+        </is>
+      </c>
     </row>
     <row r="102">
       <c r="A102" t="inlineStr">
@@ -5743,19 +5751,19 @@
       </c>
       <c r="D102" t="inlineStr">
         <is>
-          <t>MCBs (B6 x2, B16 x5, B20 x1)</t>
+          <t>PVC conduit 20 mm + boxes</t>
         </is>
       </c>
       <c r="E102" t="n">
-        <v>8</v>
+        <v>60</v>
       </c>
       <c r="F102" t="inlineStr">
         <is>
-          <t>each</t>
+          <t>m</t>
         </is>
       </c>
       <c r="G102" t="n">
-        <v>6000</v>
+        <v>600</v>
       </c>
       <c r="H102" t="inlineStr">
         <is>
@@ -5768,9 +5776,13 @@
         </is>
       </c>
       <c r="J102" t="n">
-        <v>48000</v>
-      </c>
-      <c r="K102" t="inlineStr"/>
+        <v>36000</v>
+      </c>
+      <c r="K102" t="inlineStr">
+        <is>
+          <t>per m</t>
+        </is>
+      </c>
     </row>
     <row r="103">
       <c r="A103" t="inlineStr">
@@ -5790,7 +5802,7 @@
       </c>
       <c r="D103" t="inlineStr">
         <is>
-          <t>Main switch 40 A DP + check meter (DIN kWh)</t>
+          <t>Surge protection device type 2</t>
         </is>
       </c>
       <c r="E103" t="n">
@@ -5798,11 +5810,11 @@
       </c>
       <c r="F103" t="inlineStr">
         <is>
-          <t>set</t>
+          <t>each</t>
         </is>
       </c>
       <c r="G103" t="n">
-        <v>40000</v>
+        <v>60000</v>
       </c>
       <c r="H103" t="inlineStr">
         <is>
@@ -5815,7 +5827,7 @@
         </is>
       </c>
       <c r="J103" t="n">
-        <v>40000</v>
+        <v>60000</v>
       </c>
       <c r="K103" t="inlineStr"/>
     </row>
@@ -5837,7 +5849,7 @@
       </c>
       <c r="D104" t="inlineStr">
         <is>
-          <t>Earth rod 1.5 m copper-bonded + clamp + inspection pit</t>
+          <t>RCD 40 A 30 mA type A (or RCBOs)</t>
         </is>
       </c>
       <c r="E104" t="n">
@@ -5849,7 +5861,7 @@
         </is>
       </c>
       <c r="G104" t="n">
-        <v>35000</v>
+        <v>45000</v>
       </c>
       <c r="H104" t="inlineStr">
         <is>
@@ -5862,7 +5874,7 @@
         </is>
       </c>
       <c r="J104" t="n">
-        <v>35000</v>
+        <v>45000</v>
       </c>
       <c r="K104" t="inlineStr"/>
     </row>
@@ -5874,7 +5886,7 @@
       </c>
       <c r="B105" t="inlineStr">
         <is>
-          <t>safety</t>
+          <t>electrical</t>
         </is>
       </c>
       <c r="C105" t="inlineStr">
@@ -5884,11 +5896,11 @@
       </c>
       <c r="D105" t="inlineStr">
         <is>
-          <t>Smoke alarm (10-year) + heat alarm (kitchen)</t>
+          <t>MCBs (B6 x2, B16 x5, B20 x1)</t>
         </is>
       </c>
       <c r="E105" t="n">
-        <v>2</v>
+        <v>8</v>
       </c>
       <c r="F105" t="inlineStr">
         <is>
@@ -5896,7 +5908,7 @@
         </is>
       </c>
       <c r="G105" t="n">
-        <v>20000</v>
+        <v>6000</v>
       </c>
       <c r="H105" t="inlineStr">
         <is>
@@ -5909,7 +5921,7 @@
         </is>
       </c>
       <c r="J105" t="n">
-        <v>40000</v>
+        <v>48000</v>
       </c>
       <c r="K105" t="inlineStr"/>
     </row>
@@ -5921,17 +5933,17 @@
       </c>
       <c r="B106" t="inlineStr">
         <is>
-          <t>safety</t>
+          <t>electrical</t>
         </is>
       </c>
       <c r="C106" t="inlineStr">
         <is>
-          <t>furnishing</t>
+          <t>electrical</t>
         </is>
       </c>
       <c r="D106" t="inlineStr">
         <is>
-          <t>Fire extinguisher 2 kg ABC + fire blanket</t>
+          <t>Main switch 40 A DP + check meter (DIN kWh)</t>
         </is>
       </c>
       <c r="E106" t="n">
@@ -5943,7 +5955,7 @@
         </is>
       </c>
       <c r="G106" t="n">
-        <v>55000</v>
+        <v>40000</v>
       </c>
       <c r="H106" t="inlineStr">
         <is>
@@ -5956,41 +5968,41 @@
         </is>
       </c>
       <c r="J106" t="n">
-        <v>55000</v>
+        <v>40000</v>
       </c>
       <c r="K106" t="inlineStr"/>
     </row>
     <row r="107">
       <c r="A107" t="inlineStr">
         <is>
-          <t>K9</t>
+          <t>K8</t>
         </is>
       </c>
       <c r="B107" t="inlineStr">
         <is>
-          <t>plumbing</t>
+          <t>electrical</t>
         </is>
       </c>
       <c r="C107" t="inlineStr">
         <is>
-          <t>plumbing</t>
+          <t>electrical</t>
         </is>
       </c>
       <c r="D107" t="inlineStr">
         <is>
-          <t>PPR PN20 pipe DN20</t>
+          <t>Earth rod 1.5 m copper-bonded + clamp + inspection pit</t>
         </is>
       </c>
       <c r="E107" t="n">
-        <v>9.300000000000001</v>
+        <v>1</v>
       </c>
       <c r="F107" t="inlineStr">
         <is>
-          <t>m</t>
+          <t>each</t>
         </is>
       </c>
       <c r="G107" t="n">
-        <v>2000</v>
+        <v>35000</v>
       </c>
       <c r="H107" t="inlineStr">
         <is>
@@ -6003,45 +6015,41 @@
         </is>
       </c>
       <c r="J107" t="n">
-        <v>18600</v>
-      </c>
-      <c r="K107" t="inlineStr">
-        <is>
-          <t>per m</t>
-        </is>
-      </c>
+        <v>35000</v>
+      </c>
+      <c r="K107" t="inlineStr"/>
     </row>
     <row r="108">
       <c r="A108" t="inlineStr">
         <is>
-          <t>K9</t>
+          <t>K8</t>
         </is>
       </c>
       <c r="B108" t="inlineStr">
         <is>
-          <t>plumbing</t>
+          <t>safety</t>
         </is>
       </c>
       <c r="C108" t="inlineStr">
         <is>
-          <t>plumbing</t>
+          <t>electrical</t>
         </is>
       </c>
       <c r="D108" t="inlineStr">
         <is>
-          <t>PPR PN20 pipe DN25</t>
+          <t>Smoke alarm (10-year) + heat alarm (kitchen)</t>
         </is>
       </c>
       <c r="E108" t="n">
-        <v>4.4</v>
+        <v>2</v>
       </c>
       <c r="F108" t="inlineStr">
         <is>
-          <t>m</t>
+          <t>each</t>
         </is>
       </c>
       <c r="G108" t="n">
-        <v>2800</v>
+        <v>20000</v>
       </c>
       <c r="H108" t="inlineStr">
         <is>
@@ -6054,45 +6062,41 @@
         </is>
       </c>
       <c r="J108" t="n">
-        <v>12320</v>
-      </c>
-      <c r="K108" t="inlineStr">
-        <is>
-          <t>per m</t>
-        </is>
-      </c>
+        <v>40000</v>
+      </c>
+      <c r="K108" t="inlineStr"/>
     </row>
     <row r="109">
       <c r="A109" t="inlineStr">
         <is>
-          <t>K9</t>
+          <t>K8</t>
         </is>
       </c>
       <c r="B109" t="inlineStr">
         <is>
-          <t>plumbing</t>
+          <t>safety</t>
         </is>
       </c>
       <c r="C109" t="inlineStr">
         <is>
-          <t>plumbing</t>
+          <t>furnishing</t>
         </is>
       </c>
       <c r="D109" t="inlineStr">
         <is>
-          <t>PPR PN20 pipe (hot) DN20</t>
+          <t>Fire extinguisher 2 kg ABC + fire blanket</t>
         </is>
       </c>
       <c r="E109" t="n">
-        <v>4.7</v>
+        <v>1</v>
       </c>
       <c r="F109" t="inlineStr">
         <is>
-          <t>m</t>
+          <t>set</t>
         </is>
       </c>
       <c r="G109" t="n">
-        <v>2000</v>
+        <v>55000</v>
       </c>
       <c r="H109" t="inlineStr">
         <is>
@@ -6105,13 +6109,9 @@
         </is>
       </c>
       <c r="J109" t="n">
-        <v>9400</v>
-      </c>
-      <c r="K109" t="inlineStr">
-        <is>
-          <t>per m</t>
-        </is>
-      </c>
+        <v>55000</v>
+      </c>
+      <c r="K109" t="inlineStr"/>
     </row>
     <row r="110">
       <c r="A110" t="inlineStr">
@@ -6131,11 +6131,11 @@
       </c>
       <c r="D110" t="inlineStr">
         <is>
-          <t>uPVC soil pipe DN110</t>
+          <t>PPR PN20 pipe DN20</t>
         </is>
       </c>
       <c r="E110" t="n">
-        <v>2.7</v>
+        <v>9.300000000000001</v>
       </c>
       <c r="F110" t="inlineStr">
         <is>
@@ -6143,7 +6143,7 @@
         </is>
       </c>
       <c r="G110" t="n">
-        <v>7000</v>
+        <v>2000</v>
       </c>
       <c r="H110" t="inlineStr">
         <is>
@@ -6156,7 +6156,7 @@
         </is>
       </c>
       <c r="J110" t="n">
-        <v>18900</v>
+        <v>18600</v>
       </c>
       <c r="K110" t="inlineStr">
         <is>
@@ -6182,11 +6182,11 @@
       </c>
       <c r="D111" t="inlineStr">
         <is>
-          <t>PPR PN20 pipe (tempered) DN20</t>
+          <t>PPR PN20 pipe DN25</t>
         </is>
       </c>
       <c r="E111" t="n">
-        <v>6</v>
+        <v>4.4</v>
       </c>
       <c r="F111" t="inlineStr">
         <is>
@@ -6194,7 +6194,7 @@
         </is>
       </c>
       <c r="G111" t="n">
-        <v>2000</v>
+        <v>2800</v>
       </c>
       <c r="H111" t="inlineStr">
         <is>
@@ -6207,7 +6207,7 @@
         </is>
       </c>
       <c r="J111" t="n">
-        <v>12000</v>
+        <v>12320</v>
       </c>
       <c r="K111" t="inlineStr">
         <is>
@@ -6233,11 +6233,11 @@
       </c>
       <c r="D112" t="inlineStr">
         <is>
-          <t>uPVC vent pipe DN75</t>
+          <t>PPR PN20 pipe (hot) DN20</t>
         </is>
       </c>
       <c r="E112" t="n">
-        <v>7.9</v>
+        <v>4.7</v>
       </c>
       <c r="F112" t="inlineStr">
         <is>
@@ -6245,7 +6245,7 @@
         </is>
       </c>
       <c r="G112" t="n">
-        <v>4500</v>
+        <v>2000</v>
       </c>
       <c r="H112" t="inlineStr">
         <is>
@@ -6258,7 +6258,7 @@
         </is>
       </c>
       <c r="J112" t="n">
-        <v>35550</v>
+        <v>9400</v>
       </c>
       <c r="K112" t="inlineStr">
         <is>
@@ -6284,11 +6284,11 @@
       </c>
       <c r="D113" t="inlineStr">
         <is>
-          <t>uPVC waste pipe DN40</t>
+          <t>uPVC soil pipe DN110</t>
         </is>
       </c>
       <c r="E113" t="n">
-        <v>2.5</v>
+        <v>2.7</v>
       </c>
       <c r="F113" t="inlineStr">
         <is>
@@ -6296,7 +6296,7 @@
         </is>
       </c>
       <c r="G113" t="n">
-        <v>2500</v>
+        <v>7000</v>
       </c>
       <c r="H113" t="inlineStr">
         <is>
@@ -6309,7 +6309,7 @@
         </is>
       </c>
       <c r="J113" t="n">
-        <v>6250</v>
+        <v>18900</v>
       </c>
       <c r="K113" t="inlineStr">
         <is>
@@ -6335,11 +6335,11 @@
       </c>
       <c r="D114" t="inlineStr">
         <is>
-          <t>uPVC waste pipe DN50</t>
+          <t>PPR PN20 pipe (tempered) DN20</t>
         </is>
       </c>
       <c r="E114" t="n">
-        <v>5.5</v>
+        <v>6</v>
       </c>
       <c r="F114" t="inlineStr">
         <is>
@@ -6347,7 +6347,7 @@
         </is>
       </c>
       <c r="G114" t="n">
-        <v>3000</v>
+        <v>2000</v>
       </c>
       <c r="H114" t="inlineStr">
         <is>
@@ -6360,7 +6360,7 @@
         </is>
       </c>
       <c r="J114" t="n">
-        <v>16500</v>
+        <v>12000</v>
       </c>
       <c r="K114" t="inlineStr">
         <is>
@@ -6386,19 +6386,19 @@
       </c>
       <c r="D115" t="inlineStr">
         <is>
-          <t>Pipe fittings and clips (allowance)</t>
+          <t>uPVC vent pipe DN75</t>
         </is>
       </c>
       <c r="E115" t="n">
-        <v>1</v>
+        <v>7.9</v>
       </c>
       <c r="F115" t="inlineStr">
         <is>
-          <t>set</t>
+          <t>m</t>
         </is>
       </c>
       <c r="G115" t="n">
-        <v>120000</v>
+        <v>4500</v>
       </c>
       <c r="H115" t="inlineStr">
         <is>
@@ -6411,9 +6411,13 @@
         </is>
       </c>
       <c r="J115" t="n">
-        <v>120000</v>
-      </c>
-      <c r="K115" t="inlineStr"/>
+        <v>35550</v>
+      </c>
+      <c r="K115" t="inlineStr">
+        <is>
+          <t>per m</t>
+        </is>
+      </c>
     </row>
     <row r="116">
       <c r="A116" t="inlineStr">
@@ -6433,19 +6437,19 @@
       </c>
       <c r="D116" t="inlineStr">
         <is>
-          <t>Thermostatic mixing valve (TMV) 41-44 C</t>
+          <t>uPVC waste pipe DN40</t>
         </is>
       </c>
       <c r="E116" t="n">
-        <v>1</v>
+        <v>2.5</v>
       </c>
       <c r="F116" t="inlineStr">
         <is>
-          <t>each</t>
+          <t>m</t>
         </is>
       </c>
       <c r="G116" t="n">
-        <v>60000</v>
+        <v>2500</v>
       </c>
       <c r="H116" t="inlineStr">
         <is>
@@ -6458,9 +6462,13 @@
         </is>
       </c>
       <c r="J116" t="n">
-        <v>60000</v>
-      </c>
-      <c r="K116" t="inlineStr"/>
+        <v>6250</v>
+      </c>
+      <c r="K116" t="inlineStr">
+        <is>
+          <t>per m</t>
+        </is>
+      </c>
     </row>
     <row r="117">
       <c r="A117" t="inlineStr">
@@ -6480,19 +6488,19 @@
       </c>
       <c r="D117" t="inlineStr">
         <is>
-          <t>Thermostatic shower valve + 6-7 L/min head + rail</t>
+          <t>uPVC waste pipe DN50</t>
         </is>
       </c>
       <c r="E117" t="n">
-        <v>1</v>
+        <v>5.5</v>
       </c>
       <c r="F117" t="inlineStr">
         <is>
-          <t>set</t>
+          <t>m</t>
         </is>
       </c>
       <c r="G117" t="n">
-        <v>90000</v>
+        <v>3000</v>
       </c>
       <c r="H117" t="inlineStr">
         <is>
@@ -6505,9 +6513,13 @@
         </is>
       </c>
       <c r="J117" t="n">
-        <v>90000</v>
-      </c>
-      <c r="K117" t="inlineStr"/>
+        <v>16500</v>
+      </c>
+      <c r="K117" t="inlineStr">
+        <is>
+          <t>per m</t>
+        </is>
+      </c>
     </row>
     <row r="118">
       <c r="A118" t="inlineStr">
@@ -6527,7 +6539,7 @@
       </c>
       <c r="D118" t="inlineStr">
         <is>
-          <t>Electric storage water heater 80 L, 2 kW, with T&amp;P valve</t>
+          <t>Pipe fittings and clips (allowance)</t>
         </is>
       </c>
       <c r="E118" t="n">
@@ -6535,11 +6547,11 @@
       </c>
       <c r="F118" t="inlineStr">
         <is>
-          <t>each</t>
+          <t>set</t>
         </is>
       </c>
       <c r="G118" t="n">
-        <v>300000</v>
+        <v>120000</v>
       </c>
       <c r="H118" t="inlineStr">
         <is>
@@ -6552,13 +6564,9 @@
         </is>
       </c>
       <c r="J118" t="n">
-        <v>300000</v>
-      </c>
-      <c r="K118" t="inlineStr">
-        <is>
-          <t>80 L not found; 50 L listed at RWF 144,000-252,000 (STU-P01, STU-P02)</t>
-        </is>
-      </c>
+        <v>120000</v>
+      </c>
+      <c r="K118" t="inlineStr"/>
     </row>
     <row r="119">
       <c r="A119" t="inlineStr">
@@ -6578,11 +6586,11 @@
       </c>
       <c r="D119" t="inlineStr">
         <is>
-          <t>Angle valves with filters</t>
+          <t>Thermostatic mixing valve (TMV) 41-44 C</t>
         </is>
       </c>
       <c r="E119" t="n">
-        <v>5</v>
+        <v>1</v>
       </c>
       <c r="F119" t="inlineStr">
         <is>
@@ -6590,7 +6598,7 @@
         </is>
       </c>
       <c r="G119" t="n">
-        <v>6000</v>
+        <v>60000</v>
       </c>
       <c r="H119" t="inlineStr">
         <is>
@@ -6603,7 +6611,7 @@
         </is>
       </c>
       <c r="J119" t="n">
-        <v>30000</v>
+        <v>60000</v>
       </c>
       <c r="K119" t="inlineStr"/>
     </row>
@@ -6625,7 +6633,7 @@
       </c>
       <c r="D120" t="inlineStr">
         <is>
-          <t>Air admittance valve 110 mm (spare) + rodding eyes</t>
+          <t>Thermostatic shower valve + 6-7 L/min head + rail</t>
         </is>
       </c>
       <c r="E120" t="n">
@@ -6637,7 +6645,7 @@
         </is>
       </c>
       <c r="G120" t="n">
-        <v>30000</v>
+        <v>90000</v>
       </c>
       <c r="H120" t="inlineStr">
         <is>
@@ -6650,7 +6658,7 @@
         </is>
       </c>
       <c r="J120" t="n">
-        <v>30000</v>
+        <v>90000</v>
       </c>
       <c r="K120" t="inlineStr"/>
     </row>
@@ -6672,7 +6680,7 @@
       </c>
       <c r="D121" t="inlineStr">
         <is>
-          <t>Stop valve + Y-filter + check water meter</t>
+          <t>Electric storage water heater 80 L, 2 kW, with T&amp;P valve</t>
         </is>
       </c>
       <c r="E121" t="n">
@@ -6680,11 +6688,11 @@
       </c>
       <c r="F121" t="inlineStr">
         <is>
-          <t>set</t>
+          <t>each</t>
         </is>
       </c>
       <c r="G121" t="n">
-        <v>45000</v>
+        <v>300000</v>
       </c>
       <c r="H121" t="inlineStr">
         <is>
@@ -6697,33 +6705,37 @@
         </is>
       </c>
       <c r="J121" t="n">
-        <v>45000</v>
-      </c>
-      <c r="K121" t="inlineStr"/>
+        <v>300000</v>
+      </c>
+      <c r="K121" t="inlineStr">
+        <is>
+          <t>80 L not found; 50 L listed at RWF 144,000-252,000 (STU-P01, STU-P02)</t>
+        </is>
+      </c>
     </row>
     <row r="122">
       <c r="A122" t="inlineStr">
         <is>
-          <t>K10</t>
+          <t>K9</t>
         </is>
       </c>
       <c r="B122" t="inlineStr">
         <is>
-          <t>steel</t>
+          <t>plumbing</t>
         </is>
       </c>
       <c r="C122" t="inlineStr">
         <is>
-          <t>welding</t>
+          <t>plumbing</t>
         </is>
       </c>
       <c r="D122" t="inlineStr">
         <is>
-          <t>W1 infill: 2 mm steel + 40 mm EPS, welded into the old door frame (0-1,150)</t>
+          <t>Angle valves with filters</t>
         </is>
       </c>
       <c r="E122" t="n">
-        <v>1</v>
+        <v>5</v>
       </c>
       <c r="F122" t="inlineStr">
         <is>
@@ -6731,7 +6743,7 @@
         </is>
       </c>
       <c r="G122" t="n">
-        <v>180000</v>
+        <v>6000</v>
       </c>
       <c r="H122" t="inlineStr">
         <is>
@@ -6744,33 +6756,29 @@
         </is>
       </c>
       <c r="J122" t="n">
-        <v>180000</v>
-      </c>
-      <c r="K122" t="inlineStr">
-        <is>
-          <t>incl. welding</t>
-        </is>
-      </c>
+        <v>30000</v>
+      </c>
+      <c r="K122" t="inlineStr"/>
     </row>
     <row r="123">
       <c r="A123" t="inlineStr">
         <is>
-          <t>K10</t>
+          <t>K9</t>
         </is>
       </c>
       <c r="B123" t="inlineStr">
         <is>
-          <t>glazing</t>
+          <t>plumbing</t>
         </is>
       </c>
       <c r="C123" t="inlineStr">
         <is>
-          <t>glazier</t>
+          <t>plumbing</t>
         </is>
       </c>
       <c r="D123" t="inlineStr">
         <is>
-          <t>W1 obscure louvre window 520 x 890 + insect mesh (wash lobby)</t>
+          <t>Air admittance valve 110 mm (spare) + rodding eyes</t>
         </is>
       </c>
       <c r="E123" t="n">
@@ -6778,11 +6786,11 @@
       </c>
       <c r="F123" t="inlineStr">
         <is>
-          <t>each</t>
+          <t>set</t>
         </is>
       </c>
       <c r="G123" t="n">
-        <v>120000</v>
+        <v>30000</v>
       </c>
       <c r="H123" t="inlineStr">
         <is>
@@ -6795,29 +6803,29 @@
         </is>
       </c>
       <c r="J123" t="n">
-        <v>120000</v>
+        <v>30000</v>
       </c>
       <c r="K123" t="inlineStr"/>
     </row>
     <row r="124">
       <c r="A124" t="inlineStr">
         <is>
-          <t>K10</t>
+          <t>K9</t>
         </is>
       </c>
       <c r="B124" t="inlineStr">
         <is>
-          <t>steel</t>
+          <t>plumbing</t>
         </is>
       </c>
       <c r="C124" t="inlineStr">
         <is>
-          <t>welding</t>
+          <t>plumbing</t>
         </is>
       </c>
       <c r="D124" t="inlineStr">
         <is>
-          <t>Seal and lock the end-B cargo doors (weld tabs, sealant)</t>
+          <t>Stop valve + Y-filter + check water meter</t>
         </is>
       </c>
       <c r="E124" t="n">
@@ -6825,11 +6833,11 @@
       </c>
       <c r="F124" t="inlineStr">
         <is>
-          <t>each</t>
+          <t>set</t>
         </is>
       </c>
       <c r="G124" t="n">
-        <v>60000</v>
+        <v>45000</v>
       </c>
       <c r="H124" t="inlineStr">
         <is>
@@ -6842,7 +6850,7 @@
         </is>
       </c>
       <c r="J124" t="n">
-        <v>60000</v>
+        <v>45000</v>
       </c>
       <c r="K124" t="inlineStr"/>
     </row>
@@ -6859,16 +6867,16 @@
       </c>
       <c r="C125" t="inlineStr">
         <is>
-          <t>masonry</t>
+          <t>welding</t>
         </is>
       </c>
       <c r="D125" t="inlineStr">
         <is>
-          <t>Level the corner castings: concrete pads or steel shims (rock corner)</t>
+          <t>W1 infill: 2 mm steel + 40 mm EPS, welded into the old door frame (0-1,150)</t>
         </is>
       </c>
       <c r="E125" t="n">
-        <v>4</v>
+        <v>1</v>
       </c>
       <c r="F125" t="inlineStr">
         <is>
@@ -6876,7 +6884,7 @@
         </is>
       </c>
       <c r="G125" t="n">
-        <v>25000</v>
+        <v>180000</v>
       </c>
       <c r="H125" t="inlineStr">
         <is>
@@ -6889,9 +6897,13 @@
         </is>
       </c>
       <c r="J125" t="n">
-        <v>100000</v>
-      </c>
-      <c r="K125" t="inlineStr"/>
+        <v>180000</v>
+      </c>
+      <c r="K125" t="inlineStr">
+        <is>
+          <t>incl. welding</t>
+        </is>
+      </c>
     </row>
     <row r="126">
       <c r="A126" t="inlineStr">
@@ -6901,17 +6913,17 @@
       </c>
       <c r="B126" t="inlineStr">
         <is>
-          <t>steel</t>
+          <t>glazing</t>
         </is>
       </c>
       <c r="C126" t="inlineStr">
         <is>
-          <t>welding</t>
+          <t>glazier</t>
         </is>
       </c>
       <c r="D126" t="inlineStr">
         <is>
-          <t>Steel hanging rail for wall units + heater bracket</t>
+          <t>W1 obscure louvre window 520 x 890 + insect mesh (wash lobby)</t>
         </is>
       </c>
       <c r="E126" t="n">
@@ -6919,11 +6931,11 @@
       </c>
       <c r="F126" t="inlineStr">
         <is>
-          <t>set</t>
+          <t>each</t>
         </is>
       </c>
       <c r="G126" t="n">
-        <v>40000</v>
+        <v>120000</v>
       </c>
       <c r="H126" t="inlineStr">
         <is>
@@ -6936,7 +6948,7 @@
         </is>
       </c>
       <c r="J126" t="n">
-        <v>40000</v>
+        <v>120000</v>
       </c>
       <c r="K126" t="inlineStr"/>
     </row>
@@ -6948,17 +6960,17 @@
       </c>
       <c r="B127" t="inlineStr">
         <is>
-          <t>hardware</t>
+          <t>steel</t>
         </is>
       </c>
       <c r="C127" t="inlineStr">
         <is>
-          <t>glazier</t>
+          <t>welding</t>
         </is>
       </c>
       <c r="D127" t="inlineStr">
         <is>
-          <t>Keyed lock + secondary bolt for the slider</t>
+          <t>Seal and lock the end-B cargo doors (weld tabs, sealant)</t>
         </is>
       </c>
       <c r="E127" t="n">
@@ -6966,11 +6978,11 @@
       </c>
       <c r="F127" t="inlineStr">
         <is>
-          <t>set</t>
+          <t>each</t>
         </is>
       </c>
       <c r="G127" t="n">
-        <v>45000</v>
+        <v>60000</v>
       </c>
       <c r="H127" t="inlineStr">
         <is>
@@ -6983,7 +6995,7 @@
         </is>
       </c>
       <c r="J127" t="n">
-        <v>45000</v>
+        <v>60000</v>
       </c>
       <c r="K127" t="inlineStr"/>
     </row>
@@ -6995,21 +7007,21 @@
       </c>
       <c r="B128" t="inlineStr">
         <is>
-          <t>glazing</t>
+          <t>steel</t>
         </is>
       </c>
       <c r="C128" t="inlineStr">
         <is>
-          <t>glazier</t>
+          <t>masonry</t>
         </is>
       </c>
       <c r="D128" t="inlineStr">
         <is>
-          <t>Louvred trickle-vent strip with mesh (10,000 mm2)</t>
+          <t>Level the corner castings: concrete pads or steel shims (rock corner)</t>
         </is>
       </c>
       <c r="E128" t="n">
-        <v>1</v>
+        <v>4</v>
       </c>
       <c r="F128" t="inlineStr">
         <is>
@@ -7017,7 +7029,7 @@
         </is>
       </c>
       <c r="G128" t="n">
-        <v>30000</v>
+        <v>25000</v>
       </c>
       <c r="H128" t="inlineStr">
         <is>
@@ -7030,7 +7042,7 @@
         </is>
       </c>
       <c r="J128" t="n">
-        <v>30000</v>
+        <v>100000</v>
       </c>
       <c r="K128" t="inlineStr"/>
     </row>
@@ -7052,7 +7064,7 @@
       </c>
       <c r="D129" t="inlineStr">
         <is>
-          <t>AC wall sleeve 75 mm (provision, back wall, one hole)</t>
+          <t>Steel hanging rail for wall units + heater bracket</t>
         </is>
       </c>
       <c r="E129" t="n">
@@ -7060,11 +7072,11 @@
       </c>
       <c r="F129" t="inlineStr">
         <is>
-          <t>each</t>
+          <t>set</t>
         </is>
       </c>
       <c r="G129" t="n">
-        <v>15000</v>
+        <v>40000</v>
       </c>
       <c r="H129" t="inlineStr">
         <is>
@@ -7077,29 +7089,29 @@
         </is>
       </c>
       <c r="J129" t="n">
-        <v>15000</v>
+        <v>40000</v>
       </c>
       <c r="K129" t="inlineStr"/>
     </row>
     <row r="130">
       <c r="A130" t="inlineStr">
         <is>
-          <t>K11</t>
+          <t>K10</t>
         </is>
       </c>
       <c r="B130" t="inlineStr">
         <is>
-          <t>roofing</t>
+          <t>hardware</t>
         </is>
       </c>
       <c r="C130" t="inlineStr">
         <is>
-          <t>welding</t>
+          <t>glazier</t>
         </is>
       </c>
       <c r="D130" t="inlineStr">
         <is>
-          <t>Gutter + downpipe to the rainwater tank (deck canopy)</t>
+          <t>Keyed lock + secondary bolt for the slider</t>
         </is>
       </c>
       <c r="E130" t="n">
@@ -7111,7 +7123,7 @@
         </is>
       </c>
       <c r="G130" t="n">
-        <v>90000</v>
+        <v>45000</v>
       </c>
       <c r="H130" t="inlineStr">
         <is>
@@ -7124,29 +7136,29 @@
         </is>
       </c>
       <c r="J130" t="n">
-        <v>90000</v>
+        <v>45000</v>
       </c>
       <c r="K130" t="inlineStr"/>
     </row>
     <row r="131">
       <c r="A131" t="inlineStr">
         <is>
-          <t>K11</t>
+          <t>K10</t>
         </is>
       </c>
       <c r="B131" t="inlineStr">
         <is>
-          <t>electrical</t>
+          <t>glazing</t>
         </is>
       </c>
       <c r="C131" t="inlineStr">
         <is>
-          <t>electrical</t>
+          <t>glazier</t>
         </is>
       </c>
       <c r="D131" t="inlineStr">
         <is>
-          <t>Bonding: 16 mm2 green-yellow from the frame to the earth bar</t>
+          <t>Louvred trickle-vent strip with mesh (10,000 mm2)</t>
         </is>
       </c>
       <c r="E131" t="n">
@@ -7154,11 +7166,11 @@
       </c>
       <c r="F131" t="inlineStr">
         <is>
-          <t>set</t>
+          <t>each</t>
         </is>
       </c>
       <c r="G131" t="n">
-        <v>25000</v>
+        <v>30000</v>
       </c>
       <c r="H131" t="inlineStr">
         <is>
@@ -7171,33 +7183,33 @@
         </is>
       </c>
       <c r="J131" t="n">
-        <v>25000</v>
+        <v>30000</v>
       </c>
       <c r="K131" t="inlineStr"/>
     </row>
     <row r="132">
       <c r="A132" t="inlineStr">
         <is>
-          <t>K1</t>
+          <t>K10</t>
         </is>
       </c>
       <c r="B132" t="inlineStr">
         <is>
-          <t>timber</t>
+          <t>steel</t>
         </is>
       </c>
       <c r="C132" t="inlineStr">
         <is>
-          <t>carpentry</t>
+          <t>welding</t>
         </is>
       </c>
       <c r="D132" t="inlineStr">
         <is>
-          <t>Battens 38 x 50 treated, 2.4 m</t>
+          <t>AC wall sleeve 75 mm (provision, back wall, one hole)</t>
         </is>
       </c>
       <c r="E132" t="n">
-        <v>19.8</v>
+        <v>1</v>
       </c>
       <c r="F132" t="inlineStr">
         <is>
@@ -7205,7 +7217,7 @@
         </is>
       </c>
       <c r="G132" t="n">
-        <v>2500</v>
+        <v>15000</v>
       </c>
       <c r="H132" t="inlineStr">
         <is>
@@ -7218,45 +7230,41 @@
         </is>
       </c>
       <c r="J132" t="n">
-        <v>49500</v>
-      </c>
-      <c r="K132" t="inlineStr">
-        <is>
-          <t>38 x 50 treated, 2.4 m</t>
-        </is>
-      </c>
+        <v>15000</v>
+      </c>
+      <c r="K132" t="inlineStr"/>
     </row>
     <row r="133">
       <c r="A133" t="inlineStr">
         <is>
-          <t>K2</t>
+          <t>K11</t>
         </is>
       </c>
       <c r="B133" t="inlineStr">
         <is>
-          <t>timber</t>
+          <t>roofing</t>
         </is>
       </c>
       <c r="C133" t="inlineStr">
         <is>
-          <t>carpentry</t>
+          <t>welding</t>
         </is>
       </c>
       <c r="D133" t="inlineStr">
         <is>
-          <t>Studs 40 x 40 treated, 2.4 m</t>
+          <t>Gutter + downpipe to the rainwater tank (deck canopy)</t>
         </is>
       </c>
       <c r="E133" t="n">
-        <v>5.5</v>
+        <v>1</v>
       </c>
       <c r="F133" t="inlineStr">
         <is>
-          <t>each</t>
+          <t>set</t>
         </is>
       </c>
       <c r="G133" t="n">
-        <v>3000</v>
+        <v>90000</v>
       </c>
       <c r="H133" t="inlineStr">
         <is>
@@ -7269,29 +7277,29 @@
         </is>
       </c>
       <c r="J133" t="n">
-        <v>16500</v>
-      </c>
-      <c r="K133" t="inlineStr">
-        <is>
-          <t>40 x 40, 2.4 m</t>
-        </is>
-      </c>
+        <v>90000</v>
+      </c>
+      <c r="K133" t="inlineStr"/>
     </row>
     <row r="134">
       <c r="A134" t="inlineStr">
         <is>
-          <t>labour</t>
+          <t>K11</t>
         </is>
       </c>
       <c r="B134" t="inlineStr">
         <is>
-          <t>labour</t>
-        </is>
-      </c>
-      <c r="C134" t="inlineStr"/>
+          <t>electrical</t>
+        </is>
+      </c>
+      <c r="C134" t="inlineStr">
+        <is>
+          <t>electrical</t>
+        </is>
+      </c>
       <c r="D134" t="inlineStr">
         <is>
-          <t>Carpentry workshop: cutting, edging, drilling, labelling (per unit kit)</t>
+          <t>Bonding: 16 mm2 green-yellow from the frame to the earth bar</t>
         </is>
       </c>
       <c r="E134" t="n">
@@ -7299,11 +7307,11 @@
       </c>
       <c r="F134" t="inlineStr">
         <is>
-          <t>lot</t>
+          <t>set</t>
         </is>
       </c>
       <c r="G134" t="n">
-        <v>450000</v>
+        <v>25000</v>
       </c>
       <c r="H134" t="inlineStr">
         <is>
@@ -7316,37 +7324,41 @@
         </is>
       </c>
       <c r="J134" t="n">
-        <v>450000</v>
+        <v>25000</v>
       </c>
       <c r="K134" t="inlineStr"/>
     </row>
     <row r="135">
       <c r="A135" t="inlineStr">
         <is>
-          <t>labour</t>
+          <t>K1</t>
         </is>
       </c>
       <c r="B135" t="inlineStr">
         <is>
-          <t>labour</t>
-        </is>
-      </c>
-      <c r="C135" t="inlineStr"/>
+          <t>timber</t>
+        </is>
+      </c>
+      <c r="C135" t="inlineStr">
+        <is>
+          <t>carpentry</t>
+        </is>
+      </c>
       <c r="D135" t="inlineStr">
         <is>
-          <t>Site carpentry and assembly: 2 people x 8 days</t>
+          <t>Battens 38 x 50 treated, 2.4 m</t>
         </is>
       </c>
       <c r="E135" t="n">
-        <v>1</v>
+        <v>19.8</v>
       </c>
       <c r="F135" t="inlineStr">
         <is>
-          <t>lot</t>
+          <t>each</t>
         </is>
       </c>
       <c r="G135" t="n">
-        <v>320000</v>
+        <v>2500</v>
       </c>
       <c r="H135" t="inlineStr">
         <is>
@@ -7359,37 +7371,45 @@
         </is>
       </c>
       <c r="J135" t="n">
-        <v>320000</v>
-      </c>
-      <c r="K135" t="inlineStr"/>
+        <v>49500</v>
+      </c>
+      <c r="K135" t="inlineStr">
+        <is>
+          <t>38 x 50 treated, 2.4 m</t>
+        </is>
+      </c>
     </row>
     <row r="136">
       <c r="A136" t="inlineStr">
         <is>
-          <t>labour</t>
+          <t>K2</t>
         </is>
       </c>
       <c r="B136" t="inlineStr">
         <is>
-          <t>labour</t>
-        </is>
-      </c>
-      <c r="C136" t="inlineStr"/>
+          <t>timber</t>
+        </is>
+      </c>
+      <c r="C136" t="inlineStr">
+        <is>
+          <t>carpentry</t>
+        </is>
+      </c>
       <c r="D136" t="inlineStr">
         <is>
-          <t>Electrician (RURA class A), install + certificate</t>
+          <t>Studs 40 x 40 treated, 2.4 m</t>
         </is>
       </c>
       <c r="E136" t="n">
-        <v>1</v>
+        <v>5.5</v>
       </c>
       <c r="F136" t="inlineStr">
         <is>
-          <t>lot</t>
+          <t>each</t>
         </is>
       </c>
       <c r="G136" t="n">
-        <v>250000</v>
+        <v>3000</v>
       </c>
       <c r="H136" t="inlineStr">
         <is>
@@ -7402,9 +7422,13 @@
         </is>
       </c>
       <c r="J136" t="n">
-        <v>250000</v>
-      </c>
-      <c r="K136" t="inlineStr"/>
+        <v>16500</v>
+      </c>
+      <c r="K136" t="inlineStr">
+        <is>
+          <t>40 x 40, 2.4 m</t>
+        </is>
+      </c>
     </row>
     <row r="137">
       <c r="A137" t="inlineStr">
@@ -7420,7 +7444,7 @@
       <c r="C137" t="inlineStr"/>
       <c r="D137" t="inlineStr">
         <is>
-          <t>Plumber, install + tests</t>
+          <t>Carpentry workshop: cutting, edging, drilling, labelling (per unit kit)</t>
         </is>
       </c>
       <c r="E137" t="n">
@@ -7432,7 +7456,7 @@
         </is>
       </c>
       <c r="G137" t="n">
-        <v>200000</v>
+        <v>450000</v>
       </c>
       <c r="H137" t="inlineStr">
         <is>
@@ -7445,7 +7469,7 @@
         </is>
       </c>
       <c r="J137" t="n">
-        <v>200000</v>
+        <v>450000</v>
       </c>
       <c r="K137" t="inlineStr"/>
     </row>
@@ -7463,7 +7487,7 @@
       <c r="C138" t="inlineStr"/>
       <c r="D138" t="inlineStr">
         <is>
-          <t>Tiler: wet walls and floor</t>
+          <t>Site carpentry and assembly: 2 people x 8 days</t>
         </is>
       </c>
       <c r="E138" t="n">
@@ -7475,7 +7499,7 @@
         </is>
       </c>
       <c r="G138" t="n">
-        <v>150000</v>
+        <v>320000</v>
       </c>
       <c r="H138" t="inlineStr">
         <is>
@@ -7488,7 +7512,7 @@
         </is>
       </c>
       <c r="J138" t="n">
-        <v>150000</v>
+        <v>320000</v>
       </c>
       <c r="K138" t="inlineStr"/>
     </row>
@@ -7506,7 +7530,7 @@
       <c r="C139" t="inlineStr"/>
       <c r="D139" t="inlineStr">
         <is>
-          <t>Welder: W1, roof frame, deck canopy, stair (per unit)</t>
+          <t>Electrician (RURA class A), install + certificate</t>
         </is>
       </c>
       <c r="E139" t="n">
@@ -7518,7 +7542,7 @@
         </is>
       </c>
       <c r="G139" t="n">
-        <v>600000</v>
+        <v>250000</v>
       </c>
       <c r="H139" t="inlineStr">
         <is>
@@ -7531,7 +7555,7 @@
         </is>
       </c>
       <c r="J139" t="n">
-        <v>600000</v>
+        <v>250000</v>
       </c>
       <c r="K139" t="inlineStr"/>
     </row>
@@ -7549,7 +7573,7 @@
       <c r="C140" t="inlineStr"/>
       <c r="D140" t="inlineStr">
         <is>
-          <t>Transport Kigali to site (share of 2 truck trips)</t>
+          <t>Plumber, install + tests</t>
         </is>
       </c>
       <c r="E140" t="n">
@@ -7561,22 +7585,151 @@
         </is>
       </c>
       <c r="G140" t="n">
+        <v>200000</v>
+      </c>
+      <c r="H140" t="inlineStr">
+        <is>
+          <t>A</t>
+        </is>
+      </c>
+      <c r="I140" t="inlineStr">
+        <is>
+          <t>AS-21</t>
+        </is>
+      </c>
+      <c r="J140" t="n">
+        <v>200000</v>
+      </c>
+      <c r="K140" t="inlineStr"/>
+    </row>
+    <row r="141">
+      <c r="A141" t="inlineStr">
+        <is>
+          <t>labour</t>
+        </is>
+      </c>
+      <c r="B141" t="inlineStr">
+        <is>
+          <t>labour</t>
+        </is>
+      </c>
+      <c r="C141" t="inlineStr"/>
+      <c r="D141" t="inlineStr">
+        <is>
+          <t>Tiler: wet walls and floor</t>
+        </is>
+      </c>
+      <c r="E141" t="n">
+        <v>1</v>
+      </c>
+      <c r="F141" t="inlineStr">
+        <is>
+          <t>lot</t>
+        </is>
+      </c>
+      <c r="G141" t="n">
+        <v>150000</v>
+      </c>
+      <c r="H141" t="inlineStr">
+        <is>
+          <t>A</t>
+        </is>
+      </c>
+      <c r="I141" t="inlineStr">
+        <is>
+          <t>AS-21</t>
+        </is>
+      </c>
+      <c r="J141" t="n">
+        <v>150000</v>
+      </c>
+      <c r="K141" t="inlineStr"/>
+    </row>
+    <row r="142">
+      <c r="A142" t="inlineStr">
+        <is>
+          <t>labour</t>
+        </is>
+      </c>
+      <c r="B142" t="inlineStr">
+        <is>
+          <t>labour</t>
+        </is>
+      </c>
+      <c r="C142" t="inlineStr"/>
+      <c r="D142" t="inlineStr">
+        <is>
+          <t>Welder: W1, roof frame, deck canopy, stair (per unit)</t>
+        </is>
+      </c>
+      <c r="E142" t="n">
+        <v>1</v>
+      </c>
+      <c r="F142" t="inlineStr">
+        <is>
+          <t>lot</t>
+        </is>
+      </c>
+      <c r="G142" t="n">
+        <v>600000</v>
+      </c>
+      <c r="H142" t="inlineStr">
+        <is>
+          <t>A</t>
+        </is>
+      </c>
+      <c r="I142" t="inlineStr">
+        <is>
+          <t>AS-21</t>
+        </is>
+      </c>
+      <c r="J142" t="n">
+        <v>600000</v>
+      </c>
+      <c r="K142" t="inlineStr"/>
+    </row>
+    <row r="143">
+      <c r="A143" t="inlineStr">
+        <is>
+          <t>labour</t>
+        </is>
+      </c>
+      <c r="B143" t="inlineStr">
+        <is>
+          <t>labour</t>
+        </is>
+      </c>
+      <c r="C143" t="inlineStr"/>
+      <c r="D143" t="inlineStr">
+        <is>
+          <t>Transport Kigali to site (share of 2 truck trips)</t>
+        </is>
+      </c>
+      <c r="E143" t="n">
+        <v>1</v>
+      </c>
+      <c r="F143" t="inlineStr">
+        <is>
+          <t>lot</t>
+        </is>
+      </c>
+      <c r="G143" t="n">
         <v>120000</v>
       </c>
-      <c r="H140" t="inlineStr">
-        <is>
-          <t>A</t>
-        </is>
-      </c>
-      <c r="I140" t="inlineStr">
-        <is>
-          <t>AS-21</t>
-        </is>
-      </c>
-      <c r="J140" t="n">
+      <c r="H143" t="inlineStr">
+        <is>
+          <t>A</t>
+        </is>
+      </c>
+      <c r="I143" t="inlineStr">
+        <is>
+          <t>AS-21</t>
+        </is>
+      </c>
+      <c r="J143" t="n">
         <v>120000</v>
       </c>
-      <c r="K140" t="inlineStr"/>
+      <c r="K143" t="inlineStr"/>
     </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>

</xml_diff>

<commit_message>
feat(studio): the water heater is a 30 L box above the WC; plumbing opens the bathroom
The founder asked for the heater in the bathroom, not in the galley's
storage, and a small box instead of the big cylinder. It is now a 30 L
box (2 kW, IPX4) on end wall B above the WC, on the same circuit and
inlet; the overhead cabinet is storage again. Its cold rises in end
wall B past the cistern frame, its hot comes down to the mixing valve
and back along the walls to the sink; every check still passes.

The Plumbing view also strips the bathroom's wet walls to the foam, so
the shower, WC and basin pipework shows like the cut-open sink base.

Refs D-024

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01S6J7Hh7TtJcVRMF7zFHaX8
</commit_message>
<xml_diff>
--- a/public/designs/studio/data/bom.xlsx
+++ b/public/designs/studio/data/bom.xlsx
@@ -513,27 +513,27 @@
     <row r="9">
       <c r="A9" t="inlineStr">
         <is>
-          <t>plumbing</t>
+          <t>sanitaryware</t>
         </is>
       </c>
       <c r="B9" t="n">
-        <v>898920</v>
+        <v>875000</v>
       </c>
       <c r="C9" t="n">
-        <v>2696760</v>
+        <v>2625000</v>
       </c>
     </row>
     <row r="10">
       <c r="A10" t="inlineStr">
         <is>
-          <t>sanitaryware</t>
+          <t>plumbing</t>
         </is>
       </c>
       <c r="B10" t="n">
-        <v>875000</v>
+        <v>729720</v>
       </c>
       <c r="C10" t="n">
-        <v>2625000</v>
+        <v>2189160</v>
       </c>
     </row>
     <row r="11">
@@ -736,10 +736,10 @@
         </is>
       </c>
       <c r="B26" t="n">
-        <v>2092264</v>
+        <v>2066884</v>
       </c>
       <c r="C26" t="n">
-        <v>7005191</v>
+        <v>6929051</v>
       </c>
     </row>
     <row r="27">
@@ -749,10 +749,10 @@
         </is>
       </c>
       <c r="B27" t="n">
-        <v>16040688</v>
+        <v>15846108</v>
       </c>
       <c r="C27" t="n">
-        <v>53706463</v>
+        <v>53122723</v>
       </c>
     </row>
     <row r="29">
@@ -763,7 +763,7 @@
       </c>
       <c r="B29" t="inlineStr"/>
       <c r="C29" t="n">
-        <v>36389</v>
+        <v>35993</v>
       </c>
     </row>
   </sheetData>
@@ -5775,7 +5775,7 @@
       </c>
       <c r="D102" t="inlineStr">
         <is>
-          <t>Cable 2.5 mm2 T+E/singles in conduit, 80 L water heater</t>
+          <t>Cable 2.5 mm2 T+E/singles in conduit, 30 L water heater</t>
         </is>
       </c>
       <c r="E102" t="n">
@@ -6434,7 +6434,7 @@
         </is>
       </c>
       <c r="E115" t="n">
-        <v>10.4</v>
+        <v>10.2</v>
       </c>
       <c r="F115" t="inlineStr">
         <is>
@@ -6455,7 +6455,7 @@
         </is>
       </c>
       <c r="J115" t="n">
-        <v>20800</v>
+        <v>20400</v>
       </c>
       <c r="K115" t="inlineStr">
         <is>
@@ -6536,7 +6536,7 @@
         </is>
       </c>
       <c r="E117" t="n">
-        <v>7.6</v>
+        <v>8.199999999999999</v>
       </c>
       <c r="F117" t="inlineStr">
         <is>
@@ -6557,7 +6557,7 @@
         </is>
       </c>
       <c r="J117" t="n">
-        <v>15200</v>
+        <v>16400</v>
       </c>
       <c r="K117" t="inlineStr">
         <is>
@@ -6979,7 +6979,7 @@
       </c>
       <c r="D126" t="inlineStr">
         <is>
-          <t>Electric storage water heater 80 L, 2 kW, with T&amp;P valve</t>
+          <t>Electric storage water heater 30 L, 2 kW, IPX4, with T&amp;P valve</t>
         </is>
       </c>
       <c r="E126" t="n">
@@ -6991,7 +6991,7 @@
         </is>
       </c>
       <c r="G126" t="n">
-        <v>300000</v>
+        <v>130000</v>
       </c>
       <c r="H126" t="inlineStr">
         <is>
@@ -7004,11 +7004,11 @@
         </is>
       </c>
       <c r="J126" t="n">
-        <v>300000</v>
+        <v>130000</v>
       </c>
       <c r="K126" t="inlineStr">
         <is>
-          <t>80 L not found; 50 L listed at RWF 144,000-252,000 (STU-P01, STU-P02)</t>
+          <t>30 L box not priced yet; 50 L listed at RWF 144,000-252,000 (STU-P01, STU-P02)</t>
         </is>
       </c>
     </row>
@@ -7363,7 +7363,7 @@
       </c>
       <c r="D134" t="inlineStr">
         <is>
-          <t>Steel hanging rail for wall units + heater bracket</t>
+          <t>Steel hanging rail for the wall units</t>
         </is>
       </c>
       <c r="E134" t="n">

</xml_diff>

<commit_message>
feat(studio): a 5.5 kW instant heater in the shower replaces the 30 L tank; D-053
The founder asked for a smaller box heater, like a tankless shower unit.
The heater now sits inside the shower and feeds only the hand shower
through its hose; the sink and basin go cold, so the mixing valve and the
hot and mixed runs go. Its 23.9 A raises the studio's peak to 45.3 A, so
C5 moves to B25 on 6 mm2, the contactor to 40 A, and the inlet, main and
plug to 63 A with 16 mm2 tails. The renders, water diagram, guides (with
their Kinyarwanda twins) and study docs follow. render.mjs can now save a
page's window.TAGS beside its image.

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01S6J7HgCG5ewrAWkTowrJ6N
</commit_message>
<xml_diff>
--- a/public/designs/studio/data/bom.xlsx
+++ b/public/designs/studio/data/bom.xlsx
@@ -517,10 +517,10 @@
         </is>
       </c>
       <c r="B9" t="n">
-        <v>1025400</v>
+        <v>1020650</v>
       </c>
       <c r="C9" t="n">
-        <v>2050800</v>
+        <v>2041300</v>
       </c>
     </row>
     <row r="10">
@@ -539,40 +539,40 @@
     <row r="11">
       <c r="A11" t="inlineStr">
         <is>
-          <t>plumbing</t>
+          <t>appliances</t>
         </is>
       </c>
       <c r="B11" t="n">
-        <v>729720</v>
+        <v>605000</v>
       </c>
       <c r="C11" t="n">
-        <v>1459440</v>
+        <v>1210000</v>
       </c>
     </row>
     <row r="12">
       <c r="A12" t="inlineStr">
         <is>
-          <t>appliances</t>
+          <t>furnishing</t>
         </is>
       </c>
       <c r="B12" t="n">
-        <v>605000</v>
+        <v>545000</v>
       </c>
       <c r="C12" t="n">
-        <v>1210000</v>
+        <v>1090000</v>
       </c>
     </row>
     <row r="13">
       <c r="A13" t="inlineStr">
         <is>
-          <t>furnishing</t>
+          <t>plumbing</t>
         </is>
       </c>
       <c r="B13" t="n">
-        <v>545000</v>
+        <v>537920</v>
       </c>
       <c r="C13" t="n">
-        <v>1090000</v>
+        <v>1075840</v>
       </c>
     </row>
     <row r="14">
@@ -736,10 +736,10 @@
         </is>
       </c>
       <c r="B26" t="n">
-        <v>2188839</v>
+        <v>2159356</v>
       </c>
       <c r="C26" t="n">
-        <v>5106077</v>
+        <v>5047112</v>
       </c>
     </row>
     <row r="27">
@@ -749,10 +749,10 @@
         </is>
       </c>
       <c r="B27" t="n">
-        <v>16781096</v>
+        <v>16555063</v>
       </c>
       <c r="C27" t="n">
-        <v>39146591</v>
+        <v>38694526</v>
       </c>
     </row>
     <row r="29">
@@ -763,7 +763,7 @@
       </c>
       <c r="B29" t="inlineStr"/>
       <c r="C29" t="n">
-        <v>26524</v>
+        <v>26217</v>
       </c>
     </row>
   </sheetData>
@@ -777,7 +777,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:K149"/>
+  <dimension ref="A1:K146"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -4070,7 +4070,7 @@
       </c>
       <c r="D67" t="inlineStr">
         <is>
-          <t>Power inlet 32 A IP67 (IEC 60309 blue, 2P+E), outside behind the board</t>
+          <t>Power inlet 63 A IP67 (IEC 60309 blue, 2P+E), outside behind the board</t>
         </is>
       </c>
       <c r="E67" t="n">
@@ -5081,7 +5081,7 @@
       </c>
       <c r="D88" t="inlineStr">
         <is>
-          <t>Heater DP switch + timer</t>
+          <t>Heater DP isolator, outside the bathroom</t>
         </is>
       </c>
       <c r="E88" t="n">
@@ -5093,7 +5093,7 @@
         </is>
       </c>
       <c r="G88" t="n">
-        <v>25000</v>
+        <v>9000</v>
       </c>
       <c r="H88" t="inlineStr">
         <is>
@@ -5106,13 +5106,9 @@
         </is>
       </c>
       <c r="J88" t="n">
-        <v>25000</v>
-      </c>
-      <c r="K88" t="inlineStr">
-        <is>
-          <t>DP switch + timer</t>
-        </is>
-      </c>
+        <v>9000</v>
+      </c>
+      <c r="K88" t="inlineStr"/>
     </row>
     <row r="89">
       <c r="A89" t="inlineStr">
@@ -5826,7 +5822,7 @@
       </c>
       <c r="D103" t="inlineStr">
         <is>
-          <t>Cable 2.5 mm2 T+E/singles in conduit, 30 L water heater</t>
+          <t>Cable 6.0 mm2 T+E/singles in conduit, Instant shower heater 5.5 kW</t>
         </is>
       </c>
       <c r="E103" t="n">
@@ -5838,7 +5834,7 @@
         </is>
       </c>
       <c r="G103" t="n">
-        <v>750</v>
+        <v>1800</v>
       </c>
       <c r="H103" t="inlineStr">
         <is>
@@ -5851,7 +5847,7 @@
         </is>
       </c>
       <c r="J103" t="n">
-        <v>3750</v>
+        <v>9000</v>
       </c>
       <c r="K103" t="inlineStr">
         <is>
@@ -5979,7 +5975,7 @@
       </c>
       <c r="D106" t="inlineStr">
         <is>
-          <t>Cable 6 mm2 tails, inlet to main breaker, through a gland in the back wall</t>
+          <t>Cable 16 mm2 tails, inlet to main breaker, through a gland in the back wall</t>
         </is>
       </c>
       <c r="E106" t="n">
@@ -5991,7 +5987,7 @@
         </is>
       </c>
       <c r="G106" t="n">
-        <v>1800</v>
+        <v>4800</v>
       </c>
       <c r="H106" t="inlineStr">
         <is>
@@ -6004,11 +6000,11 @@
         </is>
       </c>
       <c r="J106" t="n">
-        <v>3600</v>
+        <v>9600</v>
       </c>
       <c r="K106" t="inlineStr">
         <is>
-          <t>per m</t>
+          <t>per m, tails to the 63 A main</t>
         </is>
       </c>
     </row>
@@ -6030,7 +6026,7 @@
       </c>
       <c r="D107" t="inlineStr">
         <is>
-          <t>Matching 32 A plug (IEC 60309 blue), for whatever supply cable</t>
+          <t>Matching 63 A plug (IEC 60309 blue), for whatever supply cable</t>
         </is>
       </c>
       <c r="E107" t="n">
@@ -6183,7 +6179,7 @@
       </c>
       <c r="D110" t="inlineStr">
         <is>
-          <t>Main breaker 32 A DP (C curve) + DIN kWh check meter</t>
+          <t>Main breaker 63 A DP (C curve) + DIN kWh check meter</t>
         </is>
       </c>
       <c r="E110" t="n">
@@ -6281,7 +6277,7 @@
       </c>
       <c r="D112" t="inlineStr">
         <is>
-          <t>RCBOs 30 mA type A, 1 module (B6 x2, B16 x4, B20 x1)</t>
+          <t>RCBOs 30 mA type A, 1 module (B6 x2, B16 x3, B20 x1, B25 x1)</t>
         </is>
       </c>
       <c r="E112" t="n">
@@ -6383,7 +6379,7 @@
       </c>
       <c r="D114" t="inlineStr">
         <is>
-          <t>Contactor 2-pole 25 A, DIN: the C5 and C7 lines</t>
+          <t>Contactor 2-pole 40 A, DIN: the C5 and C7 lines</t>
         </is>
       </c>
       <c r="E114" t="n">
@@ -6485,7 +6481,7 @@
         </is>
       </c>
       <c r="E116" t="n">
-        <v>10.2</v>
+        <v>9.300000000000001</v>
       </c>
       <c r="F116" t="inlineStr">
         <is>
@@ -6506,7 +6502,7 @@
         </is>
       </c>
       <c r="J116" t="n">
-        <v>20400</v>
+        <v>18600</v>
       </c>
       <c r="K116" t="inlineStr">
         <is>
@@ -6583,11 +6579,11 @@
       </c>
       <c r="D118" t="inlineStr">
         <is>
-          <t>PPR PN20 pipe (hot) DN20</t>
+          <t>uPVC soil pipe DN110</t>
         </is>
       </c>
       <c r="E118" t="n">
-        <v>8.199999999999999</v>
+        <v>3</v>
       </c>
       <c r="F118" t="inlineStr">
         <is>
@@ -6595,7 +6591,7 @@
         </is>
       </c>
       <c r="G118" t="n">
-        <v>2000</v>
+        <v>7000</v>
       </c>
       <c r="H118" t="inlineStr">
         <is>
@@ -6608,7 +6604,7 @@
         </is>
       </c>
       <c r="J118" t="n">
-        <v>16400</v>
+        <v>21000</v>
       </c>
       <c r="K118" t="inlineStr">
         <is>
@@ -6634,11 +6630,11 @@
       </c>
       <c r="D119" t="inlineStr">
         <is>
-          <t>uPVC soil pipe DN110</t>
+          <t>uPVC vent pipe DN75</t>
         </is>
       </c>
       <c r="E119" t="n">
-        <v>3</v>
+        <v>8.800000000000001</v>
       </c>
       <c r="F119" t="inlineStr">
         <is>
@@ -6646,7 +6642,7 @@
         </is>
       </c>
       <c r="G119" t="n">
-        <v>7000</v>
+        <v>4500</v>
       </c>
       <c r="H119" t="inlineStr">
         <is>
@@ -6659,7 +6655,7 @@
         </is>
       </c>
       <c r="J119" t="n">
-        <v>21000</v>
+        <v>39600</v>
       </c>
       <c r="K119" t="inlineStr">
         <is>
@@ -6685,11 +6681,11 @@
       </c>
       <c r="D120" t="inlineStr">
         <is>
-          <t>PPR PN20 pipe (tempered) DN20</t>
+          <t>uPVC waste pipe DN40</t>
         </is>
       </c>
       <c r="E120" t="n">
-        <v>3.8</v>
+        <v>3.4</v>
       </c>
       <c r="F120" t="inlineStr">
         <is>
@@ -6697,7 +6693,7 @@
         </is>
       </c>
       <c r="G120" t="n">
-        <v>2000</v>
+        <v>2500</v>
       </c>
       <c r="H120" t="inlineStr">
         <is>
@@ -6710,7 +6706,7 @@
         </is>
       </c>
       <c r="J120" t="n">
-        <v>7600</v>
+        <v>8500</v>
       </c>
       <c r="K120" t="inlineStr">
         <is>
@@ -6736,11 +6732,11 @@
       </c>
       <c r="D121" t="inlineStr">
         <is>
-          <t>uPVC vent pipe DN75</t>
+          <t>uPVC waste pipe DN50</t>
         </is>
       </c>
       <c r="E121" t="n">
-        <v>8.800000000000001</v>
+        <v>6.3</v>
       </c>
       <c r="F121" t="inlineStr">
         <is>
@@ -6748,7 +6744,7 @@
         </is>
       </c>
       <c r="G121" t="n">
-        <v>4500</v>
+        <v>3000</v>
       </c>
       <c r="H121" t="inlineStr">
         <is>
@@ -6761,7 +6757,7 @@
         </is>
       </c>
       <c r="J121" t="n">
-        <v>39600</v>
+        <v>18900</v>
       </c>
       <c r="K121" t="inlineStr">
         <is>
@@ -6787,19 +6783,19 @@
       </c>
       <c r="D122" t="inlineStr">
         <is>
-          <t>uPVC waste pipe DN40</t>
+          <t>Pipe fittings and clips (allowance)</t>
         </is>
       </c>
       <c r="E122" t="n">
-        <v>3.4</v>
+        <v>1</v>
       </c>
       <c r="F122" t="inlineStr">
         <is>
-          <t>m</t>
+          <t>set</t>
         </is>
       </c>
       <c r="G122" t="n">
-        <v>2500</v>
+        <v>120000</v>
       </c>
       <c r="H122" t="inlineStr">
         <is>
@@ -6812,13 +6808,9 @@
         </is>
       </c>
       <c r="J122" t="n">
-        <v>8500</v>
-      </c>
-      <c r="K122" t="inlineStr">
-        <is>
-          <t>per m</t>
-        </is>
-      </c>
+        <v>120000</v>
+      </c>
+      <c r="K122" t="inlineStr"/>
     </row>
     <row r="123">
       <c r="A123" t="inlineStr">
@@ -6838,19 +6830,19 @@
       </c>
       <c r="D123" t="inlineStr">
         <is>
-          <t>uPVC waste pipe DN50</t>
+          <t>Shower slide rail with hand-shower holder</t>
         </is>
       </c>
       <c r="E123" t="n">
-        <v>6.3</v>
+        <v>1</v>
       </c>
       <c r="F123" t="inlineStr">
         <is>
-          <t>m</t>
+          <t>set</t>
         </is>
       </c>
       <c r="G123" t="n">
-        <v>3000</v>
+        <v>30000</v>
       </c>
       <c r="H123" t="inlineStr">
         <is>
@@ -6863,13 +6855,9 @@
         </is>
       </c>
       <c r="J123" t="n">
-        <v>18900</v>
-      </c>
-      <c r="K123" t="inlineStr">
-        <is>
-          <t>per m</t>
-        </is>
-      </c>
+        <v>30000</v>
+      </c>
+      <c r="K123" t="inlineStr"/>
     </row>
     <row r="124">
       <c r="A124" t="inlineStr">
@@ -6889,7 +6877,7 @@
       </c>
       <c r="D124" t="inlineStr">
         <is>
-          <t>Pipe fittings and clips (allowance)</t>
+          <t>Instant electric shower heater 5.5 kW, IPX4, digital thermostat, hand shower and hose</t>
         </is>
       </c>
       <c r="E124" t="n">
@@ -6897,11 +6885,11 @@
       </c>
       <c r="F124" t="inlineStr">
         <is>
-          <t>set</t>
+          <t>each</t>
         </is>
       </c>
       <c r="G124" t="n">
-        <v>120000</v>
+        <v>90000</v>
       </c>
       <c r="H124" t="inlineStr">
         <is>
@@ -6914,9 +6902,13 @@
         </is>
       </c>
       <c r="J124" t="n">
-        <v>120000</v>
-      </c>
-      <c r="K124" t="inlineStr"/>
+        <v>90000</v>
+      </c>
+      <c r="K124" t="inlineStr">
+        <is>
+          <t>5.5 kW instant shower heater not priced yet (D-053)</t>
+        </is>
+      </c>
     </row>
     <row r="125">
       <c r="A125" t="inlineStr">
@@ -6936,11 +6928,11 @@
       </c>
       <c r="D125" t="inlineStr">
         <is>
-          <t>Thermostatic mixing valve (TMV) 41-44 C</t>
+          <t>Angle valves with filters</t>
         </is>
       </c>
       <c r="E125" t="n">
-        <v>1</v>
+        <v>4</v>
       </c>
       <c r="F125" t="inlineStr">
         <is>
@@ -6948,7 +6940,7 @@
         </is>
       </c>
       <c r="G125" t="n">
-        <v>60000</v>
+        <v>6000</v>
       </c>
       <c r="H125" t="inlineStr">
         <is>
@@ -6961,7 +6953,7 @@
         </is>
       </c>
       <c r="J125" t="n">
-        <v>60000</v>
+        <v>24000</v>
       </c>
       <c r="K125" t="inlineStr"/>
     </row>
@@ -6983,7 +6975,7 @@
       </c>
       <c r="D126" t="inlineStr">
         <is>
-          <t>Thermostatic shower valve + 6-7 L/min head + rail</t>
+          <t>Air admittance valve 110 mm (spare) + rodding eyes</t>
         </is>
       </c>
       <c r="E126" t="n">
@@ -6995,7 +6987,7 @@
         </is>
       </c>
       <c r="G126" t="n">
-        <v>90000</v>
+        <v>30000</v>
       </c>
       <c r="H126" t="inlineStr">
         <is>
@@ -7008,7 +7000,7 @@
         </is>
       </c>
       <c r="J126" t="n">
-        <v>90000</v>
+        <v>30000</v>
       </c>
       <c r="K126" t="inlineStr"/>
     </row>
@@ -7030,7 +7022,7 @@
       </c>
       <c r="D127" t="inlineStr">
         <is>
-          <t>Electric storage water heater 30 L, 2 kW, IPX4, with T&amp;P valve</t>
+          <t>Stop valve + Y-filter + check water meter</t>
         </is>
       </c>
       <c r="E127" t="n">
@@ -7038,11 +7030,11 @@
       </c>
       <c r="F127" t="inlineStr">
         <is>
-          <t>each</t>
+          <t>set</t>
         </is>
       </c>
       <c r="G127" t="n">
-        <v>130000</v>
+        <v>45000</v>
       </c>
       <c r="H127" t="inlineStr">
         <is>
@@ -7055,37 +7047,33 @@
         </is>
       </c>
       <c r="J127" t="n">
-        <v>130000</v>
-      </c>
-      <c r="K127" t="inlineStr">
-        <is>
-          <t>30 L box not priced yet; 50 L listed at RWF 144,000-252,000 (STU-P01, STU-P02)</t>
-        </is>
-      </c>
+        <v>45000</v>
+      </c>
+      <c r="K127" t="inlineStr"/>
     </row>
     <row r="128">
       <c r="A128" t="inlineStr">
         <is>
-          <t>K9</t>
+          <t>K10</t>
         </is>
       </c>
       <c r="B128" t="inlineStr">
         <is>
-          <t>plumbing</t>
+          <t>steel</t>
         </is>
       </c>
       <c r="C128" t="inlineStr">
         <is>
-          <t>plumbing</t>
+          <t>welding</t>
         </is>
       </c>
       <c r="D128" t="inlineStr">
         <is>
-          <t>Angle valves with filters</t>
+          <t>W1 infill: 2 mm steel welded into the old door frame (0-1,150), foamed with the walls</t>
         </is>
       </c>
       <c r="E128" t="n">
-        <v>5</v>
+        <v>1</v>
       </c>
       <c r="F128" t="inlineStr">
         <is>
@@ -7093,7 +7081,7 @@
         </is>
       </c>
       <c r="G128" t="n">
-        <v>6000</v>
+        <v>180000</v>
       </c>
       <c r="H128" t="inlineStr">
         <is>
@@ -7106,29 +7094,33 @@
         </is>
       </c>
       <c r="J128" t="n">
-        <v>30000</v>
-      </c>
-      <c r="K128" t="inlineStr"/>
+        <v>180000</v>
+      </c>
+      <c r="K128" t="inlineStr">
+        <is>
+          <t>incl. welding</t>
+        </is>
+      </c>
     </row>
     <row r="129">
       <c r="A129" t="inlineStr">
         <is>
-          <t>K9</t>
+          <t>K10</t>
         </is>
       </c>
       <c r="B129" t="inlineStr">
         <is>
-          <t>plumbing</t>
+          <t>glazing</t>
         </is>
       </c>
       <c r="C129" t="inlineStr">
         <is>
-          <t>plumbing</t>
+          <t>glazier</t>
         </is>
       </c>
       <c r="D129" t="inlineStr">
         <is>
-          <t>Air admittance valve 110 mm (spare) + rodding eyes</t>
+          <t>W1 obscure louvre window 520 x 890 + insect mesh (wash lobby)</t>
         </is>
       </c>
       <c r="E129" t="n">
@@ -7136,11 +7128,11 @@
       </c>
       <c r="F129" t="inlineStr">
         <is>
-          <t>set</t>
+          <t>each</t>
         </is>
       </c>
       <c r="G129" t="n">
-        <v>30000</v>
+        <v>120000</v>
       </c>
       <c r="H129" t="inlineStr">
         <is>
@@ -7153,29 +7145,29 @@
         </is>
       </c>
       <c r="J129" t="n">
-        <v>30000</v>
+        <v>120000</v>
       </c>
       <c r="K129" t="inlineStr"/>
     </row>
     <row r="130">
       <c r="A130" t="inlineStr">
         <is>
-          <t>K9</t>
+          <t>K10</t>
         </is>
       </c>
       <c r="B130" t="inlineStr">
         <is>
-          <t>plumbing</t>
+          <t>steel</t>
         </is>
       </c>
       <c r="C130" t="inlineStr">
         <is>
-          <t>plumbing</t>
+          <t>welding</t>
         </is>
       </c>
       <c r="D130" t="inlineStr">
         <is>
-          <t>Stop valve + Y-filter + check water meter</t>
+          <t>Seal and lock the end-B cargo doors (weld tabs, sealant)</t>
         </is>
       </c>
       <c r="E130" t="n">
@@ -7183,11 +7175,11 @@
       </c>
       <c r="F130" t="inlineStr">
         <is>
-          <t>set</t>
+          <t>each</t>
         </is>
       </c>
       <c r="G130" t="n">
-        <v>45000</v>
+        <v>60000</v>
       </c>
       <c r="H130" t="inlineStr">
         <is>
@@ -7200,7 +7192,7 @@
         </is>
       </c>
       <c r="J130" t="n">
-        <v>45000</v>
+        <v>60000</v>
       </c>
       <c r="K130" t="inlineStr"/>
     </row>
@@ -7217,16 +7209,16 @@
       </c>
       <c r="C131" t="inlineStr">
         <is>
-          <t>welding</t>
+          <t>masonry</t>
         </is>
       </c>
       <c r="D131" t="inlineStr">
         <is>
-          <t>W1 infill: 2 mm steel welded into the old door frame (0-1,150), foamed with the walls</t>
+          <t>Concrete block stands 40 x 60 cm under the four corner castings, levelled (D-029)</t>
         </is>
       </c>
       <c r="E131" t="n">
-        <v>1</v>
+        <v>4</v>
       </c>
       <c r="F131" t="inlineStr">
         <is>
@@ -7234,7 +7226,7 @@
         </is>
       </c>
       <c r="G131" t="n">
-        <v>180000</v>
+        <v>25000</v>
       </c>
       <c r="H131" t="inlineStr">
         <is>
@@ -7247,13 +7239,9 @@
         </is>
       </c>
       <c r="J131" t="n">
-        <v>180000</v>
-      </c>
-      <c r="K131" t="inlineStr">
-        <is>
-          <t>incl. welding</t>
-        </is>
-      </c>
+        <v>100000</v>
+      </c>
+      <c r="K131" t="inlineStr"/>
     </row>
     <row r="132">
       <c r="A132" t="inlineStr">
@@ -7263,17 +7251,17 @@
       </c>
       <c r="B132" t="inlineStr">
         <is>
-          <t>glazing</t>
+          <t>steel</t>
         </is>
       </c>
       <c r="C132" t="inlineStr">
         <is>
-          <t>glazier</t>
+          <t>welding</t>
         </is>
       </c>
       <c r="D132" t="inlineStr">
         <is>
-          <t>W1 obscure louvre window 520 x 890 + insect mesh (wash lobby)</t>
+          <t>Steel hanging rail for the wall units</t>
         </is>
       </c>
       <c r="E132" t="n">
@@ -7281,11 +7269,11 @@
       </c>
       <c r="F132" t="inlineStr">
         <is>
-          <t>each</t>
+          <t>set</t>
         </is>
       </c>
       <c r="G132" t="n">
-        <v>120000</v>
+        <v>40000</v>
       </c>
       <c r="H132" t="inlineStr">
         <is>
@@ -7298,7 +7286,7 @@
         </is>
       </c>
       <c r="J132" t="n">
-        <v>120000</v>
+        <v>40000</v>
       </c>
       <c r="K132" t="inlineStr"/>
     </row>
@@ -7310,17 +7298,17 @@
       </c>
       <c r="B133" t="inlineStr">
         <is>
-          <t>steel</t>
+          <t>hardware</t>
         </is>
       </c>
       <c r="C133" t="inlineStr">
         <is>
-          <t>welding</t>
+          <t>glazier</t>
         </is>
       </c>
       <c r="D133" t="inlineStr">
         <is>
-          <t>Seal and lock the end-B cargo doors (weld tabs, sealant)</t>
+          <t>Keyed lock + secondary bolt for the slider</t>
         </is>
       </c>
       <c r="E133" t="n">
@@ -7328,11 +7316,11 @@
       </c>
       <c r="F133" t="inlineStr">
         <is>
-          <t>each</t>
+          <t>set</t>
         </is>
       </c>
       <c r="G133" t="n">
-        <v>60000</v>
+        <v>45000</v>
       </c>
       <c r="H133" t="inlineStr">
         <is>
@@ -7345,7 +7333,7 @@
         </is>
       </c>
       <c r="J133" t="n">
-        <v>60000</v>
+        <v>45000</v>
       </c>
       <c r="K133" t="inlineStr"/>
     </row>
@@ -7357,21 +7345,21 @@
       </c>
       <c r="B134" t="inlineStr">
         <is>
-          <t>steel</t>
+          <t>glazing</t>
         </is>
       </c>
       <c r="C134" t="inlineStr">
         <is>
-          <t>masonry</t>
+          <t>glazier</t>
         </is>
       </c>
       <c r="D134" t="inlineStr">
         <is>
-          <t>Concrete block stands 40 x 60 cm under the four corner castings, levelled (D-029)</t>
+          <t>Louvred trickle-vent strip with mesh (10,000 mm2)</t>
         </is>
       </c>
       <c r="E134" t="n">
-        <v>4</v>
+        <v>1</v>
       </c>
       <c r="F134" t="inlineStr">
         <is>
@@ -7379,7 +7367,7 @@
         </is>
       </c>
       <c r="G134" t="n">
-        <v>25000</v>
+        <v>30000</v>
       </c>
       <c r="H134" t="inlineStr">
         <is>
@@ -7392,7 +7380,7 @@
         </is>
       </c>
       <c r="J134" t="n">
-        <v>100000</v>
+        <v>30000</v>
       </c>
       <c r="K134" t="inlineStr"/>
     </row>
@@ -7414,7 +7402,7 @@
       </c>
       <c r="D135" t="inlineStr">
         <is>
-          <t>Steel hanging rail for the wall units</t>
+          <t>AC wall sleeve 75 mm (provision, back wall, one hole)</t>
         </is>
       </c>
       <c r="E135" t="n">
@@ -7422,11 +7410,11 @@
       </c>
       <c r="F135" t="inlineStr">
         <is>
-          <t>set</t>
+          <t>each</t>
         </is>
       </c>
       <c r="G135" t="n">
-        <v>40000</v>
+        <v>15000</v>
       </c>
       <c r="H135" t="inlineStr">
         <is>
@@ -7439,29 +7427,29 @@
         </is>
       </c>
       <c r="J135" t="n">
-        <v>40000</v>
+        <v>15000</v>
       </c>
       <c r="K135" t="inlineStr"/>
     </row>
     <row r="136">
       <c r="A136" t="inlineStr">
         <is>
-          <t>K10</t>
+          <t>K11</t>
         </is>
       </c>
       <c r="B136" t="inlineStr">
         <is>
-          <t>hardware</t>
+          <t>roofing</t>
         </is>
       </c>
       <c r="C136" t="inlineStr">
         <is>
-          <t>glazier</t>
+          <t>welding</t>
         </is>
       </c>
       <c r="D136" t="inlineStr">
         <is>
-          <t>Keyed lock + secondary bolt for the slider</t>
+          <t>Gutter + downpipe to the rainwater tank (deck canopy)</t>
         </is>
       </c>
       <c r="E136" t="n">
@@ -7473,7 +7461,7 @@
         </is>
       </c>
       <c r="G136" t="n">
-        <v>45000</v>
+        <v>90000</v>
       </c>
       <c r="H136" t="inlineStr">
         <is>
@@ -7486,29 +7474,29 @@
         </is>
       </c>
       <c r="J136" t="n">
-        <v>45000</v>
+        <v>90000</v>
       </c>
       <c r="K136" t="inlineStr"/>
     </row>
     <row r="137">
       <c r="A137" t="inlineStr">
         <is>
-          <t>K10</t>
+          <t>K11</t>
         </is>
       </c>
       <c r="B137" t="inlineStr">
         <is>
-          <t>glazing</t>
+          <t>electrical</t>
         </is>
       </c>
       <c r="C137" t="inlineStr">
         <is>
-          <t>glazier</t>
+          <t>electrical</t>
         </is>
       </c>
       <c r="D137" t="inlineStr">
         <is>
-          <t>Louvred trickle-vent strip with mesh (10,000 mm2)</t>
+          <t>Bonding: 16 mm2 green-yellow from the frame to the earth bar</t>
         </is>
       </c>
       <c r="E137" t="n">
@@ -7516,11 +7504,11 @@
       </c>
       <c r="F137" t="inlineStr">
         <is>
-          <t>each</t>
+          <t>set</t>
         </is>
       </c>
       <c r="G137" t="n">
-        <v>30000</v>
+        <v>25000</v>
       </c>
       <c r="H137" t="inlineStr">
         <is>
@@ -7533,33 +7521,33 @@
         </is>
       </c>
       <c r="J137" t="n">
-        <v>30000</v>
+        <v>25000</v>
       </c>
       <c r="K137" t="inlineStr"/>
     </row>
     <row r="138">
       <c r="A138" t="inlineStr">
         <is>
-          <t>K10</t>
+          <t>K1</t>
         </is>
       </c>
       <c r="B138" t="inlineStr">
         <is>
-          <t>steel</t>
+          <t>timber</t>
         </is>
       </c>
       <c r="C138" t="inlineStr">
         <is>
-          <t>welding</t>
+          <t>carpentry</t>
         </is>
       </c>
       <c r="D138" t="inlineStr">
         <is>
-          <t>AC wall sleeve 75 mm (provision, back wall, one hole)</t>
+          <t>Battens 38 x 50 treated, 2.4 m</t>
         </is>
       </c>
       <c r="E138" t="n">
-        <v>1</v>
+        <v>35.2</v>
       </c>
       <c r="F138" t="inlineStr">
         <is>
@@ -7567,7 +7555,7 @@
         </is>
       </c>
       <c r="G138" t="n">
-        <v>15000</v>
+        <v>2500</v>
       </c>
       <c r="H138" t="inlineStr">
         <is>
@@ -7580,41 +7568,45 @@
         </is>
       </c>
       <c r="J138" t="n">
-        <v>15000</v>
-      </c>
-      <c r="K138" t="inlineStr"/>
+        <v>88000</v>
+      </c>
+      <c r="K138" t="inlineStr">
+        <is>
+          <t>38 x 50 treated, 2.4 m</t>
+        </is>
+      </c>
     </row>
     <row r="139">
       <c r="A139" t="inlineStr">
         <is>
-          <t>K11</t>
+          <t>K2</t>
         </is>
       </c>
       <c r="B139" t="inlineStr">
         <is>
-          <t>roofing</t>
+          <t>timber</t>
         </is>
       </c>
       <c r="C139" t="inlineStr">
         <is>
-          <t>welding</t>
+          <t>carpentry</t>
         </is>
       </c>
       <c r="D139" t="inlineStr">
         <is>
-          <t>Gutter + downpipe to the rainwater tank (deck canopy)</t>
+          <t>Studs 40 x 40 treated, 2.4 m</t>
         </is>
       </c>
       <c r="E139" t="n">
-        <v>1</v>
+        <v>5.5</v>
       </c>
       <c r="F139" t="inlineStr">
         <is>
-          <t>set</t>
+          <t>each</t>
         </is>
       </c>
       <c r="G139" t="n">
-        <v>90000</v>
+        <v>3000</v>
       </c>
       <c r="H139" t="inlineStr">
         <is>
@@ -7627,29 +7619,29 @@
         </is>
       </c>
       <c r="J139" t="n">
-        <v>90000</v>
-      </c>
-      <c r="K139" t="inlineStr"/>
+        <v>16500</v>
+      </c>
+      <c r="K139" t="inlineStr">
+        <is>
+          <t>40 x 40, 2.4 m</t>
+        </is>
+      </c>
     </row>
     <row r="140">
       <c r="A140" t="inlineStr">
         <is>
-          <t>K11</t>
+          <t>labour</t>
         </is>
       </c>
       <c r="B140" t="inlineStr">
         <is>
-          <t>electrical</t>
-        </is>
-      </c>
-      <c r="C140" t="inlineStr">
-        <is>
-          <t>electrical</t>
-        </is>
-      </c>
+          <t>labour</t>
+        </is>
+      </c>
+      <c r="C140" t="inlineStr"/>
       <c r="D140" t="inlineStr">
         <is>
-          <t>Bonding: 16 mm2 green-yellow from the frame to the earth bar</t>
+          <t>Carpentry workshop: cutting, edging, drilling, labelling (per unit kit)</t>
         </is>
       </c>
       <c r="E140" t="n">
@@ -7657,11 +7649,11 @@
       </c>
       <c r="F140" t="inlineStr">
         <is>
-          <t>set</t>
+          <t>lot</t>
         </is>
       </c>
       <c r="G140" t="n">
-        <v>25000</v>
+        <v>450000</v>
       </c>
       <c r="H140" t="inlineStr">
         <is>
@@ -7674,41 +7666,37 @@
         </is>
       </c>
       <c r="J140" t="n">
-        <v>25000</v>
+        <v>450000</v>
       </c>
       <c r="K140" t="inlineStr"/>
     </row>
     <row r="141">
       <c r="A141" t="inlineStr">
         <is>
-          <t>K1</t>
+          <t>labour</t>
         </is>
       </c>
       <c r="B141" t="inlineStr">
         <is>
-          <t>timber</t>
-        </is>
-      </c>
-      <c r="C141" t="inlineStr">
-        <is>
-          <t>carpentry</t>
-        </is>
-      </c>
+          <t>labour</t>
+        </is>
+      </c>
+      <c r="C141" t="inlineStr"/>
       <c r="D141" t="inlineStr">
         <is>
-          <t>Battens 38 x 50 treated, 2.4 m</t>
+          <t>Site carpentry and assembly: 2 people x 8 days</t>
         </is>
       </c>
       <c r="E141" t="n">
-        <v>35.2</v>
+        <v>1</v>
       </c>
       <c r="F141" t="inlineStr">
         <is>
-          <t>each</t>
+          <t>lot</t>
         </is>
       </c>
       <c r="G141" t="n">
-        <v>2500</v>
+        <v>320000</v>
       </c>
       <c r="H141" t="inlineStr">
         <is>
@@ -7721,45 +7709,37 @@
         </is>
       </c>
       <c r="J141" t="n">
-        <v>88000</v>
-      </c>
-      <c r="K141" t="inlineStr">
-        <is>
-          <t>38 x 50 treated, 2.4 m</t>
-        </is>
-      </c>
+        <v>320000</v>
+      </c>
+      <c r="K141" t="inlineStr"/>
     </row>
     <row r="142">
       <c r="A142" t="inlineStr">
         <is>
-          <t>K2</t>
+          <t>labour</t>
         </is>
       </c>
       <c r="B142" t="inlineStr">
         <is>
-          <t>timber</t>
-        </is>
-      </c>
-      <c r="C142" t="inlineStr">
-        <is>
-          <t>carpentry</t>
-        </is>
-      </c>
+          <t>labour</t>
+        </is>
+      </c>
+      <c r="C142" t="inlineStr"/>
       <c r="D142" t="inlineStr">
         <is>
-          <t>Studs 40 x 40 treated, 2.4 m</t>
+          <t>Electrician (RURA class A), install + certificate</t>
         </is>
       </c>
       <c r="E142" t="n">
-        <v>5.5</v>
+        <v>1</v>
       </c>
       <c r="F142" t="inlineStr">
         <is>
-          <t>each</t>
+          <t>lot</t>
         </is>
       </c>
       <c r="G142" t="n">
-        <v>3000</v>
+        <v>250000</v>
       </c>
       <c r="H142" t="inlineStr">
         <is>
@@ -7772,13 +7752,9 @@
         </is>
       </c>
       <c r="J142" t="n">
-        <v>16500</v>
-      </c>
-      <c r="K142" t="inlineStr">
-        <is>
-          <t>40 x 40, 2.4 m</t>
-        </is>
-      </c>
+        <v>250000</v>
+      </c>
+      <c r="K142" t="inlineStr"/>
     </row>
     <row r="143">
       <c r="A143" t="inlineStr">
@@ -7794,7 +7770,7 @@
       <c r="C143" t="inlineStr"/>
       <c r="D143" t="inlineStr">
         <is>
-          <t>Carpentry workshop: cutting, edging, drilling, labelling (per unit kit)</t>
+          <t>Plumber, install + tests</t>
         </is>
       </c>
       <c r="E143" t="n">
@@ -7806,7 +7782,7 @@
         </is>
       </c>
       <c r="G143" t="n">
-        <v>450000</v>
+        <v>200000</v>
       </c>
       <c r="H143" t="inlineStr">
         <is>
@@ -7819,7 +7795,7 @@
         </is>
       </c>
       <c r="J143" t="n">
-        <v>450000</v>
+        <v>200000</v>
       </c>
       <c r="K143" t="inlineStr"/>
     </row>
@@ -7837,7 +7813,7 @@
       <c r="C144" t="inlineStr"/>
       <c r="D144" t="inlineStr">
         <is>
-          <t>Site carpentry and assembly: 2 people x 8 days</t>
+          <t>Tiler: wet walls and floor</t>
         </is>
       </c>
       <c r="E144" t="n">
@@ -7849,7 +7825,7 @@
         </is>
       </c>
       <c r="G144" t="n">
-        <v>320000</v>
+        <v>150000</v>
       </c>
       <c r="H144" t="inlineStr">
         <is>
@@ -7862,7 +7838,7 @@
         </is>
       </c>
       <c r="J144" t="n">
-        <v>320000</v>
+        <v>150000</v>
       </c>
       <c r="K144" t="inlineStr"/>
     </row>
@@ -7880,7 +7856,7 @@
       <c r="C145" t="inlineStr"/>
       <c r="D145" t="inlineStr">
         <is>
-          <t>Electrician (RURA class A), install + certificate</t>
+          <t>Welder: W1, roof frame, deck canopy, stair (per unit)</t>
         </is>
       </c>
       <c r="E145" t="n">
@@ -7892,7 +7868,7 @@
         </is>
       </c>
       <c r="G145" t="n">
-        <v>250000</v>
+        <v>600000</v>
       </c>
       <c r="H145" t="inlineStr">
         <is>
@@ -7905,7 +7881,7 @@
         </is>
       </c>
       <c r="J145" t="n">
-        <v>250000</v>
+        <v>600000</v>
       </c>
       <c r="K145" t="inlineStr"/>
     </row>
@@ -7923,7 +7899,7 @@
       <c r="C146" t="inlineStr"/>
       <c r="D146" t="inlineStr">
         <is>
-          <t>Plumber, install + tests</t>
+          <t>Transport Kigali to site (share of 2 truck trips)</t>
         </is>
       </c>
       <c r="E146" t="n">
@@ -7935,7 +7911,7 @@
         </is>
       </c>
       <c r="G146" t="n">
-        <v>200000</v>
+        <v>120000</v>
       </c>
       <c r="H146" t="inlineStr">
         <is>
@@ -7948,138 +7924,9 @@
         </is>
       </c>
       <c r="J146" t="n">
-        <v>200000</v>
+        <v>120000</v>
       </c>
       <c r="K146" t="inlineStr"/>
-    </row>
-    <row r="147">
-      <c r="A147" t="inlineStr">
-        <is>
-          <t>labour</t>
-        </is>
-      </c>
-      <c r="B147" t="inlineStr">
-        <is>
-          <t>labour</t>
-        </is>
-      </c>
-      <c r="C147" t="inlineStr"/>
-      <c r="D147" t="inlineStr">
-        <is>
-          <t>Tiler: wet walls and floor</t>
-        </is>
-      </c>
-      <c r="E147" t="n">
-        <v>1</v>
-      </c>
-      <c r="F147" t="inlineStr">
-        <is>
-          <t>lot</t>
-        </is>
-      </c>
-      <c r="G147" t="n">
-        <v>150000</v>
-      </c>
-      <c r="H147" t="inlineStr">
-        <is>
-          <t>A</t>
-        </is>
-      </c>
-      <c r="I147" t="inlineStr">
-        <is>
-          <t>AS-21</t>
-        </is>
-      </c>
-      <c r="J147" t="n">
-        <v>150000</v>
-      </c>
-      <c r="K147" t="inlineStr"/>
-    </row>
-    <row r="148">
-      <c r="A148" t="inlineStr">
-        <is>
-          <t>labour</t>
-        </is>
-      </c>
-      <c r="B148" t="inlineStr">
-        <is>
-          <t>labour</t>
-        </is>
-      </c>
-      <c r="C148" t="inlineStr"/>
-      <c r="D148" t="inlineStr">
-        <is>
-          <t>Welder: W1, roof frame, deck canopy, stair (per unit)</t>
-        </is>
-      </c>
-      <c r="E148" t="n">
-        <v>1</v>
-      </c>
-      <c r="F148" t="inlineStr">
-        <is>
-          <t>lot</t>
-        </is>
-      </c>
-      <c r="G148" t="n">
-        <v>600000</v>
-      </c>
-      <c r="H148" t="inlineStr">
-        <is>
-          <t>A</t>
-        </is>
-      </c>
-      <c r="I148" t="inlineStr">
-        <is>
-          <t>AS-21</t>
-        </is>
-      </c>
-      <c r="J148" t="n">
-        <v>600000</v>
-      </c>
-      <c r="K148" t="inlineStr"/>
-    </row>
-    <row r="149">
-      <c r="A149" t="inlineStr">
-        <is>
-          <t>labour</t>
-        </is>
-      </c>
-      <c r="B149" t="inlineStr">
-        <is>
-          <t>labour</t>
-        </is>
-      </c>
-      <c r="C149" t="inlineStr"/>
-      <c r="D149" t="inlineStr">
-        <is>
-          <t>Transport Kigali to site (share of 2 truck trips)</t>
-        </is>
-      </c>
-      <c r="E149" t="n">
-        <v>1</v>
-      </c>
-      <c r="F149" t="inlineStr">
-        <is>
-          <t>lot</t>
-        </is>
-      </c>
-      <c r="G149" t="n">
-        <v>120000</v>
-      </c>
-      <c r="H149" t="inlineStr">
-        <is>
-          <t>A</t>
-        </is>
-      </c>
-      <c r="I149" t="inlineStr">
-        <is>
-          <t>AS-21</t>
-        </is>
-      </c>
-      <c r="J149" t="n">
-        <v>120000</v>
-      </c>
-      <c r="K149" t="inlineStr"/>
     </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>

</xml_diff>

<commit_message>
feat(studio): sliding bathroom door, no basin, chimney hood (D-066)
The founder: hands are washed at the galley, the bathroom takes a sliding
door, and the hob gets a chimney hood like his reference picture. The leaf
parks where the basin stood; the 1.15 m cross wall caps the opening at 570
(534 clear) so it parks short of end B (R-SLIDE). The overhead cabinet
splits in two either side of the hood.

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01S6J7HinYQ9w2K8Yf8j6x7D
</commit_message>
<xml_diff>
--- a/public/designs/studio/data/bom.xlsx
+++ b/public/designs/studio/data/bom.xlsx
@@ -491,10 +491,10 @@
         </is>
       </c>
       <c r="B7" t="n">
-        <v>1426420</v>
+        <v>1419940</v>
       </c>
       <c r="C7" t="n">
-        <v>2852840</v>
+        <v>2839880</v>
       </c>
     </row>
     <row r="8">
@@ -517,10 +517,10 @@
         </is>
       </c>
       <c r="B9" t="n">
-        <v>1020650</v>
+        <v>1018150</v>
       </c>
       <c r="C9" t="n">
-        <v>2041300</v>
+        <v>2036300</v>
       </c>
     </row>
     <row r="10">
@@ -530,10 +530,10 @@
         </is>
       </c>
       <c r="B10" t="n">
-        <v>875000</v>
+        <v>785000</v>
       </c>
       <c r="C10" t="n">
-        <v>1750000</v>
+        <v>1570000</v>
       </c>
     </row>
     <row r="11">
@@ -543,10 +543,10 @@
         </is>
       </c>
       <c r="B11" t="n">
-        <v>605000</v>
+        <v>665000</v>
       </c>
       <c r="C11" t="n">
-        <v>1210000</v>
+        <v>1330000</v>
       </c>
     </row>
     <row r="12">
@@ -569,10 +569,10 @@
         </is>
       </c>
       <c r="B13" t="n">
-        <v>537920</v>
+        <v>527220</v>
       </c>
       <c r="C13" t="n">
-        <v>1075840</v>
+        <v>1054440</v>
       </c>
     </row>
     <row r="14">
@@ -595,10 +595,10 @@
         </is>
       </c>
       <c r="B15" t="n">
-        <v>452480</v>
+        <v>417120</v>
       </c>
       <c r="C15" t="n">
-        <v>904960</v>
+        <v>834240</v>
       </c>
     </row>
     <row r="16">
@@ -621,10 +621,10 @@
         </is>
       </c>
       <c r="B17" t="n">
-        <v>265000</v>
+        <v>240000</v>
       </c>
       <c r="C17" t="n">
-        <v>530000</v>
+        <v>480000</v>
       </c>
     </row>
     <row r="18">
@@ -634,10 +634,10 @@
         </is>
       </c>
       <c r="B18" t="n">
-        <v>185535</v>
+        <v>238857</v>
       </c>
       <c r="C18" t="n">
-        <v>371070</v>
+        <v>477714</v>
       </c>
     </row>
     <row r="19">
@@ -736,10 +736,10 @@
         </is>
       </c>
       <c r="B26" t="n">
-        <v>2159356</v>
+        <v>2150848</v>
       </c>
       <c r="C26" t="n">
-        <v>5047112</v>
+        <v>5030097</v>
       </c>
     </row>
     <row r="27">
@@ -749,10 +749,10 @@
         </is>
       </c>
       <c r="B27" t="n">
-        <v>16555063</v>
+        <v>16489837</v>
       </c>
       <c r="C27" t="n">
-        <v>38694526</v>
+        <v>38564075</v>
       </c>
     </row>
     <row r="29">
@@ -763,7 +763,7 @@
       </c>
       <c r="B29" t="inlineStr"/>
       <c r="C29" t="n">
-        <v>26217</v>
+        <v>26129</v>
       </c>
     </row>
   </sheetData>
@@ -777,7 +777,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:K146"/>
+  <dimension ref="A1:K143"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -1063,7 +1063,7 @@
         </is>
       </c>
       <c r="E6" t="n">
-        <v>160.7</v>
+        <v>149.9</v>
       </c>
       <c r="F6" t="inlineStr">
         <is>
@@ -1084,7 +1084,7 @@
         </is>
       </c>
       <c r="J6" t="n">
-        <v>96420</v>
+        <v>89940</v>
       </c>
       <c r="K6" t="inlineStr">
         <is>
@@ -1114,7 +1114,7 @@
         </is>
       </c>
       <c r="E7" t="n">
-        <v>37.8</v>
+        <v>50.4</v>
       </c>
       <c r="F7" t="inlineStr">
         <is>
@@ -1135,7 +1135,7 @@
         </is>
       </c>
       <c r="J7" t="n">
-        <v>2268</v>
+        <v>3024</v>
       </c>
       <c r="K7" t="inlineStr"/>
     </row>
@@ -1161,7 +1161,7 @@
         </is>
       </c>
       <c r="E8" t="n">
-        <v>25.2</v>
+        <v>33.6</v>
       </c>
       <c r="F8" t="inlineStr">
         <is>
@@ -1182,7 +1182,7 @@
         </is>
       </c>
       <c r="J8" t="n">
-        <v>504</v>
+        <v>672</v>
       </c>
       <c r="K8" t="inlineStr"/>
     </row>
@@ -1255,7 +1255,7 @@
         </is>
       </c>
       <c r="E10" t="n">
-        <v>10.5</v>
+        <v>8.4</v>
       </c>
       <c r="F10" t="inlineStr">
         <is>
@@ -1276,7 +1276,7 @@
         </is>
       </c>
       <c r="J10" t="n">
-        <v>26250</v>
+        <v>21000</v>
       </c>
       <c r="K10" t="inlineStr"/>
     </row>
@@ -1302,7 +1302,7 @@
         </is>
       </c>
       <c r="E11" t="n">
-        <v>12.6</v>
+        <v>4.2</v>
       </c>
       <c r="F11" t="inlineStr">
         <is>
@@ -1323,7 +1323,7 @@
         </is>
       </c>
       <c r="J11" t="n">
-        <v>378</v>
+        <v>126</v>
       </c>
       <c r="K11" t="inlineStr"/>
     </row>
@@ -1447,7 +1447,7 @@
         </is>
       </c>
       <c r="E14" t="n">
-        <v>7.35</v>
+        <v>6.3</v>
       </c>
       <c r="F14" t="inlineStr">
         <is>
@@ -1468,7 +1468,7 @@
         </is>
       </c>
       <c r="J14" t="n">
-        <v>14700</v>
+        <v>12600</v>
       </c>
       <c r="K14" t="inlineStr"/>
     </row>
@@ -2345,7 +2345,7 @@
       </c>
       <c r="D32" t="inlineStr">
         <is>
-          <t>Door leaf 564 x 2,030, moisture-resistant, opens into the bathroom, privacy lock</t>
+          <t>Sliding door leaf 574 x 2,055, moisture-resistant, flush pulls, privacy hook lock</t>
         </is>
       </c>
       <c r="E32" t="n">
@@ -2382,29 +2382,29 @@
       </c>
       <c r="B33" t="inlineStr">
         <is>
-          <t>wet walls</t>
+          <t>hardware</t>
         </is>
       </c>
       <c r="C33" t="inlineStr">
         <is>
-          <t>tiling</t>
+          <t>carpentry</t>
         </is>
       </c>
       <c r="D33" t="inlineStr">
         <is>
-          <t>Cement board 12 mm + liquid membrane, back wall</t>
+          <t>Surface sliding-door track 1140 mm with soft-close, end stop and floor guide, on the cross wall's lobby face</t>
         </is>
       </c>
       <c r="E33" t="n">
-        <v>2.66</v>
+        <v>1</v>
       </c>
       <c r="F33" t="inlineStr">
         <is>
-          <t>m2</t>
+          <t>set</t>
         </is>
       </c>
       <c r="G33" t="n">
-        <v>14000</v>
+        <v>60000</v>
       </c>
       <c r="H33" t="inlineStr">
         <is>
@@ -2417,11 +2417,11 @@
         </is>
       </c>
       <c r="J33" t="n">
-        <v>37240</v>
+        <v>60000</v>
       </c>
       <c r="K33" t="inlineStr">
         <is>
-          <t>per m2 incl. membrane</t>
+          <t>surface slider kit, soft-close</t>
         </is>
       </c>
     </row>
@@ -2443,11 +2443,11 @@
       </c>
       <c r="D34" t="inlineStr">
         <is>
-          <t>Wall tiles + adhesive + grout, back wall</t>
+          <t>Cement board 12 mm + liquid membrane, back wall</t>
         </is>
       </c>
       <c r="E34" t="n">
-        <v>2.93</v>
+        <v>2.66</v>
       </c>
       <c r="F34" t="inlineStr">
         <is>
@@ -2455,7 +2455,7 @@
         </is>
       </c>
       <c r="G34" t="n">
-        <v>16000</v>
+        <v>14000</v>
       </c>
       <c r="H34" t="inlineStr">
         <is>
@@ -2468,11 +2468,11 @@
         </is>
       </c>
       <c r="J34" t="n">
-        <v>46880</v>
+        <v>37240</v>
       </c>
       <c r="K34" t="inlineStr">
         <is>
-          <t>per m2 incl. adhesive and grout</t>
+          <t>per m2 incl. membrane</t>
         </is>
       </c>
     </row>
@@ -2494,11 +2494,11 @@
       </c>
       <c r="D35" t="inlineStr">
         <is>
-          <t>Cement board 12 mm + liquid membrane, end wall B, built out 30 mm over the concealed WC cistern (stud wall inside the cargo doors)</t>
+          <t>Wall tiles + adhesive + grout, back wall</t>
         </is>
       </c>
       <c r="E35" t="n">
-        <v>3.94</v>
+        <v>2.93</v>
       </c>
       <c r="F35" t="inlineStr">
         <is>
@@ -2506,7 +2506,7 @@
         </is>
       </c>
       <c r="G35" t="n">
-        <v>14000</v>
+        <v>16000</v>
       </c>
       <c r="H35" t="inlineStr">
         <is>
@@ -2519,11 +2519,11 @@
         </is>
       </c>
       <c r="J35" t="n">
-        <v>55160</v>
+        <v>46880</v>
       </c>
       <c r="K35" t="inlineStr">
         <is>
-          <t>per m2 incl. membrane</t>
+          <t>per m2 incl. adhesive and grout</t>
         </is>
       </c>
     </row>
@@ -2545,11 +2545,11 @@
       </c>
       <c r="D36" t="inlineStr">
         <is>
-          <t>Wall tiles + adhesive + grout, end wall B, built out 30 mm over the concealed WC cistern (stud wall inside the cargo doors)</t>
+          <t>Cement board 12 mm + liquid membrane, end wall B, built out 30 mm over the concealed WC cistern (stud wall inside the cargo doors)</t>
         </is>
       </c>
       <c r="E36" t="n">
-        <v>4.33</v>
+        <v>3.94</v>
       </c>
       <c r="F36" t="inlineStr">
         <is>
@@ -2557,7 +2557,7 @@
         </is>
       </c>
       <c r="G36" t="n">
-        <v>16000</v>
+        <v>14000</v>
       </c>
       <c r="H36" t="inlineStr">
         <is>
@@ -2570,11 +2570,11 @@
         </is>
       </c>
       <c r="J36" t="n">
-        <v>69280</v>
+        <v>55160</v>
       </c>
       <c r="K36" t="inlineStr">
         <is>
-          <t>per m2 incl. adhesive and grout</t>
+          <t>per m2 incl. membrane</t>
         </is>
       </c>
     </row>
@@ -2596,11 +2596,11 @@
       </c>
       <c r="D37" t="inlineStr">
         <is>
-          <t>Cement board 12 mm + liquid membrane, partition, bath face</t>
+          <t>Wall tiles + adhesive + grout, end wall B, built out 30 mm over the concealed WC cistern (stud wall inside the cargo doors)</t>
         </is>
       </c>
       <c r="E37" t="n">
-        <v>3.94</v>
+        <v>4.33</v>
       </c>
       <c r="F37" t="inlineStr">
         <is>
@@ -2608,7 +2608,7 @@
         </is>
       </c>
       <c r="G37" t="n">
-        <v>14000</v>
+        <v>16000</v>
       </c>
       <c r="H37" t="inlineStr">
         <is>
@@ -2621,11 +2621,11 @@
         </is>
       </c>
       <c r="J37" t="n">
-        <v>55160</v>
+        <v>69280</v>
       </c>
       <c r="K37" t="inlineStr">
         <is>
-          <t>per m2 incl. membrane</t>
+          <t>per m2 incl. adhesive and grout</t>
         </is>
       </c>
     </row>
@@ -2647,11 +2647,11 @@
       </c>
       <c r="D38" t="inlineStr">
         <is>
-          <t>Wall tiles + adhesive + grout, partition, bath face</t>
+          <t>Cement board 12 mm + liquid membrane, partition, bath face</t>
         </is>
       </c>
       <c r="E38" t="n">
-        <v>4.33</v>
+        <v>3.94</v>
       </c>
       <c r="F38" t="inlineStr">
         <is>
@@ -2659,7 +2659,7 @@
         </is>
       </c>
       <c r="G38" t="n">
-        <v>16000</v>
+        <v>14000</v>
       </c>
       <c r="H38" t="inlineStr">
         <is>
@@ -2672,11 +2672,11 @@
         </is>
       </c>
       <c r="J38" t="n">
-        <v>69280</v>
+        <v>55160</v>
       </c>
       <c r="K38" t="inlineStr">
         <is>
-          <t>per m2 incl. adhesive and grout</t>
+          <t>per m2 incl. membrane</t>
         </is>
       </c>
     </row>
@@ -2698,11 +2698,11 @@
       </c>
       <c r="D39" t="inlineStr">
         <is>
-          <t>Cement board 12 mm + liquid membrane, cross wall, bath face</t>
+          <t>Wall tiles + adhesive + grout, partition, bath face</t>
         </is>
       </c>
       <c r="E39" t="n">
-        <v>2.66</v>
+        <v>4.33</v>
       </c>
       <c r="F39" t="inlineStr">
         <is>
@@ -2710,7 +2710,7 @@
         </is>
       </c>
       <c r="G39" t="n">
-        <v>14000</v>
+        <v>16000</v>
       </c>
       <c r="H39" t="inlineStr">
         <is>
@@ -2723,11 +2723,11 @@
         </is>
       </c>
       <c r="J39" t="n">
-        <v>37240</v>
+        <v>69280</v>
       </c>
       <c r="K39" t="inlineStr">
         <is>
-          <t>per m2 incl. membrane</t>
+          <t>per m2 incl. adhesive and grout</t>
         </is>
       </c>
     </row>
@@ -2749,11 +2749,11 @@
       </c>
       <c r="D40" t="inlineStr">
         <is>
-          <t>Wall tiles + adhesive + grout, cross wall, bath face</t>
+          <t>Cement board 12 mm + liquid membrane, cross wall, bath face</t>
         </is>
       </c>
       <c r="E40" t="n">
-        <v>2.93</v>
+        <v>2.66</v>
       </c>
       <c r="F40" t="inlineStr">
         <is>
@@ -2761,7 +2761,7 @@
         </is>
       </c>
       <c r="G40" t="n">
-        <v>16000</v>
+        <v>14000</v>
       </c>
       <c r="H40" t="inlineStr">
         <is>
@@ -2774,11 +2774,11 @@
         </is>
       </c>
       <c r="J40" t="n">
-        <v>46880</v>
+        <v>37240</v>
       </c>
       <c r="K40" t="inlineStr">
         <is>
-          <t>per m2 incl. adhesive and grout</t>
+          <t>per m2 incl. membrane</t>
         </is>
       </c>
     </row>
@@ -2800,11 +2800,11 @@
       </c>
       <c r="D41" t="inlineStr">
         <is>
-          <t>Cement board 12 mm + liquid membrane, splashback behind the basin (end wall B, wash lobby)</t>
+          <t>Wall tiles + adhesive + grout, cross wall, bath face</t>
         </is>
       </c>
       <c r="E41" t="n">
-        <v>1.12</v>
+        <v>2.93</v>
       </c>
       <c r="F41" t="inlineStr">
         <is>
@@ -2812,7 +2812,7 @@
         </is>
       </c>
       <c r="G41" t="n">
-        <v>14000</v>
+        <v>16000</v>
       </c>
       <c r="H41" t="inlineStr">
         <is>
@@ -2825,11 +2825,11 @@
         </is>
       </c>
       <c r="J41" t="n">
-        <v>15680</v>
+        <v>46880</v>
       </c>
       <c r="K41" t="inlineStr">
         <is>
-          <t>per m2 incl. membrane</t>
+          <t>per m2 incl. adhesive and grout</t>
         </is>
       </c>
     </row>
@@ -2841,7 +2841,7 @@
       </c>
       <c r="B42" t="inlineStr">
         <is>
-          <t>wet walls</t>
+          <t>finishes</t>
         </is>
       </c>
       <c r="C42" t="inlineStr">
@@ -2851,11 +2851,11 @@
       </c>
       <c r="D42" t="inlineStr">
         <is>
-          <t>Wall tiles + adhesive + grout, splashback behind the basin (end wall B, wash lobby)</t>
+          <t>Safety vinyl sheet, coved 100 mm up the walls (bathroom and lobby)</t>
         </is>
       </c>
       <c r="E42" t="n">
-        <v>1.23</v>
+        <v>3.2</v>
       </c>
       <c r="F42" t="inlineStr">
         <is>
@@ -2863,7 +2863,7 @@
         </is>
       </c>
       <c r="G42" t="n">
-        <v>16000</v>
+        <v>15000</v>
       </c>
       <c r="H42" t="inlineStr">
         <is>
@@ -2876,11 +2876,11 @@
         </is>
       </c>
       <c r="J42" t="n">
-        <v>19680</v>
+        <v>48000</v>
       </c>
       <c r="K42" t="inlineStr">
         <is>
-          <t>per m2 incl. adhesive and grout</t>
+          <t>per m2</t>
         </is>
       </c>
     </row>
@@ -2892,29 +2892,29 @@
       </c>
       <c r="B43" t="inlineStr">
         <is>
-          <t>finishes</t>
+          <t>sanitaryware</t>
         </is>
       </c>
       <c r="C43" t="inlineStr">
         <is>
-          <t>tiling</t>
+          <t>plumbing</t>
         </is>
       </c>
       <c r="D43" t="inlineStr">
         <is>
-          <t>Safety vinyl sheet, coved 100 mm up the walls (bathroom and wash lobby)</t>
+          <t>Shower tray 1000 x 900, low profile, 90 mm waste</t>
         </is>
       </c>
       <c r="E43" t="n">
-        <v>3.2</v>
+        <v>1</v>
       </c>
       <c r="F43" t="inlineStr">
         <is>
-          <t>m2</t>
+          <t>each</t>
         </is>
       </c>
       <c r="G43" t="n">
-        <v>15000</v>
+        <v>120000</v>
       </c>
       <c r="H43" t="inlineStr">
         <is>
@@ -2927,13 +2927,9 @@
         </is>
       </c>
       <c r="J43" t="n">
-        <v>48000</v>
-      </c>
-      <c r="K43" t="inlineStr">
-        <is>
-          <t>per m2</t>
-        </is>
-      </c>
+        <v>120000</v>
+      </c>
+      <c r="K43" t="inlineStr"/>
     </row>
     <row r="44">
       <c r="A44" t="inlineStr">
@@ -2953,7 +2949,7 @@
       </c>
       <c r="D44" t="inlineStr">
         <is>
-          <t>Shower tray 1000 x 900, low profile, 90 mm waste</t>
+          <t>Fixed glass shower screen 700 x 2,000, 8 mm toughened</t>
         </is>
       </c>
       <c r="E44" t="n">
@@ -2965,7 +2961,7 @@
         </is>
       </c>
       <c r="G44" t="n">
-        <v>120000</v>
+        <v>180000</v>
       </c>
       <c r="H44" t="inlineStr">
         <is>
@@ -2978,7 +2974,7 @@
         </is>
       </c>
       <c r="J44" t="n">
-        <v>120000</v>
+        <v>180000</v>
       </c>
       <c r="K44" t="inlineStr"/>
     </row>
@@ -3000,7 +2996,7 @@
       </c>
       <c r="D45" t="inlineStr">
         <is>
-          <t>Fixed glass shower screen 700 x 2,000, 8 mm toughened</t>
+          <t>Wall-hung WC, short projection (520), soft-close seat</t>
         </is>
       </c>
       <c r="E45" t="n">
@@ -3012,7 +3008,7 @@
         </is>
       </c>
       <c r="G45" t="n">
-        <v>180000</v>
+        <v>150000</v>
       </c>
       <c r="H45" t="inlineStr">
         <is>
@@ -3025,7 +3021,7 @@
         </is>
       </c>
       <c r="J45" t="n">
-        <v>180000</v>
+        <v>150000</v>
       </c>
       <c r="K45" t="inlineStr"/>
     </row>
@@ -3047,7 +3043,7 @@
       </c>
       <c r="D46" t="inlineStr">
         <is>
-          <t>Wall-hung WC, short projection (520), soft-close seat</t>
+          <t>Slim concealed cistern frame (80 mm) with dual-flush plate, in the end-B stud wall and its 30 mm build-out</t>
         </is>
       </c>
       <c r="E46" t="n">
@@ -3055,11 +3051,11 @@
       </c>
       <c r="F46" t="inlineStr">
         <is>
-          <t>each</t>
+          <t>set</t>
         </is>
       </c>
       <c r="G46" t="n">
-        <v>150000</v>
+        <v>220000</v>
       </c>
       <c r="H46" t="inlineStr">
         <is>
@@ -3072,9 +3068,13 @@
         </is>
       </c>
       <c r="J46" t="n">
-        <v>150000</v>
-      </c>
-      <c r="K46" t="inlineStr"/>
+        <v>220000</v>
+      </c>
+      <c r="K46" t="inlineStr">
+        <is>
+          <t>slim concealed cistern frame + dual-flush plate</t>
+        </is>
+      </c>
     </row>
     <row r="47">
       <c r="A47" t="inlineStr">
@@ -3084,17 +3084,17 @@
       </c>
       <c r="B47" t="inlineStr">
         <is>
-          <t>sanitaryware</t>
+          <t>accessories</t>
         </is>
       </c>
       <c r="C47" t="inlineStr">
         <is>
-          <t>plumbing</t>
+          <t>carpentry</t>
         </is>
       </c>
       <c r="D47" t="inlineStr">
         <is>
-          <t>Slim concealed cistern frame (80 mm) with dual-flush plate, in the end-B stud wall and its 30 mm build-out</t>
+          <t>Towel rail, robe hook, toilet-roll holder, shower shelf</t>
         </is>
       </c>
       <c r="E47" t="n">
@@ -3106,7 +3106,7 @@
         </is>
       </c>
       <c r="G47" t="n">
-        <v>220000</v>
+        <v>40000</v>
       </c>
       <c r="H47" t="inlineStr">
         <is>
@@ -3119,37 +3119,33 @@
         </is>
       </c>
       <c r="J47" t="n">
-        <v>220000</v>
-      </c>
-      <c r="K47" t="inlineStr">
-        <is>
-          <t>slim concealed cistern frame + dual-flush plate</t>
-        </is>
-      </c>
+        <v>40000</v>
+      </c>
+      <c r="K47" t="inlineStr"/>
     </row>
     <row r="48">
       <c r="A48" t="inlineStr">
         <is>
-          <t>K2</t>
+          <t>K3</t>
         </is>
       </c>
       <c r="B48" t="inlineStr">
         <is>
-          <t>sanitaryware</t>
+          <t>hardware</t>
         </is>
       </c>
       <c r="C48" t="inlineStr">
         <is>
-          <t>plumbing</t>
+          <t>carpentry</t>
         </is>
       </c>
       <c r="D48" t="inlineStr">
         <is>
-          <t>Wall basin 400 x 300 + mixer + bottle trap (wash lobby)</t>
+          <t>Hob base adjustable legs</t>
         </is>
       </c>
       <c r="E48" t="n">
-        <v>1</v>
+        <v>4</v>
       </c>
       <c r="F48" t="inlineStr">
         <is>
@@ -3157,7 +3153,7 @@
         </is>
       </c>
       <c r="G48" t="n">
-        <v>90000</v>
+        <v>1500</v>
       </c>
       <c r="H48" t="inlineStr">
         <is>
@@ -3170,19 +3166,19 @@
         </is>
       </c>
       <c r="J48" t="n">
-        <v>90000</v>
+        <v>6000</v>
       </c>
       <c r="K48" t="inlineStr"/>
     </row>
     <row r="49">
       <c r="A49" t="inlineStr">
         <is>
-          <t>K2</t>
+          <t>K3</t>
         </is>
       </c>
       <c r="B49" t="inlineStr">
         <is>
-          <t>glazing</t>
+          <t>hardware</t>
         </is>
       </c>
       <c r="C49" t="inlineStr">
@@ -3192,11 +3188,11 @@
       </c>
       <c r="D49" t="inlineStr">
         <is>
-          <t>Mirror 4 mm bonded to the cabinet door</t>
+          <t>Sink base adjustable legs</t>
         </is>
       </c>
       <c r="E49" t="n">
-        <v>1</v>
+        <v>4</v>
       </c>
       <c r="F49" t="inlineStr">
         <is>
@@ -3204,7 +3200,7 @@
         </is>
       </c>
       <c r="G49" t="n">
-        <v>25000</v>
+        <v>1500</v>
       </c>
       <c r="H49" t="inlineStr">
         <is>
@@ -3217,29 +3213,29 @@
         </is>
       </c>
       <c r="J49" t="n">
-        <v>25000</v>
+        <v>6000</v>
       </c>
       <c r="K49" t="inlineStr"/>
     </row>
     <row r="50">
       <c r="A50" t="inlineStr">
         <is>
-          <t>K2</t>
+          <t>K3</t>
         </is>
       </c>
       <c r="B50" t="inlineStr">
         <is>
-          <t>accessories</t>
+          <t>appliances</t>
         </is>
       </c>
       <c r="C50" t="inlineStr">
         <is>
-          <t>carpentry</t>
+          <t>electrical</t>
         </is>
       </c>
       <c r="D50" t="inlineStr">
         <is>
-          <t>Towel rail, robe hook, toilet-roll holder, shower shelf</t>
+          <t>Two-zone induction hob, zones side by side, black glass 590 x 350, front knobs, about 3.5 kW</t>
         </is>
       </c>
       <c r="E50" t="n">
@@ -3247,11 +3243,11 @@
       </c>
       <c r="F50" t="inlineStr">
         <is>
-          <t>set</t>
+          <t>each</t>
         </is>
       </c>
       <c r="G50" t="n">
-        <v>40000</v>
+        <v>250000</v>
       </c>
       <c r="H50" t="inlineStr">
         <is>
@@ -3264,9 +3260,13 @@
         </is>
       </c>
       <c r="J50" t="n">
-        <v>40000</v>
-      </c>
-      <c r="K50" t="inlineStr"/>
+        <v>250000</v>
+      </c>
+      <c r="K50" t="inlineStr">
+        <is>
+          <t>2-zone induction, zones side by side, 590 x 350</t>
+        </is>
+      </c>
     </row>
     <row r="51">
       <c r="A51" t="inlineStr">
@@ -3276,21 +3276,21 @@
       </c>
       <c r="B51" t="inlineStr">
         <is>
-          <t>hardware</t>
+          <t>sanitaryware</t>
         </is>
       </c>
       <c r="C51" t="inlineStr">
         <is>
-          <t>carpentry</t>
+          <t>plumbing</t>
         </is>
       </c>
       <c r="D51" t="inlineStr">
         <is>
-          <t>Hob base adjustable legs</t>
+          <t>Inset stainless sink about 380 x 420, single bowl</t>
         </is>
       </c>
       <c r="E51" t="n">
-        <v>4</v>
+        <v>1</v>
       </c>
       <c r="F51" t="inlineStr">
         <is>
@@ -3298,7 +3298,7 @@
         </is>
       </c>
       <c r="G51" t="n">
-        <v>1500</v>
+        <v>70000</v>
       </c>
       <c r="H51" t="inlineStr">
         <is>
@@ -3311,7 +3311,7 @@
         </is>
       </c>
       <c r="J51" t="n">
-        <v>6000</v>
+        <v>70000</v>
       </c>
       <c r="K51" t="inlineStr"/>
     </row>
@@ -3323,21 +3323,21 @@
       </c>
       <c r="B52" t="inlineStr">
         <is>
-          <t>hardware</t>
+          <t>sanitaryware</t>
         </is>
       </c>
       <c r="C52" t="inlineStr">
         <is>
-          <t>carpentry</t>
+          <t>plumbing</t>
         </is>
       </c>
       <c r="D52" t="inlineStr">
         <is>
-          <t>Sink base adjustable legs</t>
+          <t>Kitchen mixer tap</t>
         </is>
       </c>
       <c r="E52" t="n">
-        <v>4</v>
+        <v>1</v>
       </c>
       <c r="F52" t="inlineStr">
         <is>
@@ -3345,7 +3345,7 @@
         </is>
       </c>
       <c r="G52" t="n">
-        <v>1500</v>
+        <v>45000</v>
       </c>
       <c r="H52" t="inlineStr">
         <is>
@@ -3358,7 +3358,7 @@
         </is>
       </c>
       <c r="J52" t="n">
-        <v>6000</v>
+        <v>45000</v>
       </c>
       <c r="K52" t="inlineStr"/>
     </row>
@@ -3380,7 +3380,7 @@
       </c>
       <c r="D53" t="inlineStr">
         <is>
-          <t>Two-zone induction hob, zones side by side, black glass 590 x 350, front knobs, about 3.5 kW</t>
+          <t>Under-counter fridge about 90 L (A-class)</t>
         </is>
       </c>
       <c r="E53" t="n">
@@ -3392,24 +3392,24 @@
         </is>
       </c>
       <c r="G53" t="n">
-        <v>250000</v>
+        <v>265000</v>
       </c>
       <c r="H53" t="inlineStr">
         <is>
-          <t>A</t>
+          <t>V</t>
         </is>
       </c>
       <c r="I53" t="inlineStr">
         <is>
-          <t>AS-21</t>
+          <t>STU-P03</t>
         </is>
       </c>
       <c r="J53" t="n">
-        <v>250000</v>
+        <v>265000</v>
       </c>
       <c r="K53" t="inlineStr">
         <is>
-          <t>2-zone induction, zones side by side, 590 x 350</t>
+          <t>90 L mini fridge, Kanis 2026-10-26</t>
         </is>
       </c>
     </row>
@@ -3421,17 +3421,17 @@
       </c>
       <c r="B54" t="inlineStr">
         <is>
-          <t>sanitaryware</t>
+          <t>appliances</t>
         </is>
       </c>
       <c r="C54" t="inlineStr">
         <is>
-          <t>plumbing</t>
+          <t>electrical</t>
         </is>
       </c>
       <c r="D54" t="inlineStr">
         <is>
-          <t>Inset stainless sink about 380 x 420, single bowl</t>
+          <t>Chimney hood 600 mm, black, recirculating with a charcoal filter</t>
         </is>
       </c>
       <c r="E54" t="n">
@@ -3443,7 +3443,7 @@
         </is>
       </c>
       <c r="G54" t="n">
-        <v>70000</v>
+        <v>150000</v>
       </c>
       <c r="H54" t="inlineStr">
         <is>
@@ -3456,9 +3456,13 @@
         </is>
       </c>
       <c r="J54" t="n">
-        <v>70000</v>
-      </c>
-      <c r="K54" t="inlineStr"/>
+        <v>150000</v>
+      </c>
+      <c r="K54" t="inlineStr">
+        <is>
+          <t>chimney hood 600 mm, black</t>
+        </is>
+      </c>
     </row>
     <row r="55">
       <c r="A55" t="inlineStr">
@@ -3468,17 +3472,17 @@
       </c>
       <c r="B55" t="inlineStr">
         <is>
-          <t>sanitaryware</t>
+          <t>appliances</t>
         </is>
       </c>
       <c r="C55" t="inlineStr">
         <is>
-          <t>plumbing</t>
+          <t>electrical</t>
         </is>
       </c>
       <c r="D55" t="inlineStr">
         <is>
-          <t>Kitchen mixer tap</t>
+          <t>Telescopic chimney cover 260 x 220, hood to the ceiling (comes with the hood)</t>
         </is>
       </c>
       <c r="E55" t="n">
@@ -3490,7 +3494,7 @@
         </is>
       </c>
       <c r="G55" t="n">
-        <v>45000</v>
+        <v>0</v>
       </c>
       <c r="H55" t="inlineStr">
         <is>
@@ -3503,9 +3507,13 @@
         </is>
       </c>
       <c r="J55" t="n">
-        <v>45000</v>
-      </c>
-      <c r="K55" t="inlineStr"/>
+        <v>0</v>
+      </c>
+      <c r="K55" t="inlineStr">
+        <is>
+          <t>telescopic cover, comes with the hood</t>
+        </is>
+      </c>
     </row>
     <row r="56">
       <c r="A56" t="inlineStr">
@@ -3515,17 +3523,17 @@
       </c>
       <c r="B56" t="inlineStr">
         <is>
-          <t>appliances</t>
+          <t>plumbing</t>
         </is>
       </c>
       <c r="C56" t="inlineStr">
         <is>
-          <t>electrical</t>
+          <t>plumbing</t>
         </is>
       </c>
       <c r="D56" t="inlineStr">
         <is>
-          <t>Under-counter fridge about 90 L (A-class)</t>
+          <t>Under-sink drinking-water filter + faucet</t>
         </is>
       </c>
       <c r="E56" t="n">
@@ -3537,46 +3545,42 @@
         </is>
       </c>
       <c r="G56" t="n">
-        <v>265000</v>
+        <v>80000</v>
       </c>
       <c r="H56" t="inlineStr">
         <is>
-          <t>V</t>
+          <t>A</t>
         </is>
       </c>
       <c r="I56" t="inlineStr">
         <is>
-          <t>STU-P03</t>
+          <t>AS-21</t>
         </is>
       </c>
       <c r="J56" t="n">
-        <v>265000</v>
-      </c>
-      <c r="K56" t="inlineStr">
-        <is>
-          <t>90 L mini fridge, Kanis 2026-10-26</t>
-        </is>
-      </c>
+        <v>80000</v>
+      </c>
+      <c r="K56" t="inlineStr"/>
     </row>
     <row r="57">
       <c r="A57" t="inlineStr">
         <is>
-          <t>K3</t>
+          <t>K4</t>
         </is>
       </c>
       <c r="B57" t="inlineStr">
         <is>
-          <t>appliances</t>
+          <t>bedding</t>
         </is>
       </c>
       <c r="C57" t="inlineStr">
         <is>
-          <t>electrical</t>
+          <t>furnishing</t>
         </is>
       </c>
       <c r="D57" t="inlineStr">
         <is>
-          <t>Slim recirculating hood 600 mm, black, charcoal filter</t>
+          <t>Mattress up to 1,600 x 2,000 (local size, e.g. 5 x 6 ft), 200 mm</t>
         </is>
       </c>
       <c r="E57" t="n">
@@ -3588,7 +3592,7 @@
         </is>
       </c>
       <c r="G57" t="n">
-        <v>90000</v>
+        <v>180000</v>
       </c>
       <c r="H57" t="inlineStr">
         <is>
@@ -3601,33 +3605,33 @@
         </is>
       </c>
       <c r="J57" t="n">
-        <v>90000</v>
+        <v>180000</v>
       </c>
       <c r="K57" t="inlineStr">
         <is>
-          <t>slim 600 mm, black</t>
+          <t>local foam, size to field-check (STU-51)</t>
         </is>
       </c>
     </row>
     <row r="58">
       <c r="A58" t="inlineStr">
         <is>
-          <t>K3</t>
+          <t>K5</t>
         </is>
       </c>
       <c r="B58" t="inlineStr">
         <is>
-          <t>plumbing</t>
+          <t>furnishing</t>
         </is>
       </c>
       <c r="C58" t="inlineStr">
         <is>
-          <t>plumbing</t>
+          <t>furnishing</t>
         </is>
       </c>
       <c r="D58" t="inlineStr">
         <is>
-          <t>Under-sink drinking-water filter + faucet</t>
+          <t>Table lamp, linen drum shade, LED E27 (reading lamp)</t>
         </is>
       </c>
       <c r="E58" t="n">
@@ -3639,7 +3643,7 @@
         </is>
       </c>
       <c r="G58" t="n">
-        <v>80000</v>
+        <v>35000</v>
       </c>
       <c r="H58" t="inlineStr">
         <is>
@@ -3652,29 +3656,33 @@
         </is>
       </c>
       <c r="J58" t="n">
-        <v>80000</v>
-      </c>
-      <c r="K58" t="inlineStr"/>
+        <v>35000</v>
+      </c>
+      <c r="K58" t="inlineStr">
+        <is>
+          <t>table lamp with linen shade, LED bulb</t>
+        </is>
+      </c>
     </row>
     <row r="59">
       <c r="A59" t="inlineStr">
         <is>
-          <t>K4</t>
+          <t>K5</t>
         </is>
       </c>
       <c r="B59" t="inlineStr">
         <is>
-          <t>bedding</t>
+          <t>hardware</t>
         </is>
       </c>
       <c r="C59" t="inlineStr">
         <is>
-          <t>furnishing</t>
+          <t>carpentry</t>
         </is>
       </c>
       <c r="D59" t="inlineStr">
         <is>
-          <t>Mattress up to 1,600 x 2,000 (local size, e.g. 5 x 6 ft), 200 mm</t>
+          <t>Coat hooks, hanging rail by the door and a folding luggage rack</t>
         </is>
       </c>
       <c r="E59" t="n">
@@ -3682,11 +3690,11 @@
       </c>
       <c r="F59" t="inlineStr">
         <is>
-          <t>each</t>
+          <t>set</t>
         </is>
       </c>
       <c r="G59" t="n">
-        <v>180000</v>
+        <v>8000</v>
       </c>
       <c r="H59" t="inlineStr">
         <is>
@@ -3699,18 +3707,14 @@
         </is>
       </c>
       <c r="J59" t="n">
-        <v>180000</v>
-      </c>
-      <c r="K59" t="inlineStr">
-        <is>
-          <t>local foam, size to field-check (STU-51)</t>
-        </is>
-      </c>
+        <v>8000</v>
+      </c>
+      <c r="K59" t="inlineStr"/>
     </row>
     <row r="60">
       <c r="A60" t="inlineStr">
         <is>
-          <t>K5</t>
+          <t>K6</t>
         </is>
       </c>
       <c r="B60" t="inlineStr">
@@ -3725,7 +3729,7 @@
       </c>
       <c r="D60" t="inlineStr">
         <is>
-          <t>Table lamp, linen drum shade, LED E27 (reading lamp)</t>
+          <t>Low two-seat sofa about 1300 x 750, 700 high, soft dark grey washable covers</t>
         </is>
       </c>
       <c r="E60" t="n">
@@ -3737,7 +3741,7 @@
         </is>
       </c>
       <c r="G60" t="n">
-        <v>35000</v>
+        <v>450000</v>
       </c>
       <c r="H60" t="inlineStr">
         <is>
@@ -3750,33 +3754,33 @@
         </is>
       </c>
       <c r="J60" t="n">
-        <v>35000</v>
+        <v>450000</v>
       </c>
       <c r="K60" t="inlineStr">
         <is>
-          <t>table lamp with linen shade, LED bulb</t>
+          <t>compact two-seat sofa, washable covers</t>
         </is>
       </c>
     </row>
     <row r="61">
       <c r="A61" t="inlineStr">
         <is>
-          <t>K5</t>
+          <t>K6</t>
         </is>
       </c>
       <c r="B61" t="inlineStr">
         <is>
-          <t>hardware</t>
+          <t>furnishing</t>
         </is>
       </c>
       <c r="C61" t="inlineStr">
         <is>
-          <t>carpentry</t>
+          <t>furnishing</t>
         </is>
       </c>
       <c r="D61" t="inlineStr">
         <is>
-          <t>Coat hooks, hanging rail by the door and a folding luggage rack</t>
+          <t>Blackout curtain + track for the 3 m slider</t>
         </is>
       </c>
       <c r="E61" t="n">
@@ -3788,7 +3792,7 @@
         </is>
       </c>
       <c r="G61" t="n">
-        <v>8000</v>
+        <v>60000</v>
       </c>
       <c r="H61" t="inlineStr">
         <is>
@@ -3801,7 +3805,7 @@
         </is>
       </c>
       <c r="J61" t="n">
-        <v>8000</v>
+        <v>60000</v>
       </c>
       <c r="K61" t="inlineStr"/>
     </row>
@@ -3813,17 +3817,17 @@
       </c>
       <c r="B62" t="inlineStr">
         <is>
-          <t>furnishing</t>
+          <t>glazing</t>
         </is>
       </c>
       <c r="C62" t="inlineStr">
         <is>
-          <t>furnishing</t>
+          <t>glazier</t>
         </is>
       </c>
       <c r="D62" t="inlineStr">
         <is>
-          <t>Low two-seat sofa about 1300 x 750, 700 high, soft dark grey washable covers</t>
+          <t>Insect screens: slider (sliding), W1, vents</t>
         </is>
       </c>
       <c r="E62" t="n">
@@ -3831,11 +3835,11 @@
       </c>
       <c r="F62" t="inlineStr">
         <is>
-          <t>each</t>
+          <t>set</t>
         </is>
       </c>
       <c r="G62" t="n">
-        <v>450000</v>
+        <v>90000</v>
       </c>
       <c r="H62" t="inlineStr">
         <is>
@@ -3848,45 +3852,41 @@
         </is>
       </c>
       <c r="J62" t="n">
-        <v>450000</v>
-      </c>
-      <c r="K62" t="inlineStr">
-        <is>
-          <t>compact two-seat sofa, washable covers</t>
-        </is>
-      </c>
+        <v>90000</v>
+      </c>
+      <c r="K62" t="inlineStr"/>
     </row>
     <row r="63">
       <c r="A63" t="inlineStr">
         <is>
-          <t>K6</t>
+          <t>K7</t>
         </is>
       </c>
       <c r="B63" t="inlineStr">
         <is>
-          <t>furnishing</t>
+          <t>finishes</t>
         </is>
       </c>
       <c r="C63" t="inlineStr">
         <is>
-          <t>furnishing</t>
+          <t>painting</t>
         </is>
       </c>
       <c r="D63" t="inlineStr">
         <is>
-          <t>Blackout curtain + track for the 3 m slider</t>
+          <t>Joinery finish: medium-oak stain + clear matte PU varnish over pine (all furniture)</t>
         </is>
       </c>
       <c r="E63" t="n">
-        <v>1</v>
+        <v>6</v>
       </c>
       <c r="F63" t="inlineStr">
         <is>
-          <t>set</t>
+          <t>L</t>
         </is>
       </c>
       <c r="G63" t="n">
-        <v>60000</v>
+        <v>14000</v>
       </c>
       <c r="H63" t="inlineStr">
         <is>
@@ -3899,29 +3899,33 @@
         </is>
       </c>
       <c r="J63" t="n">
-        <v>60000</v>
-      </c>
-      <c r="K63" t="inlineStr"/>
+        <v>84000</v>
+      </c>
+      <c r="K63" t="inlineStr">
+        <is>
+          <t>medium-oak stain + clear matte PU varnish for pine, per L</t>
+        </is>
+      </c>
     </row>
     <row r="64">
       <c r="A64" t="inlineStr">
         <is>
-          <t>K6</t>
+          <t>K8</t>
         </is>
       </c>
       <c r="B64" t="inlineStr">
         <is>
-          <t>glazing</t>
+          <t>electrical</t>
         </is>
       </c>
       <c r="C64" t="inlineStr">
         <is>
-          <t>glazier</t>
+          <t>electrical</t>
         </is>
       </c>
       <c r="D64" t="inlineStr">
         <is>
-          <t>Insect screens: slider (sliding), W1, vents</t>
+          <t>Unit board, 24 modules (2 x 12), by the galley</t>
         </is>
       </c>
       <c r="E64" t="n">
@@ -3929,11 +3933,11 @@
       </c>
       <c r="F64" t="inlineStr">
         <is>
-          <t>set</t>
+          <t>each</t>
         </is>
       </c>
       <c r="G64" t="n">
-        <v>90000</v>
+        <v>65000</v>
       </c>
       <c r="H64" t="inlineStr">
         <is>
@@ -3946,41 +3950,45 @@
         </is>
       </c>
       <c r="J64" t="n">
-        <v>90000</v>
-      </c>
-      <c r="K64" t="inlineStr"/>
+        <v>65000</v>
+      </c>
+      <c r="K64" t="inlineStr">
+        <is>
+          <t>enclosure, 24 modules (2 x 12)</t>
+        </is>
+      </c>
     </row>
     <row r="65">
       <c r="A65" t="inlineStr">
         <is>
-          <t>K7</t>
+          <t>K8</t>
         </is>
       </c>
       <c r="B65" t="inlineStr">
         <is>
-          <t>finishes</t>
+          <t>electrical</t>
         </is>
       </c>
       <c r="C65" t="inlineStr">
         <is>
-          <t>painting</t>
+          <t>electrical</t>
         </is>
       </c>
       <c r="D65" t="inlineStr">
         <is>
-          <t>Joinery finish: medium-oak stain + clear matte PU varnish over pine (all furniture)</t>
+          <t>Power inlet 63 A IP67 (IEC 60309 blue, 2P+E), outside behind the board</t>
         </is>
       </c>
       <c r="E65" t="n">
-        <v>6</v>
+        <v>1</v>
       </c>
       <c r="F65" t="inlineStr">
         <is>
-          <t>L</t>
+          <t>each</t>
         </is>
       </c>
       <c r="G65" t="n">
-        <v>14000</v>
+        <v>35000</v>
       </c>
       <c r="H65" t="inlineStr">
         <is>
@@ -3993,11 +4001,11 @@
         </is>
       </c>
       <c r="J65" t="n">
-        <v>84000</v>
+        <v>35000</v>
       </c>
       <c r="K65" t="inlineStr">
         <is>
-          <t>medium-oak stain + clear matte PU varnish for pine, per L</t>
+          <t>surface, IP67</t>
         </is>
       </c>
     </row>
@@ -4019,7 +4027,7 @@
       </c>
       <c r="D66" t="inlineStr">
         <is>
-          <t>Unit board, 24 modules (2 x 12), by the galley</t>
+          <t>Ceiling light, bed</t>
         </is>
       </c>
       <c r="E66" t="n">
@@ -4031,7 +4039,7 @@
         </is>
       </c>
       <c r="G66" t="n">
-        <v>65000</v>
+        <v>15000</v>
       </c>
       <c r="H66" t="inlineStr">
         <is>
@@ -4044,13 +4052,9 @@
         </is>
       </c>
       <c r="J66" t="n">
-        <v>65000</v>
-      </c>
-      <c r="K66" t="inlineStr">
-        <is>
-          <t>enclosure, 24 modules (2 x 12)</t>
-        </is>
-      </c>
+        <v>15000</v>
+      </c>
+      <c r="K66" t="inlineStr"/>
     </row>
     <row r="67">
       <c r="A67" t="inlineStr">
@@ -4070,7 +4074,7 @@
       </c>
       <c r="D67" t="inlineStr">
         <is>
-          <t>Power inlet 63 A IP67 (IEC 60309 blue, 2P+E), outside behind the board</t>
+          <t>Ceiling light, living</t>
         </is>
       </c>
       <c r="E67" t="n">
@@ -4082,7 +4086,7 @@
         </is>
       </c>
       <c r="G67" t="n">
-        <v>35000</v>
+        <v>15000</v>
       </c>
       <c r="H67" t="inlineStr">
         <is>
@@ -4095,13 +4099,9 @@
         </is>
       </c>
       <c r="J67" t="n">
-        <v>35000</v>
-      </c>
-      <c r="K67" t="inlineStr">
-        <is>
-          <t>surface, IP67</t>
-        </is>
-      </c>
+        <v>15000</v>
+      </c>
+      <c r="K67" t="inlineStr"/>
     </row>
     <row r="68">
       <c r="A68" t="inlineStr">
@@ -4121,7 +4121,7 @@
       </c>
       <c r="D68" t="inlineStr">
         <is>
-          <t>Ceiling light, bed</t>
+          <t>Ceiling light, galley</t>
         </is>
       </c>
       <c r="E68" t="n">
@@ -4168,7 +4168,7 @@
       </c>
       <c r="D69" t="inlineStr">
         <is>
-          <t>Ceiling light, living</t>
+          <t>Bathroom light IP65</t>
         </is>
       </c>
       <c r="E69" t="n">
@@ -4180,7 +4180,7 @@
         </is>
       </c>
       <c r="G69" t="n">
-        <v>15000</v>
+        <v>18000</v>
       </c>
       <c r="H69" t="inlineStr">
         <is>
@@ -4193,9 +4193,13 @@
         </is>
       </c>
       <c r="J69" t="n">
-        <v>15000</v>
-      </c>
-      <c r="K69" t="inlineStr"/>
+        <v>18000</v>
+      </c>
+      <c r="K69" t="inlineStr">
+        <is>
+          <t>IP65</t>
+        </is>
+      </c>
     </row>
     <row r="70">
       <c r="A70" t="inlineStr">
@@ -4215,7 +4219,7 @@
       </c>
       <c r="D70" t="inlineStr">
         <is>
-          <t>Ceiling light, galley</t>
+          <t>Wall reading light over the bed (wall side)</t>
         </is>
       </c>
       <c r="E70" t="n">
@@ -4262,7 +4266,7 @@
       </c>
       <c r="D71" t="inlineStr">
         <is>
-          <t>Bathroom light IP65</t>
+          <t>Under-cabinet LED strip</t>
         </is>
       </c>
       <c r="E71" t="n">
@@ -4274,7 +4278,7 @@
         </is>
       </c>
       <c r="G71" t="n">
-        <v>18000</v>
+        <v>15000</v>
       </c>
       <c r="H71" t="inlineStr">
         <is>
@@ -4287,13 +4291,9 @@
         </is>
       </c>
       <c r="J71" t="n">
-        <v>18000</v>
-      </c>
-      <c r="K71" t="inlineStr">
-        <is>
-          <t>IP65</t>
-        </is>
-      </c>
+        <v>15000</v>
+      </c>
+      <c r="K71" t="inlineStr"/>
     </row>
     <row r="72">
       <c r="A72" t="inlineStr">
@@ -4313,7 +4313,7 @@
       </c>
       <c r="D72" t="inlineStr">
         <is>
-          <t>Wall reading light over the bed (wall side)</t>
+          <t>Entry: bed (2-way), living and galley lights</t>
         </is>
       </c>
       <c r="E72" t="n">
@@ -4325,7 +4325,7 @@
         </is>
       </c>
       <c r="G72" t="n">
-        <v>15000</v>
+        <v>3500</v>
       </c>
       <c r="H72" t="inlineStr">
         <is>
@@ -4338,7 +4338,7 @@
         </is>
       </c>
       <c r="J72" t="n">
-        <v>15000</v>
+        <v>3500</v>
       </c>
       <c r="K72" t="inlineStr"/>
     </row>
@@ -4360,7 +4360,7 @@
       </c>
       <c r="D73" t="inlineStr">
         <is>
-          <t>Under-cabinet LED strip</t>
+          <t>Bed: ceiling light (2-way), over the bedside table</t>
         </is>
       </c>
       <c r="E73" t="n">
@@ -4372,7 +4372,7 @@
         </is>
       </c>
       <c r="G73" t="n">
-        <v>15000</v>
+        <v>3500</v>
       </c>
       <c r="H73" t="inlineStr">
         <is>
@@ -4385,7 +4385,7 @@
         </is>
       </c>
       <c r="J73" t="n">
-        <v>15000</v>
+        <v>3500</v>
       </c>
       <c r="K73" t="inlineStr"/>
     </row>
@@ -4407,7 +4407,7 @@
       </c>
       <c r="D74" t="inlineStr">
         <is>
-          <t>Entry: bed (2-way), living and galley lights</t>
+          <t>Bathroom light + fan (outside, by the door)</t>
         </is>
       </c>
       <c r="E74" t="n">
@@ -4454,7 +4454,7 @@
       </c>
       <c r="D75" t="inlineStr">
         <is>
-          <t>Bed: ceiling light (2-way), over the bedside table</t>
+          <t>Bathroom extract 100 mm, IPX4 for zone 1, with run-on</t>
         </is>
       </c>
       <c r="E75" t="n">
@@ -4466,7 +4466,7 @@
         </is>
       </c>
       <c r="G75" t="n">
-        <v>3500</v>
+        <v>35000</v>
       </c>
       <c r="H75" t="inlineStr">
         <is>
@@ -4479,7 +4479,7 @@
         </is>
       </c>
       <c r="J75" t="n">
-        <v>3500</v>
+        <v>35000</v>
       </c>
       <c r="K75" t="inlineStr"/>
     </row>
@@ -4501,7 +4501,7 @@
       </c>
       <c r="D76" t="inlineStr">
         <is>
-          <t>Bathroom light + fan (outside)</t>
+          <t>Wall fan 300 mm</t>
         </is>
       </c>
       <c r="E76" t="n">
@@ -4513,7 +4513,7 @@
         </is>
       </c>
       <c r="G76" t="n">
-        <v>3500</v>
+        <v>35000</v>
       </c>
       <c r="H76" t="inlineStr">
         <is>
@@ -4526,7 +4526,7 @@
         </is>
       </c>
       <c r="J76" t="n">
-        <v>3500</v>
+        <v>35000</v>
       </c>
       <c r="K76" t="inlineStr"/>
     </row>
@@ -4548,7 +4548,7 @@
       </c>
       <c r="D77" t="inlineStr">
         <is>
-          <t>Bathroom extract 100 mm, IPX4 for zone 1, with run-on</t>
+          <t>Socket + USB-C in the headboard (wall side)</t>
         </is>
       </c>
       <c r="E77" t="n">
@@ -4560,7 +4560,7 @@
         </is>
       </c>
       <c r="G77" t="n">
-        <v>35000</v>
+        <v>15000</v>
       </c>
       <c r="H77" t="inlineStr">
         <is>
@@ -4573,7 +4573,7 @@
         </is>
       </c>
       <c r="J77" t="n">
-        <v>35000</v>
+        <v>15000</v>
       </c>
       <c r="K77" t="inlineStr"/>
     </row>
@@ -4595,7 +4595,7 @@
       </c>
       <c r="D78" t="inlineStr">
         <is>
-          <t>Wall fan 300 mm</t>
+          <t>Bedside socket + USB-C (reading lamp)</t>
         </is>
       </c>
       <c r="E78" t="n">
@@ -4607,7 +4607,7 @@
         </is>
       </c>
       <c r="G78" t="n">
-        <v>35000</v>
+        <v>15000</v>
       </c>
       <c r="H78" t="inlineStr">
         <is>
@@ -4620,7 +4620,7 @@
         </is>
       </c>
       <c r="J78" t="n">
-        <v>35000</v>
+        <v>15000</v>
       </c>
       <c r="K78" t="inlineStr"/>
     </row>
@@ -4642,7 +4642,7 @@
       </c>
       <c r="D79" t="inlineStr">
         <is>
-          <t>Socket + USB-C in the headboard (wall side)</t>
+          <t>Socket + USB-C over the sofa arm, for the sofa and the table</t>
         </is>
       </c>
       <c r="E79" t="n">
@@ -4689,7 +4689,7 @@
       </c>
       <c r="D80" t="inlineStr">
         <is>
-          <t>Bedside socket + USB-C (reading lamp)</t>
+          <t>Deck socket IP66, outside by the slider</t>
         </is>
       </c>
       <c r="E80" t="n">
@@ -4716,7 +4716,11 @@
       <c r="J80" t="n">
         <v>15000</v>
       </c>
-      <c r="K80" t="inlineStr"/>
+      <c r="K80" t="inlineStr">
+        <is>
+          <t>IP66, lidded</t>
+        </is>
+      </c>
     </row>
     <row r="81">
       <c r="A81" t="inlineStr">
@@ -4736,7 +4740,7 @@
       </c>
       <c r="D81" t="inlineStr">
         <is>
-          <t>Socket + USB-C over the sofa arm, for the sofa and the table</t>
+          <t>Worktop double socket 1</t>
         </is>
       </c>
       <c r="E81" t="n">
@@ -4748,7 +4752,7 @@
         </is>
       </c>
       <c r="G81" t="n">
-        <v>15000</v>
+        <v>9000</v>
       </c>
       <c r="H81" t="inlineStr">
         <is>
@@ -4761,9 +4765,13 @@
         </is>
       </c>
       <c r="J81" t="n">
-        <v>15000</v>
-      </c>
-      <c r="K81" t="inlineStr"/>
+        <v>9000</v>
+      </c>
+      <c r="K81" t="inlineStr">
+        <is>
+          <t>double</t>
+        </is>
+      </c>
     </row>
     <row r="82">
       <c r="A82" t="inlineStr">
@@ -4783,7 +4791,7 @@
       </c>
       <c r="D82" t="inlineStr">
         <is>
-          <t>Deck socket IP66, outside by the slider</t>
+          <t>Worktop double socket 2 (back wall)</t>
         </is>
       </c>
       <c r="E82" t="n">
@@ -4795,7 +4803,7 @@
         </is>
       </c>
       <c r="G82" t="n">
-        <v>15000</v>
+        <v>9000</v>
       </c>
       <c r="H82" t="inlineStr">
         <is>
@@ -4808,11 +4816,11 @@
         </is>
       </c>
       <c r="J82" t="n">
-        <v>15000</v>
+        <v>9000</v>
       </c>
       <c r="K82" t="inlineStr">
         <is>
-          <t>IP66, lidded</t>
+          <t>double</t>
         </is>
       </c>
     </row>
@@ -4834,7 +4842,7 @@
       </c>
       <c r="D83" t="inlineStr">
         <is>
-          <t>Worktop double socket 1</t>
+          <t>Fridge socket</t>
         </is>
       </c>
       <c r="E83" t="n">
@@ -4846,7 +4854,7 @@
         </is>
       </c>
       <c r="G83" t="n">
-        <v>9000</v>
+        <v>5000</v>
       </c>
       <c r="H83" t="inlineStr">
         <is>
@@ -4859,13 +4867,9 @@
         </is>
       </c>
       <c r="J83" t="n">
-        <v>9000</v>
-      </c>
-      <c r="K83" t="inlineStr">
-        <is>
-          <t>double</t>
-        </is>
-      </c>
+        <v>5000</v>
+      </c>
+      <c r="K83" t="inlineStr"/>
     </row>
     <row r="84">
       <c r="A84" t="inlineStr">
@@ -4885,7 +4889,7 @@
       </c>
       <c r="D84" t="inlineStr">
         <is>
-          <t>Worktop double socket 2 (back wall)</t>
+          <t>Double socket behind the hood's chimney: hood + Wi-Fi router</t>
         </is>
       </c>
       <c r="E84" t="n">
@@ -4936,7 +4940,7 @@
       </c>
       <c r="D85" t="inlineStr">
         <is>
-          <t>Fridge socket</t>
+          <t>Hob outlet plate, isolated at its RCBO on the board</t>
         </is>
       </c>
       <c r="E85" t="n">
@@ -4948,7 +4952,7 @@
         </is>
       </c>
       <c r="G85" t="n">
-        <v>5000</v>
+        <v>9000</v>
       </c>
       <c r="H85" t="inlineStr">
         <is>
@@ -4961,7 +4965,7 @@
         </is>
       </c>
       <c r="J85" t="n">
-        <v>5000</v>
+        <v>9000</v>
       </c>
       <c r="K85" t="inlineStr"/>
     </row>
@@ -4983,7 +4987,7 @@
       </c>
       <c r="D86" t="inlineStr">
         <is>
-          <t>Double socket above the hood: hood + Wi-Fi router</t>
+          <t>Heater DP isolator, outside the bathroom</t>
         </is>
       </c>
       <c r="E86" t="n">
@@ -5010,11 +5014,7 @@
       <c r="J86" t="n">
         <v>9000</v>
       </c>
-      <c r="K86" t="inlineStr">
-        <is>
-          <t>double</t>
-        </is>
-      </c>
+      <c r="K86" t="inlineStr"/>
     </row>
     <row r="87">
       <c r="A87" t="inlineStr">
@@ -5034,7 +5034,7 @@
       </c>
       <c r="D87" t="inlineStr">
         <is>
-          <t>Hob outlet plate, isolated at its RCBO on the board</t>
+          <t>Deck light IP65, under the veranda canopy</t>
         </is>
       </c>
       <c r="E87" t="n">
@@ -5046,7 +5046,7 @@
         </is>
       </c>
       <c r="G87" t="n">
-        <v>9000</v>
+        <v>18000</v>
       </c>
       <c r="H87" t="inlineStr">
         <is>
@@ -5059,9 +5059,13 @@
         </is>
       </c>
       <c r="J87" t="n">
-        <v>9000</v>
-      </c>
-      <c r="K87" t="inlineStr"/>
+        <v>18000</v>
+      </c>
+      <c r="K87" t="inlineStr">
+        <is>
+          <t>IP65</t>
+        </is>
+      </c>
     </row>
     <row r="88">
       <c r="A88" t="inlineStr">
@@ -5081,7 +5085,7 @@
       </c>
       <c r="D88" t="inlineStr">
         <is>
-          <t>Heater DP isolator, outside the bathroom</t>
+          <t>Deck light, beside the entry switch</t>
         </is>
       </c>
       <c r="E88" t="n">
@@ -5093,7 +5097,7 @@
         </is>
       </c>
       <c r="G88" t="n">
-        <v>9000</v>
+        <v>3500</v>
       </c>
       <c r="H88" t="inlineStr">
         <is>
@@ -5106,7 +5110,7 @@
         </is>
       </c>
       <c r="J88" t="n">
-        <v>9000</v>
+        <v>3500</v>
       </c>
       <c r="K88" t="inlineStr"/>
     </row>
@@ -5128,7 +5132,7 @@
       </c>
       <c r="D89" t="inlineStr">
         <is>
-          <t>Deck light IP65, under the veranda canopy</t>
+          <t>Stair and roof lights (2-way), IP65 at the stair foot</t>
         </is>
       </c>
       <c r="E89" t="n">
@@ -5140,7 +5144,7 @@
         </is>
       </c>
       <c r="G89" t="n">
-        <v>18000</v>
+        <v>8000</v>
       </c>
       <c r="H89" t="inlineStr">
         <is>
@@ -5153,7 +5157,7 @@
         </is>
       </c>
       <c r="J89" t="n">
-        <v>18000</v>
+        <v>8000</v>
       </c>
       <c r="K89" t="inlineStr">
         <is>
@@ -5179,7 +5183,7 @@
       </c>
       <c r="D90" t="inlineStr">
         <is>
-          <t>Deck light, beside the entry switch</t>
+          <t>Stair light IP65</t>
         </is>
       </c>
       <c r="E90" t="n">
@@ -5191,7 +5195,7 @@
         </is>
       </c>
       <c r="G90" t="n">
-        <v>3500</v>
+        <v>18000</v>
       </c>
       <c r="H90" t="inlineStr">
         <is>
@@ -5204,9 +5208,13 @@
         </is>
       </c>
       <c r="J90" t="n">
-        <v>3500</v>
-      </c>
-      <c r="K90" t="inlineStr"/>
+        <v>18000</v>
+      </c>
+      <c r="K90" t="inlineStr">
+        <is>
+          <t>IP65</t>
+        </is>
+      </c>
     </row>
     <row r="91">
       <c r="A91" t="inlineStr">
@@ -5226,7 +5234,7 @@
       </c>
       <c r="D91" t="inlineStr">
         <is>
-          <t>Stair and roof lights (2-way), IP65 at the stair foot</t>
+          <t>Stair and roof lights (2-way), IP65 at the stair head</t>
         </is>
       </c>
       <c r="E91" t="n">
@@ -5277,7 +5285,7 @@
       </c>
       <c r="D92" t="inlineStr">
         <is>
-          <t>Stair light IP65</t>
+          <t>Roof terrace lights IP65 (x2), under the front top rail</t>
         </is>
       </c>
       <c r="E92" t="n">
@@ -5328,7 +5336,7 @@
       </c>
       <c r="D93" t="inlineStr">
         <is>
-          <t>Stair and roof lights (2-way), IP65 at the stair head</t>
+          <t>AC provision: isolator</t>
         </is>
       </c>
       <c r="E93" t="n">
@@ -5340,7 +5348,7 @@
         </is>
       </c>
       <c r="G93" t="n">
-        <v>8000</v>
+        <v>9000</v>
       </c>
       <c r="H93" t="inlineStr">
         <is>
@@ -5353,13 +5361,9 @@
         </is>
       </c>
       <c r="J93" t="n">
-        <v>8000</v>
-      </c>
-      <c r="K93" t="inlineStr">
-        <is>
-          <t>IP65</t>
-        </is>
-      </c>
+        <v>9000</v>
+      </c>
+      <c r="K93" t="inlineStr"/>
     </row>
     <row r="94">
       <c r="A94" t="inlineStr">
@@ -5369,7 +5373,7 @@
       </c>
       <c r="B94" t="inlineStr">
         <is>
-          <t>electrical</t>
+          <t>safety</t>
         </is>
       </c>
       <c r="C94" t="inlineStr">
@@ -5379,7 +5383,7 @@
       </c>
       <c r="D94" t="inlineStr">
         <is>
-          <t>Roof terrace lights IP65 (x2), under the front top rail</t>
+          <t>Smoke alarm, 10-year battery</t>
         </is>
       </c>
       <c r="E94" t="n">
@@ -5391,7 +5395,7 @@
         </is>
       </c>
       <c r="G94" t="n">
-        <v>18000</v>
+        <v>20000</v>
       </c>
       <c r="H94" t="inlineStr">
         <is>
@@ -5404,13 +5408,9 @@
         </is>
       </c>
       <c r="J94" t="n">
-        <v>18000</v>
-      </c>
-      <c r="K94" t="inlineStr">
-        <is>
-          <t>IP65</t>
-        </is>
-      </c>
+        <v>20000</v>
+      </c>
+      <c r="K94" t="inlineStr"/>
     </row>
     <row r="95">
       <c r="A95" t="inlineStr">
@@ -5420,7 +5420,7 @@
       </c>
       <c r="B95" t="inlineStr">
         <is>
-          <t>electrical</t>
+          <t>safety</t>
         </is>
       </c>
       <c r="C95" t="inlineStr">
@@ -5430,7 +5430,7 @@
       </c>
       <c r="D95" t="inlineStr">
         <is>
-          <t>AC provision: isolator</t>
+          <t>Heat alarm, kitchen, 10-year battery</t>
         </is>
       </c>
       <c r="E95" t="n">
@@ -5442,7 +5442,7 @@
         </is>
       </c>
       <c r="G95" t="n">
-        <v>9000</v>
+        <v>20000</v>
       </c>
       <c r="H95" t="inlineStr">
         <is>
@@ -5455,7 +5455,7 @@
         </is>
       </c>
       <c r="J95" t="n">
-        <v>9000</v>
+        <v>20000</v>
       </c>
       <c r="K95" t="inlineStr"/>
     </row>
@@ -5467,7 +5467,7 @@
       </c>
       <c r="B96" t="inlineStr">
         <is>
-          <t>safety</t>
+          <t>electrical</t>
         </is>
       </c>
       <c r="C96" t="inlineStr">
@@ -5477,7 +5477,7 @@
       </c>
       <c r="D96" t="inlineStr">
         <is>
-          <t>Smoke alarm, 10-year battery</t>
+          <t>Earth rod 1.5 m copper-bonded in an inspection pit, behind the board</t>
         </is>
       </c>
       <c r="E96" t="n">
@@ -5489,7 +5489,7 @@
         </is>
       </c>
       <c r="G96" t="n">
-        <v>20000</v>
+        <v>35000</v>
       </c>
       <c r="H96" t="inlineStr">
         <is>
@@ -5502,7 +5502,7 @@
         </is>
       </c>
       <c r="J96" t="n">
-        <v>20000</v>
+        <v>35000</v>
       </c>
       <c r="K96" t="inlineStr"/>
     </row>
@@ -5514,7 +5514,7 @@
       </c>
       <c r="B97" t="inlineStr">
         <is>
-          <t>safety</t>
+          <t>electrical</t>
         </is>
       </c>
       <c r="C97" t="inlineStr">
@@ -5524,19 +5524,19 @@
       </c>
       <c r="D97" t="inlineStr">
         <is>
-          <t>Heat alarm, kitchen, 10-year battery</t>
+          <t>Cable 1.5 mm2 T+E/singles in conduit, Indoor lights and fans</t>
         </is>
       </c>
       <c r="E97" t="n">
-        <v>1</v>
+        <v>31</v>
       </c>
       <c r="F97" t="inlineStr">
         <is>
-          <t>each</t>
+          <t>m</t>
         </is>
       </c>
       <c r="G97" t="n">
-        <v>20000</v>
+        <v>500</v>
       </c>
       <c r="H97" t="inlineStr">
         <is>
@@ -5549,9 +5549,13 @@
         </is>
       </c>
       <c r="J97" t="n">
-        <v>20000</v>
-      </c>
-      <c r="K97" t="inlineStr"/>
+        <v>15500</v>
+      </c>
+      <c r="K97" t="inlineStr">
+        <is>
+          <t>per m</t>
+        </is>
+      </c>
     </row>
     <row r="98">
       <c r="A98" t="inlineStr">
@@ -5571,19 +5575,19 @@
       </c>
       <c r="D98" t="inlineStr">
         <is>
-          <t>Earth rod 1.5 m copper-bonded in an inspection pit, behind the board</t>
+          <t>Cable 2.5 mm2 T+E/singles in conduit, Sockets: bed, sofa and deck</t>
         </is>
       </c>
       <c r="E98" t="n">
-        <v>1</v>
+        <v>26</v>
       </c>
       <c r="F98" t="inlineStr">
         <is>
-          <t>each</t>
+          <t>m</t>
         </is>
       </c>
       <c r="G98" t="n">
-        <v>35000</v>
+        <v>750</v>
       </c>
       <c r="H98" t="inlineStr">
         <is>
@@ -5596,9 +5600,13 @@
         </is>
       </c>
       <c r="J98" t="n">
-        <v>35000</v>
-      </c>
-      <c r="K98" t="inlineStr"/>
+        <v>19500</v>
+      </c>
+      <c r="K98" t="inlineStr">
+        <is>
+          <t>per m</t>
+        </is>
+      </c>
     </row>
     <row r="99">
       <c r="A99" t="inlineStr">
@@ -5618,11 +5626,11 @@
       </c>
       <c r="D99" t="inlineStr">
         <is>
-          <t>Cable 1.5 mm2 T+E/singles in conduit, Indoor lights and fans</t>
+          <t>Cable 2.5 mm2 T+E/singles in conduit, Kitchen sockets, fridge and hood</t>
         </is>
       </c>
       <c r="E99" t="n">
-        <v>36</v>
+        <v>14</v>
       </c>
       <c r="F99" t="inlineStr">
         <is>
@@ -5630,7 +5638,7 @@
         </is>
       </c>
       <c r="G99" t="n">
-        <v>500</v>
+        <v>750</v>
       </c>
       <c r="H99" t="inlineStr">
         <is>
@@ -5643,7 +5651,7 @@
         </is>
       </c>
       <c r="J99" t="n">
-        <v>18000</v>
+        <v>10500</v>
       </c>
       <c r="K99" t="inlineStr">
         <is>
@@ -5669,11 +5677,11 @@
       </c>
       <c r="D100" t="inlineStr">
         <is>
-          <t>Cable 2.5 mm2 T+E/singles in conduit, Sockets: bed, sofa and deck</t>
+          <t>Cable 4.0 mm2 T+E/singles in conduit, Induction hob</t>
         </is>
       </c>
       <c r="E100" t="n">
-        <v>26</v>
+        <v>6</v>
       </c>
       <c r="F100" t="inlineStr">
         <is>
@@ -5681,7 +5689,7 @@
         </is>
       </c>
       <c r="G100" t="n">
-        <v>750</v>
+        <v>1200</v>
       </c>
       <c r="H100" t="inlineStr">
         <is>
@@ -5694,7 +5702,7 @@
         </is>
       </c>
       <c r="J100" t="n">
-        <v>19500</v>
+        <v>7200</v>
       </c>
       <c r="K100" t="inlineStr">
         <is>
@@ -5720,11 +5728,11 @@
       </c>
       <c r="D101" t="inlineStr">
         <is>
-          <t>Cable 2.5 mm2 T+E/singles in conduit, Kitchen sockets, fridge and hood</t>
+          <t>Cable 6.0 mm2 T+E/singles in conduit, Instant shower heater 5.5 kW</t>
         </is>
       </c>
       <c r="E101" t="n">
-        <v>14</v>
+        <v>5</v>
       </c>
       <c r="F101" t="inlineStr">
         <is>
@@ -5732,7 +5740,7 @@
         </is>
       </c>
       <c r="G101" t="n">
-        <v>750</v>
+        <v>1800</v>
       </c>
       <c r="H101" t="inlineStr">
         <is>
@@ -5745,7 +5753,7 @@
         </is>
       </c>
       <c r="J101" t="n">
-        <v>10500</v>
+        <v>9000</v>
       </c>
       <c r="K101" t="inlineStr">
         <is>
@@ -5771,11 +5779,11 @@
       </c>
       <c r="D102" t="inlineStr">
         <is>
-          <t>Cable 4.0 mm2 T+E/singles in conduit, Induction hob</t>
+          <t>Cable 1.5 mm2 T+E/singles in conduit, Outdoor lights: deck, stair and roof</t>
         </is>
       </c>
       <c r="E102" t="n">
-        <v>6</v>
+        <v>21</v>
       </c>
       <c r="F102" t="inlineStr">
         <is>
@@ -5783,7 +5791,7 @@
         </is>
       </c>
       <c r="G102" t="n">
-        <v>1200</v>
+        <v>500</v>
       </c>
       <c r="H102" t="inlineStr">
         <is>
@@ -5796,7 +5804,7 @@
         </is>
       </c>
       <c r="J102" t="n">
-        <v>7200</v>
+        <v>10500</v>
       </c>
       <c r="K102" t="inlineStr">
         <is>
@@ -5822,7 +5830,7 @@
       </c>
       <c r="D103" t="inlineStr">
         <is>
-          <t>Cable 6.0 mm2 T+E/singles in conduit, Instant shower heater 5.5 kW</t>
+          <t>Cable 2.5 mm2 T+E/singles in conduit, AC provision</t>
         </is>
       </c>
       <c r="E103" t="n">
@@ -5834,7 +5842,7 @@
         </is>
       </c>
       <c r="G103" t="n">
-        <v>1800</v>
+        <v>750</v>
       </c>
       <c r="H103" t="inlineStr">
         <is>
@@ -5847,7 +5855,7 @@
         </is>
       </c>
       <c r="J103" t="n">
-        <v>9000</v>
+        <v>3750</v>
       </c>
       <c r="K103" t="inlineStr">
         <is>
@@ -5873,11 +5881,11 @@
       </c>
       <c r="D104" t="inlineStr">
         <is>
-          <t>Cable 1.5 mm2 T+E/singles in conduit, Outdoor lights: deck, stair and roof</t>
+          <t>Cable 16 mm2 tails, inlet to main breaker, through a gland in the back wall</t>
         </is>
       </c>
       <c r="E104" t="n">
-        <v>21</v>
+        <v>2</v>
       </c>
       <c r="F104" t="inlineStr">
         <is>
@@ -5885,7 +5893,7 @@
         </is>
       </c>
       <c r="G104" t="n">
-        <v>500</v>
+        <v>4800</v>
       </c>
       <c r="H104" t="inlineStr">
         <is>
@@ -5898,11 +5906,11 @@
         </is>
       </c>
       <c r="J104" t="n">
-        <v>10500</v>
+        <v>9600</v>
       </c>
       <c r="K104" t="inlineStr">
         <is>
-          <t>per m</t>
+          <t>per m, tails to the 63 A main</t>
         </is>
       </c>
     </row>
@@ -5924,19 +5932,19 @@
       </c>
       <c r="D105" t="inlineStr">
         <is>
-          <t>Cable 2.5 mm2 T+E/singles in conduit, AC provision</t>
+          <t>Matching 63 A plug (IEC 60309 blue), for whatever supply cable</t>
         </is>
       </c>
       <c r="E105" t="n">
-        <v>5</v>
+        <v>1</v>
       </c>
       <c r="F105" t="inlineStr">
         <is>
-          <t>m</t>
+          <t>each</t>
         </is>
       </c>
       <c r="G105" t="n">
-        <v>750</v>
+        <v>20000</v>
       </c>
       <c r="H105" t="inlineStr">
         <is>
@@ -5949,11 +5957,11 @@
         </is>
       </c>
       <c r="J105" t="n">
-        <v>3750</v>
+        <v>20000</v>
       </c>
       <c r="K105" t="inlineStr">
         <is>
-          <t>per m</t>
+          <t>IP67</t>
         </is>
       </c>
     </row>
@@ -5975,11 +5983,11 @@
       </c>
       <c r="D106" t="inlineStr">
         <is>
-          <t>Cable 16 mm2 tails, inlet to main breaker, through a gland in the back wall</t>
+          <t>PVC conduit 20 mm + boxes, in the lining</t>
         </is>
       </c>
       <c r="E106" t="n">
-        <v>2</v>
+        <v>53</v>
       </c>
       <c r="F106" t="inlineStr">
         <is>
@@ -5987,7 +5995,7 @@
         </is>
       </c>
       <c r="G106" t="n">
-        <v>4800</v>
+        <v>600</v>
       </c>
       <c r="H106" t="inlineStr">
         <is>
@@ -6000,11 +6008,11 @@
         </is>
       </c>
       <c r="J106" t="n">
-        <v>9600</v>
+        <v>31800</v>
       </c>
       <c r="K106" t="inlineStr">
         <is>
-          <t>per m, tails to the 63 A main</t>
+          <t>per m</t>
         </is>
       </c>
     </row>
@@ -6026,19 +6034,19 @@
       </c>
       <c r="D107" t="inlineStr">
         <is>
-          <t>Matching 63 A plug (IEC 60309 blue), for whatever supply cable</t>
+          <t>UV-stable conduit 20 mm + IP66 glands, outdoor runs</t>
         </is>
       </c>
       <c r="E107" t="n">
-        <v>1</v>
+        <v>12</v>
       </c>
       <c r="F107" t="inlineStr">
         <is>
-          <t>each</t>
+          <t>m</t>
         </is>
       </c>
       <c r="G107" t="n">
-        <v>20000</v>
+        <v>900</v>
       </c>
       <c r="H107" t="inlineStr">
         <is>
@@ -6051,11 +6059,11 @@
         </is>
       </c>
       <c r="J107" t="n">
-        <v>20000</v>
+        <v>10800</v>
       </c>
       <c r="K107" t="inlineStr">
         <is>
-          <t>IP67</t>
+          <t>per m, UV-stable</t>
         </is>
       </c>
     </row>
@@ -6077,19 +6085,19 @@
       </c>
       <c r="D108" t="inlineStr">
         <is>
-          <t>PVC conduit 20 mm + boxes, in the lining</t>
+          <t>Main breaker 63 A DP (C curve) + DIN kWh check meter</t>
         </is>
       </c>
       <c r="E108" t="n">
-        <v>53</v>
+        <v>1</v>
       </c>
       <c r="F108" t="inlineStr">
         <is>
-          <t>m</t>
+          <t>set</t>
         </is>
       </c>
       <c r="G108" t="n">
-        <v>600</v>
+        <v>45000</v>
       </c>
       <c r="H108" t="inlineStr">
         <is>
@@ -6102,11 +6110,11 @@
         </is>
       </c>
       <c r="J108" t="n">
-        <v>31800</v>
+        <v>45000</v>
       </c>
       <c r="K108" t="inlineStr">
         <is>
-          <t>per m</t>
+          <t>DP breaker + DIN kWh meter</t>
         </is>
       </c>
     </row>
@@ -6128,19 +6136,19 @@
       </c>
       <c r="D109" t="inlineStr">
         <is>
-          <t>UV-stable conduit 20 mm + IP66 glands, outdoor runs</t>
+          <t>Surge protection device type 2</t>
         </is>
       </c>
       <c r="E109" t="n">
-        <v>12</v>
+        <v>1</v>
       </c>
       <c r="F109" t="inlineStr">
         <is>
-          <t>m</t>
+          <t>each</t>
         </is>
       </c>
       <c r="G109" t="n">
-        <v>900</v>
+        <v>60000</v>
       </c>
       <c r="H109" t="inlineStr">
         <is>
@@ -6153,13 +6161,9 @@
         </is>
       </c>
       <c r="J109" t="n">
-        <v>10800</v>
-      </c>
-      <c r="K109" t="inlineStr">
-        <is>
-          <t>per m, UV-stable</t>
-        </is>
-      </c>
+        <v>60000</v>
+      </c>
+      <c r="K109" t="inlineStr"/>
     </row>
     <row r="110">
       <c r="A110" t="inlineStr">
@@ -6179,19 +6183,19 @@
       </c>
       <c r="D110" t="inlineStr">
         <is>
-          <t>Main breaker 63 A DP (C curve) + DIN kWh check meter</t>
+          <t>RCBOs 30 mA type A, 1 module (B6 x2, B16 x3, B20 x1, B25 x1)</t>
         </is>
       </c>
       <c r="E110" t="n">
-        <v>1</v>
+        <v>7</v>
       </c>
       <c r="F110" t="inlineStr">
         <is>
-          <t>set</t>
+          <t>each</t>
         </is>
       </c>
       <c r="G110" t="n">
-        <v>45000</v>
+        <v>22000</v>
       </c>
       <c r="H110" t="inlineStr">
         <is>
@@ -6204,11 +6208,11 @@
         </is>
       </c>
       <c r="J110" t="n">
-        <v>45000</v>
+        <v>154000</v>
       </c>
       <c r="K110" t="inlineStr">
         <is>
-          <t>DP breaker + DIN kWh meter</t>
+          <t>1 module</t>
         </is>
       </c>
     </row>
@@ -6230,7 +6234,7 @@
       </c>
       <c r="D111" t="inlineStr">
         <is>
-          <t>Surge protection device type 2</t>
+          <t>Priority relay, DIN: senses the hob (C4) and sheds C5 and C7</t>
         </is>
       </c>
       <c r="E111" t="n">
@@ -6257,7 +6261,11 @@
       <c r="J111" t="n">
         <v>60000</v>
       </c>
-      <c r="K111" t="inlineStr"/>
+      <c r="K111" t="inlineStr">
+        <is>
+          <t>load shedding, DIN</t>
+        </is>
+      </c>
     </row>
     <row r="112">
       <c r="A112" t="inlineStr">
@@ -6277,11 +6285,11 @@
       </c>
       <c r="D112" t="inlineStr">
         <is>
-          <t>RCBOs 30 mA type A, 1 module (B6 x2, B16 x3, B20 x1, B25 x1)</t>
+          <t>Contactor 2-pole 40 A, DIN: the C5 and C7 lines</t>
         </is>
       </c>
       <c r="E112" t="n">
-        <v>7</v>
+        <v>1</v>
       </c>
       <c r="F112" t="inlineStr">
         <is>
@@ -6289,7 +6297,7 @@
         </is>
       </c>
       <c r="G112" t="n">
-        <v>22000</v>
+        <v>25000</v>
       </c>
       <c r="H112" t="inlineStr">
         <is>
@@ -6302,11 +6310,11 @@
         </is>
       </c>
       <c r="J112" t="n">
-        <v>154000</v>
+        <v>25000</v>
       </c>
       <c r="K112" t="inlineStr">
         <is>
-          <t>1 module</t>
+          <t>DIN</t>
         </is>
       </c>
     </row>
@@ -6318,17 +6326,17 @@
       </c>
       <c r="B113" t="inlineStr">
         <is>
-          <t>electrical</t>
+          <t>safety</t>
         </is>
       </c>
       <c r="C113" t="inlineStr">
         <is>
-          <t>electrical</t>
+          <t>furnishing</t>
         </is>
       </c>
       <c r="D113" t="inlineStr">
         <is>
-          <t>Priority relay, DIN: senses the hob (C4) and sheds C5 and C7</t>
+          <t>Fire extinguisher 2 kg ABC + fire blanket</t>
         </is>
       </c>
       <c r="E113" t="n">
@@ -6336,11 +6344,11 @@
       </c>
       <c r="F113" t="inlineStr">
         <is>
-          <t>each</t>
+          <t>set</t>
         </is>
       </c>
       <c r="G113" t="n">
-        <v>60000</v>
+        <v>55000</v>
       </c>
       <c r="H113" t="inlineStr">
         <is>
@@ -6353,45 +6361,41 @@
         </is>
       </c>
       <c r="J113" t="n">
-        <v>60000</v>
-      </c>
-      <c r="K113" t="inlineStr">
-        <is>
-          <t>load shedding, DIN</t>
-        </is>
-      </c>
+        <v>55000</v>
+      </c>
+      <c r="K113" t="inlineStr"/>
     </row>
     <row r="114">
       <c r="A114" t="inlineStr">
         <is>
-          <t>K8</t>
+          <t>K9</t>
         </is>
       </c>
       <c r="B114" t="inlineStr">
         <is>
-          <t>electrical</t>
+          <t>plumbing</t>
         </is>
       </c>
       <c r="C114" t="inlineStr">
         <is>
-          <t>electrical</t>
+          <t>plumbing</t>
         </is>
       </c>
       <c r="D114" t="inlineStr">
         <is>
-          <t>Contactor 2-pole 40 A, DIN: the C5 and C7 lines</t>
+          <t>PPR PN20 pipe DN20</t>
         </is>
       </c>
       <c r="E114" t="n">
-        <v>1</v>
+        <v>8.199999999999999</v>
       </c>
       <c r="F114" t="inlineStr">
         <is>
-          <t>each</t>
+          <t>m</t>
         </is>
       </c>
       <c r="G114" t="n">
-        <v>25000</v>
+        <v>2000</v>
       </c>
       <c r="H114" t="inlineStr">
         <is>
@@ -6404,45 +6408,45 @@
         </is>
       </c>
       <c r="J114" t="n">
-        <v>25000</v>
+        <v>16400</v>
       </c>
       <c r="K114" t="inlineStr">
         <is>
-          <t>DIN</t>
+          <t>per m</t>
         </is>
       </c>
     </row>
     <row r="115">
       <c r="A115" t="inlineStr">
         <is>
-          <t>K8</t>
+          <t>K9</t>
         </is>
       </c>
       <c r="B115" t="inlineStr">
         <is>
-          <t>safety</t>
+          <t>plumbing</t>
         </is>
       </c>
       <c r="C115" t="inlineStr">
         <is>
-          <t>furnishing</t>
+          <t>plumbing</t>
         </is>
       </c>
       <c r="D115" t="inlineStr">
         <is>
-          <t>Fire extinguisher 2 kg ABC + fire blanket</t>
+          <t>PPR PN20 pipe DN25</t>
         </is>
       </c>
       <c r="E115" t="n">
-        <v>1</v>
+        <v>4.4</v>
       </c>
       <c r="F115" t="inlineStr">
         <is>
-          <t>set</t>
+          <t>m</t>
         </is>
       </c>
       <c r="G115" t="n">
-        <v>55000</v>
+        <v>2800</v>
       </c>
       <c r="H115" t="inlineStr">
         <is>
@@ -6455,9 +6459,13 @@
         </is>
       </c>
       <c r="J115" t="n">
-        <v>55000</v>
-      </c>
-      <c r="K115" t="inlineStr"/>
+        <v>12320</v>
+      </c>
+      <c r="K115" t="inlineStr">
+        <is>
+          <t>per m</t>
+        </is>
+      </c>
     </row>
     <row r="116">
       <c r="A116" t="inlineStr">
@@ -6477,11 +6485,11 @@
       </c>
       <c r="D116" t="inlineStr">
         <is>
-          <t>PPR PN20 pipe DN20</t>
+          <t>uPVC soil pipe DN110</t>
         </is>
       </c>
       <c r="E116" t="n">
-        <v>9.300000000000001</v>
+        <v>3</v>
       </c>
       <c r="F116" t="inlineStr">
         <is>
@@ -6489,7 +6497,7 @@
         </is>
       </c>
       <c r="G116" t="n">
-        <v>2000</v>
+        <v>7000</v>
       </c>
       <c r="H116" t="inlineStr">
         <is>
@@ -6502,7 +6510,7 @@
         </is>
       </c>
       <c r="J116" t="n">
-        <v>18600</v>
+        <v>21000</v>
       </c>
       <c r="K116" t="inlineStr">
         <is>
@@ -6528,11 +6536,11 @@
       </c>
       <c r="D117" t="inlineStr">
         <is>
-          <t>PPR PN20 pipe DN25</t>
+          <t>uPVC vent pipe DN75</t>
         </is>
       </c>
       <c r="E117" t="n">
-        <v>4.4</v>
+        <v>8.800000000000001</v>
       </c>
       <c r="F117" t="inlineStr">
         <is>
@@ -6540,7 +6548,7 @@
         </is>
       </c>
       <c r="G117" t="n">
-        <v>2800</v>
+        <v>4500</v>
       </c>
       <c r="H117" t="inlineStr">
         <is>
@@ -6553,7 +6561,7 @@
         </is>
       </c>
       <c r="J117" t="n">
-        <v>12320</v>
+        <v>39600</v>
       </c>
       <c r="K117" t="inlineStr">
         <is>
@@ -6579,11 +6587,11 @@
       </c>
       <c r="D118" t="inlineStr">
         <is>
-          <t>uPVC soil pipe DN110</t>
+          <t>uPVC waste pipe DN50</t>
         </is>
       </c>
       <c r="E118" t="n">
-        <v>3</v>
+        <v>6.3</v>
       </c>
       <c r="F118" t="inlineStr">
         <is>
@@ -6591,7 +6599,7 @@
         </is>
       </c>
       <c r="G118" t="n">
-        <v>7000</v>
+        <v>3000</v>
       </c>
       <c r="H118" t="inlineStr">
         <is>
@@ -6604,7 +6612,7 @@
         </is>
       </c>
       <c r="J118" t="n">
-        <v>21000</v>
+        <v>18900</v>
       </c>
       <c r="K118" t="inlineStr">
         <is>
@@ -6630,19 +6638,19 @@
       </c>
       <c r="D119" t="inlineStr">
         <is>
-          <t>uPVC vent pipe DN75</t>
+          <t>Pipe fittings and clips (allowance)</t>
         </is>
       </c>
       <c r="E119" t="n">
-        <v>8.800000000000001</v>
+        <v>1</v>
       </c>
       <c r="F119" t="inlineStr">
         <is>
-          <t>m</t>
+          <t>set</t>
         </is>
       </c>
       <c r="G119" t="n">
-        <v>4500</v>
+        <v>120000</v>
       </c>
       <c r="H119" t="inlineStr">
         <is>
@@ -6655,13 +6663,9 @@
         </is>
       </c>
       <c r="J119" t="n">
-        <v>39600</v>
-      </c>
-      <c r="K119" t="inlineStr">
-        <is>
-          <t>per m</t>
-        </is>
-      </c>
+        <v>120000</v>
+      </c>
+      <c r="K119" t="inlineStr"/>
     </row>
     <row r="120">
       <c r="A120" t="inlineStr">
@@ -6681,19 +6685,19 @@
       </c>
       <c r="D120" t="inlineStr">
         <is>
-          <t>uPVC waste pipe DN40</t>
+          <t>Shower slide rail with hand-shower holder</t>
         </is>
       </c>
       <c r="E120" t="n">
-        <v>3.4</v>
+        <v>1</v>
       </c>
       <c r="F120" t="inlineStr">
         <is>
-          <t>m</t>
+          <t>set</t>
         </is>
       </c>
       <c r="G120" t="n">
-        <v>2500</v>
+        <v>30000</v>
       </c>
       <c r="H120" t="inlineStr">
         <is>
@@ -6706,13 +6710,9 @@
         </is>
       </c>
       <c r="J120" t="n">
-        <v>8500</v>
-      </c>
-      <c r="K120" t="inlineStr">
-        <is>
-          <t>per m</t>
-        </is>
-      </c>
+        <v>30000</v>
+      </c>
+      <c r="K120" t="inlineStr"/>
     </row>
     <row r="121">
       <c r="A121" t="inlineStr">
@@ -6732,19 +6732,19 @@
       </c>
       <c r="D121" t="inlineStr">
         <is>
-          <t>uPVC waste pipe DN50</t>
+          <t>Instant electric shower heater 5.5 kW, IPX4, digital thermostat, hand shower and hose</t>
         </is>
       </c>
       <c r="E121" t="n">
-        <v>6.3</v>
+        <v>1</v>
       </c>
       <c r="F121" t="inlineStr">
         <is>
-          <t>m</t>
+          <t>each</t>
         </is>
       </c>
       <c r="G121" t="n">
-        <v>3000</v>
+        <v>90000</v>
       </c>
       <c r="H121" t="inlineStr">
         <is>
@@ -6757,11 +6757,11 @@
         </is>
       </c>
       <c r="J121" t="n">
-        <v>18900</v>
+        <v>90000</v>
       </c>
       <c r="K121" t="inlineStr">
         <is>
-          <t>per m</t>
+          <t>5.5 kW instant shower heater not priced yet (D-053)</t>
         </is>
       </c>
     </row>
@@ -6783,19 +6783,19 @@
       </c>
       <c r="D122" t="inlineStr">
         <is>
-          <t>Pipe fittings and clips (allowance)</t>
+          <t>Angle valves with filters</t>
         </is>
       </c>
       <c r="E122" t="n">
-        <v>1</v>
+        <v>4</v>
       </c>
       <c r="F122" t="inlineStr">
         <is>
-          <t>set</t>
+          <t>each</t>
         </is>
       </c>
       <c r="G122" t="n">
-        <v>120000</v>
+        <v>6000</v>
       </c>
       <c r="H122" t="inlineStr">
         <is>
@@ -6808,7 +6808,7 @@
         </is>
       </c>
       <c r="J122" t="n">
-        <v>120000</v>
+        <v>24000</v>
       </c>
       <c r="K122" t="inlineStr"/>
     </row>
@@ -6830,7 +6830,7 @@
       </c>
       <c r="D123" t="inlineStr">
         <is>
-          <t>Shower slide rail with hand-shower holder</t>
+          <t>Air admittance valve 110 mm (spare) + rodding eyes</t>
         </is>
       </c>
       <c r="E123" t="n">
@@ -6877,7 +6877,7 @@
       </c>
       <c r="D124" t="inlineStr">
         <is>
-          <t>Instant electric shower heater 5.5 kW, IPX4, digital thermostat, hand shower and hose</t>
+          <t>Stop valve + Y-filter + check water meter</t>
         </is>
       </c>
       <c r="E124" t="n">
@@ -6885,11 +6885,11 @@
       </c>
       <c r="F124" t="inlineStr">
         <is>
-          <t>each</t>
+          <t>set</t>
         </is>
       </c>
       <c r="G124" t="n">
-        <v>90000</v>
+        <v>45000</v>
       </c>
       <c r="H124" t="inlineStr">
         <is>
@@ -6902,37 +6902,33 @@
         </is>
       </c>
       <c r="J124" t="n">
-        <v>90000</v>
-      </c>
-      <c r="K124" t="inlineStr">
-        <is>
-          <t>5.5 kW instant shower heater not priced yet (D-053)</t>
-        </is>
-      </c>
+        <v>45000</v>
+      </c>
+      <c r="K124" t="inlineStr"/>
     </row>
     <row r="125">
       <c r="A125" t="inlineStr">
         <is>
-          <t>K9</t>
+          <t>K10</t>
         </is>
       </c>
       <c r="B125" t="inlineStr">
         <is>
-          <t>plumbing</t>
+          <t>steel</t>
         </is>
       </c>
       <c r="C125" t="inlineStr">
         <is>
-          <t>plumbing</t>
+          <t>welding</t>
         </is>
       </c>
       <c r="D125" t="inlineStr">
         <is>
-          <t>Angle valves with filters</t>
+          <t>W1 infill: 2 mm steel welded into the old door frame (0-1,150), foamed with the walls</t>
         </is>
       </c>
       <c r="E125" t="n">
-        <v>4</v>
+        <v>1</v>
       </c>
       <c r="F125" t="inlineStr">
         <is>
@@ -6940,7 +6936,7 @@
         </is>
       </c>
       <c r="G125" t="n">
-        <v>6000</v>
+        <v>180000</v>
       </c>
       <c r="H125" t="inlineStr">
         <is>
@@ -6953,29 +6949,33 @@
         </is>
       </c>
       <c r="J125" t="n">
-        <v>24000</v>
-      </c>
-      <c r="K125" t="inlineStr"/>
+        <v>180000</v>
+      </c>
+      <c r="K125" t="inlineStr">
+        <is>
+          <t>incl. welding</t>
+        </is>
+      </c>
     </row>
     <row r="126">
       <c r="A126" t="inlineStr">
         <is>
-          <t>K9</t>
+          <t>K10</t>
         </is>
       </c>
       <c r="B126" t="inlineStr">
         <is>
-          <t>plumbing</t>
+          <t>glazing</t>
         </is>
       </c>
       <c r="C126" t="inlineStr">
         <is>
-          <t>plumbing</t>
+          <t>glazier</t>
         </is>
       </c>
       <c r="D126" t="inlineStr">
         <is>
-          <t>Air admittance valve 110 mm (spare) + rodding eyes</t>
+          <t>W1 obscure louvre window 520 x 890 + insect mesh (bathroom lobby)</t>
         </is>
       </c>
       <c r="E126" t="n">
@@ -6983,11 +6983,11 @@
       </c>
       <c r="F126" t="inlineStr">
         <is>
-          <t>set</t>
+          <t>each</t>
         </is>
       </c>
       <c r="G126" t="n">
-        <v>30000</v>
+        <v>120000</v>
       </c>
       <c r="H126" t="inlineStr">
         <is>
@@ -7000,29 +7000,29 @@
         </is>
       </c>
       <c r="J126" t="n">
-        <v>30000</v>
+        <v>120000</v>
       </c>
       <c r="K126" t="inlineStr"/>
     </row>
     <row r="127">
       <c r="A127" t="inlineStr">
         <is>
-          <t>K9</t>
+          <t>K10</t>
         </is>
       </c>
       <c r="B127" t="inlineStr">
         <is>
-          <t>plumbing</t>
+          <t>steel</t>
         </is>
       </c>
       <c r="C127" t="inlineStr">
         <is>
-          <t>plumbing</t>
+          <t>welding</t>
         </is>
       </c>
       <c r="D127" t="inlineStr">
         <is>
-          <t>Stop valve + Y-filter + check water meter</t>
+          <t>Seal and lock the end-B cargo doors (weld tabs, sealant)</t>
         </is>
       </c>
       <c r="E127" t="n">
@@ -7030,11 +7030,11 @@
       </c>
       <c r="F127" t="inlineStr">
         <is>
-          <t>set</t>
+          <t>each</t>
         </is>
       </c>
       <c r="G127" t="n">
-        <v>45000</v>
+        <v>60000</v>
       </c>
       <c r="H127" t="inlineStr">
         <is>
@@ -7047,7 +7047,7 @@
         </is>
       </c>
       <c r="J127" t="n">
-        <v>45000</v>
+        <v>60000</v>
       </c>
       <c r="K127" t="inlineStr"/>
     </row>
@@ -7064,16 +7064,16 @@
       </c>
       <c r="C128" t="inlineStr">
         <is>
-          <t>welding</t>
+          <t>masonry</t>
         </is>
       </c>
       <c r="D128" t="inlineStr">
         <is>
-          <t>W1 infill: 2 mm steel welded into the old door frame (0-1,150), foamed with the walls</t>
+          <t>Concrete block stands 40 x 60 cm under the four corner castings, levelled (D-029)</t>
         </is>
       </c>
       <c r="E128" t="n">
-        <v>1</v>
+        <v>4</v>
       </c>
       <c r="F128" t="inlineStr">
         <is>
@@ -7081,7 +7081,7 @@
         </is>
       </c>
       <c r="G128" t="n">
-        <v>180000</v>
+        <v>25000</v>
       </c>
       <c r="H128" t="inlineStr">
         <is>
@@ -7094,13 +7094,9 @@
         </is>
       </c>
       <c r="J128" t="n">
-        <v>180000</v>
-      </c>
-      <c r="K128" t="inlineStr">
-        <is>
-          <t>incl. welding</t>
-        </is>
-      </c>
+        <v>100000</v>
+      </c>
+      <c r="K128" t="inlineStr"/>
     </row>
     <row r="129">
       <c r="A129" t="inlineStr">
@@ -7110,17 +7106,17 @@
       </c>
       <c r="B129" t="inlineStr">
         <is>
-          <t>glazing</t>
+          <t>steel</t>
         </is>
       </c>
       <c r="C129" t="inlineStr">
         <is>
-          <t>glazier</t>
+          <t>welding</t>
         </is>
       </c>
       <c r="D129" t="inlineStr">
         <is>
-          <t>W1 obscure louvre window 520 x 890 + insect mesh (wash lobby)</t>
+          <t>Steel hanging rail for the wall units</t>
         </is>
       </c>
       <c r="E129" t="n">
@@ -7128,11 +7124,11 @@
       </c>
       <c r="F129" t="inlineStr">
         <is>
-          <t>each</t>
+          <t>set</t>
         </is>
       </c>
       <c r="G129" t="n">
-        <v>120000</v>
+        <v>40000</v>
       </c>
       <c r="H129" t="inlineStr">
         <is>
@@ -7145,7 +7141,7 @@
         </is>
       </c>
       <c r="J129" t="n">
-        <v>120000</v>
+        <v>40000</v>
       </c>
       <c r="K129" t="inlineStr"/>
     </row>
@@ -7157,17 +7153,17 @@
       </c>
       <c r="B130" t="inlineStr">
         <is>
-          <t>steel</t>
+          <t>hardware</t>
         </is>
       </c>
       <c r="C130" t="inlineStr">
         <is>
-          <t>welding</t>
+          <t>glazier</t>
         </is>
       </c>
       <c r="D130" t="inlineStr">
         <is>
-          <t>Seal and lock the end-B cargo doors (weld tabs, sealant)</t>
+          <t>Keyed lock + secondary bolt for the slider</t>
         </is>
       </c>
       <c r="E130" t="n">
@@ -7175,11 +7171,11 @@
       </c>
       <c r="F130" t="inlineStr">
         <is>
-          <t>each</t>
+          <t>set</t>
         </is>
       </c>
       <c r="G130" t="n">
-        <v>60000</v>
+        <v>45000</v>
       </c>
       <c r="H130" t="inlineStr">
         <is>
@@ -7192,7 +7188,7 @@
         </is>
       </c>
       <c r="J130" t="n">
-        <v>60000</v>
+        <v>45000</v>
       </c>
       <c r="K130" t="inlineStr"/>
     </row>
@@ -7204,21 +7200,21 @@
       </c>
       <c r="B131" t="inlineStr">
         <is>
-          <t>steel</t>
+          <t>glazing</t>
         </is>
       </c>
       <c r="C131" t="inlineStr">
         <is>
-          <t>masonry</t>
+          <t>glazier</t>
         </is>
       </c>
       <c r="D131" t="inlineStr">
         <is>
-          <t>Concrete block stands 40 x 60 cm under the four corner castings, levelled (D-029)</t>
+          <t>Louvred trickle-vent strip with mesh (10,000 mm2)</t>
         </is>
       </c>
       <c r="E131" t="n">
-        <v>4</v>
+        <v>1</v>
       </c>
       <c r="F131" t="inlineStr">
         <is>
@@ -7226,7 +7222,7 @@
         </is>
       </c>
       <c r="G131" t="n">
-        <v>25000</v>
+        <v>30000</v>
       </c>
       <c r="H131" t="inlineStr">
         <is>
@@ -7239,7 +7235,7 @@
         </is>
       </c>
       <c r="J131" t="n">
-        <v>100000</v>
+        <v>30000</v>
       </c>
       <c r="K131" t="inlineStr"/>
     </row>
@@ -7261,7 +7257,7 @@
       </c>
       <c r="D132" t="inlineStr">
         <is>
-          <t>Steel hanging rail for the wall units</t>
+          <t>AC wall sleeve 75 mm (provision, back wall, one hole)</t>
         </is>
       </c>
       <c r="E132" t="n">
@@ -7269,11 +7265,11 @@
       </c>
       <c r="F132" t="inlineStr">
         <is>
-          <t>set</t>
+          <t>each</t>
         </is>
       </c>
       <c r="G132" t="n">
-        <v>40000</v>
+        <v>15000</v>
       </c>
       <c r="H132" t="inlineStr">
         <is>
@@ -7286,29 +7282,29 @@
         </is>
       </c>
       <c r="J132" t="n">
-        <v>40000</v>
+        <v>15000</v>
       </c>
       <c r="K132" t="inlineStr"/>
     </row>
     <row r="133">
       <c r="A133" t="inlineStr">
         <is>
-          <t>K10</t>
+          <t>K11</t>
         </is>
       </c>
       <c r="B133" t="inlineStr">
         <is>
-          <t>hardware</t>
+          <t>roofing</t>
         </is>
       </c>
       <c r="C133" t="inlineStr">
         <is>
-          <t>glazier</t>
+          <t>welding</t>
         </is>
       </c>
       <c r="D133" t="inlineStr">
         <is>
-          <t>Keyed lock + secondary bolt for the slider</t>
+          <t>Gutter + downpipe to the rainwater tank (deck canopy)</t>
         </is>
       </c>
       <c r="E133" t="n">
@@ -7320,7 +7316,7 @@
         </is>
       </c>
       <c r="G133" t="n">
-        <v>45000</v>
+        <v>90000</v>
       </c>
       <c r="H133" t="inlineStr">
         <is>
@@ -7333,29 +7329,29 @@
         </is>
       </c>
       <c r="J133" t="n">
-        <v>45000</v>
+        <v>90000</v>
       </c>
       <c r="K133" t="inlineStr"/>
     </row>
     <row r="134">
       <c r="A134" t="inlineStr">
         <is>
-          <t>K10</t>
+          <t>K11</t>
         </is>
       </c>
       <c r="B134" t="inlineStr">
         <is>
-          <t>glazing</t>
+          <t>electrical</t>
         </is>
       </c>
       <c r="C134" t="inlineStr">
         <is>
-          <t>glazier</t>
+          <t>electrical</t>
         </is>
       </c>
       <c r="D134" t="inlineStr">
         <is>
-          <t>Louvred trickle-vent strip with mesh (10,000 mm2)</t>
+          <t>Bonding: 16 mm2 green-yellow from the frame to the earth bar</t>
         </is>
       </c>
       <c r="E134" t="n">
@@ -7363,11 +7359,11 @@
       </c>
       <c r="F134" t="inlineStr">
         <is>
-          <t>each</t>
+          <t>set</t>
         </is>
       </c>
       <c r="G134" t="n">
-        <v>30000</v>
+        <v>25000</v>
       </c>
       <c r="H134" t="inlineStr">
         <is>
@@ -7380,33 +7376,33 @@
         </is>
       </c>
       <c r="J134" t="n">
-        <v>30000</v>
+        <v>25000</v>
       </c>
       <c r="K134" t="inlineStr"/>
     </row>
     <row r="135">
       <c r="A135" t="inlineStr">
         <is>
-          <t>K10</t>
+          <t>K1</t>
         </is>
       </c>
       <c r="B135" t="inlineStr">
         <is>
-          <t>steel</t>
+          <t>timber</t>
         </is>
       </c>
       <c r="C135" t="inlineStr">
         <is>
-          <t>welding</t>
+          <t>carpentry</t>
         </is>
       </c>
       <c r="D135" t="inlineStr">
         <is>
-          <t>AC wall sleeve 75 mm (provision, back wall, one hole)</t>
+          <t>Battens 38 x 50 treated, 2.4 m</t>
         </is>
       </c>
       <c r="E135" t="n">
-        <v>1</v>
+        <v>35.2</v>
       </c>
       <c r="F135" t="inlineStr">
         <is>
@@ -7414,7 +7410,7 @@
         </is>
       </c>
       <c r="G135" t="n">
-        <v>15000</v>
+        <v>2500</v>
       </c>
       <c r="H135" t="inlineStr">
         <is>
@@ -7427,41 +7423,45 @@
         </is>
       </c>
       <c r="J135" t="n">
-        <v>15000</v>
-      </c>
-      <c r="K135" t="inlineStr"/>
+        <v>88000</v>
+      </c>
+      <c r="K135" t="inlineStr">
+        <is>
+          <t>38 x 50 treated, 2.4 m</t>
+        </is>
+      </c>
     </row>
     <row r="136">
       <c r="A136" t="inlineStr">
         <is>
-          <t>K11</t>
+          <t>K2</t>
         </is>
       </c>
       <c r="B136" t="inlineStr">
         <is>
-          <t>roofing</t>
+          <t>timber</t>
         </is>
       </c>
       <c r="C136" t="inlineStr">
         <is>
-          <t>welding</t>
+          <t>carpentry</t>
         </is>
       </c>
       <c r="D136" t="inlineStr">
         <is>
-          <t>Gutter + downpipe to the rainwater tank (deck canopy)</t>
+          <t>Studs 40 x 40 treated, 2.4 m</t>
         </is>
       </c>
       <c r="E136" t="n">
-        <v>1</v>
+        <v>5.5</v>
       </c>
       <c r="F136" t="inlineStr">
         <is>
-          <t>set</t>
+          <t>each</t>
         </is>
       </c>
       <c r="G136" t="n">
-        <v>90000</v>
+        <v>3000</v>
       </c>
       <c r="H136" t="inlineStr">
         <is>
@@ -7474,29 +7474,29 @@
         </is>
       </c>
       <c r="J136" t="n">
-        <v>90000</v>
-      </c>
-      <c r="K136" t="inlineStr"/>
+        <v>16500</v>
+      </c>
+      <c r="K136" t="inlineStr">
+        <is>
+          <t>40 x 40, 2.4 m</t>
+        </is>
+      </c>
     </row>
     <row r="137">
       <c r="A137" t="inlineStr">
         <is>
-          <t>K11</t>
+          <t>labour</t>
         </is>
       </c>
       <c r="B137" t="inlineStr">
         <is>
-          <t>electrical</t>
-        </is>
-      </c>
-      <c r="C137" t="inlineStr">
-        <is>
-          <t>electrical</t>
-        </is>
-      </c>
+          <t>labour</t>
+        </is>
+      </c>
+      <c r="C137" t="inlineStr"/>
       <c r="D137" t="inlineStr">
         <is>
-          <t>Bonding: 16 mm2 green-yellow from the frame to the earth bar</t>
+          <t>Carpentry workshop: cutting, edging, drilling, labelling (per unit kit)</t>
         </is>
       </c>
       <c r="E137" t="n">
@@ -7504,11 +7504,11 @@
       </c>
       <c r="F137" t="inlineStr">
         <is>
-          <t>set</t>
+          <t>lot</t>
         </is>
       </c>
       <c r="G137" t="n">
-        <v>25000</v>
+        <v>450000</v>
       </c>
       <c r="H137" t="inlineStr">
         <is>
@@ -7521,41 +7521,37 @@
         </is>
       </c>
       <c r="J137" t="n">
-        <v>25000</v>
+        <v>450000</v>
       </c>
       <c r="K137" t="inlineStr"/>
     </row>
     <row r="138">
       <c r="A138" t="inlineStr">
         <is>
-          <t>K1</t>
+          <t>labour</t>
         </is>
       </c>
       <c r="B138" t="inlineStr">
         <is>
-          <t>timber</t>
-        </is>
-      </c>
-      <c r="C138" t="inlineStr">
-        <is>
-          <t>carpentry</t>
-        </is>
-      </c>
+          <t>labour</t>
+        </is>
+      </c>
+      <c r="C138" t="inlineStr"/>
       <c r="D138" t="inlineStr">
         <is>
-          <t>Battens 38 x 50 treated, 2.4 m</t>
+          <t>Site carpentry and assembly: 2 people x 8 days</t>
         </is>
       </c>
       <c r="E138" t="n">
-        <v>35.2</v>
+        <v>1</v>
       </c>
       <c r="F138" t="inlineStr">
         <is>
-          <t>each</t>
+          <t>lot</t>
         </is>
       </c>
       <c r="G138" t="n">
-        <v>2500</v>
+        <v>320000</v>
       </c>
       <c r="H138" t="inlineStr">
         <is>
@@ -7568,45 +7564,37 @@
         </is>
       </c>
       <c r="J138" t="n">
-        <v>88000</v>
-      </c>
-      <c r="K138" t="inlineStr">
-        <is>
-          <t>38 x 50 treated, 2.4 m</t>
-        </is>
-      </c>
+        <v>320000</v>
+      </c>
+      <c r="K138" t="inlineStr"/>
     </row>
     <row r="139">
       <c r="A139" t="inlineStr">
         <is>
-          <t>K2</t>
+          <t>labour</t>
         </is>
       </c>
       <c r="B139" t="inlineStr">
         <is>
-          <t>timber</t>
-        </is>
-      </c>
-      <c r="C139" t="inlineStr">
-        <is>
-          <t>carpentry</t>
-        </is>
-      </c>
+          <t>labour</t>
+        </is>
+      </c>
+      <c r="C139" t="inlineStr"/>
       <c r="D139" t="inlineStr">
         <is>
-          <t>Studs 40 x 40 treated, 2.4 m</t>
+          <t>Electrician (RURA class A), install + certificate</t>
         </is>
       </c>
       <c r="E139" t="n">
-        <v>5.5</v>
+        <v>1</v>
       </c>
       <c r="F139" t="inlineStr">
         <is>
-          <t>each</t>
+          <t>lot</t>
         </is>
       </c>
       <c r="G139" t="n">
-        <v>3000</v>
+        <v>250000</v>
       </c>
       <c r="H139" t="inlineStr">
         <is>
@@ -7619,13 +7607,9 @@
         </is>
       </c>
       <c r="J139" t="n">
-        <v>16500</v>
-      </c>
-      <c r="K139" t="inlineStr">
-        <is>
-          <t>40 x 40, 2.4 m</t>
-        </is>
-      </c>
+        <v>250000</v>
+      </c>
+      <c r="K139" t="inlineStr"/>
     </row>
     <row r="140">
       <c r="A140" t="inlineStr">
@@ -7641,7 +7625,7 @@
       <c r="C140" t="inlineStr"/>
       <c r="D140" t="inlineStr">
         <is>
-          <t>Carpentry workshop: cutting, edging, drilling, labelling (per unit kit)</t>
+          <t>Plumber, install + tests</t>
         </is>
       </c>
       <c r="E140" t="n">
@@ -7653,7 +7637,7 @@
         </is>
       </c>
       <c r="G140" t="n">
-        <v>450000</v>
+        <v>200000</v>
       </c>
       <c r="H140" t="inlineStr">
         <is>
@@ -7666,7 +7650,7 @@
         </is>
       </c>
       <c r="J140" t="n">
-        <v>450000</v>
+        <v>200000</v>
       </c>
       <c r="K140" t="inlineStr"/>
     </row>
@@ -7684,7 +7668,7 @@
       <c r="C141" t="inlineStr"/>
       <c r="D141" t="inlineStr">
         <is>
-          <t>Site carpentry and assembly: 2 people x 8 days</t>
+          <t>Tiler: wet walls and floor</t>
         </is>
       </c>
       <c r="E141" t="n">
@@ -7696,7 +7680,7 @@
         </is>
       </c>
       <c r="G141" t="n">
-        <v>320000</v>
+        <v>150000</v>
       </c>
       <c r="H141" t="inlineStr">
         <is>
@@ -7709,7 +7693,7 @@
         </is>
       </c>
       <c r="J141" t="n">
-        <v>320000</v>
+        <v>150000</v>
       </c>
       <c r="K141" t="inlineStr"/>
     </row>
@@ -7727,7 +7711,7 @@
       <c r="C142" t="inlineStr"/>
       <c r="D142" t="inlineStr">
         <is>
-          <t>Electrician (RURA class A), install + certificate</t>
+          <t>Welder: W1, roof frame, deck canopy, stair (per unit)</t>
         </is>
       </c>
       <c r="E142" t="n">
@@ -7739,7 +7723,7 @@
         </is>
       </c>
       <c r="G142" t="n">
-        <v>250000</v>
+        <v>600000</v>
       </c>
       <c r="H142" t="inlineStr">
         <is>
@@ -7752,7 +7736,7 @@
         </is>
       </c>
       <c r="J142" t="n">
-        <v>250000</v>
+        <v>600000</v>
       </c>
       <c r="K142" t="inlineStr"/>
     </row>
@@ -7770,7 +7754,7 @@
       <c r="C143" t="inlineStr"/>
       <c r="D143" t="inlineStr">
         <is>
-          <t>Plumber, install + tests</t>
+          <t>Transport Kigali to site (share of 2 truck trips)</t>
         </is>
       </c>
       <c r="E143" t="n">
@@ -7782,7 +7766,7 @@
         </is>
       </c>
       <c r="G143" t="n">
-        <v>200000</v>
+        <v>120000</v>
       </c>
       <c r="H143" t="inlineStr">
         <is>
@@ -7795,138 +7779,9 @@
         </is>
       </c>
       <c r="J143" t="n">
-        <v>200000</v>
+        <v>120000</v>
       </c>
       <c r="K143" t="inlineStr"/>
-    </row>
-    <row r="144">
-      <c r="A144" t="inlineStr">
-        <is>
-          <t>labour</t>
-        </is>
-      </c>
-      <c r="B144" t="inlineStr">
-        <is>
-          <t>labour</t>
-        </is>
-      </c>
-      <c r="C144" t="inlineStr"/>
-      <c r="D144" t="inlineStr">
-        <is>
-          <t>Tiler: wet walls and floor</t>
-        </is>
-      </c>
-      <c r="E144" t="n">
-        <v>1</v>
-      </c>
-      <c r="F144" t="inlineStr">
-        <is>
-          <t>lot</t>
-        </is>
-      </c>
-      <c r="G144" t="n">
-        <v>150000</v>
-      </c>
-      <c r="H144" t="inlineStr">
-        <is>
-          <t>A</t>
-        </is>
-      </c>
-      <c r="I144" t="inlineStr">
-        <is>
-          <t>AS-21</t>
-        </is>
-      </c>
-      <c r="J144" t="n">
-        <v>150000</v>
-      </c>
-      <c r="K144" t="inlineStr"/>
-    </row>
-    <row r="145">
-      <c r="A145" t="inlineStr">
-        <is>
-          <t>labour</t>
-        </is>
-      </c>
-      <c r="B145" t="inlineStr">
-        <is>
-          <t>labour</t>
-        </is>
-      </c>
-      <c r="C145" t="inlineStr"/>
-      <c r="D145" t="inlineStr">
-        <is>
-          <t>Welder: W1, roof frame, deck canopy, stair (per unit)</t>
-        </is>
-      </c>
-      <c r="E145" t="n">
-        <v>1</v>
-      </c>
-      <c r="F145" t="inlineStr">
-        <is>
-          <t>lot</t>
-        </is>
-      </c>
-      <c r="G145" t="n">
-        <v>600000</v>
-      </c>
-      <c r="H145" t="inlineStr">
-        <is>
-          <t>A</t>
-        </is>
-      </c>
-      <c r="I145" t="inlineStr">
-        <is>
-          <t>AS-21</t>
-        </is>
-      </c>
-      <c r="J145" t="n">
-        <v>600000</v>
-      </c>
-      <c r="K145" t="inlineStr"/>
-    </row>
-    <row r="146">
-      <c r="A146" t="inlineStr">
-        <is>
-          <t>labour</t>
-        </is>
-      </c>
-      <c r="B146" t="inlineStr">
-        <is>
-          <t>labour</t>
-        </is>
-      </c>
-      <c r="C146" t="inlineStr"/>
-      <c r="D146" t="inlineStr">
-        <is>
-          <t>Transport Kigali to site (share of 2 truck trips)</t>
-        </is>
-      </c>
-      <c r="E146" t="n">
-        <v>1</v>
-      </c>
-      <c r="F146" t="inlineStr">
-        <is>
-          <t>lot</t>
-        </is>
-      </c>
-      <c r="G146" t="n">
-        <v>120000</v>
-      </c>
-      <c r="H146" t="inlineStr">
-        <is>
-          <t>A</t>
-        </is>
-      </c>
-      <c r="I146" t="inlineStr">
-        <is>
-          <t>AS-21</t>
-        </is>
-      </c>
-      <c r="J146" t="n">
-        <v>120000</v>
-      </c>
-      <c r="K146" t="inlineStr"/>
     </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>

</xml_diff>

<commit_message>
feat(studio): a 1 m bathroom across the width, door slides inside (D-067)
The founder: the bathroom side 1 m, the shower and WC spread out, and the
slider inside along the partition. The cross wall goes; the shower takes
the back wall, the WC end wall B, and the door opens through the partition
past the galley. The WC front space drops to 430 to the parked leaf, under
the 600 guide; the sofa walkway grows to 778.

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01S6J7HinYQ9w2K8Yf8j6x7D
</commit_message>
<xml_diff>
--- a/public/designs/studio/data/bom.xlsx
+++ b/public/designs/studio/data/bom.xlsx
@@ -491,10 +491,10 @@
         </is>
       </c>
       <c r="B7" t="n">
-        <v>1419940</v>
+        <v>1359940</v>
       </c>
       <c r="C7" t="n">
-        <v>2839880</v>
+        <v>2719880</v>
       </c>
     </row>
     <row r="8">
@@ -517,10 +517,10 @@
         </is>
       </c>
       <c r="B9" t="n">
-        <v>1018150</v>
+        <v>1020800</v>
       </c>
       <c r="C9" t="n">
-        <v>2036300</v>
+        <v>2041600</v>
       </c>
     </row>
     <row r="10">
@@ -569,10 +569,10 @@
         </is>
       </c>
       <c r="B13" t="n">
-        <v>527220</v>
+        <v>525660</v>
       </c>
       <c r="C13" t="n">
-        <v>1054440</v>
+        <v>1051320</v>
       </c>
     </row>
     <row r="14">
@@ -582,10 +582,10 @@
         </is>
       </c>
       <c r="B14" t="n">
-        <v>476750</v>
+        <v>477650</v>
       </c>
       <c r="C14" t="n">
-        <v>953500</v>
+        <v>955300</v>
       </c>
     </row>
     <row r="15">
@@ -595,10 +595,10 @@
         </is>
       </c>
       <c r="B15" t="n">
-        <v>417120</v>
+        <v>436980</v>
       </c>
       <c r="C15" t="n">
-        <v>834240</v>
+        <v>873960</v>
       </c>
     </row>
     <row r="16">
@@ -660,10 +660,10 @@
         </is>
       </c>
       <c r="B20" t="n">
-        <v>104500</v>
+        <v>97900</v>
       </c>
       <c r="C20" t="n">
-        <v>209000</v>
+        <v>195800</v>
       </c>
     </row>
     <row r="21">
@@ -736,10 +736,10 @@
         </is>
       </c>
       <c r="B26" t="n">
-        <v>2150848</v>
+        <v>2144136</v>
       </c>
       <c r="C26" t="n">
-        <v>5030097</v>
+        <v>5016672</v>
       </c>
     </row>
     <row r="27">
@@ -749,10 +749,10 @@
         </is>
       </c>
       <c r="B27" t="n">
-        <v>16489837</v>
+        <v>16438375</v>
       </c>
       <c r="C27" t="n">
-        <v>38564075</v>
+        <v>38461150</v>
       </c>
     </row>
     <row r="29">
@@ -763,7 +763,7 @@
       </c>
       <c r="B29" t="inlineStr"/>
       <c r="C29" t="n">
-        <v>26129</v>
+        <v>26059</v>
       </c>
     </row>
   </sheetData>
@@ -859,7 +859,7 @@
         </is>
       </c>
       <c r="E2" t="n">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="F2" t="inlineStr">
         <is>
@@ -880,7 +880,7 @@
         </is>
       </c>
       <c r="J2" t="n">
-        <v>180000</v>
+        <v>120000</v>
       </c>
       <c r="K2" t="inlineStr">
         <is>
@@ -2196,7 +2196,7 @@
         </is>
       </c>
       <c r="E29" t="n">
-        <v>11.1</v>
+        <v>11.4</v>
       </c>
       <c r="F29" t="inlineStr">
         <is>
@@ -2217,7 +2217,7 @@
         </is>
       </c>
       <c r="J29" t="n">
-        <v>199800</v>
+        <v>205200</v>
       </c>
       <c r="K29" t="inlineStr">
         <is>
@@ -2345,7 +2345,7 @@
       </c>
       <c r="D32" t="inlineStr">
         <is>
-          <t>Sliding door leaf 574 x 2,055, moisture-resistant, flush pulls, privacy hook lock</t>
+          <t>Sliding door leaf 602 x 2,055, moisture-resistant, flush pulls, privacy hook lock</t>
         </is>
       </c>
       <c r="E32" t="n">
@@ -2392,7 +2392,7 @@
       </c>
       <c r="D33" t="inlineStr">
         <is>
-          <t>Surface sliding-door track 1140 mm with soft-close, end stop and floor guide, on the cross wall's lobby face</t>
+          <t>Surface sliding-door track 1184 mm with soft-close, end stop and floor guide, inside the bathroom on the partition</t>
         </is>
       </c>
       <c r="E33" t="n">
@@ -2447,7 +2447,7 @@
         </is>
       </c>
       <c r="E34" t="n">
-        <v>2.66</v>
+        <v>2.39</v>
       </c>
       <c r="F34" t="inlineStr">
         <is>
@@ -2468,7 +2468,7 @@
         </is>
       </c>
       <c r="J34" t="n">
-        <v>37240</v>
+        <v>33460</v>
       </c>
       <c r="K34" t="inlineStr">
         <is>
@@ -2498,7 +2498,7 @@
         </is>
       </c>
       <c r="E35" t="n">
-        <v>2.93</v>
+        <v>2.63</v>
       </c>
       <c r="F35" t="inlineStr">
         <is>
@@ -2519,7 +2519,7 @@
         </is>
       </c>
       <c r="J35" t="n">
-        <v>46880</v>
+        <v>42080</v>
       </c>
       <c r="K35" t="inlineStr">
         <is>
@@ -2549,7 +2549,7 @@
         </is>
       </c>
       <c r="E36" t="n">
-        <v>3.94</v>
+        <v>5.22</v>
       </c>
       <c r="F36" t="inlineStr">
         <is>
@@ -2570,7 +2570,7 @@
         </is>
       </c>
       <c r="J36" t="n">
-        <v>55160</v>
+        <v>73080</v>
       </c>
       <c r="K36" t="inlineStr">
         <is>
@@ -2600,7 +2600,7 @@
         </is>
       </c>
       <c r="E37" t="n">
-        <v>4.33</v>
+        <v>5.74</v>
       </c>
       <c r="F37" t="inlineStr">
         <is>
@@ -2621,7 +2621,7 @@
         </is>
       </c>
       <c r="J37" t="n">
-        <v>69280</v>
+        <v>91840</v>
       </c>
       <c r="K37" t="inlineStr">
         <is>
@@ -2651,7 +2651,7 @@
         </is>
       </c>
       <c r="E38" t="n">
-        <v>3.94</v>
+        <v>3.83</v>
       </c>
       <c r="F38" t="inlineStr">
         <is>
@@ -2672,7 +2672,7 @@
         </is>
       </c>
       <c r="J38" t="n">
-        <v>55160</v>
+        <v>53620</v>
       </c>
       <c r="K38" t="inlineStr">
         <is>
@@ -2702,7 +2702,7 @@
         </is>
       </c>
       <c r="E39" t="n">
-        <v>4.33</v>
+        <v>4.21</v>
       </c>
       <c r="F39" t="inlineStr">
         <is>
@@ -2723,7 +2723,7 @@
         </is>
       </c>
       <c r="J39" t="n">
-        <v>69280</v>
+        <v>67360</v>
       </c>
       <c r="K39" t="inlineStr">
         <is>
@@ -2749,11 +2749,11 @@
       </c>
       <c r="D40" t="inlineStr">
         <is>
-          <t>Cement board 12 mm + liquid membrane, cross wall, bath face</t>
+          <t>Cement board 12 mm + liquid membrane, front wall around W1</t>
         </is>
       </c>
       <c r="E40" t="n">
-        <v>2.66</v>
+        <v>2.39</v>
       </c>
       <c r="F40" t="inlineStr">
         <is>
@@ -2774,7 +2774,7 @@
         </is>
       </c>
       <c r="J40" t="n">
-        <v>37240</v>
+        <v>33460</v>
       </c>
       <c r="K40" t="inlineStr">
         <is>
@@ -2800,11 +2800,11 @@
       </c>
       <c r="D41" t="inlineStr">
         <is>
-          <t>Wall tiles + adhesive + grout, cross wall, bath face</t>
+          <t>Wall tiles + adhesive + grout, front wall around W1</t>
         </is>
       </c>
       <c r="E41" t="n">
-        <v>2.93</v>
+        <v>2.63</v>
       </c>
       <c r="F41" t="inlineStr">
         <is>
@@ -2825,7 +2825,7 @@
         </is>
       </c>
       <c r="J41" t="n">
-        <v>46880</v>
+        <v>42080</v>
       </c>
       <c r="K41" t="inlineStr">
         <is>
@@ -2851,11 +2851,11 @@
       </c>
       <c r="D42" t="inlineStr">
         <is>
-          <t>Safety vinyl sheet, coved 100 mm up the walls (bathroom and lobby)</t>
+          <t>Safety vinyl sheet, coved 100 mm up the walls (bathroom)</t>
         </is>
       </c>
       <c r="E42" t="n">
-        <v>3.2</v>
+        <v>2.9</v>
       </c>
       <c r="F42" t="inlineStr">
         <is>
@@ -2876,7 +2876,7 @@
         </is>
       </c>
       <c r="J42" t="n">
-        <v>48000</v>
+        <v>43500</v>
       </c>
       <c r="K42" t="inlineStr">
         <is>
@@ -2949,7 +2949,7 @@
       </c>
       <c r="D44" t="inlineStr">
         <is>
-          <t>Fixed glass shower screen 700 x 2,000, 8 mm toughened</t>
+          <t>Fixed glass shower screen 520 x 2,000, 8 mm toughened</t>
         </is>
       </c>
       <c r="E44" t="n">
@@ -4407,7 +4407,7 @@
       </c>
       <c r="D74" t="inlineStr">
         <is>
-          <t>Bathroom light + fan (outside, by the door)</t>
+          <t>Bathroom light + fan (inside, by the door)</t>
         </is>
       </c>
       <c r="E74" t="n">
@@ -5528,7 +5528,7 @@
         </is>
       </c>
       <c r="E97" t="n">
-        <v>31</v>
+        <v>36</v>
       </c>
       <c r="F97" t="inlineStr">
         <is>
@@ -5549,7 +5549,7 @@
         </is>
       </c>
       <c r="J97" t="n">
-        <v>15500</v>
+        <v>18000</v>
       </c>
       <c r="K97" t="inlineStr">
         <is>
@@ -5834,7 +5834,7 @@
         </is>
       </c>
       <c r="E103" t="n">
-        <v>5</v>
+        <v>6</v>
       </c>
       <c r="F103" t="inlineStr">
         <is>
@@ -5855,7 +5855,7 @@
         </is>
       </c>
       <c r="J103" t="n">
-        <v>3750</v>
+        <v>4500</v>
       </c>
       <c r="K103" t="inlineStr">
         <is>
@@ -5987,7 +5987,7 @@
         </is>
       </c>
       <c r="E106" t="n">
-        <v>53</v>
+        <v>52</v>
       </c>
       <c r="F106" t="inlineStr">
         <is>
@@ -6008,7 +6008,7 @@
         </is>
       </c>
       <c r="J106" t="n">
-        <v>31800</v>
+        <v>31200</v>
       </c>
       <c r="K106" t="inlineStr">
         <is>
@@ -6387,7 +6387,7 @@
         </is>
       </c>
       <c r="E114" t="n">
-        <v>8.199999999999999</v>
+        <v>8</v>
       </c>
       <c r="F114" t="inlineStr">
         <is>
@@ -6408,7 +6408,7 @@
         </is>
       </c>
       <c r="J114" t="n">
-        <v>16400</v>
+        <v>16000</v>
       </c>
       <c r="K114" t="inlineStr">
         <is>
@@ -6438,7 +6438,7 @@
         </is>
       </c>
       <c r="E115" t="n">
-        <v>4.4</v>
+        <v>4.2</v>
       </c>
       <c r="F115" t="inlineStr">
         <is>
@@ -6459,7 +6459,7 @@
         </is>
       </c>
       <c r="J115" t="n">
-        <v>12320</v>
+        <v>11760</v>
       </c>
       <c r="K115" t="inlineStr">
         <is>
@@ -6591,7 +6591,7 @@
         </is>
       </c>
       <c r="E118" t="n">
-        <v>6.3</v>
+        <v>6.1</v>
       </c>
       <c r="F118" t="inlineStr">
         <is>
@@ -6612,7 +6612,7 @@
         </is>
       </c>
       <c r="J118" t="n">
-        <v>18900</v>
+        <v>18300</v>
       </c>
       <c r="K118" t="inlineStr">
         <is>
@@ -6975,7 +6975,7 @@
       </c>
       <c r="D126" t="inlineStr">
         <is>
-          <t>W1 obscure louvre window 520 x 890 + insect mesh (bathroom lobby)</t>
+          <t>W1 obscure louvre window 520 x 890 + insect mesh (bathroom)</t>
         </is>
       </c>
       <c r="E126" t="n">
@@ -7453,7 +7453,7 @@
         </is>
       </c>
       <c r="E136" t="n">
-        <v>5.5</v>
+        <v>3.3</v>
       </c>
       <c r="F136" t="inlineStr">
         <is>
@@ -7474,7 +7474,7 @@
         </is>
       </c>
       <c r="J136" t="n">
-        <v>16500</v>
+        <v>9900</v>
       </c>
       <c r="K136" t="inlineStr">
         <is>

</xml_diff>